<commit_message>
Smartbank o'rniga Openbank (2025-yilda nomi o'zgargan), sayti openbank.uz
- banks.json: openbank, https://openbank.uz; bo'limlar: /mortgage, /installment, /faq
- Qo'lda tekshirilgan qator, izoh va saytdan o'qilgan ma'lumotda nom yangilandi
- O'zbekistondan o'qiladigan banklar ro'yxatida ham openbank

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WBEE3seDEXSJoGf4V5Zkid
</commit_message>
<xml_diff>
--- a/docs/banklar_kreditlar.xlsx
+++ b/docs/banklar_kreditlar.xlsx
@@ -1643,7 +1643,7 @@
     <row r="54">
       <c r="A54" s="3" t="inlineStr">
         <is>
-          <t>Smartbank</t>
+          <t>Openbank</t>
         </is>
       </c>
       <c r="B54" s="3" t="inlineStr">
@@ -1660,7 +1660,7 @@
       <c r="E54" s="3" t="inlineStr"/>
       <c r="F54" s="6" t="inlineStr">
         <is>
-          <t>https://smartbank.uz/useful/faq</t>
+          <t>https://openbank.uz/faq</t>
         </is>
       </c>
     </row>
@@ -20616,7 +20616,7 @@
     <row r="319">
       <c r="A319" s="3" t="inlineStr">
         <is>
-          <t>Orient Finans Bank</t>
+          <t>Openbank</t>
         </is>
       </c>
       <c r="B319" s="3" t="inlineStr">
@@ -20626,31 +20626,23 @@
       </c>
       <c r="C319" s="3" t="inlineStr">
         <is>
-          <t>Avtokredit</t>
+          <t>Iste'mol</t>
         </is>
       </c>
       <c r="D319" s="3" t="inlineStr">
         <is>
-          <t>Avtokredit Ikkilamchi bozorga</t>
+          <t>Kredit</t>
         </is>
       </c>
       <c r="E319" s="3" t="n">
-        <v>24.9</v>
+        <v>24.99</v>
       </c>
       <c r="F319" s="3" t="n">
-        <v>24.9</v>
+        <v>25.99</v>
       </c>
       <c r="G319" s="3" t="inlineStr"/>
-      <c r="H319" s="3" t="inlineStr">
-        <is>
-          <t>4 yilgacha</t>
-        </is>
-      </c>
-      <c r="I319" s="3" t="inlineStr">
-        <is>
-          <t>800 mln gacha</t>
-        </is>
-      </c>
+      <c r="H319" s="3" t="inlineStr"/>
+      <c r="I319" s="3" t="inlineStr"/>
       <c r="J319" s="3" t="inlineStr">
         <is>
           <t>UZS</t>
@@ -20658,18 +20650,18 @@
       </c>
       <c r="K319" s="3" t="inlineStr">
         <is>
-          <t>Saytdan avtomatik</t>
-        </is>
-      </c>
-      <c r="L319" s="3" t="inlineStr">
-        <is>
-          <t>2026-10-15</t>
-        </is>
-      </c>
-      <c r="M319" s="3" t="inlineStr"/>
+          <t>Qo'lda tekshirilgan</t>
+        </is>
+      </c>
+      <c r="L319" s="3" t="inlineStr"/>
+      <c r="M319" s="3" t="inlineStr">
+        <is>
+          <t>Rasmiy daromadli 24.99%, o'zini band qilganlar 25.99%</t>
+        </is>
+      </c>
       <c r="N319" s="6" t="inlineStr">
         <is>
-          <t>https://ofb.uz/kreditlar/ikkilamchi-bozor-uchun-avtokredit</t>
+          <t>https://openbank.uz/faq</t>
         </is>
       </c>
     </row>
@@ -20691,19 +20683,19 @@
       </c>
       <c r="D320" s="3" t="inlineStr">
         <is>
-          <t>Avtokredit Import</t>
+          <t>Avtokredit Ikkilamchi bozorga</t>
         </is>
       </c>
       <c r="E320" s="3" t="n">
-        <v>22.9</v>
+        <v>24.9</v>
       </c>
       <c r="F320" s="3" t="n">
-        <v>22.9</v>
+        <v>24.9</v>
       </c>
       <c r="G320" s="3" t="inlineStr"/>
       <c r="H320" s="3" t="inlineStr">
         <is>
-          <t>5 yilgacha</t>
+          <t>4 yilgacha</t>
         </is>
       </c>
       <c r="I320" s="3" t="inlineStr">
@@ -20729,7 +20721,7 @@
       <c r="M320" s="3" t="inlineStr"/>
       <c r="N320" s="6" t="inlineStr">
         <is>
-          <t>https://ofb.uz/kreditlar/import-avtokredit</t>
+          <t>https://ofb.uz/kreditlar/ikkilamchi-bozor-uchun-avtokredit</t>
         </is>
       </c>
     </row>
@@ -20751,19 +20743,19 @@
       </c>
       <c r="D321" s="3" t="inlineStr">
         <is>
-          <t>Avtokredit Foydali</t>
+          <t>Avtokredit Import</t>
         </is>
       </c>
       <c r="E321" s="3" t="n">
-        <v>22</v>
+        <v>22.9</v>
       </c>
       <c r="F321" s="3" t="n">
-        <v>22</v>
+        <v>22.9</v>
       </c>
       <c r="G321" s="3" t="inlineStr"/>
       <c r="H321" s="3" t="inlineStr">
         <is>
-          <t>1 yilgacha</t>
+          <t>5 yilgacha</t>
         </is>
       </c>
       <c r="I321" s="3" t="inlineStr">
@@ -20789,7 +20781,7 @@
       <c r="M321" s="3" t="inlineStr"/>
       <c r="N321" s="6" t="inlineStr">
         <is>
-          <t>https://ofb.uz/kreditlar/avtokredit-foydali</t>
+          <t>https://ofb.uz/kreditlar/import-avtokredit</t>
         </is>
       </c>
     </row>
@@ -20811,19 +20803,19 @@
       </c>
       <c r="D322" s="3" t="inlineStr">
         <is>
-          <t>Oson avtokredit</t>
+          <t>Avtokredit Foydali</t>
         </is>
       </c>
       <c r="E322" s="3" t="n">
-        <v>21.9</v>
+        <v>22</v>
       </c>
       <c r="F322" s="3" t="n">
-        <v>21.9</v>
+        <v>22</v>
       </c>
       <c r="G322" s="3" t="inlineStr"/>
       <c r="H322" s="3" t="inlineStr">
         <is>
-          <t>5 yilgacha</t>
+          <t>1 yilgacha</t>
         </is>
       </c>
       <c r="I322" s="3" t="inlineStr">
@@ -20849,7 +20841,7 @@
       <c r="M322" s="3" t="inlineStr"/>
       <c r="N322" s="6" t="inlineStr">
         <is>
-          <t>https://ofb.uz/kreditlar/oson-avtokredit</t>
+          <t>https://ofb.uz/kreditlar/avtokredit-foydali</t>
         </is>
       </c>
     </row>
@@ -20871,21 +20863,19 @@
       </c>
       <c r="D323" s="3" t="inlineStr">
         <is>
-          <t>Byudjet tashkilotlari xodimlari uchun</t>
+          <t>Oson avtokredit</t>
         </is>
       </c>
       <c r="E323" s="3" t="n">
-        <v>20.9</v>
-      </c>
-      <c r="F323" s="3" t="n"/>
-      <c r="G323" s="3" t="inlineStr">
-        <is>
-          <t>20.9</t>
-        </is>
-      </c>
+        <v>21.9</v>
+      </c>
+      <c r="F323" s="3" t="n">
+        <v>21.9</v>
+      </c>
+      <c r="G323" s="3" t="inlineStr"/>
       <c r="H323" s="3" t="inlineStr">
         <is>
-          <t>60 oygacha</t>
+          <t>5 yilgacha</t>
         </is>
       </c>
       <c r="I323" s="3" t="inlineStr">
@@ -20900,18 +20890,18 @@
       </c>
       <c r="K323" s="3" t="inlineStr">
         <is>
-          <t>Qo'lda tekshirilgan</t>
-        </is>
-      </c>
-      <c r="L323" s="3" t="inlineStr"/>
-      <c r="M323" s="3" t="inlineStr">
-        <is>
-          <t>Boshlang'ich badalga qarab pasayadi</t>
-        </is>
-      </c>
+          <t>Saytdan avtomatik</t>
+        </is>
+      </c>
+      <c r="L323" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="M323" s="3" t="inlineStr"/>
       <c r="N323" s="6" t="inlineStr">
         <is>
-          <t>https://ofb.uz/kreditlar/byudjet-tashkilotlari-xodimlari-uchun-avtokredit</t>
+          <t>https://ofb.uz/kreditlar/oson-avtokredit</t>
         </is>
       </c>
     </row>
@@ -20933,17 +20923,21 @@
       </c>
       <c r="D324" s="3" t="inlineStr">
         <is>
-          <t>BYD Special Plus</t>
+          <t>Byudjet tashkilotlari xodimlari uchun</t>
         </is>
       </c>
       <c r="E324" s="3" t="n">
-        <v>12.5</v>
+        <v>20.9</v>
       </c>
       <c r="F324" s="3" t="n"/>
-      <c r="G324" s="3" t="inlineStr"/>
+      <c r="G324" s="3" t="inlineStr">
+        <is>
+          <t>20.9</t>
+        </is>
+      </c>
       <c r="H324" s="3" t="inlineStr">
         <is>
-          <t>36 / 60 oy</t>
+          <t>60 oygacha</t>
         </is>
       </c>
       <c r="I324" s="3" t="inlineStr">
@@ -20964,12 +20958,12 @@
       <c r="L324" s="3" t="inlineStr"/>
       <c r="M324" s="3" t="inlineStr">
         <is>
-          <t>Yangi BYD avtomobillari</t>
+          <t>Boshlang'ich badalga qarab pasayadi</t>
         </is>
       </c>
       <c r="N324" s="6" t="inlineStr">
         <is>
-          <t>https://ofb.uz/kreditlar/byd-special-plus</t>
+          <t>https://ofb.uz/kreditlar/byudjet-tashkilotlari-xodimlari-uchun-avtokredit</t>
         </is>
       </c>
     </row>
@@ -20986,29 +20980,27 @@
       </c>
       <c r="C325" s="3" t="inlineStr">
         <is>
-          <t>Biznes</t>
+          <t>Avtokredit</t>
         </is>
       </c>
       <c r="D325" s="3" t="inlineStr">
         <is>
-          <t>OFB Start</t>
+          <t>BYD Special Plus</t>
         </is>
       </c>
       <c r="E325" s="3" t="n">
-        <v>25</v>
-      </c>
-      <c r="F325" s="3" t="n">
-        <v>28</v>
-      </c>
+        <v>12.5</v>
+      </c>
+      <c r="F325" s="3" t="n"/>
       <c r="G325" s="3" t="inlineStr"/>
       <c r="H325" s="3" t="inlineStr">
         <is>
-          <t>3 oy – 3 yil</t>
+          <t>36 / 60 oy</t>
         </is>
       </c>
       <c r="I325" s="3" t="inlineStr">
         <is>
-          <t>5.33715 mln – 1 mlrd</t>
+          <t>800 mln gacha</t>
         </is>
       </c>
       <c r="J325" s="3" t="inlineStr">
@@ -21018,18 +21010,18 @@
       </c>
       <c r="K325" s="3" t="inlineStr">
         <is>
-          <t>Saytdan avtomatik</t>
-        </is>
-      </c>
-      <c r="L325" s="3" t="inlineStr">
-        <is>
-          <t>2026-10-15</t>
-        </is>
-      </c>
-      <c r="M325" s="3" t="inlineStr"/>
+          <t>Qo'lda tekshirilgan</t>
+        </is>
+      </c>
+      <c r="L325" s="3" t="inlineStr"/>
+      <c r="M325" s="3" t="inlineStr">
+        <is>
+          <t>Yangi BYD avtomobillari</t>
+        </is>
+      </c>
       <c r="N325" s="6" t="inlineStr">
         <is>
-          <t>https://ofb.uz/biznes/kreditlar/ofb-start</t>
+          <t>https://ofb.uz/kreditlar/byd-special-plus</t>
         </is>
       </c>
     </row>
@@ -21051,11 +21043,11 @@
       </c>
       <c r="D326" s="3" t="inlineStr">
         <is>
-          <t>OFB Ishonchli</t>
+          <t>OFB Start</t>
         </is>
       </c>
       <c r="E326" s="3" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F326" s="3" t="n">
         <v>28</v>
@@ -21063,12 +21055,12 @@
       <c r="G326" s="3" t="inlineStr"/>
       <c r="H326" s="3" t="inlineStr">
         <is>
-          <t>2 oy – 2 yil</t>
+          <t>3 oy – 3 yil</t>
         </is>
       </c>
       <c r="I326" s="3" t="inlineStr">
         <is>
-          <t>18.0539 mln – 2 mlrd</t>
+          <t>5.33715 mln – 1 mlrd</t>
         </is>
       </c>
       <c r="J326" s="3" t="inlineStr">
@@ -21089,7 +21081,7 @@
       <c r="M326" s="3" t="inlineStr"/>
       <c r="N326" s="6" t="inlineStr">
         <is>
-          <t>https://ofb.uz/biznes/kreditlar/ofb-ishonchli</t>
+          <t>https://ofb.uz/biznes/kreditlar/ofb-start</t>
         </is>
       </c>
     </row>
@@ -21111,14 +21103,14 @@
       </c>
       <c r="D327" s="3" t="inlineStr">
         <is>
-          <t>OFB Cash</t>
+          <t>OFB Ishonchli</t>
         </is>
       </c>
       <c r="E327" s="3" t="n">
         <v>26</v>
       </c>
       <c r="F327" s="3" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="G327" s="3" t="inlineStr"/>
       <c r="H327" s="3" t="inlineStr">
@@ -21128,7 +21120,7 @@
       </c>
       <c r="I327" s="3" t="inlineStr">
         <is>
-          <t>17.9531 mln – 1 mlrd</t>
+          <t>18.0539 mln – 2 mlrd</t>
         </is>
       </c>
       <c r="J327" s="3" t="inlineStr">
@@ -21149,7 +21141,7 @@
       <c r="M327" s="3" t="inlineStr"/>
       <c r="N327" s="6" t="inlineStr">
         <is>
-          <t>https://ofb.uz/biznes/kreditlar/ofb-cash</t>
+          <t>https://ofb.uz/biznes/kreditlar/ofb-ishonchli</t>
         </is>
       </c>
     </row>
@@ -21171,11 +21163,11 @@
       </c>
       <c r="D328" s="3" t="inlineStr">
         <is>
-          <t>OFB Kapital</t>
+          <t>OFB Cash</t>
         </is>
       </c>
       <c r="E328" s="3" t="n">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="F328" s="3" t="n">
         <v>26</v>
@@ -21183,12 +21175,12 @@
       <c r="G328" s="3" t="inlineStr"/>
       <c r="H328" s="3" t="inlineStr">
         <is>
-          <t>3 oy – 3 yil</t>
+          <t>2 oy – 2 yil</t>
         </is>
       </c>
       <c r="I328" s="3" t="inlineStr">
         <is>
-          <t>9.55301 mln – 3 mlrd</t>
+          <t>17.9531 mln – 1 mlrd</t>
         </is>
       </c>
       <c r="J328" s="3" t="inlineStr">
@@ -21209,7 +21201,7 @@
       <c r="M328" s="3" t="inlineStr"/>
       <c r="N328" s="6" t="inlineStr">
         <is>
-          <t>https://ofb.uz/biznes/kreditlar/ofb-kapital</t>
+          <t>https://ofb.uz/biznes/kreditlar/ofb-cash</t>
         </is>
       </c>
     </row>
@@ -21231,14 +21223,14 @@
       </c>
       <c r="D329" s="3" t="inlineStr">
         <is>
-          <t>OFB Garant</t>
+          <t>OFB Kapital</t>
         </is>
       </c>
       <c r="E329" s="3" t="n">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="F329" s="3" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G329" s="3" t="inlineStr"/>
       <c r="H329" s="3" t="inlineStr">
@@ -21248,7 +21240,7 @@
       </c>
       <c r="I329" s="3" t="inlineStr">
         <is>
-          <t>93.75 ming – 5 mln</t>
+          <t>9.55301 mln – 3 mlrd</t>
         </is>
       </c>
       <c r="J329" s="3" t="inlineStr">
@@ -21269,7 +21261,7 @@
       <c r="M329" s="3" t="inlineStr"/>
       <c r="N329" s="6" t="inlineStr">
         <is>
-          <t>https://ofb.uz/biznes/kreditlar/ofb-garant</t>
+          <t>https://ofb.uz/biznes/kreditlar/ofb-kapital</t>
         </is>
       </c>
     </row>
@@ -21291,24 +21283,24 @@
       </c>
       <c r="D330" s="3" t="inlineStr">
         <is>
-          <t>OFB Kelajak</t>
+          <t>OFB Garant</t>
         </is>
       </c>
       <c r="E330" s="3" t="n">
-        <v>12.5</v>
+        <v>25</v>
       </c>
       <c r="F330" s="3" t="n">
-        <v>12.5</v>
+        <v>25</v>
       </c>
       <c r="G330" s="3" t="inlineStr"/>
       <c r="H330" s="3" t="inlineStr">
         <is>
-          <t>2 oy – 2 yil</t>
+          <t>3 oy – 3 yil</t>
         </is>
       </c>
       <c r="I330" s="3" t="inlineStr">
         <is>
-          <t>259.193 ming – 1.64891 mln</t>
+          <t>93.75 ming – 5 mln</t>
         </is>
       </c>
       <c r="J330" s="3" t="inlineStr">
@@ -21329,7 +21321,7 @@
       <c r="M330" s="3" t="inlineStr"/>
       <c r="N330" s="6" t="inlineStr">
         <is>
-          <t>https://ofb.uz/biznes/kreditlar/ofb-kelajak</t>
+          <t>https://ofb.uz/biznes/kreditlar/ofb-garant</t>
         </is>
       </c>
     </row>
@@ -21346,29 +21338,29 @@
       </c>
       <c r="C331" s="3" t="inlineStr">
         <is>
-          <t>Ipoteka</t>
+          <t>Biznes</t>
         </is>
       </c>
       <c r="D331" s="3" t="inlineStr">
         <is>
-          <t>Foydali ipoteka</t>
+          <t>OFB Kelajak</t>
         </is>
       </c>
       <c r="E331" s="3" t="n">
-        <v>16</v>
+        <v>12.5</v>
       </c>
       <c r="F331" s="3" t="n">
-        <v>25</v>
+        <v>12.5</v>
       </c>
       <c r="G331" s="3" t="inlineStr"/>
       <c r="H331" s="3" t="inlineStr">
         <is>
-          <t>6 oy – 20 yil</t>
+          <t>2 oy – 2 yil</t>
         </is>
       </c>
       <c r="I331" s="3" t="inlineStr">
         <is>
-          <t>7.82892 mln – 1.06 mlrd</t>
+          <t>259.193 ming – 1.64891 mln</t>
         </is>
       </c>
       <c r="J331" s="3" t="inlineStr">
@@ -21389,7 +21381,7 @@
       <c r="M331" s="3" t="inlineStr"/>
       <c r="N331" s="6" t="inlineStr">
         <is>
-          <t>https://ofb.uz/kreditlar/foydali-ipoteka</t>
+          <t>https://ofb.uz/biznes/kreditlar/ofb-kelajak</t>
         </is>
       </c>
     </row>
@@ -21411,24 +21403,24 @@
       </c>
       <c r="D332" s="3" t="inlineStr">
         <is>
-          <t>Uy-joy ta'miri uchun ipoteka</t>
+          <t>Foydali ipoteka</t>
         </is>
       </c>
       <c r="E332" s="3" t="n">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="F332" s="3" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="G332" s="3" t="inlineStr"/>
       <c r="H332" s="3" t="inlineStr">
         <is>
-          <t>10 yilgacha</t>
+          <t>6 oy – 20 yil</t>
         </is>
       </c>
       <c r="I332" s="3" t="inlineStr">
         <is>
-          <t>400 mln gacha</t>
+          <t>7.82892 mln – 1.06 mlrd</t>
         </is>
       </c>
       <c r="J332" s="3" t="inlineStr">
@@ -21438,14 +21430,18 @@
       </c>
       <c r="K332" s="3" t="inlineStr">
         <is>
-          <t>Qo'lda tekshirilgan</t>
-        </is>
-      </c>
-      <c r="L332" s="3" t="inlineStr"/>
+          <t>Saytdan avtomatik</t>
+        </is>
+      </c>
+      <c r="L332" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
       <c r="M332" s="3" t="inlineStr"/>
       <c r="N332" s="6" t="inlineStr">
         <is>
-          <t>https://ofb.uz/kreditlar/tamirlash-uchun-ipoteka-krediti</t>
+          <t>https://ofb.uz/kreditlar/foydali-ipoteka</t>
         </is>
       </c>
     </row>
@@ -21467,7 +21463,7 @@
       </c>
       <c r="D333" s="3" t="inlineStr">
         <is>
-          <t>Ta’mirlash uchun ipoteka krediti</t>
+          <t>Uy-joy ta'miri uchun ipoteka</t>
         </is>
       </c>
       <c r="E333" s="3" t="n">
@@ -21494,14 +21490,10 @@
       </c>
       <c r="K333" s="3" t="inlineStr">
         <is>
-          <t>Saytdan avtomatik</t>
-        </is>
-      </c>
-      <c r="L333" s="3" t="inlineStr">
-        <is>
-          <t>2026-10-15</t>
-        </is>
-      </c>
+          <t>Qo'lda tekshirilgan</t>
+        </is>
+      </c>
+      <c r="L333" s="3" t="inlineStr"/>
       <c r="M333" s="3" t="inlineStr"/>
       <c r="N333" s="6" t="inlineStr">
         <is>
@@ -21527,7 +21519,7 @@
       </c>
       <c r="D334" s="3" t="inlineStr">
         <is>
-          <t>Yashil ipoteka</t>
+          <t>Ta’mirlash uchun ipoteka krediti</t>
         </is>
       </c>
       <c r="E334" s="3" t="n">
@@ -21539,12 +21531,12 @@
       <c r="G334" s="3" t="inlineStr"/>
       <c r="H334" s="3" t="inlineStr">
         <is>
-          <t>7 yilgacha</t>
+          <t>10 yilgacha</t>
         </is>
       </c>
       <c r="I334" s="3" t="inlineStr">
         <is>
-          <t>350 mln gacha</t>
+          <t>400 mln gacha</t>
         </is>
       </c>
       <c r="J334" s="3" t="inlineStr">
@@ -21565,7 +21557,7 @@
       <c r="M334" s="3" t="inlineStr"/>
       <c r="N334" s="6" t="inlineStr">
         <is>
-          <t>https://ofb.uz/kreditlar/yashil-ipoteka</t>
+          <t>https://ofb.uz/kreditlar/tamirlash-uchun-ipoteka-krediti</t>
         </is>
       </c>
     </row>
@@ -21587,24 +21579,24 @@
       </c>
       <c r="D335" s="3" t="inlineStr">
         <is>
-          <t>Navro‘z ipoteka krediti</t>
+          <t>Yashil ipoteka</t>
         </is>
       </c>
       <c r="E335" s="3" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="F335" s="3" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="G335" s="3" t="inlineStr"/>
       <c r="H335" s="3" t="inlineStr">
         <is>
-          <t>20 yilgacha</t>
+          <t>7 yilgacha</t>
         </is>
       </c>
       <c r="I335" s="3" t="inlineStr">
         <is>
-          <t>1.06 mlrd gacha</t>
+          <t>350 mln gacha</t>
         </is>
       </c>
       <c r="J335" s="3" t="inlineStr">
@@ -21625,7 +21617,7 @@
       <c r="M335" s="3" t="inlineStr"/>
       <c r="N335" s="6" t="inlineStr">
         <is>
-          <t>https://ofb.uz/kreditlar/navroz-ipoteka-krediti</t>
+          <t>https://ofb.uz/kreditlar/yashil-ipoteka</t>
         </is>
       </c>
     </row>
@@ -21647,14 +21639,14 @@
       </c>
       <c r="D336" s="3" t="inlineStr">
         <is>
-          <t>Birlamchi bozor uchun ipoteka 2.0</t>
+          <t>Navro‘z ipoteka krediti</t>
         </is>
       </c>
       <c r="E336" s="3" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="F336" s="3" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="G336" s="3" t="inlineStr"/>
       <c r="H336" s="3" t="inlineStr">
@@ -21664,7 +21656,7 @@
       </c>
       <c r="I336" s="3" t="inlineStr">
         <is>
-          <t>800 mln gacha</t>
+          <t>1.06 mlrd gacha</t>
         </is>
       </c>
       <c r="J336" s="3" t="inlineStr">
@@ -21685,7 +21677,7 @@
       <c r="M336" s="3" t="inlineStr"/>
       <c r="N336" s="6" t="inlineStr">
         <is>
-          <t>https://ofb.uz/kreditlar/birlamchi-bozor-uchun-2-0</t>
+          <t>https://ofb.uz/kreditlar/navroz-ipoteka-krediti</t>
         </is>
       </c>
     </row>
@@ -21707,24 +21699,24 @@
       </c>
       <c r="D337" s="3" t="inlineStr">
         <is>
-          <t>Ipoteka O‘qituvchi</t>
+          <t>Birlamchi bozor uchun ipoteka 2.0</t>
         </is>
       </c>
       <c r="E337" s="3" t="n">
-        <v>16.7</v>
+        <v>19</v>
       </c>
       <c r="F337" s="3" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="G337" s="3" t="inlineStr"/>
       <c r="H337" s="3" t="inlineStr">
         <is>
-          <t>6 oy – 20 yil</t>
+          <t>20 yilgacha</t>
         </is>
       </c>
       <c r="I337" s="3" t="inlineStr">
         <is>
-          <t>8.26814 mln – 496.088 mln</t>
+          <t>800 mln gacha</t>
         </is>
       </c>
       <c r="J337" s="3" t="inlineStr">
@@ -21745,7 +21737,7 @@
       <c r="M337" s="3" t="inlineStr"/>
       <c r="N337" s="6" t="inlineStr">
         <is>
-          <t>https://ofb.uz/kreditlar/ipoteka-oqituvchi</t>
+          <t>https://ofb.uz/kreditlar/birlamchi-bozor-uchun-2-0</t>
         </is>
       </c>
     </row>
@@ -21767,14 +21759,14 @@
       </c>
       <c r="D338" s="3" t="inlineStr">
         <is>
-          <t>Oilaviy ipoteka</t>
+          <t>Ipoteka O‘qituvchi</t>
         </is>
       </c>
       <c r="E338" s="3" t="n">
         <v>16.7</v>
       </c>
       <c r="F338" s="3" t="n">
-        <v>16.7</v>
+        <v>17</v>
       </c>
       <c r="G338" s="3" t="inlineStr"/>
       <c r="H338" s="3" t="inlineStr">
@@ -21805,7 +21797,7 @@
       <c r="M338" s="3" t="inlineStr"/>
       <c r="N338" s="6" t="inlineStr">
         <is>
-          <t>https://ofb.uz/kreditlar/oilaviy-ipoteka</t>
+          <t>https://ofb.uz/kreditlar/ipoteka-oqituvchi</t>
         </is>
       </c>
     </row>
@@ -21822,29 +21814,29 @@
       </c>
       <c r="C339" s="3" t="inlineStr">
         <is>
-          <t>Iste'mol</t>
+          <t>Ipoteka</t>
         </is>
       </c>
       <c r="D339" s="3" t="inlineStr">
         <is>
-          <t>Corporate Plus</t>
+          <t>Oilaviy ipoteka</t>
         </is>
       </c>
       <c r="E339" s="3" t="n">
-        <v>25</v>
+        <v>16.7</v>
       </c>
       <c r="F339" s="3" t="n">
-        <v>25</v>
+        <v>16.7</v>
       </c>
       <c r="G339" s="3" t="inlineStr"/>
       <c r="H339" s="3" t="inlineStr">
         <is>
-          <t>3 yilgacha</t>
+          <t>6 oy – 20 yil</t>
         </is>
       </c>
       <c r="I339" s="3" t="inlineStr">
         <is>
-          <t>100 mln gacha</t>
+          <t>8.26814 mln – 496.088 mln</t>
         </is>
       </c>
       <c r="J339" s="3" t="inlineStr">
@@ -21865,7 +21857,7 @@
       <c r="M339" s="3" t="inlineStr"/>
       <c r="N339" s="6" t="inlineStr">
         <is>
-          <t>https://ofb.uz/kreditlar/corporate-plus</t>
+          <t>https://ofb.uz/kreditlar/oilaviy-ipoteka</t>
         </is>
       </c>
     </row>
@@ -21887,20 +21879,24 @@
       </c>
       <c r="D340" s="3" t="inlineStr">
         <is>
-          <t>Qulay qayta moliyalashtirish</t>
+          <t>Corporate Plus</t>
         </is>
       </c>
       <c r="E340" s="3" t="n">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="F340" s="3" t="n">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="G340" s="3" t="inlineStr"/>
-      <c r="H340" s="3" t="inlineStr"/>
+      <c r="H340" s="3" t="inlineStr">
+        <is>
+          <t>3 yilgacha</t>
+        </is>
+      </c>
       <c r="I340" s="3" t="inlineStr">
         <is>
-          <t>1.72392 mln – 1 mlrd</t>
+          <t>100 mln gacha</t>
         </is>
       </c>
       <c r="J340" s="3" t="inlineStr">
@@ -21921,7 +21917,7 @@
       <c r="M340" s="3" t="inlineStr"/>
       <c r="N340" s="6" t="inlineStr">
         <is>
-          <t>https://ofb.uz/kreditlar/qulay-qayta-moliyalashtirish</t>
+          <t>https://ofb.uz/kreditlar/corporate-plus</t>
         </is>
       </c>
     </row>
@@ -21943,20 +21939,20 @@
       </c>
       <c r="D341" s="3" t="inlineStr">
         <is>
-          <t>Bashkent</t>
+          <t>Qulay qayta moliyalashtirish</t>
         </is>
       </c>
       <c r="E341" s="3" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F341" s="3" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G341" s="3" t="inlineStr"/>
       <c r="H341" s="3" t="inlineStr"/>
       <c r="I341" s="3" t="inlineStr">
         <is>
-          <t>1.06 mlrd gacha</t>
+          <t>1.72392 mln – 1 mlrd</t>
         </is>
       </c>
       <c r="J341" s="3" t="inlineStr">
@@ -21977,7 +21973,7 @@
       <c r="M341" s="3" t="inlineStr"/>
       <c r="N341" s="6" t="inlineStr">
         <is>
-          <t>https://ofb.uz/kreditlar/bashkent</t>
+          <t>https://ofb.uz/kreditlar/qulay-qayta-moliyalashtirish</t>
         </is>
       </c>
     </row>
@@ -21994,29 +21990,25 @@
       </c>
       <c r="C342" s="3" t="inlineStr">
         <is>
-          <t>Kredit karta</t>
+          <t>Iste'mol</t>
         </is>
       </c>
       <c r="D342" s="3" t="inlineStr">
         <is>
-          <t>Biznes Karta</t>
+          <t>Bashkent</t>
         </is>
       </c>
       <c r="E342" s="3" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="F342" s="3" t="n">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="G342" s="3" t="inlineStr"/>
-      <c r="H342" s="3" t="inlineStr">
-        <is>
-          <t>2 oy – 1 yil</t>
-        </is>
-      </c>
+      <c r="H342" s="3" t="inlineStr"/>
       <c r="I342" s="3" t="inlineStr">
         <is>
-          <t>17.9028 mln – 500 mln</t>
+          <t>1.06 mlrd gacha</t>
         </is>
       </c>
       <c r="J342" s="3" t="inlineStr">
@@ -22037,7 +22029,7 @@
       <c r="M342" s="3" t="inlineStr"/>
       <c r="N342" s="6" t="inlineStr">
         <is>
-          <t>https://ofb.uz/biznes/kreditlar/biznes-karta</t>
+          <t>https://ofb.uz/kreditlar/bashkent</t>
         </is>
       </c>
     </row>
@@ -22059,24 +22051,24 @@
       </c>
       <c r="D343" s="3" t="inlineStr">
         <is>
-          <t>Biznes Overdraft</t>
+          <t>Biznes Karta</t>
         </is>
       </c>
       <c r="E343" s="3" t="n">
         <v>25</v>
       </c>
       <c r="F343" s="3" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G343" s="3" t="inlineStr"/>
       <c r="H343" s="3" t="inlineStr">
         <is>
-          <t>2 oy – 18 oy</t>
+          <t>2 oy – 1 yil</t>
         </is>
       </c>
       <c r="I343" s="3" t="inlineStr">
         <is>
-          <t>17.9028 mln – 1.5 mlrd</t>
+          <t>17.9028 mln – 500 mln</t>
         </is>
       </c>
       <c r="J343" s="3" t="inlineStr">
@@ -22097,7 +22089,7 @@
       <c r="M343" s="3" t="inlineStr"/>
       <c r="N343" s="6" t="inlineStr">
         <is>
-          <t>https://ofb.uz/biznes/kreditlar/biznes-overdraft</t>
+          <t>https://ofb.uz/biznes/kreditlar/biznes-karta</t>
         </is>
       </c>
     </row>
@@ -22119,24 +22111,24 @@
       </c>
       <c r="D344" s="3" t="inlineStr">
         <is>
-          <t>Overdraft</t>
+          <t>Biznes Overdraft</t>
         </is>
       </c>
       <c r="E344" s="3" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F344" s="3" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G344" s="3" t="inlineStr"/>
       <c r="H344" s="3" t="inlineStr">
         <is>
-          <t>2 yilgacha</t>
+          <t>2 oy – 18 oy</t>
         </is>
       </c>
       <c r="I344" s="3" t="inlineStr">
         <is>
-          <t>50 mln gacha</t>
+          <t>17.9028 mln – 1.5 mlrd</t>
         </is>
       </c>
       <c r="J344" s="3" t="inlineStr">
@@ -22157,7 +22149,7 @@
       <c r="M344" s="3" t="inlineStr"/>
       <c r="N344" s="6" t="inlineStr">
         <is>
-          <t>https://ofb.uz/kreditlar/overdraft</t>
+          <t>https://ofb.uz/biznes/kreditlar/biznes-overdraft</t>
         </is>
       </c>
     </row>
@@ -22174,24 +22166,24 @@
       </c>
       <c r="C345" s="3" t="inlineStr">
         <is>
-          <t>Mikroqarz</t>
+          <t>Kredit karta</t>
         </is>
       </c>
       <c r="D345" s="3" t="inlineStr">
         <is>
-          <t>Onlayn mikroqarz (ilova)</t>
+          <t>Overdraft</t>
         </is>
       </c>
       <c r="E345" s="3" t="n">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="F345" s="3" t="n">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="G345" s="3" t="inlineStr"/>
       <c r="H345" s="3" t="inlineStr">
         <is>
-          <t>24 oygacha</t>
+          <t>2 yilgacha</t>
         </is>
       </c>
       <c r="I345" s="3" t="inlineStr">
@@ -22206,14 +22198,18 @@
       </c>
       <c r="K345" s="3" t="inlineStr">
         <is>
-          <t>Qo'lda tekshirilgan</t>
-        </is>
-      </c>
-      <c r="L345" s="3" t="inlineStr"/>
+          <t>Saytdan avtomatik</t>
+        </is>
+      </c>
+      <c r="L345" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
       <c r="M345" s="3" t="inlineStr"/>
       <c r="N345" s="6" t="inlineStr">
         <is>
-          <t>https://ofb.uz/en/credits/online-microloan</t>
+          <t>https://ofb.uz/kreditlar/overdraft</t>
         </is>
       </c>
     </row>
@@ -22235,7 +22231,7 @@
       </c>
       <c r="D346" s="3" t="inlineStr">
         <is>
-          <t>Onlayn mikroqarz</t>
+          <t>Onlayn mikroqarz (ilova)</t>
         </is>
       </c>
       <c r="E346" s="3" t="n">
@@ -22245,7 +22241,11 @@
         <v>30</v>
       </c>
       <c r="G346" s="3" t="inlineStr"/>
-      <c r="H346" s="3" t="inlineStr"/>
+      <c r="H346" s="3" t="inlineStr">
+        <is>
+          <t>24 oygacha</t>
+        </is>
+      </c>
       <c r="I346" s="3" t="inlineStr">
         <is>
           <t>50 mln gacha</t>
@@ -22258,18 +22258,14 @@
       </c>
       <c r="K346" s="3" t="inlineStr">
         <is>
-          <t>Saytdan avtomatik</t>
-        </is>
-      </c>
-      <c r="L346" s="3" t="inlineStr">
-        <is>
-          <t>2026-10-15</t>
-        </is>
-      </c>
+          <t>Qo'lda tekshirilgan</t>
+        </is>
+      </c>
+      <c r="L346" s="3" t="inlineStr"/>
       <c r="M346" s="3" t="inlineStr"/>
       <c r="N346" s="6" t="inlineStr">
         <is>
-          <t>https://ofb.uz/kreditlar/onlayn-mikroqarz</t>
+          <t>https://ofb.uz/en/credits/online-microloan</t>
         </is>
       </c>
     </row>
@@ -22291,24 +22287,20 @@
       </c>
       <c r="D347" s="3" t="inlineStr">
         <is>
-          <t>Kichik biznesga qadam</t>
+          <t>Onlayn mikroqarz</t>
         </is>
       </c>
       <c r="E347" s="3" t="n">
-        <v>27.4</v>
+        <v>30</v>
       </c>
       <c r="F347" s="3" t="n">
-        <v>27.4</v>
+        <v>30</v>
       </c>
       <c r="G347" s="3" t="inlineStr"/>
-      <c r="H347" s="3" t="inlineStr">
-        <is>
-          <t>2 yilgacha</t>
-        </is>
-      </c>
+      <c r="H347" s="3" t="inlineStr"/>
       <c r="I347" s="3" t="inlineStr">
         <is>
-          <t>5 mln gacha</t>
+          <t>50 mln gacha</t>
         </is>
       </c>
       <c r="J347" s="3" t="inlineStr">
@@ -22329,7 +22321,7 @@
       <c r="M347" s="3" t="inlineStr"/>
       <c r="N347" s="6" t="inlineStr">
         <is>
-          <t>https://ofb.uz/kreditlar/kichik-biznesga-qadam-mikrozaymi</t>
+          <t>https://ofb.uz/kreditlar/onlayn-mikroqarz</t>
         </is>
       </c>
     </row>
@@ -22351,24 +22343,24 @@
       </c>
       <c r="D348" s="3" t="inlineStr">
         <is>
-          <t>O‘simlikchilik</t>
+          <t>Kichik biznesga qadam</t>
         </is>
       </c>
       <c r="E348" s="3" t="n">
-        <v>26.9</v>
+        <v>27.4</v>
       </c>
       <c r="F348" s="3" t="n">
-        <v>26.9</v>
+        <v>27.4</v>
       </c>
       <c r="G348" s="3" t="inlineStr"/>
       <c r="H348" s="3" t="inlineStr">
         <is>
-          <t>3 yilgacha</t>
+          <t>2 yilgacha</t>
         </is>
       </c>
       <c r="I348" s="3" t="inlineStr">
         <is>
-          <t>30 mln gacha</t>
+          <t>5 mln gacha</t>
         </is>
       </c>
       <c r="J348" s="3" t="inlineStr">
@@ -22389,7 +22381,7 @@
       <c r="M348" s="3" t="inlineStr"/>
       <c r="N348" s="6" t="inlineStr">
         <is>
-          <t>https://ofb.uz/kreditlar/osimlikchilik-mikrozaymi</t>
+          <t>https://ofb.uz/kreditlar/kichik-biznesga-qadam-mikrozaymi</t>
         </is>
       </c>
     </row>
@@ -22411,7 +22403,7 @@
       </c>
       <c r="D349" s="3" t="inlineStr">
         <is>
-          <t>Bog‘bon</t>
+          <t>O‘simlikchilik</t>
         </is>
       </c>
       <c r="E349" s="3" t="n">
@@ -22428,7 +22420,7 @@
       </c>
       <c r="I349" s="3" t="inlineStr">
         <is>
-          <t>20 mln gacha</t>
+          <t>30 mln gacha</t>
         </is>
       </c>
       <c r="J349" s="3" t="inlineStr">
@@ -22449,7 +22441,7 @@
       <c r="M349" s="3" t="inlineStr"/>
       <c r="N349" s="6" t="inlineStr">
         <is>
-          <t>https://ofb.uz/kreditlar/bogbon-mikrozaymi</t>
+          <t>https://ofb.uz/kreditlar/osimlikchilik-mikrozaymi</t>
         </is>
       </c>
     </row>
@@ -22471,28 +22463,24 @@
       </c>
       <c r="D350" s="3" t="inlineStr">
         <is>
-          <t>Mikroqarz Ichki turizm</t>
+          <t>Bog‘bon</t>
         </is>
       </c>
       <c r="E350" s="3" t="n">
-        <v>26</v>
+        <v>26.9</v>
       </c>
       <c r="F350" s="3" t="n">
-        <v>26</v>
-      </c>
-      <c r="G350" s="3" t="inlineStr">
-        <is>
-          <t>27</t>
-        </is>
-      </c>
+        <v>26.9</v>
+      </c>
+      <c r="G350" s="3" t="inlineStr"/>
       <c r="H350" s="3" t="inlineStr">
         <is>
-          <t>12 oygacha</t>
+          <t>3 yilgacha</t>
         </is>
       </c>
       <c r="I350" s="3" t="inlineStr">
         <is>
-          <t>15 mln gacha</t>
+          <t>20 mln gacha</t>
         </is>
       </c>
       <c r="J350" s="3" t="inlineStr">
@@ -22502,14 +22490,18 @@
       </c>
       <c r="K350" s="3" t="inlineStr">
         <is>
-          <t>Qo'lda tekshirilgan</t>
-        </is>
-      </c>
-      <c r="L350" s="3" t="inlineStr"/>
+          <t>Saytdan avtomatik</t>
+        </is>
+      </c>
+      <c r="L350" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
       <c r="M350" s="3" t="inlineStr"/>
       <c r="N350" s="6" t="inlineStr">
         <is>
-          <t>https://ofb.uz/kreditlar/mikroqarz-ichki-turizm</t>
+          <t>https://ofb.uz/kreditlar/bogbon-mikrozaymi</t>
         </is>
       </c>
     </row>
@@ -22531,19 +22523,23 @@
       </c>
       <c r="D351" s="3" t="inlineStr">
         <is>
-          <t>Start Up</t>
+          <t>Mikroqarz Ichki turizm</t>
         </is>
       </c>
       <c r="E351" s="3" t="n">
-        <v>25.9</v>
+        <v>26</v>
       </c>
       <c r="F351" s="3" t="n">
-        <v>25.9</v>
-      </c>
-      <c r="G351" s="3" t="inlineStr"/>
+        <v>26</v>
+      </c>
+      <c r="G351" s="3" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
       <c r="H351" s="3" t="inlineStr">
         <is>
-          <t>1 yilgacha</t>
+          <t>12 oygacha</t>
         </is>
       </c>
       <c r="I351" s="3" t="inlineStr">
@@ -22558,18 +22554,14 @@
       </c>
       <c r="K351" s="3" t="inlineStr">
         <is>
-          <t>Saytdan avtomatik</t>
-        </is>
-      </c>
-      <c r="L351" s="3" t="inlineStr">
-        <is>
-          <t>2026-10-15</t>
-        </is>
-      </c>
+          <t>Qo'lda tekshirilgan</t>
+        </is>
+      </c>
+      <c r="L351" s="3" t="inlineStr"/>
       <c r="M351" s="3" t="inlineStr"/>
       <c r="N351" s="6" t="inlineStr">
         <is>
-          <t>https://ofb.uz/kreditlar/start-up-mikrozaymi</t>
+          <t>https://ofb.uz/kreditlar/mikroqarz-ichki-turizm</t>
         </is>
       </c>
     </row>
@@ -22591,7 +22583,7 @@
       </c>
       <c r="D352" s="3" t="inlineStr">
         <is>
-          <t>Oilaviy biznes</t>
+          <t>Start Up</t>
         </is>
       </c>
       <c r="E352" s="3" t="n">
@@ -22603,12 +22595,12 @@
       <c r="G352" s="3" t="inlineStr"/>
       <c r="H352" s="3" t="inlineStr">
         <is>
-          <t>3 yilgacha</t>
+          <t>1 yilgacha</t>
         </is>
       </c>
       <c r="I352" s="3" t="inlineStr">
         <is>
-          <t>25 mln gacha</t>
+          <t>15 mln gacha</t>
         </is>
       </c>
       <c r="J352" s="3" t="inlineStr">
@@ -22629,7 +22621,7 @@
       <c r="M352" s="3" t="inlineStr"/>
       <c r="N352" s="6" t="inlineStr">
         <is>
-          <t>https://ofb.uz/kreditlar/oilaviy-biznes-mikrozaymi</t>
+          <t>https://ofb.uz/kreditlar/start-up-mikrozaymi</t>
         </is>
       </c>
     </row>
@@ -22651,14 +22643,14 @@
       </c>
       <c r="D353" s="3" t="inlineStr">
         <is>
-          <t>Ishonch</t>
+          <t>Oilaviy biznes</t>
         </is>
       </c>
       <c r="E353" s="3" t="n">
-        <v>25.5</v>
+        <v>25.9</v>
       </c>
       <c r="F353" s="3" t="n">
-        <v>25.5</v>
+        <v>25.9</v>
       </c>
       <c r="G353" s="3" t="inlineStr"/>
       <c r="H353" s="3" t="inlineStr">
@@ -22668,7 +22660,7 @@
       </c>
       <c r="I353" s="3" t="inlineStr">
         <is>
-          <t>100 mln gacha</t>
+          <t>25 mln gacha</t>
         </is>
       </c>
       <c r="J353" s="3" t="inlineStr">
@@ -22689,7 +22681,7 @@
       <c r="M353" s="3" t="inlineStr"/>
       <c r="N353" s="6" t="inlineStr">
         <is>
-          <t>https://ofb.uz/kreditlar/ishonch-mikroqarz</t>
+          <t>https://ofb.uz/kreditlar/oilaviy-biznes-mikrozaymi</t>
         </is>
       </c>
     </row>
@@ -22711,24 +22703,24 @@
       </c>
       <c r="D354" s="3" t="inlineStr">
         <is>
-          <t>Green mikroqarz</t>
+          <t>Ishonch</t>
         </is>
       </c>
       <c r="E354" s="3" t="n">
-        <v>20</v>
+        <v>25.5</v>
       </c>
       <c r="F354" s="3" t="n">
-        <v>20</v>
+        <v>25.5</v>
       </c>
       <c r="G354" s="3" t="inlineStr"/>
       <c r="H354" s="3" t="inlineStr">
         <is>
-          <t>36 oygacha</t>
+          <t>3 yilgacha</t>
         </is>
       </c>
       <c r="I354" s="3" t="inlineStr">
         <is>
-          <t>5–50 mln</t>
+          <t>100 mln gacha</t>
         </is>
       </c>
       <c r="J354" s="3" t="inlineStr">
@@ -22738,14 +22730,18 @@
       </c>
       <c r="K354" s="3" t="inlineStr">
         <is>
-          <t>Qo'lda tekshirilgan</t>
-        </is>
-      </c>
-      <c r="L354" s="3" t="inlineStr"/>
+          <t>Saytdan avtomatik</t>
+        </is>
+      </c>
+      <c r="L354" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
       <c r="M354" s="3" t="inlineStr"/>
       <c r="N354" s="6" t="inlineStr">
         <is>
-          <t>https://ofb.uz/kreditlar/green-mikroqarz</t>
+          <t>https://ofb.uz/kreditlar/ishonch-mikroqarz</t>
         </is>
       </c>
     </row>
@@ -22762,29 +22758,29 @@
       </c>
       <c r="C355" s="3" t="inlineStr">
         <is>
-          <t>Ta'lim</t>
+          <t>Mikroqarz</t>
         </is>
       </c>
       <c r="D355" s="3" t="inlineStr">
         <is>
-          <t>Ta’lim uchun</t>
+          <t>Green mikroqarz</t>
         </is>
       </c>
       <c r="E355" s="3" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="F355" s="3" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="G355" s="3" t="inlineStr"/>
       <c r="H355" s="3" t="inlineStr">
         <is>
-          <t>4 yilgacha</t>
+          <t>36 oygacha</t>
         </is>
       </c>
       <c r="I355" s="3" t="inlineStr">
         <is>
-          <t>250 mln gacha</t>
+          <t>5–50 mln</t>
         </is>
       </c>
       <c r="J355" s="3" t="inlineStr">
@@ -22794,18 +22790,14 @@
       </c>
       <c r="K355" s="3" t="inlineStr">
         <is>
-          <t>Saytdan avtomatik</t>
-        </is>
-      </c>
-      <c r="L355" s="3" t="inlineStr">
-        <is>
-          <t>2026-10-15</t>
-        </is>
-      </c>
+          <t>Qo'lda tekshirilgan</t>
+        </is>
+      </c>
+      <c r="L355" s="3" t="inlineStr"/>
       <c r="M355" s="3" t="inlineStr"/>
       <c r="N355" s="6" t="inlineStr">
         <is>
-          <t>https://ofb.uz/kreditlar/talim-uchun-istemol-krediti</t>
+          <t>https://ofb.uz/kreditlar/green-mikroqarz</t>
         </is>
       </c>
     </row>
@@ -22817,36 +22809,34 @@
       </c>
       <c r="B356" s="3" t="inlineStr">
         <is>
-          <t>Yuridik</t>
+          <t>Jismoniy</t>
         </is>
       </c>
       <c r="C356" s="3" t="inlineStr">
         <is>
-          <t>Biznes</t>
+          <t>Ta'lim</t>
         </is>
       </c>
       <c r="D356" s="3" t="inlineStr">
         <is>
-          <t>OFB Express (aylanma mablag')</t>
+          <t>Ta’lim uchun</t>
         </is>
       </c>
       <c r="E356" s="3" t="n">
-        <v>26</v>
-      </c>
-      <c r="F356" s="3" t="n"/>
-      <c r="G356" s="3" t="inlineStr">
-        <is>
-          <t>26</t>
-        </is>
-      </c>
+        <v>25</v>
+      </c>
+      <c r="F356" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="G356" s="3" t="inlineStr"/>
       <c r="H356" s="3" t="inlineStr">
         <is>
-          <t>24 oygacha</t>
+          <t>4 yilgacha</t>
         </is>
       </c>
       <c r="I356" s="3" t="inlineStr">
         <is>
-          <t>1 mlrd gacha</t>
+          <t>250 mln gacha</t>
         </is>
       </c>
       <c r="J356" s="3" t="inlineStr">
@@ -22856,49 +22846,59 @@
       </c>
       <c r="K356" s="3" t="inlineStr">
         <is>
-          <t>Qo'lda tekshirilgan</t>
-        </is>
-      </c>
-      <c r="L356" s="3" t="inlineStr"/>
+          <t>Saytdan avtomatik</t>
+        </is>
+      </c>
+      <c r="L356" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
       <c r="M356" s="3" t="inlineStr"/>
       <c r="N356" s="6" t="inlineStr">
         <is>
-          <t>https://ofb.uz/biznes/kreditlar/ofb-express</t>
+          <t>https://ofb.uz/kreditlar/talim-uchun-istemol-krediti</t>
         </is>
       </c>
     </row>
     <row r="357">
       <c r="A357" s="3" t="inlineStr">
         <is>
-          <t>Poytaxt bank</t>
+          <t>Orient Finans Bank</t>
         </is>
       </c>
       <c r="B357" s="3" t="inlineStr">
         <is>
-          <t>Jismoniy</t>
+          <t>Yuridik</t>
         </is>
       </c>
       <c r="C357" s="3" t="inlineStr">
         <is>
-          <t>Avtokredit</t>
+          <t>Biznes</t>
         </is>
       </c>
       <c r="D357" s="3" t="inlineStr">
         <is>
-          <t>"Milliy" avtokredit</t>
+          <t>OFB Express (aylanma mablag')</t>
         </is>
       </c>
       <c r="E357" s="3" t="n">
-        <v>20</v>
-      </c>
-      <c r="F357" s="3" t="n">
-        <v>28</v>
-      </c>
-      <c r="G357" s="3" t="inlineStr"/>
-      <c r="H357" s="3" t="inlineStr"/>
+        <v>26</v>
+      </c>
+      <c r="F357" s="3" t="n"/>
+      <c r="G357" s="3" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="H357" s="3" t="inlineStr">
+        <is>
+          <t>24 oygacha</t>
+        </is>
+      </c>
       <c r="I357" s="3" t="inlineStr">
         <is>
-          <t>100 mln – 300 mln</t>
+          <t>1 mlrd gacha</t>
         </is>
       </c>
       <c r="J357" s="3" t="inlineStr">
@@ -22908,18 +22908,14 @@
       </c>
       <c r="K357" s="3" t="inlineStr">
         <is>
-          <t>Saytdan avtomatik</t>
-        </is>
-      </c>
-      <c r="L357" s="3" t="inlineStr">
-        <is>
-          <t>2026-10-15</t>
-        </is>
-      </c>
+          <t>Qo'lda tekshirilgan</t>
+        </is>
+      </c>
+      <c r="L357" s="3" t="inlineStr"/>
       <c r="M357" s="3" t="inlineStr"/>
       <c r="N357" s="6" t="inlineStr">
         <is>
-          <t>https://poytaxtbank.uz/uz/private/crediting/milliy-avtokredit/</t>
+          <t>https://ofb.uz/biznes/kreditlar/ofb-express</t>
         </is>
       </c>
     </row>
@@ -22941,7 +22937,7 @@
       </c>
       <c r="D358" s="3" t="inlineStr">
         <is>
-          <t>"Mini Truck Avto" krediti</t>
+          <t>"Milliy" avtokredit</t>
         </is>
       </c>
       <c r="E358" s="3" t="n">
@@ -22954,7 +22950,7 @@
       <c r="H358" s="3" t="inlineStr"/>
       <c r="I358" s="3" t="inlineStr">
         <is>
-          <t>1 mln – 450 mln</t>
+          <t>100 mln – 300 mln</t>
         </is>
       </c>
       <c r="J358" s="3" t="inlineStr">
@@ -22975,7 +22971,7 @@
       <c r="M358" s="3" t="inlineStr"/>
       <c r="N358" s="6" t="inlineStr">
         <is>
-          <t>https://poytaxtbank.uz/uz/private/crediting/mini-truck-avto-krediti/</t>
+          <t>https://poytaxtbank.uz/uz/private/crediting/milliy-avtokredit/</t>
         </is>
       </c>
     </row>
@@ -22997,22 +22993,22 @@
       </c>
       <c r="D359" s="3" t="inlineStr">
         <is>
-          <t>BYD / UzAuto / Hyundai</t>
+          <t>"Mini Truck Avto" krediti</t>
         </is>
       </c>
       <c r="E359" s="3" t="n">
-        <v>24.9</v>
+        <v>20</v>
       </c>
       <c r="F359" s="3" t="n">
-        <v>26.9</v>
+        <v>28</v>
       </c>
       <c r="G359" s="3" t="inlineStr"/>
-      <c r="H359" s="3" t="inlineStr">
-        <is>
-          <t>48 oy</t>
-        </is>
-      </c>
-      <c r="I359" s="3" t="inlineStr"/>
+      <c r="H359" s="3" t="inlineStr"/>
+      <c r="I359" s="3" t="inlineStr">
+        <is>
+          <t>1 mln – 450 mln</t>
+        </is>
+      </c>
       <c r="J359" s="3" t="inlineStr">
         <is>
           <t>UZS</t>
@@ -23020,18 +23016,18 @@
       </c>
       <c r="K359" s="3" t="inlineStr">
         <is>
-          <t>Qo'lda tekshirilgan</t>
-        </is>
-      </c>
-      <c r="L359" s="3" t="inlineStr"/>
-      <c r="M359" s="3" t="inlineStr">
-        <is>
-          <t>Ayrim Chevrolet modellari uchun 0%, 60 oygacha</t>
-        </is>
-      </c>
+          <t>Saytdan avtomatik</t>
+        </is>
+      </c>
+      <c r="L359" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="M359" s="3" t="inlineStr"/>
       <c r="N359" s="6" t="inlineStr">
         <is>
-          <t>https://poytaxtbank.uz/uz/private/</t>
+          <t>https://poytaxtbank.uz/uz/private/crediting/mini-truck-avto-krediti/</t>
         </is>
       </c>
     </row>
@@ -23053,19 +23049,19 @@
       </c>
       <c r="D360" s="3" t="inlineStr">
         <is>
-          <t>"Komfort AVTO" avtok... YANGI</t>
+          <t>BYD / UzAuto / Hyundai</t>
         </is>
       </c>
       <c r="E360" s="3" t="n">
-        <v>20</v>
+        <v>24.9</v>
       </c>
       <c r="F360" s="3" t="n">
-        <v>24</v>
+        <v>26.9</v>
       </c>
       <c r="G360" s="3" t="inlineStr"/>
       <c r="H360" s="3" t="inlineStr">
         <is>
-          <t>5 yilgacha</t>
+          <t>48 oy</t>
         </is>
       </c>
       <c r="I360" s="3" t="inlineStr"/>
@@ -23076,18 +23072,18 @@
       </c>
       <c r="K360" s="3" t="inlineStr">
         <is>
-          <t>Saytdan avtomatik</t>
-        </is>
-      </c>
-      <c r="L360" s="3" t="inlineStr">
-        <is>
-          <t>2026-10-15</t>
-        </is>
-      </c>
-      <c r="M360" s="3" t="inlineStr"/>
+          <t>Qo'lda tekshirilgan</t>
+        </is>
+      </c>
+      <c r="L360" s="3" t="inlineStr"/>
+      <c r="M360" s="3" t="inlineStr">
+        <is>
+          <t>Ayrim Chevrolet modellari uchun 0%, 60 oygacha</t>
+        </is>
+      </c>
       <c r="N360" s="6" t="inlineStr">
         <is>
-          <t>https://poytaxtbank.uz/uz/private/crediting/komfort-avto-avtokrediti/</t>
+          <t>https://poytaxtbank.uz/uz/private/</t>
         </is>
       </c>
     </row>
@@ -23104,27 +23100,27 @@
       </c>
       <c r="C361" s="3" t="inlineStr">
         <is>
-          <t>Biznes</t>
+          <t>Avtokredit</t>
         </is>
       </c>
       <c r="D361" s="3" t="inlineStr">
         <is>
-          <t>"Biznesga birinchi qadam" krediti</t>
+          <t>"Komfort AVTO" avtok... YANGI</t>
         </is>
       </c>
       <c r="E361" s="3" t="n">
         <v>20</v>
       </c>
       <c r="F361" s="3" t="n">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="G361" s="3" t="inlineStr"/>
-      <c r="H361" s="3" t="inlineStr"/>
-      <c r="I361" s="3" t="inlineStr">
-        <is>
-          <t>18 ming – 15 mln</t>
-        </is>
-      </c>
+      <c r="H361" s="3" t="inlineStr">
+        <is>
+          <t>5 yilgacha</t>
+        </is>
+      </c>
+      <c r="I361" s="3" t="inlineStr"/>
       <c r="J361" s="3" t="inlineStr">
         <is>
           <t>UZS</t>
@@ -23143,7 +23139,7 @@
       <c r="M361" s="3" t="inlineStr"/>
       <c r="N361" s="6" t="inlineStr">
         <is>
-          <t>https://poytaxtbank.uz/uz/private/crediting/first-step-to-business/</t>
+          <t>https://poytaxtbank.uz/uz/private/crediting/komfort-avto-avtokrediti/</t>
         </is>
       </c>
     </row>
@@ -23165,7 +23161,7 @@
       </c>
       <c r="D362" s="3" t="inlineStr">
         <is>
-          <t>"Biznesga ikkinchi qadam" krediti</t>
+          <t>"Biznesga birinchi qadam" krediti</t>
         </is>
       </c>
       <c r="E362" s="3" t="n">
@@ -23178,7 +23174,7 @@
       <c r="H362" s="3" t="inlineStr"/>
       <c r="I362" s="3" t="inlineStr">
         <is>
-          <t>42 ming – 17 mln</t>
+          <t>18 ming – 15 mln</t>
         </is>
       </c>
       <c r="J362" s="3" t="inlineStr">
@@ -23199,7 +23195,7 @@
       <c r="M362" s="3" t="inlineStr"/>
       <c r="N362" s="6" t="inlineStr">
         <is>
-          <t>https://poytaxtbank.uz/uz/private/crediting/second-step-to-business/</t>
+          <t>https://poytaxtbank.uz/uz/private/crediting/first-step-to-business/</t>
         </is>
       </c>
     </row>
@@ -23216,27 +23212,27 @@
       </c>
       <c r="C363" s="3" t="inlineStr">
         <is>
-          <t>Ipoteka</t>
+          <t>Biznes</t>
         </is>
       </c>
       <c r="D363" s="3" t="inlineStr">
         <is>
-          <t>Maskan</t>
+          <t>"Biznesga ikkinchi qadam" krediti</t>
         </is>
       </c>
       <c r="E363" s="3" t="n">
-        <v>27.99</v>
+        <v>20</v>
       </c>
       <c r="F363" s="3" t="n">
-        <v>31.99</v>
+        <v>28</v>
       </c>
       <c r="G363" s="3" t="inlineStr"/>
-      <c r="H363" s="3" t="inlineStr">
-        <is>
-          <t>5–10 yil</t>
-        </is>
-      </c>
-      <c r="I363" s="3" t="inlineStr"/>
+      <c r="H363" s="3" t="inlineStr"/>
+      <c r="I363" s="3" t="inlineStr">
+        <is>
+          <t>42 ming – 17 mln</t>
+        </is>
+      </c>
       <c r="J363" s="3" t="inlineStr">
         <is>
           <t>UZS</t>
@@ -23244,18 +23240,18 @@
       </c>
       <c r="K363" s="3" t="inlineStr">
         <is>
-          <t>Qo'lda tekshirilgan</t>
-        </is>
-      </c>
-      <c r="L363" s="3" t="inlineStr"/>
-      <c r="M363" s="3" t="inlineStr">
-        <is>
-          <t>Boshlang'ich badal 25%</t>
-        </is>
-      </c>
+          <t>Saytdan avtomatik</t>
+        </is>
+      </c>
+      <c r="L363" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="M363" s="3" t="inlineStr"/>
       <c r="N363" s="6" t="inlineStr">
         <is>
-          <t>https://poytaxtbank.uz/uz/private/crediting/mortgage-loan</t>
+          <t>https://poytaxtbank.uz/uz/private/crediting/second-step-to-business/</t>
         </is>
       </c>
     </row>
@@ -23277,19 +23273,19 @@
       </c>
       <c r="D364" s="3" t="inlineStr">
         <is>
-          <t>«Tayyor Uy» ipoteka krediti YANGI</t>
+          <t>Maskan</t>
         </is>
       </c>
       <c r="E364" s="3" t="n">
-        <v>22.5</v>
+        <v>27.99</v>
       </c>
       <c r="F364" s="3" t="n">
-        <v>24.5</v>
+        <v>31.99</v>
       </c>
       <c r="G364" s="3" t="inlineStr"/>
       <c r="H364" s="3" t="inlineStr">
         <is>
-          <t>20 yilgacha</t>
+          <t>5–10 yil</t>
         </is>
       </c>
       <c r="I364" s="3" t="inlineStr"/>
@@ -23300,18 +23296,18 @@
       </c>
       <c r="K364" s="3" t="inlineStr">
         <is>
-          <t>Saytdan avtomatik</t>
-        </is>
-      </c>
-      <c r="L364" s="3" t="inlineStr">
-        <is>
-          <t>2026-10-15</t>
-        </is>
-      </c>
-      <c r="M364" s="3" t="inlineStr"/>
+          <t>Qo'lda tekshirilgan</t>
+        </is>
+      </c>
+      <c r="L364" s="3" t="inlineStr"/>
+      <c r="M364" s="3" t="inlineStr">
+        <is>
+          <t>Boshlang'ich badal 25%</t>
+        </is>
+      </c>
       <c r="N364" s="6" t="inlineStr">
         <is>
-          <t>https://poytaxtbank.uz/uz/private/crediting/tayyor-uy-ipoteka-krediti/</t>
+          <t>https://poytaxtbank.uz/uz/private/crediting/mortgage-loan</t>
         </is>
       </c>
     </row>
@@ -23328,24 +23324,24 @@
       </c>
       <c r="C365" s="3" t="inlineStr">
         <is>
-          <t>Iste'mol</t>
+          <t>Ipoteka</t>
         </is>
       </c>
       <c r="D365" s="3" t="inlineStr">
         <is>
-          <t>Iste'mol krediti</t>
+          <t>«Tayyor Uy» ipoteka krediti YANGI</t>
         </is>
       </c>
       <c r="E365" s="3" t="n">
-        <v>28</v>
+        <v>22.5</v>
       </c>
       <c r="F365" s="3" t="n">
-        <v>30</v>
+        <v>24.5</v>
       </c>
       <c r="G365" s="3" t="inlineStr"/>
       <c r="H365" s="3" t="inlineStr">
         <is>
-          <t>12–36 oy</t>
+          <t>20 yilgacha</t>
         </is>
       </c>
       <c r="I365" s="3" t="inlineStr"/>
@@ -23356,18 +23352,18 @@
       </c>
       <c r="K365" s="3" t="inlineStr">
         <is>
-          <t>Qo'lda tekshirilgan</t>
-        </is>
-      </c>
-      <c r="L365" s="3" t="inlineStr"/>
-      <c r="M365" s="3" t="inlineStr">
-        <is>
-          <t>'Sayohat' krediti: 28%, 12 oy</t>
-        </is>
-      </c>
+          <t>Saytdan avtomatik</t>
+        </is>
+      </c>
+      <c r="L365" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="M365" s="3" t="inlineStr"/>
       <c r="N365" s="6" t="inlineStr">
         <is>
-          <t>https://poytaxtbank.uz/uz/private/</t>
+          <t>https://poytaxtbank.uz/uz/private/crediting/tayyor-uy-ipoteka-krediti/</t>
         </is>
       </c>
     </row>
@@ -23389,22 +23385,22 @@
       </c>
       <c r="D366" s="3" t="inlineStr">
         <is>
-          <t>Mahalla loyihasi krediti</t>
+          <t>Iste'mol krediti</t>
         </is>
       </c>
       <c r="E366" s="3" t="n">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="F366" s="3" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="G366" s="3" t="inlineStr"/>
-      <c r="H366" s="3" t="inlineStr"/>
-      <c r="I366" s="3" t="inlineStr">
-        <is>
-          <t>18 ming – 30 mln</t>
-        </is>
-      </c>
+      <c r="H366" s="3" t="inlineStr">
+        <is>
+          <t>12–36 oy</t>
+        </is>
+      </c>
+      <c r="I366" s="3" t="inlineStr"/>
       <c r="J366" s="3" t="inlineStr">
         <is>
           <t>UZS</t>
@@ -23412,18 +23408,18 @@
       </c>
       <c r="K366" s="3" t="inlineStr">
         <is>
-          <t>Saytdan avtomatik</t>
-        </is>
-      </c>
-      <c r="L366" s="3" t="inlineStr">
-        <is>
-          <t>2026-10-15</t>
-        </is>
-      </c>
-      <c r="M366" s="3" t="inlineStr"/>
+          <t>Qo'lda tekshirilgan</t>
+        </is>
+      </c>
+      <c r="L366" s="3" t="inlineStr"/>
+      <c r="M366" s="3" t="inlineStr">
+        <is>
+          <t>'Sayohat' krediti: 28%, 12 oy</t>
+        </is>
+      </c>
       <c r="N366" s="6" t="inlineStr">
         <is>
-          <t>https://poytaxtbank.uz/uz/private/crediting/mahalla-loyihasi-krediti/</t>
+          <t>https://poytaxtbank.uz/uz/private/</t>
         </is>
       </c>
     </row>
@@ -23440,29 +23436,25 @@
       </c>
       <c r="C367" s="3" t="inlineStr">
         <is>
-          <t>Mikroqarz</t>
+          <t>Iste'mol</t>
         </is>
       </c>
       <c r="D367" s="3" t="inlineStr">
         <is>
-          <t>Mikroqarz</t>
+          <t>Mahalla loyihasi krediti</t>
         </is>
       </c>
       <c r="E367" s="3" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="F367" s="3" t="n">
         <v>28</v>
       </c>
       <c r="G367" s="3" t="inlineStr"/>
-      <c r="H367" s="3" t="inlineStr">
-        <is>
-          <t>36 oygacha</t>
-        </is>
-      </c>
+      <c r="H367" s="3" t="inlineStr"/>
       <c r="I367" s="3" t="inlineStr">
         <is>
-          <t>100 mln gacha</t>
+          <t>18 ming – 30 mln</t>
         </is>
       </c>
       <c r="J367" s="3" t="inlineStr">
@@ -23472,18 +23464,18 @@
       </c>
       <c r="K367" s="3" t="inlineStr">
         <is>
-          <t>Qo'lda tekshirilgan</t>
-        </is>
-      </c>
-      <c r="L367" s="3" t="inlineStr"/>
-      <c r="M367" s="3" t="inlineStr">
-        <is>
-          <t>Boshlang'ich badal yo'q</t>
-        </is>
-      </c>
+          <t>Saytdan avtomatik</t>
+        </is>
+      </c>
+      <c r="L367" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="M367" s="3" t="inlineStr"/>
       <c r="N367" s="6" t="inlineStr">
         <is>
-          <t>https://poytaxtbank.uz/uz/private/crediting/microloan/</t>
+          <t>https://poytaxtbank.uz/uz/private/crediting/mahalla-loyihasi-krediti/</t>
         </is>
       </c>
     </row>
@@ -23505,7 +23497,7 @@
       </c>
       <c r="D368" s="3" t="inlineStr">
         <is>
-          <t>Mikroqarz KASSA ORQALI</t>
+          <t>Mikroqarz</t>
         </is>
       </c>
       <c r="E368" s="3" t="n">
@@ -23517,10 +23509,14 @@
       <c r="G368" s="3" t="inlineStr"/>
       <c r="H368" s="3" t="inlineStr">
         <is>
-          <t>3 yilgacha</t>
-        </is>
-      </c>
-      <c r="I368" s="3" t="inlineStr"/>
+          <t>36 oygacha</t>
+        </is>
+      </c>
+      <c r="I368" s="3" t="inlineStr">
+        <is>
+          <t>100 mln gacha</t>
+        </is>
+      </c>
       <c r="J368" s="3" t="inlineStr">
         <is>
           <t>UZS</t>
@@ -23528,15 +23524,15 @@
       </c>
       <c r="K368" s="3" t="inlineStr">
         <is>
-          <t>Saytdan avtomatik</t>
-        </is>
-      </c>
-      <c r="L368" s="3" t="inlineStr">
-        <is>
-          <t>2026-10-15</t>
-        </is>
-      </c>
-      <c r="M368" s="3" t="inlineStr"/>
+          <t>Qo'lda tekshirilgan</t>
+        </is>
+      </c>
+      <c r="L368" s="3" t="inlineStr"/>
+      <c r="M368" s="3" t="inlineStr">
+        <is>
+          <t>Boshlang'ich badal yo'q</t>
+        </is>
+      </c>
       <c r="N368" s="6" t="inlineStr">
         <is>
           <t>https://poytaxtbank.uz/uz/private/crediting/microloan/</t>
@@ -23561,11 +23557,11 @@
       </c>
       <c r="D369" s="3" t="inlineStr">
         <is>
-          <t>Mikroqarz "Bir to‘lov... YANGI</t>
+          <t>Mikroqarz KASSA ORQALI</t>
         </is>
       </c>
       <c r="E369" s="3" t="n">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="F369" s="3" t="n">
         <v>28</v>
@@ -23595,7 +23591,7 @@
       <c r="M369" s="3" t="inlineStr"/>
       <c r="N369" s="6" t="inlineStr">
         <is>
-          <t>https://poytaxtbank.uz/uz/private/crediting/mikroqarz-bir-to-lov/</t>
+          <t>https://poytaxtbank.uz/uz/private/crediting/microloan/</t>
         </is>
       </c>
     </row>
@@ -23617,22 +23613,22 @@
       </c>
       <c r="D370" s="3" t="inlineStr">
         <is>
-          <t>Oylik ish haqi loyihasida Mikroqarz</t>
+          <t>Mikroqarz "Bir to‘lov... YANGI</t>
         </is>
       </c>
       <c r="E370" s="3" t="n">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="F370" s="3" t="n">
         <v>28</v>
       </c>
       <c r="G370" s="3" t="inlineStr"/>
-      <c r="H370" s="3" t="inlineStr"/>
-      <c r="I370" s="3" t="inlineStr">
-        <is>
-          <t>600 ming – 100 mln</t>
-        </is>
-      </c>
+      <c r="H370" s="3" t="inlineStr">
+        <is>
+          <t>3 yilgacha</t>
+        </is>
+      </c>
+      <c r="I370" s="3" t="inlineStr"/>
       <c r="J370" s="3" t="inlineStr">
         <is>
           <t>UZS</t>
@@ -23651,7 +23647,7 @@
       <c r="M370" s="3" t="inlineStr"/>
       <c r="N370" s="6" t="inlineStr">
         <is>
-          <t>https://poytaxtbank.uz/uz/private/crediting/oylik-ish-haqi-loyihasida-mikroqarz/</t>
+          <t>https://poytaxtbank.uz/uz/private/crediting/mikroqarz-bir-to-lov/</t>
         </is>
       </c>
     </row>
@@ -23663,32 +23659,32 @@
       </c>
       <c r="B371" s="3" t="inlineStr">
         <is>
-          <t>Yuridik</t>
+          <t>Jismoniy</t>
         </is>
       </c>
       <c r="C371" s="3" t="inlineStr">
         <is>
-          <t>Avtokredit</t>
+          <t>Mikroqarz</t>
         </is>
       </c>
       <c r="D371" s="3" t="inlineStr">
         <is>
-          <t>Avto kredit</t>
+          <t>Oylik ish haqi loyihasida Mikroqarz</t>
         </is>
       </c>
       <c r="E371" s="3" t="n">
-        <v>27.99</v>
+        <v>20</v>
       </c>
       <c r="F371" s="3" t="n">
-        <v>27.99</v>
+        <v>28</v>
       </c>
       <c r="G371" s="3" t="inlineStr"/>
-      <c r="H371" s="3" t="inlineStr">
-        <is>
-          <t>3 yilgacha</t>
-        </is>
-      </c>
-      <c r="I371" s="3" t="inlineStr"/>
+      <c r="H371" s="3" t="inlineStr"/>
+      <c r="I371" s="3" t="inlineStr">
+        <is>
+          <t>600 ming – 100 mln</t>
+        </is>
+      </c>
       <c r="J371" s="3" t="inlineStr">
         <is>
           <t>UZS</t>
@@ -23707,7 +23703,7 @@
       <c r="M371" s="3" t="inlineStr"/>
       <c r="N371" s="6" t="inlineStr">
         <is>
-          <t>https://poytaxtbank.uz/uz/corporate/crediting/avto-kredit-/</t>
+          <t>https://poytaxtbank.uz/uz/private/crediting/oylik-ish-haqi-loyihasida-mikroqarz/</t>
         </is>
       </c>
     </row>
@@ -23729,7 +23725,7 @@
       </c>
       <c r="D372" s="3" t="inlineStr">
         <is>
-          <t>Avto kredit (5 tonnagacha bo‘l... YANGI</t>
+          <t>Avto kredit</t>
         </is>
       </c>
       <c r="E372" s="3" t="n">
@@ -23763,7 +23759,7 @@
       <c r="M372" s="3" t="inlineStr"/>
       <c r="N372" s="6" t="inlineStr">
         <is>
-          <t>https://poytaxtbank.uz/uz/corporate/crediting/avto-kredit-5-tonnagacha-bo-lgan-yo-lovchi-va-yuk-tashish-uchun/</t>
+          <t>https://poytaxtbank.uz/uz/corporate/crediting/avto-kredit-/</t>
         </is>
       </c>
     </row>
@@ -23785,7 +23781,7 @@
       </c>
       <c r="D373" s="3" t="inlineStr">
         <is>
-          <t>Avto kredit YANGI</t>
+          <t>Avto kredit (5 tonnagacha bo‘l... YANGI</t>
         </is>
       </c>
       <c r="E373" s="3" t="n">
@@ -23819,7 +23815,7 @@
       <c r="M373" s="3" t="inlineStr"/>
       <c r="N373" s="6" t="inlineStr">
         <is>
-          <t>https://poytaxtbank.uz/uz/small-business/crediting/avto-kredit-/</t>
+          <t>https://poytaxtbank.uz/uz/corporate/crediting/avto-kredit-5-tonnagacha-bo-lgan-yo-lovchi-va-yuk-tashish-uchun/</t>
         </is>
       </c>
     </row>
@@ -23836,12 +23832,12 @@
       </c>
       <c r="C374" s="3" t="inlineStr">
         <is>
-          <t>Biznes</t>
+          <t>Avtokredit</t>
         </is>
       </c>
       <c r="D374" s="3" t="inlineStr">
         <is>
-          <t>“Faol tadbirkor” krediti YANGI</t>
+          <t>Avto kredit YANGI</t>
         </is>
       </c>
       <c r="E374" s="3" t="n">
@@ -23853,7 +23849,7 @@
       <c r="G374" s="3" t="inlineStr"/>
       <c r="H374" s="3" t="inlineStr">
         <is>
-          <t>1 yilgacha</t>
+          <t>3 yilgacha</t>
         </is>
       </c>
       <c r="I374" s="3" t="inlineStr"/>
@@ -23875,7 +23871,7 @@
       <c r="M374" s="3" t="inlineStr"/>
       <c r="N374" s="6" t="inlineStr">
         <is>
-          <t>https://poytaxtbank.uz/uz/corporate/crediting/faol-tadbirkor-krediti/</t>
+          <t>https://poytaxtbank.uz/uz/small-business/crediting/avto-kredit-/</t>
         </is>
       </c>
     </row>
@@ -23897,7 +23893,7 @@
       </c>
       <c r="D375" s="3" t="inlineStr">
         <is>
-          <t>Revolver kreditlar</t>
+          <t>“Faol tadbirkor” krediti YANGI</t>
         </is>
       </c>
       <c r="E375" s="3" t="n">
@@ -23909,7 +23905,7 @@
       <c r="G375" s="3" t="inlineStr"/>
       <c r="H375" s="3" t="inlineStr">
         <is>
-          <t>3 yilgacha</t>
+          <t>1 yilgacha</t>
         </is>
       </c>
       <c r="I375" s="3" t="inlineStr"/>
@@ -23931,7 +23927,7 @@
       <c r="M375" s="3" t="inlineStr"/>
       <c r="N375" s="6" t="inlineStr">
         <is>
-          <t>https://poytaxtbank.uz/uz/corporate/crediting/revolver-kreditlar/</t>
+          <t>https://poytaxtbank.uz/uz/corporate/crediting/faol-tadbirkor-krediti/</t>
         </is>
       </c>
     </row>
@@ -23953,7 +23949,7 @@
       </c>
       <c r="D376" s="3" t="inlineStr">
         <is>
-          <t>Aylanma mablagʻlarni toʻldiris...</t>
+          <t>Revolver kreditlar</t>
         </is>
       </c>
       <c r="E376" s="3" t="n">
@@ -23987,7 +23983,7 @@
       <c r="M376" s="3" t="inlineStr"/>
       <c r="N376" s="6" t="inlineStr">
         <is>
-          <t>https://poytaxtbank.uz/uz/corporate/crediting/aylanma-mablag-larni-to-ldirish-/</t>
+          <t>https://poytaxtbank.uz/uz/corporate/crediting/revolver-kreditlar/</t>
         </is>
       </c>
     </row>
@@ -24009,7 +24005,7 @@
       </c>
       <c r="D377" s="3" t="inlineStr">
         <is>
-          <t>Asosiy vosita hamda investitsi...</t>
+          <t>Aylanma mablagʻlarni toʻldiris...</t>
         </is>
       </c>
       <c r="E377" s="3" t="n">
@@ -24043,7 +24039,7 @@
       <c r="M377" s="3" t="inlineStr"/>
       <c r="N377" s="6" t="inlineStr">
         <is>
-          <t>https://poytaxtbank.uz/uz/small-business/crediting/asosiy-vosita-hamda-investitsiya-loyihalarni-moliyalashtirish/</t>
+          <t>https://poytaxtbank.uz/uz/corporate/crediting/aylanma-mablag-larni-to-ldirish-/</t>
         </is>
       </c>
     </row>
@@ -24065,14 +24061,14 @@
       </c>
       <c r="D378" s="3" t="inlineStr">
         <is>
-          <t>Poytaxt Biznes 2 YANGI</t>
+          <t>Asosiy vosita hamda investitsi...</t>
         </is>
       </c>
       <c r="E378" s="3" t="n">
-        <v>25</v>
+        <v>27.99</v>
       </c>
       <c r="F378" s="3" t="n">
-        <v>25</v>
+        <v>27.99</v>
       </c>
       <c r="G378" s="3" t="inlineStr"/>
       <c r="H378" s="3" t="inlineStr">
@@ -24099,7 +24095,7 @@
       <c r="M378" s="3" t="inlineStr"/>
       <c r="N378" s="6" t="inlineStr">
         <is>
-          <t>https://poytaxtbank.uz/uz/corporate/crediting/poytaxt-biznes-2/</t>
+          <t>https://poytaxtbank.uz/uz/small-business/crediting/asosiy-vosita-hamda-investitsiya-loyihalarni-moliyalashtirish/</t>
         </is>
       </c>
     </row>
@@ -24121,7 +24117,7 @@
       </c>
       <c r="D379" s="3" t="inlineStr">
         <is>
-          <t>Asosiy vosita hamda investitsi...</t>
+          <t>Poytaxt Biznes 2 YANGI</t>
         </is>
       </c>
       <c r="E379" s="3" t="n">
@@ -24133,7 +24129,7 @@
       <c r="G379" s="3" t="inlineStr"/>
       <c r="H379" s="3" t="inlineStr">
         <is>
-          <t>5 yilgacha</t>
+          <t>3 yilgacha</t>
         </is>
       </c>
       <c r="I379" s="3" t="inlineStr"/>
@@ -24155,7 +24151,7 @@
       <c r="M379" s="3" t="inlineStr"/>
       <c r="N379" s="6" t="inlineStr">
         <is>
-          <t>https://poytaxtbank.uz/uz/corporate/crediting/asosiy-vosita-hamda-investitsiya-loyihalarni-moliyalashtirish/</t>
+          <t>https://poytaxtbank.uz/uz/corporate/crediting/poytaxt-biznes-2/</t>
         </is>
       </c>
     </row>
@@ -24172,24 +24168,24 @@
       </c>
       <c r="C380" s="3" t="inlineStr">
         <is>
-          <t>Ipoteka</t>
+          <t>Biznes</t>
         </is>
       </c>
       <c r="D380" s="3" t="inlineStr">
         <is>
-          <t>Koʻp qavatli uy-joylar qurish ... YANGI</t>
+          <t>Asosiy vosita hamda investitsi...</t>
         </is>
       </c>
       <c r="E380" s="3" t="n">
-        <v>27.99</v>
+        <v>25</v>
       </c>
       <c r="F380" s="3" t="n">
-        <v>27.99</v>
+        <v>25</v>
       </c>
       <c r="G380" s="3" t="inlineStr"/>
       <c r="H380" s="3" t="inlineStr">
         <is>
-          <t>3 yilgacha</t>
+          <t>5 yilgacha</t>
         </is>
       </c>
       <c r="I380" s="3" t="inlineStr"/>
@@ -24211,39 +24207,43 @@
       <c r="M380" s="3" t="inlineStr"/>
       <c r="N380" s="6" t="inlineStr">
         <is>
-          <t>https://poytaxtbank.uz/uz/corporate/crediting/ko-p-qavatli-uy-joylar-qurish-va-rekonstruksiya-qilish-uchun/</t>
+          <t>https://poytaxtbank.uz/uz/corporate/crediting/asosiy-vosita-hamda-investitsiya-loyihalarni-moliyalashtirish/</t>
         </is>
       </c>
     </row>
     <row r="381">
       <c r="A381" s="3" t="inlineStr">
         <is>
-          <t>Smartbank</t>
+          <t>Poytaxt bank</t>
         </is>
       </c>
       <c r="B381" s="3" t="inlineStr">
         <is>
-          <t>Jismoniy</t>
+          <t>Yuridik</t>
         </is>
       </c>
       <c r="C381" s="3" t="inlineStr">
         <is>
-          <t>Iste'mol</t>
+          <t>Ipoteka</t>
         </is>
       </c>
       <c r="D381" s="3" t="inlineStr">
         <is>
-          <t>Kredit</t>
+          <t>Koʻp qavatli uy-joylar qurish ... YANGI</t>
         </is>
       </c>
       <c r="E381" s="3" t="n">
-        <v>24.99</v>
+        <v>27.99</v>
       </c>
       <c r="F381" s="3" t="n">
-        <v>25.99</v>
+        <v>27.99</v>
       </c>
       <c r="G381" s="3" t="inlineStr"/>
-      <c r="H381" s="3" t="inlineStr"/>
+      <c r="H381" s="3" t="inlineStr">
+        <is>
+          <t>3 yilgacha</t>
+        </is>
+      </c>
       <c r="I381" s="3" t="inlineStr"/>
       <c r="J381" s="3" t="inlineStr">
         <is>
@@ -24252,18 +24252,18 @@
       </c>
       <c r="K381" s="3" t="inlineStr">
         <is>
-          <t>Qo'lda tekshirilgan</t>
-        </is>
-      </c>
-      <c r="L381" s="3" t="inlineStr"/>
-      <c r="M381" s="3" t="inlineStr">
-        <is>
-          <t>Rasmiy daromadli 24.99%, o'zini band qilganlar 25.99%; sahifa 'Openbank' nomida</t>
-        </is>
-      </c>
+          <t>Saytdan avtomatik</t>
+        </is>
+      </c>
+      <c r="L381" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="M381" s="3" t="inlineStr"/>
       <c r="N381" s="6" t="inlineStr">
         <is>
-          <t>https://smartbank.uz/useful/faq</t>
+          <t>https://poytaxtbank.uz/uz/corporate/crediting/ko-p-qavatli-uy-joylar-qurish-va-rekonstruksiya-qilish-uchun/</t>
         </is>
       </c>
     </row>
@@ -29336,85 +29336,81 @@
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>Orient Finans Bank</t>
+          <t>Openbank</t>
         </is>
       </c>
       <c r="B21" s="3" t="n">
-        <v>37</v>
+        <v>1</v>
       </c>
       <c r="C21" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>12.5 – 30</t>
+          <t>24.99 – 25.99</t>
         </is>
       </c>
       <c r="E21" s="3" t="n">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="F21" s="3" t="inlineStr"/>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>ofb.uz</t>
+          <t>openbank.uz</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>Poytaxt bank</t>
+          <t>Orient Finans Bank</t>
         </is>
       </c>
       <c r="B22" s="3" t="n">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="C22" s="3" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>20 – 31.99</t>
+          <t>12.5 – 30</t>
         </is>
       </c>
       <c r="E22" s="3" t="n">
-        <v>20</v>
+        <v>31</v>
       </c>
       <c r="F22" s="3" t="inlineStr"/>
       <c r="G22" s="3" t="inlineStr">
         <is>
-          <t>poytaxtbank.uz</t>
+          <t>ofb.uz</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>Smartbank</t>
+          <t>Poytaxt bank</t>
         </is>
       </c>
       <c r="B23" s="3" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="C23" s="3" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>24.99 – 25.99</t>
+          <t>20 – 31.99</t>
         </is>
       </c>
       <c r="E23" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F23" s="3" t="inlineStr">
-        <is>
-          <t>Sayt 'Openbank' nomida</t>
-        </is>
-      </c>
+        <v>20</v>
+      </c>
+      <c r="F23" s="3" t="inlineStr"/>
       <c r="G23" s="3" t="inlineStr">
         <is>
-          <t>smartbank.uz</t>
+          <t>poytaxtbank.uz</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Ma'lumot avtomatik yangilandi (2026-10-15)
</commit_message>
<xml_diff>
--- a/docs/banklar_kreditlar.xlsx
+++ b/docs/banklar_kreditlar.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Xulosalar" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kreditlar" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Banklar xulosasi" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Izoh" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Xulosalar" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Kreditlar" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Banklar xulosasi" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Izoh" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Kreditlar'!$A$1:$N$453</definedName>

</xml_diff>

<commit_message>
Ma'lumot avtomatik yangilandi (2026-10-16)
</commit_message>
<xml_diff>
--- a/docs/banklar_kreditlar.xlsx
+++ b/docs/banklar_kreditlar.xlsx
@@ -2223,7 +2223,7 @@
       </c>
       <c r="L3" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M3" s="3" t="inlineStr"/>
@@ -2283,7 +2283,7 @@
       </c>
       <c r="L4" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M4" s="3" t="inlineStr"/>
@@ -2343,7 +2343,7 @@
       </c>
       <c r="L5" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M5" s="3" t="inlineStr"/>
@@ -2403,7 +2403,7 @@
       </c>
       <c r="L6" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M6" s="3" t="inlineStr"/>
@@ -2463,7 +2463,7 @@
       </c>
       <c r="L7" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M7" s="3" t="inlineStr"/>
@@ -2523,7 +2523,7 @@
       </c>
       <c r="L8" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M8" s="3" t="inlineStr"/>
@@ -2639,7 +2639,7 @@
       </c>
       <c r="L10" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M10" s="3" t="inlineStr"/>
@@ -2699,7 +2699,7 @@
       </c>
       <c r="L11" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M11" s="3" t="inlineStr"/>
@@ -2815,7 +2815,7 @@
       </c>
       <c r="L13" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M13" s="3" t="inlineStr"/>
@@ -2875,7 +2875,7 @@
       </c>
       <c r="L14" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M14" s="3" t="inlineStr"/>
@@ -2935,7 +2935,7 @@
       </c>
       <c r="L15" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M15" s="3" t="inlineStr"/>
@@ -3047,7 +3047,7 @@
       </c>
       <c r="L17" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M17" s="3" t="inlineStr"/>
@@ -3107,7 +3107,7 @@
       </c>
       <c r="L18" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M18" s="3" t="inlineStr"/>
@@ -3223,7 +3223,7 @@
       </c>
       <c r="L20" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M20" s="3" t="inlineStr"/>
@@ -3283,7 +3283,7 @@
       </c>
       <c r="L21" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M21" s="3" t="inlineStr"/>
@@ -3343,7 +3343,7 @@
       </c>
       <c r="L22" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M22" s="3" t="inlineStr"/>
@@ -3403,7 +3403,7 @@
       </c>
       <c r="L23" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M23" s="3" t="inlineStr"/>
@@ -3463,7 +3463,7 @@
       </c>
       <c r="L24" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M24" s="3" t="inlineStr"/>
@@ -3631,7 +3631,7 @@
       </c>
       <c r="L27" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M27" s="3" t="inlineStr"/>
@@ -3691,7 +3691,7 @@
       </c>
       <c r="L28" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M28" s="3" t="inlineStr"/>
@@ -3751,7 +3751,7 @@
       </c>
       <c r="L29" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M29" s="3" t="inlineStr"/>
@@ -3811,7 +3811,7 @@
       </c>
       <c r="L30" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M30" s="3" t="inlineStr"/>
@@ -3871,7 +3871,7 @@
       </c>
       <c r="L31" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M31" s="3" t="inlineStr"/>
@@ -3931,7 +3931,7 @@
       </c>
       <c r="L32" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M32" s="3" t="inlineStr"/>
@@ -3991,7 +3991,7 @@
       </c>
       <c r="L33" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M33" s="3" t="inlineStr"/>
@@ -4051,7 +4051,7 @@
       </c>
       <c r="L34" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M34" s="3" t="inlineStr"/>
@@ -4111,7 +4111,7 @@
       </c>
       <c r="L35" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M35" s="3" t="inlineStr"/>
@@ -4171,7 +4171,7 @@
       </c>
       <c r="L36" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M36" s="3" t="inlineStr"/>
@@ -4227,7 +4227,7 @@
       </c>
       <c r="L37" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M37" s="3" t="inlineStr"/>
@@ -4339,7 +4339,7 @@
       </c>
       <c r="L39" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M39" s="3" t="inlineStr"/>
@@ -4395,7 +4395,7 @@
       </c>
       <c r="L40" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M40" s="3" t="inlineStr"/>
@@ -4451,7 +4451,7 @@
       </c>
       <c r="L41" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M41" s="3" t="inlineStr"/>
@@ -4507,7 +4507,7 @@
       </c>
       <c r="L42" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M42" s="3" t="inlineStr"/>
@@ -4567,7 +4567,7 @@
       </c>
       <c r="L43" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M43" s="3" t="inlineStr"/>
@@ -4627,7 +4627,7 @@
       </c>
       <c r="L44" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M44" s="3" t="inlineStr"/>
@@ -4687,7 +4687,7 @@
       </c>
       <c r="L45" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M45" s="3" t="inlineStr"/>
@@ -4743,7 +4743,7 @@
       </c>
       <c r="L46" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M46" s="3" t="inlineStr"/>
@@ -4799,7 +4799,7 @@
       </c>
       <c r="L47" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M47" s="3" t="inlineStr"/>
@@ -4859,7 +4859,7 @@
       </c>
       <c r="L48" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M48" s="3" t="inlineStr"/>
@@ -4919,7 +4919,7 @@
       </c>
       <c r="L49" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M49" s="3" t="inlineStr"/>
@@ -4979,7 +4979,7 @@
       </c>
       <c r="L50" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M50" s="3" t="inlineStr"/>
@@ -5093,7 +5093,7 @@
       </c>
       <c r="L52" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M52" s="3" t="inlineStr"/>
@@ -5153,7 +5153,7 @@
       </c>
       <c r="L53" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M53" s="3" t="inlineStr"/>
@@ -5213,7 +5213,7 @@
       </c>
       <c r="L54" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M54" s="3" t="inlineStr"/>
@@ -5273,7 +5273,7 @@
       </c>
       <c r="L55" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M55" s="3" t="inlineStr"/>
@@ -5333,7 +5333,7 @@
       </c>
       <c r="L56" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M56" s="3" t="inlineStr"/>
@@ -5445,7 +5445,7 @@
       </c>
       <c r="L58" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M58" s="3" t="inlineStr"/>
@@ -5501,7 +5501,7 @@
       </c>
       <c r="L59" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M59" s="3" t="inlineStr"/>
@@ -6257,7 +6257,7 @@
       </c>
       <c r="L72" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M72" s="3" t="inlineStr"/>
@@ -6369,7 +6369,7 @@
       </c>
       <c r="L74" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M74" s="3" t="inlineStr"/>
@@ -6481,7 +6481,7 @@
       </c>
       <c r="L76" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M76" s="3" t="inlineStr"/>
@@ -6537,7 +6537,7 @@
       </c>
       <c r="L77" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M77" s="3" t="inlineStr"/>
@@ -6593,7 +6593,7 @@
       </c>
       <c r="L78" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M78" s="3" t="inlineStr"/>
@@ -6649,7 +6649,7 @@
       </c>
       <c r="L79" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M79" s="3" t="inlineStr"/>
@@ -6705,7 +6705,7 @@
       </c>
       <c r="L80" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M80" s="3" t="inlineStr"/>
@@ -6761,7 +6761,7 @@
       </c>
       <c r="L81" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M81" s="3" t="inlineStr"/>
@@ -6817,7 +6817,7 @@
       </c>
       <c r="L82" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M82" s="3" t="inlineStr"/>
@@ -6869,7 +6869,7 @@
       </c>
       <c r="L83" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M83" s="3" t="inlineStr"/>
@@ -6929,7 +6929,7 @@
       </c>
       <c r="L84" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M84" s="3" t="inlineStr"/>
@@ -6989,7 +6989,7 @@
       </c>
       <c r="L85" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M85" s="3" t="inlineStr"/>
@@ -7049,7 +7049,7 @@
       </c>
       <c r="L86" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M86" s="3" t="inlineStr"/>
@@ -7109,7 +7109,7 @@
       </c>
       <c r="L87" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M87" s="3" t="inlineStr"/>
@@ -7169,7 +7169,7 @@
       </c>
       <c r="L88" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M88" s="3" t="inlineStr"/>
@@ -7225,7 +7225,7 @@
       </c>
       <c r="L89" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M89" s="3" t="inlineStr"/>
@@ -7277,7 +7277,7 @@
       </c>
       <c r="L90" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M90" s="3" t="inlineStr"/>
@@ -7389,7 +7389,7 @@
       </c>
       <c r="L92" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M92" s="3" t="inlineStr"/>
@@ -7445,7 +7445,7 @@
       </c>
       <c r="L93" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M93" s="3" t="inlineStr"/>
@@ -7505,7 +7505,7 @@
       </c>
       <c r="L94" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M94" s="3" t="inlineStr"/>
@@ -7565,7 +7565,7 @@
       </c>
       <c r="L95" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M95" s="3" t="inlineStr"/>
@@ -7625,7 +7625,7 @@
       </c>
       <c r="L96" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M96" s="3" t="inlineStr"/>
@@ -7685,7 +7685,7 @@
       </c>
       <c r="L97" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M97" s="3" t="inlineStr"/>
@@ -7745,7 +7745,7 @@
       </c>
       <c r="L98" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M98" s="3" t="inlineStr"/>
@@ -7805,7 +7805,7 @@
       </c>
       <c r="L99" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M99" s="3" t="inlineStr"/>
@@ -7865,7 +7865,7 @@
       </c>
       <c r="L100" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M100" s="3" t="inlineStr"/>
@@ -7925,7 +7925,7 @@
       </c>
       <c r="L101" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M101" s="3" t="inlineStr"/>
@@ -7985,7 +7985,7 @@
       </c>
       <c r="L102" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M102" s="3" t="inlineStr"/>
@@ -8105,7 +8105,7 @@
       </c>
       <c r="L104" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M104" s="3" t="inlineStr"/>
@@ -8165,7 +8165,7 @@
       </c>
       <c r="L105" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M105" s="3" t="inlineStr"/>
@@ -8225,7 +8225,7 @@
       </c>
       <c r="L106" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M106" s="3" t="inlineStr"/>
@@ -8285,7 +8285,7 @@
       </c>
       <c r="L107" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M107" s="3" t="inlineStr"/>
@@ -8401,7 +8401,7 @@
       </c>
       <c r="L109" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M109" s="3" t="inlineStr"/>
@@ -8461,7 +8461,7 @@
       </c>
       <c r="L110" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M110" s="3" t="inlineStr"/>
@@ -8521,7 +8521,7 @@
       </c>
       <c r="L111" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M111" s="3" t="inlineStr"/>
@@ -8581,7 +8581,7 @@
       </c>
       <c r="L112" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M112" s="3" t="inlineStr"/>
@@ -8641,7 +8641,7 @@
       </c>
       <c r="L113" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M113" s="3" t="inlineStr"/>
@@ -8697,7 +8697,7 @@
       </c>
       <c r="L114" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M114" s="3" t="inlineStr"/>
@@ -8757,7 +8757,7 @@
       </c>
       <c r="L115" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M115" s="3" t="inlineStr"/>
@@ -8813,7 +8813,7 @@
       </c>
       <c r="L116" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M116" s="3" t="inlineStr"/>
@@ -8869,7 +8869,7 @@
       </c>
       <c r="L117" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M117" s="3" t="inlineStr"/>
@@ -8929,7 +8929,7 @@
       </c>
       <c r="L118" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M118" s="3" t="inlineStr"/>
@@ -8989,7 +8989,7 @@
       </c>
       <c r="L119" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M119" s="3" t="inlineStr"/>
@@ -9049,7 +9049,7 @@
       </c>
       <c r="L120" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M120" s="3" t="inlineStr"/>
@@ -9109,7 +9109,7 @@
       </c>
       <c r="L121" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M121" s="3" t="inlineStr"/>
@@ -9169,7 +9169,7 @@
       </c>
       <c r="L122" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M122" s="3" t="inlineStr"/>
@@ -9229,7 +9229,7 @@
       </c>
       <c r="L123" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M123" s="3" t="inlineStr"/>
@@ -9289,7 +9289,7 @@
       </c>
       <c r="L124" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M124" s="3" t="inlineStr"/>
@@ -9349,7 +9349,7 @@
       </c>
       <c r="L125" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M125" s="3" t="inlineStr"/>
@@ -9409,7 +9409,7 @@
       </c>
       <c r="L126" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M126" s="3" t="inlineStr"/>
@@ -9469,7 +9469,7 @@
       </c>
       <c r="L127" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M127" s="3" t="inlineStr"/>
@@ -9529,7 +9529,7 @@
       </c>
       <c r="L128" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M128" s="3" t="inlineStr"/>
@@ -9589,7 +9589,7 @@
       </c>
       <c r="L129" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M129" s="3" t="inlineStr"/>
@@ -9649,7 +9649,7 @@
       </c>
       <c r="L130" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M130" s="3" t="inlineStr"/>
@@ -9709,7 +9709,7 @@
       </c>
       <c r="L131" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M131" s="3" t="inlineStr"/>
@@ -9769,7 +9769,7 @@
       </c>
       <c r="L132" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M132" s="3" t="inlineStr"/>
@@ -9829,7 +9829,7 @@
       </c>
       <c r="L133" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M133" s="3" t="inlineStr"/>
@@ -10061,7 +10061,7 @@
       </c>
       <c r="L137" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M137" s="3" t="inlineStr"/>
@@ -10121,7 +10121,7 @@
       </c>
       <c r="L138" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M138" s="3" t="inlineStr"/>
@@ -10181,7 +10181,7 @@
       </c>
       <c r="L139" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M139" s="3" t="inlineStr"/>
@@ -10241,7 +10241,7 @@
       </c>
       <c r="L140" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M140" s="3" t="inlineStr"/>
@@ -10409,7 +10409,7 @@
       </c>
       <c r="L143" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M143" s="3" t="inlineStr"/>
@@ -10697,7 +10697,7 @@
       </c>
       <c r="L148" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M148" s="3" t="inlineStr"/>
@@ -10817,7 +10817,7 @@
       </c>
       <c r="L150" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M150" s="3" t="inlineStr"/>
@@ -11081,7 +11081,7 @@
       </c>
       <c r="L155" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M155" s="3" t="inlineStr"/>
@@ -11197,7 +11197,7 @@
       </c>
       <c r="L157" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M157" s="3" t="inlineStr"/>
@@ -11257,7 +11257,7 @@
       </c>
       <c r="L158" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M158" s="3" t="inlineStr"/>
@@ -11317,7 +11317,7 @@
       </c>
       <c r="L159" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M159" s="3" t="inlineStr"/>
@@ -11487,7 +11487,7 @@
       </c>
       <c r="L162" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M162" s="3" t="inlineStr"/>
@@ -11543,7 +11543,7 @@
       </c>
       <c r="L163" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M163" s="3" t="inlineStr"/>
@@ -11603,7 +11603,7 @@
       </c>
       <c r="L164" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M164" s="3" t="inlineStr"/>
@@ -11663,7 +11663,7 @@
       </c>
       <c r="L165" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M165" s="3" t="inlineStr"/>
@@ -11773,7 +11773,7 @@
       </c>
       <c r="L167" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M167" s="3" t="inlineStr"/>
@@ -11833,7 +11833,7 @@
       </c>
       <c r="L168" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M168" s="3" t="inlineStr"/>
@@ -11889,7 +11889,7 @@
       </c>
       <c r="L169" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M169" s="3" t="inlineStr"/>
@@ -11949,7 +11949,7 @@
       </c>
       <c r="L170" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M170" s="3" t="inlineStr"/>
@@ -12129,7 +12129,7 @@
       </c>
       <c r="L173" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M173" s="3" t="inlineStr"/>
@@ -12189,7 +12189,7 @@
       </c>
       <c r="L174" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M174" s="3" t="inlineStr"/>
@@ -12305,7 +12305,7 @@
       </c>
       <c r="L176" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M176" s="3" t="inlineStr"/>
@@ -12365,7 +12365,7 @@
       </c>
       <c r="L177" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M177" s="3" t="inlineStr"/>
@@ -12421,7 +12421,7 @@
       </c>
       <c r="L178" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M178" s="3" t="inlineStr"/>
@@ -12481,7 +12481,7 @@
       </c>
       <c r="L179" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M179" s="3" t="inlineStr"/>
@@ -12541,7 +12541,7 @@
       </c>
       <c r="L180" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M180" s="3" t="inlineStr"/>
@@ -12597,7 +12597,7 @@
       </c>
       <c r="L181" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M181" s="3" t="inlineStr"/>
@@ -12653,7 +12653,7 @@
       </c>
       <c r="L182" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M182" s="3" t="inlineStr"/>
@@ -12705,7 +12705,7 @@
       </c>
       <c r="L183" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M183" s="3" t="inlineStr"/>
@@ -12877,7 +12877,7 @@
       </c>
       <c r="L186" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M186" s="3" t="inlineStr"/>
@@ -12933,7 +12933,7 @@
       </c>
       <c r="L187" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M187" s="3" t="inlineStr"/>
@@ -12989,7 +12989,7 @@
       </c>
       <c r="L188" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M188" s="3" t="inlineStr"/>
@@ -13045,7 +13045,7 @@
       </c>
       <c r="L189" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M189" s="3" t="inlineStr"/>
@@ -13105,7 +13105,7 @@
       </c>
       <c r="L190" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M190" s="3" t="inlineStr"/>
@@ -13225,7 +13225,7 @@
       </c>
       <c r="L192" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M192" s="3" t="inlineStr"/>
@@ -13285,7 +13285,7 @@
       </c>
       <c r="L193" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M193" s="3" t="inlineStr"/>
@@ -13401,7 +13401,7 @@
       </c>
       <c r="L195" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M195" s="3" t="inlineStr"/>
@@ -13461,7 +13461,7 @@
       </c>
       <c r="L196" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M196" s="3" t="inlineStr"/>
@@ -13521,7 +13521,7 @@
       </c>
       <c r="L197" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M197" s="3" t="inlineStr"/>
@@ -13581,7 +13581,7 @@
       </c>
       <c r="L198" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M198" s="3" t="inlineStr"/>
@@ -13641,7 +13641,7 @@
       </c>
       <c r="L199" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M199" s="3" t="inlineStr"/>
@@ -13701,7 +13701,7 @@
       </c>
       <c r="L200" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M200" s="3" t="inlineStr"/>
@@ -13821,7 +13821,7 @@
       </c>
       <c r="L202" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M202" s="3" t="inlineStr"/>
@@ -13881,7 +13881,7 @@
       </c>
       <c r="L203" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M203" s="3" t="inlineStr"/>
@@ -13941,7 +13941,7 @@
       </c>
       <c r="L204" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M204" s="3" t="inlineStr"/>
@@ -14001,7 +14001,7 @@
       </c>
       <c r="L205" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M205" s="3" t="inlineStr"/>
@@ -14061,7 +14061,7 @@
       </c>
       <c r="L206" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M206" s="3" t="inlineStr"/>
@@ -14121,7 +14121,7 @@
       </c>
       <c r="L207" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M207" s="3" t="inlineStr"/>
@@ -14181,7 +14181,7 @@
       </c>
       <c r="L208" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M208" s="3" t="inlineStr"/>
@@ -14305,7 +14305,7 @@
       </c>
       <c r="L210" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M210" s="3" t="inlineStr"/>
@@ -14423,7 +14423,7 @@
       </c>
       <c r="L212" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M212" s="3" t="inlineStr"/>
@@ -14483,7 +14483,7 @@
       </c>
       <c r="L213" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M213" s="3" t="inlineStr"/>
@@ -14597,7 +14597,7 @@
       </c>
       <c r="L215" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M215" s="3" t="inlineStr"/>
@@ -14713,7 +14713,7 @@
       </c>
       <c r="L217" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M217" s="3" t="inlineStr"/>
@@ -14765,7 +14765,7 @@
       </c>
       <c r="L218" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M218" s="3" t="inlineStr"/>
@@ -14817,7 +14817,7 @@
       </c>
       <c r="L219" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M219" s="3" t="inlineStr"/>
@@ -14927,7 +14927,7 @@
       </c>
       <c r="L221" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M221" s="3" t="inlineStr"/>
@@ -14987,7 +14987,7 @@
       </c>
       <c r="L222" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M222" s="3" t="inlineStr"/>
@@ -15155,7 +15155,7 @@
       </c>
       <c r="L225" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M225" s="3" t="inlineStr"/>
@@ -15263,7 +15263,7 @@
       </c>
       <c r="L227" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M227" s="3" t="inlineStr"/>
@@ -15323,7 +15323,7 @@
       </c>
       <c r="L228" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M228" s="3" t="inlineStr"/>
@@ -15383,7 +15383,7 @@
       </c>
       <c r="L229" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M229" s="3" t="inlineStr"/>
@@ -15443,7 +15443,7 @@
       </c>
       <c r="L230" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M230" s="3" t="inlineStr"/>
@@ -15499,7 +15499,7 @@
       </c>
       <c r="L231" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M231" s="3" t="inlineStr"/>
@@ -15559,7 +15559,7 @@
       </c>
       <c r="L232" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M232" s="3" t="inlineStr"/>
@@ -15619,7 +15619,7 @@
       </c>
       <c r="L233" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M233" s="3" t="inlineStr"/>
@@ -15679,7 +15679,7 @@
       </c>
       <c r="L234" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M234" s="3" t="inlineStr"/>
@@ -15799,7 +15799,7 @@
       </c>
       <c r="L236" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M236" s="3" t="inlineStr"/>
@@ -15859,7 +15859,7 @@
       </c>
       <c r="L237" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M237" s="3" t="inlineStr"/>
@@ -15919,7 +15919,7 @@
       </c>
       <c r="L238" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M238" s="3" t="inlineStr"/>
@@ -15975,7 +15975,7 @@
       </c>
       <c r="L239" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M239" s="3" t="inlineStr"/>
@@ -16199,7 +16199,7 @@
       </c>
       <c r="L243" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M243" s="3" t="inlineStr"/>
@@ -16311,7 +16311,7 @@
       </c>
       <c r="L245" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M245" s="3" t="inlineStr"/>
@@ -16367,7 +16367,7 @@
       </c>
       <c r="L246" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M246" s="3" t="inlineStr"/>
@@ -16427,7 +16427,7 @@
       </c>
       <c r="L247" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M247" s="3" t="inlineStr"/>
@@ -16541,7 +16541,7 @@
       </c>
       <c r="L249" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M249" s="3" t="inlineStr"/>
@@ -16597,7 +16597,7 @@
       </c>
       <c r="L250" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M250" s="3" t="inlineStr"/>
@@ -16657,7 +16657,7 @@
       </c>
       <c r="L251" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M251" s="3" t="inlineStr"/>
@@ -16717,7 +16717,7 @@
       </c>
       <c r="L252" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M252" s="3" t="inlineStr"/>
@@ -16777,7 +16777,7 @@
       </c>
       <c r="L253" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M253" s="3" t="inlineStr"/>
@@ -16837,7 +16837,7 @@
       </c>
       <c r="L254" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M254" s="3" t="inlineStr"/>
@@ -16897,7 +16897,7 @@
       </c>
       <c r="L255" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M255" s="3" t="inlineStr"/>
@@ -16957,7 +16957,7 @@
       </c>
       <c r="L256" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M256" s="3" t="inlineStr"/>
@@ -17017,7 +17017,7 @@
       </c>
       <c r="L257" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M257" s="3" t="inlineStr"/>
@@ -17077,7 +17077,7 @@
       </c>
       <c r="L258" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M258" s="3" t="inlineStr"/>
@@ -17137,7 +17137,7 @@
       </c>
       <c r="L259" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M259" s="3" t="inlineStr"/>
@@ -17197,7 +17197,7 @@
       </c>
       <c r="L260" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M260" s="3" t="inlineStr"/>
@@ -17257,7 +17257,7 @@
       </c>
       <c r="L261" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M261" s="3" t="inlineStr"/>
@@ -17313,7 +17313,7 @@
       </c>
       <c r="L262" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M262" s="3" t="inlineStr"/>
@@ -17373,7 +17373,7 @@
       </c>
       <c r="L263" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M263" s="3" t="inlineStr"/>
@@ -17497,7 +17497,7 @@
       </c>
       <c r="L265" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M265" s="3" t="inlineStr"/>
@@ -17617,7 +17617,7 @@
       </c>
       <c r="L267" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M267" s="3" t="inlineStr"/>
@@ -17677,7 +17677,7 @@
       </c>
       <c r="L268" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M268" s="3" t="inlineStr"/>
@@ -17797,7 +17797,7 @@
       </c>
       <c r="L270" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M270" s="3" t="inlineStr"/>
@@ -17857,7 +17857,7 @@
       </c>
       <c r="L271" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M271" s="3" t="inlineStr"/>
@@ -17917,7 +17917,7 @@
       </c>
       <c r="L272" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M272" s="3" t="inlineStr"/>
@@ -17973,7 +17973,7 @@
       </c>
       <c r="L273" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M273" s="3" t="inlineStr"/>
@@ -18033,7 +18033,7 @@
       </c>
       <c r="L274" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M274" s="3" t="inlineStr"/>
@@ -18213,7 +18213,7 @@
       </c>
       <c r="L277" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M277" s="3" t="inlineStr"/>
@@ -18273,7 +18273,7 @@
       </c>
       <c r="L278" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M278" s="3" t="inlineStr"/>
@@ -18333,7 +18333,7 @@
       </c>
       <c r="L279" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M279" s="3" t="inlineStr"/>
@@ -18393,7 +18393,7 @@
       </c>
       <c r="L280" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M280" s="3" t="inlineStr"/>
@@ -18453,7 +18453,7 @@
       </c>
       <c r="L281" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M281" s="3" t="inlineStr"/>
@@ -18513,7 +18513,7 @@
       </c>
       <c r="L282" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M282" s="3" t="inlineStr"/>
@@ -18573,7 +18573,7 @@
       </c>
       <c r="L283" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M283" s="3" t="inlineStr"/>
@@ -18633,7 +18633,7 @@
       </c>
       <c r="L284" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M284" s="3" t="inlineStr"/>
@@ -18693,7 +18693,7 @@
       </c>
       <c r="L285" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M285" s="3" t="inlineStr"/>
@@ -18753,7 +18753,7 @@
       </c>
       <c r="L286" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M286" s="3" t="inlineStr"/>
@@ -18813,7 +18813,7 @@
       </c>
       <c r="L287" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M287" s="3" t="inlineStr"/>
@@ -18865,7 +18865,7 @@
       </c>
       <c r="L288" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M288" s="3" t="inlineStr"/>
@@ -18925,7 +18925,7 @@
       </c>
       <c r="L289" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M289" s="3" t="inlineStr"/>
@@ -18985,7 +18985,7 @@
       </c>
       <c r="L290" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M290" s="3" t="inlineStr"/>
@@ -19045,7 +19045,7 @@
       </c>
       <c r="L291" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M291" s="3" t="inlineStr"/>
@@ -19157,7 +19157,7 @@
       </c>
       <c r="L293" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M293" s="3" t="inlineStr"/>
@@ -19217,7 +19217,7 @@
       </c>
       <c r="L294" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M294" s="3" t="inlineStr"/>
@@ -19277,7 +19277,7 @@
       </c>
       <c r="L295" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M295" s="3" t="inlineStr"/>
@@ -19337,7 +19337,7 @@
       </c>
       <c r="L296" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M296" s="3" t="inlineStr"/>
@@ -19509,7 +19509,7 @@
       </c>
       <c r="L299" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M299" s="3" t="inlineStr"/>
@@ -19569,7 +19569,7 @@
       </c>
       <c r="L300" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M300" s="3" t="inlineStr"/>
@@ -19629,7 +19629,7 @@
       </c>
       <c r="L301" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M301" s="3" t="inlineStr"/>
@@ -19747,7 +19747,7 @@
       </c>
       <c r="L303" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M303" s="3" t="inlineStr"/>
@@ -19807,7 +19807,7 @@
       </c>
       <c r="L304" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M304" s="3" t="inlineStr"/>
@@ -19867,7 +19867,7 @@
       </c>
       <c r="L305" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M305" s="3" t="inlineStr"/>
@@ -19927,7 +19927,7 @@
       </c>
       <c r="L306" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M306" s="3" t="inlineStr"/>
@@ -19987,7 +19987,7 @@
       </c>
       <c r="L307" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M307" s="3" t="inlineStr"/>
@@ -20047,7 +20047,7 @@
       </c>
       <c r="L308" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M308" s="3" t="inlineStr"/>
@@ -20107,7 +20107,7 @@
       </c>
       <c r="L309" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M309" s="3" t="inlineStr"/>
@@ -20167,7 +20167,7 @@
       </c>
       <c r="L310" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M310" s="3" t="inlineStr"/>
@@ -20223,7 +20223,7 @@
       </c>
       <c r="L311" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M311" s="3" t="inlineStr"/>
@@ -20435,7 +20435,7 @@
       <c r="G315" s="3" t="inlineStr"/>
       <c r="H315" s="3" t="inlineStr">
         <is>
-          <t>2.53 oygacha</t>
+          <t>2.5 oygacha</t>
         </is>
       </c>
       <c r="I315" s="3" t="inlineStr"/>
@@ -20451,7 +20451,7 @@
       </c>
       <c r="L315" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M315" s="3" t="inlineStr"/>
@@ -20847,7 +20847,7 @@
       </c>
       <c r="L322" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M322" s="3" t="inlineStr"/>
@@ -20907,7 +20907,7 @@
       </c>
       <c r="L323" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M323" s="3" t="inlineStr"/>
@@ -20967,7 +20967,7 @@
       </c>
       <c r="L324" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M324" s="3" t="inlineStr"/>
@@ -21027,7 +21027,7 @@
       </c>
       <c r="L325" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M325" s="3" t="inlineStr"/>
@@ -21207,7 +21207,7 @@
       </c>
       <c r="L328" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M328" s="3" t="inlineStr"/>
@@ -21267,7 +21267,7 @@
       </c>
       <c r="L329" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M329" s="3" t="inlineStr"/>
@@ -21327,7 +21327,7 @@
       </c>
       <c r="L330" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M330" s="3" t="inlineStr"/>
@@ -21387,7 +21387,7 @@
       </c>
       <c r="L331" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M331" s="3" t="inlineStr"/>
@@ -21447,7 +21447,7 @@
       </c>
       <c r="L332" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M332" s="3" t="inlineStr"/>
@@ -21507,7 +21507,7 @@
       </c>
       <c r="L333" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M333" s="3" t="inlineStr"/>
@@ -21567,7 +21567,7 @@
       </c>
       <c r="L334" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M334" s="3" t="inlineStr"/>
@@ -21683,7 +21683,7 @@
       </c>
       <c r="L336" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M336" s="3" t="inlineStr"/>
@@ -21743,7 +21743,7 @@
       </c>
       <c r="L337" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M337" s="3" t="inlineStr"/>
@@ -21803,7 +21803,7 @@
       </c>
       <c r="L338" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M338" s="3" t="inlineStr"/>
@@ -21863,7 +21863,7 @@
       </c>
       <c r="L339" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M339" s="3" t="inlineStr"/>
@@ -21923,7 +21923,7 @@
       </c>
       <c r="L340" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M340" s="3" t="inlineStr"/>
@@ -21983,7 +21983,7 @@
       </c>
       <c r="L341" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M341" s="3" t="inlineStr"/>
@@ -22043,7 +22043,7 @@
       </c>
       <c r="L342" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M342" s="3" t="inlineStr"/>
@@ -22099,7 +22099,7 @@
       </c>
       <c r="L343" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M343" s="3" t="inlineStr"/>
@@ -22155,7 +22155,7 @@
       </c>
       <c r="L344" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M344" s="3" t="inlineStr"/>
@@ -22215,7 +22215,7 @@
       </c>
       <c r="L345" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M345" s="3" t="inlineStr"/>
@@ -22275,7 +22275,7 @@
       </c>
       <c r="L346" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M346" s="3" t="inlineStr"/>
@@ -22335,7 +22335,7 @@
       </c>
       <c r="L347" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M347" s="3" t="inlineStr"/>
@@ -22447,7 +22447,7 @@
       </c>
       <c r="L349" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M349" s="3" t="inlineStr"/>
@@ -22507,7 +22507,7 @@
       </c>
       <c r="L350" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M350" s="3" t="inlineStr"/>
@@ -22567,7 +22567,7 @@
       </c>
       <c r="L351" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M351" s="3" t="inlineStr"/>
@@ -22627,7 +22627,7 @@
       </c>
       <c r="L352" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M352" s="3" t="inlineStr"/>
@@ -22747,7 +22747,7 @@
       </c>
       <c r="L354" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M354" s="3" t="inlineStr"/>
@@ -22807,7 +22807,7 @@
       </c>
       <c r="L355" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M355" s="3" t="inlineStr"/>
@@ -22867,7 +22867,7 @@
       </c>
       <c r="L356" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M356" s="3" t="inlineStr"/>
@@ -22983,7 +22983,7 @@
       </c>
       <c r="L358" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M358" s="3" t="inlineStr"/>
@@ -23097,7 +23097,7 @@
       </c>
       <c r="L360" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M360" s="3" t="inlineStr"/>
@@ -23153,7 +23153,7 @@
       </c>
       <c r="L361" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M361" s="3" t="inlineStr"/>
@@ -23265,7 +23265,7 @@
       </c>
       <c r="L363" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M363" s="3" t="inlineStr"/>
@@ -23321,7 +23321,7 @@
       </c>
       <c r="L364" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M364" s="3" t="inlineStr"/>
@@ -23377,7 +23377,7 @@
       </c>
       <c r="L365" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M365" s="3" t="inlineStr"/>
@@ -23489,7 +23489,7 @@
       </c>
       <c r="L367" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M367" s="3" t="inlineStr"/>
@@ -23601,7 +23601,7 @@
       </c>
       <c r="L369" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M369" s="3" t="inlineStr"/>
@@ -23717,7 +23717,7 @@
       </c>
       <c r="L371" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M371" s="3" t="inlineStr"/>
@@ -23773,7 +23773,7 @@
       </c>
       <c r="L372" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M372" s="3" t="inlineStr"/>
@@ -23829,7 +23829,7 @@
       </c>
       <c r="L373" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M373" s="3" t="inlineStr"/>
@@ -23885,7 +23885,7 @@
       </c>
       <c r="L374" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M374" s="3" t="inlineStr"/>
@@ -23941,7 +23941,7 @@
       </c>
       <c r="L375" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M375" s="3" t="inlineStr"/>
@@ -23997,7 +23997,7 @@
       </c>
       <c r="L376" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M376" s="3" t="inlineStr"/>
@@ -24053,7 +24053,7 @@
       </c>
       <c r="L377" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M377" s="3" t="inlineStr"/>
@@ -24109,7 +24109,7 @@
       </c>
       <c r="L378" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M378" s="3" t="inlineStr"/>
@@ -24165,7 +24165,7 @@
       </c>
       <c r="L379" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M379" s="3" t="inlineStr"/>
@@ -24221,7 +24221,7 @@
       </c>
       <c r="L380" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M380" s="3" t="inlineStr"/>
@@ -24277,7 +24277,7 @@
       </c>
       <c r="L381" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M381" s="3" t="inlineStr"/>
@@ -24333,7 +24333,7 @@
       </c>
       <c r="L382" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M382" s="3" t="inlineStr"/>
@@ -24389,7 +24389,7 @@
       </c>
       <c r="L383" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M383" s="3" t="inlineStr"/>
@@ -24449,7 +24449,7 @@
       </c>
       <c r="L384" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M384" s="3" t="inlineStr"/>
@@ -24509,7 +24509,7 @@
       </c>
       <c r="L385" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M385" s="3" t="inlineStr"/>
@@ -24569,7 +24569,7 @@
       </c>
       <c r="L386" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M386" s="3" t="inlineStr"/>
@@ -24789,7 +24789,7 @@
       </c>
       <c r="L390" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M390" s="3" t="inlineStr"/>
@@ -24845,7 +24845,7 @@
       </c>
       <c r="L391" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M391" s="3" t="inlineStr"/>
@@ -24901,7 +24901,7 @@
       </c>
       <c r="L392" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M392" s="3" t="inlineStr"/>
@@ -25021,7 +25021,7 @@
       </c>
       <c r="L394" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M394" s="3" t="inlineStr"/>
@@ -25077,7 +25077,7 @@
       </c>
       <c r="L395" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M395" s="3" t="inlineStr"/>
@@ -25309,7 +25309,7 @@
       </c>
       <c r="L399" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M399" s="3" t="inlineStr"/>
@@ -25365,7 +25365,7 @@
       </c>
       <c r="L400" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M400" s="3" t="inlineStr"/>
@@ -25425,7 +25425,7 @@
       </c>
       <c r="L401" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M401" s="3" t="inlineStr"/>
@@ -25537,7 +25537,7 @@
       </c>
       <c r="L403" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M403" s="3" t="inlineStr"/>
@@ -25593,7 +25593,7 @@
       </c>
       <c r="L404" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M404" s="3" t="inlineStr"/>
@@ -25649,7 +25649,7 @@
       </c>
       <c r="L405" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M405" s="3" t="inlineStr"/>
@@ -25705,7 +25705,7 @@
       </c>
       <c r="L406" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M406" s="3" t="inlineStr"/>
@@ -25761,7 +25761,7 @@
       </c>
       <c r="L407" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M407" s="3" t="inlineStr"/>
@@ -25817,7 +25817,7 @@
       </c>
       <c r="L408" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M408" s="3" t="inlineStr"/>
@@ -25873,7 +25873,7 @@
       </c>
       <c r="L409" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M409" s="3" t="inlineStr"/>
@@ -25981,7 +25981,7 @@
       </c>
       <c r="L411" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M411" s="3" t="inlineStr"/>
@@ -26041,7 +26041,7 @@
       </c>
       <c r="L412" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M412" s="3" t="inlineStr"/>
@@ -26101,7 +26101,7 @@
       </c>
       <c r="L413" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M413" s="3" t="inlineStr"/>
@@ -26217,7 +26217,7 @@
       </c>
       <c r="L415" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M415" s="3" t="inlineStr"/>
@@ -26385,7 +26385,7 @@
       </c>
       <c r="L418" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M418" s="3" t="inlineStr"/>
@@ -26445,7 +26445,7 @@
       </c>
       <c r="L419" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M419" s="3" t="inlineStr"/>
@@ -26505,7 +26505,7 @@
       </c>
       <c r="L420" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M420" s="3" t="inlineStr"/>
@@ -26565,7 +26565,7 @@
       </c>
       <c r="L421" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M421" s="3" t="inlineStr"/>
@@ -26901,7 +26901,7 @@
       </c>
       <c r="L427" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M427" s="3" t="inlineStr"/>
@@ -26961,7 +26961,7 @@
       </c>
       <c r="L428" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M428" s="3" t="inlineStr"/>
@@ -27021,7 +27021,7 @@
       </c>
       <c r="L429" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M429" s="3" t="inlineStr"/>
@@ -27081,7 +27081,7 @@
       </c>
       <c r="L430" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M430" s="3" t="inlineStr"/>
@@ -27137,7 +27137,7 @@
       </c>
       <c r="L431" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M431" s="3" t="inlineStr"/>
@@ -27377,7 +27377,7 @@
       </c>
       <c r="L435" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M435" s="3" t="inlineStr"/>
@@ -27437,7 +27437,7 @@
       </c>
       <c r="L436" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M436" s="3" t="inlineStr"/>
@@ -27549,7 +27549,7 @@
       </c>
       <c r="L438" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M438" s="3" t="inlineStr"/>
@@ -27605,7 +27605,7 @@
       </c>
       <c r="L439" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M439" s="3" t="inlineStr"/>
@@ -27661,7 +27661,7 @@
       </c>
       <c r="L440" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M440" s="3" t="inlineStr"/>
@@ -27717,7 +27717,7 @@
       </c>
       <c r="L441" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M441" s="3" t="inlineStr"/>
@@ -27773,7 +27773,7 @@
       </c>
       <c r="L442" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M442" s="3" t="inlineStr"/>
@@ -27833,7 +27833,7 @@
       </c>
       <c r="L443" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M443" s="3" t="inlineStr"/>
@@ -27893,7 +27893,7 @@
       </c>
       <c r="L444" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M444" s="3" t="inlineStr"/>
@@ -28129,7 +28129,7 @@
       </c>
       <c r="L448" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M448" s="3" t="inlineStr"/>
@@ -28185,7 +28185,7 @@
       </c>
       <c r="L449" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M449" s="3" t="inlineStr"/>
@@ -28241,7 +28241,7 @@
       </c>
       <c r="L450" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M450" s="3" t="inlineStr"/>
@@ -28297,7 +28297,7 @@
       </c>
       <c r="L451" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M451" s="3" t="inlineStr"/>
@@ -28413,7 +28413,7 @@
       </c>
       <c r="L453" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M453" s="3" t="inlineStr"/>

</xml_diff>

<commit_message>
Ma'lumot avtomatik yangilandi (2026-10-18)
</commit_message>
<xml_diff>
--- a/docs/banklar_kreditlar.xlsx
+++ b/docs/banklar_kreditlar.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Izoh" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Kreditlar'!$A$1:$N$461</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Kreditlar'!$A$1:$N$449</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Banklar xulosasi'!$A$1:$G$31</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Izoh'!$A$1:$A$9</definedName>
   </definedNames>
@@ -2028,7 +2028,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N461"/>
+  <dimension ref="A1:N449"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -2223,7 +2223,7 @@
       </c>
       <c r="L3" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M3" s="3" t="inlineStr"/>
@@ -2283,7 +2283,7 @@
       </c>
       <c r="L4" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M4" s="3" t="inlineStr"/>
@@ -2343,7 +2343,7 @@
       </c>
       <c r="L5" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M5" s="3" t="inlineStr"/>
@@ -2403,7 +2403,7 @@
       </c>
       <c r="L6" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M6" s="3" t="inlineStr"/>
@@ -2463,7 +2463,7 @@
       </c>
       <c r="L7" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M7" s="3" t="inlineStr"/>
@@ -2523,7 +2523,7 @@
       </c>
       <c r="L8" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M8" s="3" t="inlineStr"/>
@@ -2639,7 +2639,7 @@
       </c>
       <c r="L10" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M10" s="3" t="inlineStr"/>
@@ -2699,7 +2699,7 @@
       </c>
       <c r="L11" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M11" s="3" t="inlineStr"/>
@@ -2815,7 +2815,7 @@
       </c>
       <c r="L13" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M13" s="3" t="inlineStr"/>
@@ -2875,7 +2875,7 @@
       </c>
       <c r="L14" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M14" s="3" t="inlineStr"/>
@@ -2935,7 +2935,7 @@
       </c>
       <c r="L15" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M15" s="3" t="inlineStr"/>
@@ -3047,7 +3047,7 @@
       </c>
       <c r="L17" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M17" s="3" t="inlineStr"/>
@@ -3107,7 +3107,7 @@
       </c>
       <c r="L18" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M18" s="3" t="inlineStr"/>
@@ -3223,7 +3223,7 @@
       </c>
       <c r="L20" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M20" s="3" t="inlineStr"/>
@@ -3283,7 +3283,7 @@
       </c>
       <c r="L21" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M21" s="3" t="inlineStr"/>
@@ -3343,7 +3343,7 @@
       </c>
       <c r="L22" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M22" s="3" t="inlineStr"/>
@@ -3403,7 +3403,7 @@
       </c>
       <c r="L23" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M23" s="3" t="inlineStr"/>
@@ -3463,7 +3463,7 @@
       </c>
       <c r="L24" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M24" s="3" t="inlineStr"/>
@@ -3631,7 +3631,7 @@
       </c>
       <c r="L27" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M27" s="3" t="inlineStr"/>
@@ -3691,7 +3691,7 @@
       </c>
       <c r="L28" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M28" s="3" t="inlineStr"/>
@@ -3751,7 +3751,7 @@
       </c>
       <c r="L29" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M29" s="3" t="inlineStr"/>
@@ -3811,7 +3811,7 @@
       </c>
       <c r="L30" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M30" s="3" t="inlineStr"/>
@@ -3871,7 +3871,7 @@
       </c>
       <c r="L31" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M31" s="3" t="inlineStr"/>
@@ -3931,7 +3931,7 @@
       </c>
       <c r="L32" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M32" s="3" t="inlineStr"/>
@@ -3991,7 +3991,7 @@
       </c>
       <c r="L33" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M33" s="3" t="inlineStr"/>
@@ -4051,7 +4051,7 @@
       </c>
       <c r="L34" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M34" s="3" t="inlineStr"/>
@@ -4111,7 +4111,7 @@
       </c>
       <c r="L35" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M35" s="3" t="inlineStr"/>
@@ -4171,7 +4171,7 @@
       </c>
       <c r="L36" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M36" s="3" t="inlineStr"/>
@@ -4227,7 +4227,7 @@
       </c>
       <c r="L37" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M37" s="3" t="inlineStr"/>
@@ -4339,7 +4339,7 @@
       </c>
       <c r="L39" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M39" s="3" t="inlineStr"/>
@@ -4395,7 +4395,7 @@
       </c>
       <c r="L40" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M40" s="3" t="inlineStr"/>
@@ -4451,7 +4451,7 @@
       </c>
       <c r="L41" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M41" s="3" t="inlineStr"/>
@@ -4507,7 +4507,7 @@
       </c>
       <c r="L42" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M42" s="3" t="inlineStr"/>
@@ -4567,7 +4567,7 @@
       </c>
       <c r="L43" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M43" s="3" t="inlineStr"/>
@@ -4627,7 +4627,7 @@
       </c>
       <c r="L44" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M44" s="3" t="inlineStr"/>
@@ -4687,7 +4687,7 @@
       </c>
       <c r="L45" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M45" s="3" t="inlineStr"/>
@@ -4743,7 +4743,7 @@
       </c>
       <c r="L46" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M46" s="3" t="inlineStr"/>
@@ -4799,7 +4799,7 @@
       </c>
       <c r="L47" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M47" s="3" t="inlineStr"/>
@@ -4859,7 +4859,7 @@
       </c>
       <c r="L48" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M48" s="3" t="inlineStr"/>
@@ -4919,7 +4919,7 @@
       </c>
       <c r="L49" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M49" s="3" t="inlineStr"/>
@@ -4979,7 +4979,7 @@
       </c>
       <c r="L50" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M50" s="3" t="inlineStr"/>
@@ -5093,7 +5093,7 @@
       </c>
       <c r="L52" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M52" s="3" t="inlineStr"/>
@@ -5153,7 +5153,7 @@
       </c>
       <c r="L53" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M53" s="3" t="inlineStr"/>
@@ -5213,7 +5213,7 @@
       </c>
       <c r="L54" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M54" s="3" t="inlineStr"/>
@@ -5273,7 +5273,7 @@
       </c>
       <c r="L55" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M55" s="3" t="inlineStr"/>
@@ -5333,7 +5333,7 @@
       </c>
       <c r="L56" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M56" s="3" t="inlineStr"/>
@@ -5445,7 +5445,7 @@
       </c>
       <c r="L58" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M58" s="3" t="inlineStr"/>
@@ -5501,7 +5501,7 @@
       </c>
       <c r="L59" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M59" s="3" t="inlineStr"/>
@@ -6257,7 +6257,7 @@
       </c>
       <c r="L72" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M72" s="3" t="inlineStr"/>
@@ -6369,7 +6369,7 @@
       </c>
       <c r="L74" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M74" s="3" t="inlineStr"/>
@@ -6481,7 +6481,7 @@
       </c>
       <c r="L76" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M76" s="3" t="inlineStr"/>
@@ -6537,7 +6537,7 @@
       </c>
       <c r="L77" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M77" s="3" t="inlineStr"/>
@@ -6593,7 +6593,7 @@
       </c>
       <c r="L78" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M78" s="3" t="inlineStr"/>
@@ -6649,7 +6649,7 @@
       </c>
       <c r="L79" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M79" s="3" t="inlineStr"/>
@@ -6705,7 +6705,7 @@
       </c>
       <c r="L80" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M80" s="3" t="inlineStr"/>
@@ -6761,7 +6761,7 @@
       </c>
       <c r="L81" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M81" s="3" t="inlineStr"/>
@@ -6817,7 +6817,7 @@
       </c>
       <c r="L82" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M82" s="3" t="inlineStr"/>
@@ -6869,7 +6869,7 @@
       </c>
       <c r="L83" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M83" s="3" t="inlineStr"/>
@@ -6929,7 +6929,7 @@
       </c>
       <c r="L84" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M84" s="3" t="inlineStr"/>
@@ -6989,7 +6989,7 @@
       </c>
       <c r="L85" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M85" s="3" t="inlineStr"/>
@@ -7049,7 +7049,7 @@
       </c>
       <c r="L86" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M86" s="3" t="inlineStr"/>
@@ -7109,7 +7109,7 @@
       </c>
       <c r="L87" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M87" s="3" t="inlineStr"/>
@@ -7169,7 +7169,7 @@
       </c>
       <c r="L88" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M88" s="3" t="inlineStr"/>
@@ -7225,7 +7225,7 @@
       </c>
       <c r="L89" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M89" s="3" t="inlineStr"/>
@@ -7277,7 +7277,7 @@
       </c>
       <c r="L90" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M90" s="3" t="inlineStr"/>
@@ -7389,7 +7389,7 @@
       </c>
       <c r="L92" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M92" s="3" t="inlineStr"/>
@@ -7445,7 +7445,7 @@
       </c>
       <c r="L93" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M93" s="3" t="inlineStr"/>
@@ -7505,7 +7505,7 @@
       </c>
       <c r="L94" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M94" s="3" t="inlineStr"/>
@@ -7565,7 +7565,7 @@
       </c>
       <c r="L95" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M95" s="3" t="inlineStr"/>
@@ -7625,7 +7625,7 @@
       </c>
       <c r="L96" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M96" s="3" t="inlineStr"/>
@@ -7685,7 +7685,7 @@
       </c>
       <c r="L97" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M97" s="3" t="inlineStr"/>
@@ -7745,7 +7745,7 @@
       </c>
       <c r="L98" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M98" s="3" t="inlineStr"/>
@@ -7805,7 +7805,7 @@
       </c>
       <c r="L99" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M99" s="3" t="inlineStr"/>
@@ -7865,7 +7865,7 @@
       </c>
       <c r="L100" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M100" s="3" t="inlineStr"/>
@@ -7985,7 +7985,7 @@
       </c>
       <c r="L102" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M102" s="3" t="inlineStr"/>
@@ -8045,7 +8045,7 @@
       </c>
       <c r="L103" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M103" s="3" t="inlineStr"/>
@@ -8105,7 +8105,7 @@
       </c>
       <c r="L104" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M104" s="3" t="inlineStr"/>
@@ -8165,7 +8165,7 @@
       </c>
       <c r="L105" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M105" s="3" t="inlineStr"/>
@@ -8281,7 +8281,7 @@
       </c>
       <c r="L107" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M107" s="3" t="inlineStr"/>
@@ -8341,7 +8341,7 @@
       </c>
       <c r="L108" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M108" s="3" t="inlineStr"/>
@@ -8401,7 +8401,7 @@
       </c>
       <c r="L109" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M109" s="3" t="inlineStr"/>
@@ -8461,7 +8461,7 @@
       </c>
       <c r="L110" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M110" s="3" t="inlineStr"/>
@@ -8521,7 +8521,7 @@
       </c>
       <c r="L111" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M111" s="3" t="inlineStr"/>
@@ -8581,7 +8581,7 @@
       </c>
       <c r="L112" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M112" s="3" t="inlineStr"/>
@@ -8637,7 +8637,7 @@
       </c>
       <c r="L113" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M113" s="3" t="inlineStr"/>
@@ -8693,7 +8693,7 @@
       </c>
       <c r="L114" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M114" s="3" t="inlineStr"/>
@@ -8749,7 +8749,7 @@
       </c>
       <c r="L115" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M115" s="3" t="inlineStr"/>
@@ -8809,7 +8809,7 @@
       </c>
       <c r="L116" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M116" s="3" t="inlineStr"/>
@@ -8869,7 +8869,7 @@
       </c>
       <c r="L117" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M117" s="3" t="inlineStr"/>
@@ -8929,7 +8929,7 @@
       </c>
       <c r="L118" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M118" s="3" t="inlineStr"/>
@@ -8989,7 +8989,7 @@
       </c>
       <c r="L119" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M119" s="3" t="inlineStr"/>
@@ -9049,7 +9049,7 @@
       </c>
       <c r="L120" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M120" s="3" t="inlineStr"/>
@@ -9109,7 +9109,7 @@
       </c>
       <c r="L121" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M121" s="3" t="inlineStr"/>
@@ -9169,7 +9169,7 @@
       </c>
       <c r="L122" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M122" s="3" t="inlineStr"/>
@@ -9229,7 +9229,7 @@
       </c>
       <c r="L123" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M123" s="3" t="inlineStr"/>
@@ -9289,7 +9289,7 @@
       </c>
       <c r="L124" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M124" s="3" t="inlineStr"/>
@@ -9349,7 +9349,7 @@
       </c>
       <c r="L125" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M125" s="3" t="inlineStr"/>
@@ -9409,7 +9409,7 @@
       </c>
       <c r="L126" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M126" s="3" t="inlineStr"/>
@@ -9469,7 +9469,7 @@
       </c>
       <c r="L127" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M127" s="3" t="inlineStr"/>
@@ -9529,7 +9529,7 @@
       </c>
       <c r="L128" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M128" s="3" t="inlineStr"/>
@@ -9589,7 +9589,7 @@
       </c>
       <c r="L129" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M129" s="3" t="inlineStr"/>
@@ -9821,7 +9821,7 @@
       </c>
       <c r="L133" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M133" s="3" t="inlineStr"/>
@@ -9881,7 +9881,7 @@
       </c>
       <c r="L134" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M134" s="3" t="inlineStr"/>
@@ -9941,7 +9941,7 @@
       </c>
       <c r="L135" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M135" s="3" t="inlineStr"/>
@@ -10001,7 +10001,7 @@
       </c>
       <c r="L136" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M136" s="3" t="inlineStr"/>
@@ -10169,7 +10169,7 @@
       </c>
       <c r="L139" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M139" s="3" t="inlineStr"/>
@@ -10457,7 +10457,7 @@
       </c>
       <c r="L144" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M144" s="3" t="inlineStr"/>
@@ -10577,7 +10577,7 @@
       </c>
       <c r="L146" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M146" s="3" t="inlineStr"/>
@@ -10841,7 +10841,7 @@
       </c>
       <c r="L151" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M151" s="3" t="inlineStr"/>
@@ -10957,7 +10957,7 @@
       </c>
       <c r="L153" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M153" s="3" t="inlineStr"/>
@@ -11017,7 +11017,7 @@
       </c>
       <c r="L154" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M154" s="3" t="inlineStr"/>
@@ -11077,7 +11077,7 @@
       </c>
       <c r="L155" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M155" s="3" t="inlineStr"/>
@@ -11247,7 +11247,7 @@
       </c>
       <c r="L158" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M158" s="3" t="inlineStr"/>
@@ -11303,7 +11303,7 @@
       </c>
       <c r="L159" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M159" s="3" t="inlineStr"/>
@@ -11363,7 +11363,7 @@
       </c>
       <c r="L160" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M160" s="3" t="inlineStr"/>
@@ -11423,7 +11423,7 @@
       </c>
       <c r="L161" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M161" s="3" t="inlineStr"/>
@@ -11533,7 +11533,7 @@
       </c>
       <c r="L163" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M163" s="3" t="inlineStr"/>
@@ -11593,7 +11593,7 @@
       </c>
       <c r="L164" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M164" s="3" t="inlineStr"/>
@@ -11649,7 +11649,7 @@
       </c>
       <c r="L165" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M165" s="3" t="inlineStr"/>
@@ -11709,7 +11709,7 @@
       </c>
       <c r="L166" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M166" s="3" t="inlineStr"/>
@@ -11889,7 +11889,7 @@
       </c>
       <c r="L169" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M169" s="3" t="inlineStr"/>
@@ -11949,7 +11949,7 @@
       </c>
       <c r="L170" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M170" s="3" t="inlineStr"/>
@@ -12065,7 +12065,7 @@
       </c>
       <c r="L172" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M172" s="3" t="inlineStr"/>
@@ -12125,7 +12125,7 @@
       </c>
       <c r="L173" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M173" s="3" t="inlineStr"/>
@@ -12181,7 +12181,7 @@
       </c>
       <c r="L174" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M174" s="3" t="inlineStr"/>
@@ -12241,7 +12241,7 @@
       </c>
       <c r="L175" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M175" s="3" t="inlineStr"/>
@@ -12301,7 +12301,7 @@
       </c>
       <c r="L176" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M176" s="3" t="inlineStr"/>
@@ -12357,7 +12357,7 @@
       </c>
       <c r="L177" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M177" s="3" t="inlineStr"/>
@@ -12413,7 +12413,7 @@
       </c>
       <c r="L178" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M178" s="3" t="inlineStr"/>
@@ -12465,7 +12465,7 @@
       </c>
       <c r="L179" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M179" s="3" t="inlineStr"/>
@@ -12637,7 +12637,7 @@
       </c>
       <c r="L182" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M182" s="3" t="inlineStr"/>
@@ -12693,7 +12693,7 @@
       </c>
       <c r="L183" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M183" s="3" t="inlineStr"/>
@@ -12749,7 +12749,7 @@
       </c>
       <c r="L184" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M184" s="3" t="inlineStr"/>
@@ -12805,7 +12805,7 @@
       </c>
       <c r="L185" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M185" s="3" t="inlineStr"/>
@@ -12865,7 +12865,7 @@
       </c>
       <c r="L186" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M186" s="3" t="inlineStr"/>
@@ -12985,7 +12985,7 @@
       </c>
       <c r="L188" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M188" s="3" t="inlineStr"/>
@@ -13045,7 +13045,7 @@
       </c>
       <c r="L189" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M189" s="3" t="inlineStr"/>
@@ -13161,7 +13161,7 @@
       </c>
       <c r="L191" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M191" s="3" t="inlineStr"/>
@@ -13221,7 +13221,7 @@
       </c>
       <c r="L192" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M192" s="3" t="inlineStr"/>
@@ -13281,7 +13281,7 @@
       </c>
       <c r="L193" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M193" s="3" t="inlineStr"/>
@@ -13341,7 +13341,7 @@
       </c>
       <c r="L194" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M194" s="3" t="inlineStr"/>
@@ -13401,7 +13401,7 @@
       </c>
       <c r="L195" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M195" s="3" t="inlineStr"/>
@@ -13461,7 +13461,7 @@
       </c>
       <c r="L196" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M196" s="3" t="inlineStr"/>
@@ -13581,7 +13581,7 @@
       </c>
       <c r="L198" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M198" s="3" t="inlineStr"/>
@@ -13641,7 +13641,7 @@
       </c>
       <c r="L199" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M199" s="3" t="inlineStr"/>
@@ -13701,7 +13701,7 @@
       </c>
       <c r="L200" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M200" s="3" t="inlineStr"/>
@@ -13761,7 +13761,7 @@
       </c>
       <c r="L201" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M201" s="3" t="inlineStr"/>
@@ -13821,7 +13821,7 @@
       </c>
       <c r="L202" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M202" s="3" t="inlineStr"/>
@@ -13881,7 +13881,7 @@
       </c>
       <c r="L203" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M203" s="3" t="inlineStr"/>
@@ -13941,7 +13941,7 @@
       </c>
       <c r="L204" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M204" s="3" t="inlineStr"/>
@@ -14065,7 +14065,7 @@
       </c>
       <c r="L206" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M206" s="3" t="inlineStr"/>
@@ -14183,7 +14183,7 @@
       </c>
       <c r="L208" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M208" s="3" t="inlineStr"/>
@@ -14243,7 +14243,7 @@
       </c>
       <c r="L209" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M209" s="3" t="inlineStr"/>
@@ -14357,7 +14357,7 @@
       </c>
       <c r="L211" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M211" s="3" t="inlineStr"/>
@@ -14473,7 +14473,7 @@
       </c>
       <c r="L213" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M213" s="3" t="inlineStr"/>
@@ -14525,7 +14525,7 @@
       </c>
       <c r="L214" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M214" s="3" t="inlineStr"/>
@@ -14577,7 +14577,7 @@
       </c>
       <c r="L215" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M215" s="3" t="inlineStr"/>
@@ -14687,7 +14687,7 @@
       </c>
       <c r="L217" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M217" s="3" t="inlineStr"/>
@@ -14747,7 +14747,7 @@
       </c>
       <c r="L218" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M218" s="3" t="inlineStr"/>
@@ -14915,7 +14915,7 @@
       </c>
       <c r="L221" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M221" s="3" t="inlineStr"/>
@@ -15023,7 +15023,7 @@
       </c>
       <c r="L223" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M223" s="3" t="inlineStr"/>
@@ -15083,7 +15083,7 @@
       </c>
       <c r="L224" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M224" s="3" t="inlineStr"/>
@@ -15143,7 +15143,7 @@
       </c>
       <c r="L225" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M225" s="3" t="inlineStr"/>
@@ -15203,7 +15203,7 @@
       </c>
       <c r="L226" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M226" s="3" t="inlineStr"/>
@@ -15259,7 +15259,7 @@
       </c>
       <c r="L227" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M227" s="3" t="inlineStr"/>
@@ -15319,7 +15319,7 @@
       </c>
       <c r="L228" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M228" s="3" t="inlineStr"/>
@@ -15379,7 +15379,7 @@
       </c>
       <c r="L229" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M229" s="3" t="inlineStr"/>
@@ -15439,7 +15439,7 @@
       </c>
       <c r="L230" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M230" s="3" t="inlineStr"/>
@@ -15559,7 +15559,7 @@
       </c>
       <c r="L232" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M232" s="3" t="inlineStr"/>
@@ -15619,7 +15619,7 @@
       </c>
       <c r="L233" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M233" s="3" t="inlineStr"/>
@@ -15679,7 +15679,7 @@
       </c>
       <c r="L234" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M234" s="3" t="inlineStr"/>
@@ -15735,7 +15735,7 @@
       </c>
       <c r="L235" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M235" s="3" t="inlineStr"/>
@@ -15959,7 +15959,7 @@
       </c>
       <c r="L239" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M239" s="3" t="inlineStr"/>
@@ -16071,7 +16071,7 @@
       </c>
       <c r="L241" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M241" s="3" t="inlineStr"/>
@@ -16127,7 +16127,7 @@
       </c>
       <c r="L242" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M242" s="3" t="inlineStr"/>
@@ -16187,7 +16187,7 @@
       </c>
       <c r="L243" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M243" s="3" t="inlineStr"/>
@@ -16301,7 +16301,7 @@
       </c>
       <c r="L245" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M245" s="3" t="inlineStr"/>
@@ -16357,7 +16357,7 @@
       </c>
       <c r="L246" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M246" s="3" t="inlineStr"/>
@@ -16417,7 +16417,7 @@
       </c>
       <c r="L247" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M247" s="3" t="inlineStr"/>
@@ -16477,7 +16477,7 @@
       </c>
       <c r="L248" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M248" s="3" t="inlineStr"/>
@@ -16537,7 +16537,7 @@
       </c>
       <c r="L249" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M249" s="3" t="inlineStr"/>
@@ -16597,7 +16597,7 @@
       </c>
       <c r="L250" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M250" s="3" t="inlineStr"/>
@@ -16657,7 +16657,7 @@
       </c>
       <c r="L251" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M251" s="3" t="inlineStr"/>
@@ -16717,7 +16717,7 @@
       </c>
       <c r="L252" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M252" s="3" t="inlineStr"/>
@@ -16777,7 +16777,7 @@
       </c>
       <c r="L253" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M253" s="3" t="inlineStr"/>
@@ -16837,7 +16837,7 @@
       </c>
       <c r="L254" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M254" s="3" t="inlineStr"/>
@@ -16897,7 +16897,7 @@
       </c>
       <c r="L255" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M255" s="3" t="inlineStr"/>
@@ -16957,7 +16957,7 @@
       </c>
       <c r="L256" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M256" s="3" t="inlineStr"/>
@@ -17017,7 +17017,7 @@
       </c>
       <c r="L257" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M257" s="3" t="inlineStr"/>
@@ -17073,7 +17073,7 @@
       </c>
       <c r="L258" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M258" s="3" t="inlineStr"/>
@@ -17133,7 +17133,7 @@
       </c>
       <c r="L259" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M259" s="3" t="inlineStr"/>
@@ -17257,7 +17257,7 @@
       </c>
       <c r="L261" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M261" s="3" t="inlineStr"/>
@@ -17377,7 +17377,7 @@
       </c>
       <c r="L263" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M263" s="3" t="inlineStr"/>
@@ -17437,7 +17437,7 @@
       </c>
       <c r="L264" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M264" s="3" t="inlineStr"/>
@@ -17557,7 +17557,7 @@
       </c>
       <c r="L266" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M266" s="3" t="inlineStr"/>
@@ -17617,7 +17617,7 @@
       </c>
       <c r="L267" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M267" s="3" t="inlineStr"/>
@@ -17677,7 +17677,7 @@
       </c>
       <c r="L268" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M268" s="3" t="inlineStr"/>
@@ -17733,7 +17733,7 @@
       </c>
       <c r="L269" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M269" s="3" t="inlineStr"/>
@@ -17793,7 +17793,7 @@
       </c>
       <c r="L270" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M270" s="3" t="inlineStr"/>
@@ -17973,7 +17973,7 @@
       </c>
       <c r="L273" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M273" s="3" t="inlineStr"/>
@@ -18033,7 +18033,7 @@
       </c>
       <c r="L274" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M274" s="3" t="inlineStr"/>
@@ -18093,7 +18093,7 @@
       </c>
       <c r="L275" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M275" s="3" t="inlineStr"/>
@@ -18153,7 +18153,7 @@
       </c>
       <c r="L276" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M276" s="3" t="inlineStr"/>
@@ -18213,7 +18213,7 @@
       </c>
       <c r="L277" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M277" s="3" t="inlineStr"/>
@@ -18273,7 +18273,7 @@
       </c>
       <c r="L278" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M278" s="3" t="inlineStr"/>
@@ -18333,7 +18333,7 @@
       </c>
       <c r="L279" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M279" s="3" t="inlineStr"/>
@@ -18393,7 +18393,7 @@
       </c>
       <c r="L280" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M280" s="3" t="inlineStr"/>
@@ -18453,7 +18453,7 @@
       </c>
       <c r="L281" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M281" s="3" t="inlineStr"/>
@@ -18513,7 +18513,7 @@
       </c>
       <c r="L282" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M282" s="3" t="inlineStr"/>
@@ -18573,7 +18573,7 @@
       </c>
       <c r="L283" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M283" s="3" t="inlineStr"/>
@@ -18625,7 +18625,7 @@
       </c>
       <c r="L284" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M284" s="3" t="inlineStr"/>
@@ -18685,7 +18685,7 @@
       </c>
       <c r="L285" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M285" s="3" t="inlineStr"/>
@@ -18745,7 +18745,7 @@
       </c>
       <c r="L286" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M286" s="3" t="inlineStr"/>
@@ -18805,7 +18805,7 @@
       </c>
       <c r="L287" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M287" s="3" t="inlineStr"/>
@@ -18917,7 +18917,7 @@
       </c>
       <c r="L289" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M289" s="3" t="inlineStr"/>
@@ -18977,7 +18977,7 @@
       </c>
       <c r="L290" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M290" s="3" t="inlineStr"/>
@@ -19037,7 +19037,7 @@
       </c>
       <c r="L291" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M291" s="3" t="inlineStr"/>
@@ -19097,7 +19097,7 @@
       </c>
       <c r="L292" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M292" s="3" t="inlineStr"/>
@@ -19269,7 +19269,7 @@
       </c>
       <c r="L295" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M295" s="3" t="inlineStr"/>
@@ -19329,7 +19329,7 @@
       </c>
       <c r="L296" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M296" s="3" t="inlineStr"/>
@@ -19389,7 +19389,7 @@
       </c>
       <c r="L297" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M297" s="3" t="inlineStr"/>
@@ -19507,7 +19507,7 @@
       </c>
       <c r="L299" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M299" s="3" t="inlineStr"/>
@@ -19567,7 +19567,7 @@
       </c>
       <c r="L300" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M300" s="3" t="inlineStr"/>
@@ -19627,7 +19627,7 @@
       </c>
       <c r="L301" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M301" s="3" t="inlineStr"/>
@@ -19687,7 +19687,7 @@
       </c>
       <c r="L302" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M302" s="3" t="inlineStr"/>
@@ -19747,7 +19747,7 @@
       </c>
       <c r="L303" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M303" s="3" t="inlineStr"/>
@@ -19807,7 +19807,7 @@
       </c>
       <c r="L304" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M304" s="3" t="inlineStr"/>
@@ -19867,7 +19867,7 @@
       </c>
       <c r="L305" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M305" s="3" t="inlineStr"/>
@@ -19927,7 +19927,7 @@
       </c>
       <c r="L306" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M306" s="3" t="inlineStr"/>
@@ -19983,7 +19983,7 @@
       </c>
       <c r="L307" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M307" s="3" t="inlineStr"/>
@@ -20195,7 +20195,7 @@
       <c r="G311" s="3" t="inlineStr"/>
       <c r="H311" s="3" t="inlineStr">
         <is>
-          <t>2.47 oygacha</t>
+          <t>2.43 oygacha</t>
         </is>
       </c>
       <c r="I311" s="3" t="inlineStr"/>
@@ -20211,7 +20211,7 @@
       </c>
       <c r="L311" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M311" s="3" t="inlineStr"/>
@@ -20607,7 +20607,7 @@
       </c>
       <c r="L318" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M318" s="3" t="inlineStr"/>
@@ -20667,7 +20667,7 @@
       </c>
       <c r="L319" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M319" s="3" t="inlineStr"/>
@@ -20727,7 +20727,7 @@
       </c>
       <c r="L320" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M320" s="3" t="inlineStr"/>
@@ -20787,7 +20787,7 @@
       </c>
       <c r="L321" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M321" s="3" t="inlineStr"/>
@@ -20967,7 +20967,7 @@
       </c>
       <c r="L324" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M324" s="3" t="inlineStr"/>
@@ -21027,7 +21027,7 @@
       </c>
       <c r="L325" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M325" s="3" t="inlineStr"/>
@@ -21087,7 +21087,7 @@
       </c>
       <c r="L326" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M326" s="3" t="inlineStr"/>
@@ -21147,7 +21147,7 @@
       </c>
       <c r="L327" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M327" s="3" t="inlineStr"/>
@@ -21207,7 +21207,7 @@
       </c>
       <c r="L328" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M328" s="3" t="inlineStr"/>
@@ -21267,7 +21267,7 @@
       </c>
       <c r="L329" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M329" s="3" t="inlineStr"/>
@@ -21327,7 +21327,7 @@
       </c>
       <c r="L330" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M330" s="3" t="inlineStr"/>
@@ -21443,7 +21443,7 @@
       </c>
       <c r="L332" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M332" s="3" t="inlineStr"/>
@@ -21503,7 +21503,7 @@
       </c>
       <c r="L333" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M333" s="3" t="inlineStr"/>
@@ -21563,7 +21563,7 @@
       </c>
       <c r="L334" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M334" s="3" t="inlineStr"/>
@@ -21623,7 +21623,7 @@
       </c>
       <c r="L335" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M335" s="3" t="inlineStr"/>
@@ -21683,7 +21683,7 @@
       </c>
       <c r="L336" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M336" s="3" t="inlineStr"/>
@@ -21743,7 +21743,7 @@
       </c>
       <c r="L337" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M337" s="3" t="inlineStr"/>
@@ -21803,7 +21803,7 @@
       </c>
       <c r="L338" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M338" s="3" t="inlineStr"/>
@@ -21863,7 +21863,7 @@
       </c>
       <c r="L339" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M339" s="3" t="inlineStr"/>
@@ -21919,7 +21919,7 @@
       </c>
       <c r="L340" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M340" s="3" t="inlineStr"/>
@@ -21979,7 +21979,7 @@
       </c>
       <c r="L341" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M341" s="3" t="inlineStr"/>
@@ -22039,7 +22039,7 @@
       </c>
       <c r="L342" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M342" s="3" t="inlineStr"/>
@@ -22099,7 +22099,7 @@
       </c>
       <c r="L343" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M343" s="3" t="inlineStr"/>
@@ -22211,7 +22211,7 @@
       </c>
       <c r="L345" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M345" s="3" t="inlineStr"/>
@@ -22271,7 +22271,7 @@
       </c>
       <c r="L346" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M346" s="3" t="inlineStr"/>
@@ -22331,7 +22331,7 @@
       </c>
       <c r="L347" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M347" s="3" t="inlineStr"/>
@@ -22391,7 +22391,7 @@
       </c>
       <c r="L348" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M348" s="3" t="inlineStr"/>
@@ -22511,7 +22511,7 @@
       </c>
       <c r="L350" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M350" s="3" t="inlineStr"/>
@@ -22571,7 +22571,7 @@
       </c>
       <c r="L351" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M351" s="3" t="inlineStr"/>
@@ -22631,7 +22631,7 @@
       </c>
       <c r="L352" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M352" s="3" t="inlineStr"/>
@@ -22747,7 +22747,7 @@
       </c>
       <c r="L354" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M354" s="3" t="inlineStr"/>
@@ -22861,7 +22861,7 @@
       </c>
       <c r="L356" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M356" s="3" t="inlineStr"/>
@@ -22917,7 +22917,7 @@
       </c>
       <c r="L357" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M357" s="3" t="inlineStr"/>
@@ -23029,7 +23029,7 @@
       </c>
       <c r="L359" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M359" s="3" t="inlineStr"/>
@@ -23085,7 +23085,7 @@
       </c>
       <c r="L360" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M360" s="3" t="inlineStr"/>
@@ -23141,7 +23141,7 @@
       </c>
       <c r="L361" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M361" s="3" t="inlineStr"/>
@@ -23253,7 +23253,7 @@
       </c>
       <c r="L363" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M363" s="3" t="inlineStr"/>
@@ -23365,7 +23365,7 @@
       </c>
       <c r="L365" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M365" s="3" t="inlineStr"/>
@@ -23481,7 +23481,7 @@
       </c>
       <c r="L367" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M367" s="3" t="inlineStr"/>
@@ -23537,7 +23537,7 @@
       </c>
       <c r="L368" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M368" s="3" t="inlineStr"/>
@@ -23593,7 +23593,7 @@
       </c>
       <c r="L369" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M369" s="3" t="inlineStr"/>
@@ -23649,7 +23649,7 @@
       </c>
       <c r="L370" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M370" s="3" t="inlineStr"/>
@@ -23705,7 +23705,7 @@
       </c>
       <c r="L371" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M371" s="3" t="inlineStr"/>
@@ -23761,7 +23761,7 @@
       </c>
       <c r="L372" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M372" s="3" t="inlineStr"/>
@@ -23817,7 +23817,7 @@
       </c>
       <c r="L373" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M373" s="3" t="inlineStr"/>
@@ -23873,7 +23873,7 @@
       </c>
       <c r="L374" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M374" s="3" t="inlineStr"/>
@@ -23929,7 +23929,7 @@
       </c>
       <c r="L375" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M375" s="3" t="inlineStr"/>
@@ -23985,7 +23985,7 @@
       </c>
       <c r="L376" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M376" s="3" t="inlineStr"/>
@@ -24041,7 +24041,7 @@
       </c>
       <c r="L377" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M377" s="3" t="inlineStr"/>
@@ -24097,7 +24097,7 @@
       </c>
       <c r="L378" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M378" s="3" t="inlineStr"/>
@@ -24153,7 +24153,7 @@
       </c>
       <c r="L379" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M379" s="3" t="inlineStr"/>
@@ -24213,7 +24213,7 @@
       </c>
       <c r="L380" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M380" s="3" t="inlineStr"/>
@@ -24273,7 +24273,7 @@
       </c>
       <c r="L381" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M381" s="3" t="inlineStr"/>
@@ -24333,7 +24333,7 @@
       </c>
       <c r="L382" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M382" s="3" t="inlineStr"/>
@@ -24553,7 +24553,7 @@
       </c>
       <c r="L386" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M386" s="3" t="inlineStr"/>
@@ -24609,7 +24609,7 @@
       </c>
       <c r="L387" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M387" s="3" t="inlineStr"/>
@@ -24665,7 +24665,7 @@
       </c>
       <c r="L388" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M388" s="3" t="inlineStr"/>
@@ -24785,7 +24785,7 @@
       </c>
       <c r="L390" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M390" s="3" t="inlineStr"/>
@@ -24841,7 +24841,7 @@
       </c>
       <c r="L391" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M391" s="3" t="inlineStr"/>
@@ -25073,7 +25073,7 @@
       </c>
       <c r="L395" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M395" s="3" t="inlineStr"/>
@@ -25129,7 +25129,7 @@
       </c>
       <c r="L396" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M396" s="3" t="inlineStr"/>
@@ -25189,7 +25189,7 @@
       </c>
       <c r="L397" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M397" s="3" t="inlineStr"/>
@@ -25301,7 +25301,7 @@
       </c>
       <c r="L399" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M399" s="3" t="inlineStr"/>
@@ -25357,7 +25357,7 @@
       </c>
       <c r="L400" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M400" s="3" t="inlineStr"/>
@@ -25413,7 +25413,7 @@
       </c>
       <c r="L401" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M401" s="3" t="inlineStr"/>
@@ -25469,7 +25469,7 @@
       </c>
       <c r="L402" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M402" s="3" t="inlineStr"/>
@@ -25525,7 +25525,7 @@
       </c>
       <c r="L403" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M403" s="3" t="inlineStr"/>
@@ -25581,7 +25581,7 @@
       </c>
       <c r="L404" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M404" s="3" t="inlineStr"/>
@@ -25637,7 +25637,7 @@
       </c>
       <c r="L405" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M405" s="3" t="inlineStr"/>
@@ -25745,7 +25745,7 @@
       </c>
       <c r="L407" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M407" s="3" t="inlineStr"/>
@@ -25805,7 +25805,7 @@
       </c>
       <c r="L408" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M408" s="3" t="inlineStr"/>
@@ -25865,7 +25865,7 @@
       </c>
       <c r="L409" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M409" s="3" t="inlineStr"/>
@@ -25981,7 +25981,7 @@
       </c>
       <c r="L411" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M411" s="3" t="inlineStr"/>
@@ -26149,7 +26149,7 @@
       </c>
       <c r="L414" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M414" s="3" t="inlineStr"/>
@@ -26209,7 +26209,7 @@
       </c>
       <c r="L415" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M415" s="3" t="inlineStr"/>
@@ -26269,7 +26269,7 @@
       </c>
       <c r="L416" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M416" s="3" t="inlineStr"/>
@@ -26329,7 +26329,7 @@
       </c>
       <c r="L417" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M417" s="3" t="inlineStr"/>
@@ -26665,7 +26665,7 @@
       </c>
       <c r="L423" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M423" s="3" t="inlineStr"/>
@@ -26725,7 +26725,7 @@
       </c>
       <c r="L424" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M424" s="3" t="inlineStr"/>
@@ -26785,7 +26785,7 @@
       </c>
       <c r="L425" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M425" s="3" t="inlineStr"/>
@@ -26845,7 +26845,7 @@
       </c>
       <c r="L426" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M426" s="3" t="inlineStr"/>
@@ -26901,7 +26901,7 @@
       </c>
       <c r="L427" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M427" s="3" t="inlineStr"/>
@@ -27141,7 +27141,7 @@
       </c>
       <c r="L431" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M431" s="3" t="inlineStr"/>
@@ -27201,7 +27201,7 @@
       </c>
       <c r="L432" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M432" s="3" t="inlineStr"/>
@@ -27313,7 +27313,7 @@
       </c>
       <c r="L434" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M434" s="3" t="inlineStr"/>
@@ -27369,7 +27369,7 @@
       </c>
       <c r="L435" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M435" s="3" t="inlineStr"/>
@@ -27425,7 +27425,7 @@
       </c>
       <c r="L436" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M436" s="3" t="inlineStr"/>
@@ -27481,7 +27481,7 @@
       </c>
       <c r="L437" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M437" s="3" t="inlineStr"/>
@@ -27537,7 +27537,7 @@
       </c>
       <c r="L438" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M438" s="3" t="inlineStr"/>
@@ -27597,7 +27597,7 @@
       </c>
       <c r="L439" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M439" s="3" t="inlineStr"/>
@@ -27657,7 +27657,7 @@
       </c>
       <c r="L440" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M440" s="3" t="inlineStr"/>
@@ -27740,31 +27740,27 @@
       </c>
       <c r="C442" s="3" t="inlineStr">
         <is>
-          <t>Ipoteka</t>
+          <t>Iste'mol</t>
         </is>
       </c>
       <c r="D442" s="3" t="inlineStr">
         <is>
-          <t>"Oilaviy" ipoteka krediti</t>
+          <t>Byudjet tashkiloti xodimlari uchun</t>
         </is>
       </c>
       <c r="E442" s="3" t="n">
-        <v>21.5</v>
+        <v>27</v>
       </c>
       <c r="F442" s="3" t="n">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="G442" s="3" t="inlineStr"/>
       <c r="H442" s="3" t="inlineStr">
         <is>
-          <t>1 oy – 20 yil</t>
-        </is>
-      </c>
-      <c r="I442" s="3" t="inlineStr">
-        <is>
-          <t>763.438 ming – 1 mlrd</t>
-        </is>
-      </c>
+          <t>4 yilgacha</t>
+        </is>
+      </c>
+      <c r="I442" s="3" t="inlineStr"/>
       <c r="J442" s="3" t="inlineStr">
         <is>
           <t>UZS</t>
@@ -27772,18 +27768,22 @@
       </c>
       <c r="K442" s="3" t="inlineStr">
         <is>
-          <t>Saytdan avtomatik</t>
+          <t>Qo'lda tekshirilgan</t>
         </is>
       </c>
       <c r="L442" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="M442" s="3" t="inlineStr"/>
+          <t>2024-03</t>
+        </is>
+      </c>
+      <c r="M442" s="3" t="inlineStr">
+        <is>
+          <t>2024 yilgi hujjat</t>
+        </is>
+      </c>
       <c r="N442" s="6" t="inlineStr">
         <is>
-          <t>https://xb.uz/page/oilaviy-ipoteka-krediti</t>
+          <t>https://xb.uz/cdn/2/uploads/2024/03/13/10/37/xFOk3qk78QLp4M9iml5Dtfxdpf4RAJg9WlWzWtIymDeLH1KET7RIL94TKXcXfUC7.pdf</t>
         </is>
       </c>
     </row>
@@ -27800,31 +27800,27 @@
       </c>
       <c r="C443" s="3" t="inlineStr">
         <is>
-          <t>Ipoteka</t>
+          <t>Iste'mol</t>
         </is>
       </c>
       <c r="D443" s="3" t="inlineStr">
         <is>
-          <t>"Farovon" ipoteka krediti</t>
+          <t>Ish haqi loyihasi ishtirokchilari uchun</t>
         </is>
       </c>
       <c r="E443" s="3" t="n">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="F443" s="3" t="n">
-        <v>21.5</v>
+        <v>30</v>
       </c>
       <c r="G443" s="3" t="inlineStr"/>
       <c r="H443" s="3" t="inlineStr">
         <is>
-          <t>10 yil – 20 yil</t>
-        </is>
-      </c>
-      <c r="I443" s="3" t="inlineStr">
-        <is>
-          <t>170 mln – 1 mlrd</t>
-        </is>
-      </c>
+          <t>1–4 yil</t>
+        </is>
+      </c>
+      <c r="I443" s="3" t="inlineStr"/>
       <c r="J443" s="3" t="inlineStr">
         <is>
           <t>UZS</t>
@@ -27832,18 +27828,22 @@
       </c>
       <c r="K443" s="3" t="inlineStr">
         <is>
-          <t>Saytdan avtomatik</t>
+          <t>Qo'lda tekshirilgan</t>
         </is>
       </c>
       <c r="L443" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="M443" s="3" t="inlineStr"/>
+          <t>2024-03</t>
+        </is>
+      </c>
+      <c r="M443" s="3" t="inlineStr">
+        <is>
+          <t>1 yil 25%, 2 yil 26%, 3 yil 28%, 4 yil 30%; 2024 yilgi hujjat</t>
+        </is>
+      </c>
       <c r="N443" s="6" t="inlineStr">
         <is>
-          <t>https://xb.uz/page/ipoteka-kreditlari</t>
+          <t>https://xb.uz/cdn/2/uploads/2024/03/13/10/37/xFOk3qk78QLp4M9iml5Dtfxdpf4RAJg9WlWzWtIymDeLH1KET7RIL94TKXcXfUC7.pdf</t>
         </is>
       </c>
     </row>
@@ -27860,31 +27860,27 @@
       </c>
       <c r="C444" s="3" t="inlineStr">
         <is>
-          <t>Ipoteka</t>
+          <t>Iste'mol</t>
         </is>
       </c>
       <c r="D444" s="3" t="inlineStr">
         <is>
-          <t>Ipoteka kreditini sotib olish</t>
+          <t>"Moliyaviy ommabop" krediti</t>
         </is>
       </c>
       <c r="E444" s="3" t="n">
-        <v>21.5</v>
+        <v>23</v>
       </c>
       <c r="F444" s="3" t="n">
-        <v>21.5</v>
+        <v>24</v>
       </c>
       <c r="G444" s="3" t="inlineStr"/>
       <c r="H444" s="3" t="inlineStr">
         <is>
-          <t>1 oy – 15 yil</t>
-        </is>
-      </c>
-      <c r="I444" s="3" t="inlineStr">
-        <is>
-          <t>18.6808 mln – 1 mlrd</t>
-        </is>
-      </c>
+          <t>3 yilgacha</t>
+        </is>
+      </c>
+      <c r="I444" s="3" t="inlineStr"/>
       <c r="J444" s="3" t="inlineStr">
         <is>
           <t>UZS</t>
@@ -27897,20 +27893,20 @@
       </c>
       <c r="L444" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M444" s="3" t="inlineStr"/>
       <c r="N444" s="6" t="inlineStr">
         <is>
-          <t>https://xb.uz/page/ipoteka-kreditini-sotib-olish</t>
+          <t>https://xb.uz/page/moliyaviy-ommabop-krediti</t>
         </is>
       </c>
     </row>
     <row r="445">
       <c r="A445" s="3" t="inlineStr">
         <is>
-          <t>Xalq banki</t>
+          <t>Ziraat Bank O'zbekiston</t>
         </is>
       </c>
       <c r="B445" s="3" t="inlineStr">
@@ -27920,31 +27916,27 @@
       </c>
       <c r="C445" s="3" t="inlineStr">
         <is>
-          <t>Ipoteka</t>
+          <t>Iste'mol</t>
         </is>
       </c>
       <c r="D445" s="3" t="inlineStr">
         <is>
-          <t>“Imkon” ipoteka krediti</t>
+          <t>Iste`mol kredit "Shinam uy"</t>
         </is>
       </c>
       <c r="E445" s="3" t="n">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="F445" s="3" t="n">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="G445" s="3" t="inlineStr"/>
       <c r="H445" s="3" t="inlineStr">
         <is>
-          <t>1 oy – 20 yil</t>
-        </is>
-      </c>
-      <c r="I445" s="3" t="inlineStr">
-        <is>
-          <t>6.9312 mln – 480 mln</t>
-        </is>
-      </c>
+          <t>1 oy – 3 yil</t>
+        </is>
+      </c>
+      <c r="I445" s="3" t="inlineStr"/>
       <c r="J445" s="3" t="inlineStr">
         <is>
           <t>UZS</t>
@@ -27957,20 +27949,20 @@
       </c>
       <c r="L445" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M445" s="3" t="inlineStr"/>
       <c r="N445" s="6" t="inlineStr">
         <is>
-          <t>https://xb.uz/page/imkon-ipoteka-krediti</t>
+          <t>https://ziraatbank.uz/uz/%D1%88%D0%B8%D0%BD%D0%B0%D0%BC-%D1%83%D0%B9</t>
         </is>
       </c>
     </row>
     <row r="446">
       <c r="A446" s="3" t="inlineStr">
         <is>
-          <t>Xalq banki</t>
+          <t>Ziraat Bank O'zbekiston</t>
         </is>
       </c>
       <c r="B446" s="3" t="inlineStr">
@@ -27980,31 +27972,27 @@
       </c>
       <c r="C446" s="3" t="inlineStr">
         <is>
-          <t>Ipoteka</t>
+          <t>Iste'mol</t>
         </is>
       </c>
       <c r="D446" s="3" t="inlineStr">
         <is>
-          <t>"Yashil ipoteka 1" ipoteka krediti</t>
+          <t>Iste'mol kredit "Yashil Komfort"</t>
         </is>
       </c>
       <c r="E446" s="3" t="n">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="F446" s="3" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="G446" s="3" t="inlineStr"/>
       <c r="H446" s="3" t="inlineStr">
         <is>
-          <t>1 oy – 10 yil</t>
-        </is>
-      </c>
-      <c r="I446" s="3" t="inlineStr">
-        <is>
-          <t>17 mln – 172.833 mln</t>
-        </is>
-      </c>
+          <t>6 oy – 5 yil</t>
+        </is>
+      </c>
+      <c r="I446" s="3" t="inlineStr"/>
       <c r="J446" s="3" t="inlineStr">
         <is>
           <t>UZS</t>
@@ -28017,20 +28005,20 @@
       </c>
       <c r="L446" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M446" s="3" t="inlineStr"/>
       <c r="N446" s="6" t="inlineStr">
         <is>
-          <t>https://xb.uz/page/yashil-ipoteka-1-ipoteka-krediti</t>
+          <t>https://ziraatbank.uz/uz/iste-mol-kredit----yashil-komfort---</t>
         </is>
       </c>
     </row>
     <row r="447">
       <c r="A447" s="3" t="inlineStr">
         <is>
-          <t>Xalq banki</t>
+          <t>Ziraat Bank O'zbekiston</t>
         </is>
       </c>
       <c r="B447" s="3" t="inlineStr">
@@ -28045,19 +28033,19 @@
       </c>
       <c r="D447" s="3" t="inlineStr">
         <is>
-          <t>Byudjet tashkiloti xodimlari uchun</t>
+          <t>ECO SARMOYA</t>
         </is>
       </c>
       <c r="E447" s="3" t="n">
-        <v>27</v>
+        <v>23.5</v>
       </c>
       <c r="F447" s="3" t="n">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="G447" s="3" t="inlineStr"/>
       <c r="H447" s="3" t="inlineStr">
         <is>
-          <t>4 yilgacha</t>
+          <t>6 oy – 5 yil</t>
         </is>
       </c>
       <c r="I447" s="3" t="inlineStr"/>
@@ -28068,29 +28056,25 @@
       </c>
       <c r="K447" s="3" t="inlineStr">
         <is>
-          <t>Qo'lda tekshirilgan</t>
+          <t>Saytdan avtomatik</t>
         </is>
       </c>
       <c r="L447" s="3" t="inlineStr">
         <is>
-          <t>2024-03</t>
-        </is>
-      </c>
-      <c r="M447" s="3" t="inlineStr">
-        <is>
-          <t>2024 yilgi hujjat</t>
-        </is>
-      </c>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="M447" s="3" t="inlineStr"/>
       <c r="N447" s="6" t="inlineStr">
         <is>
-          <t>https://xb.uz/cdn/2/uploads/2024/03/13/10/37/xFOk3qk78QLp4M9iml5Dtfxdpf4RAJg9WlWzWtIymDeLH1KET7RIL94TKXcXfUC7.pdf</t>
+          <t>https://ziraatbank.uz/uz/eco-sarmoya</t>
         </is>
       </c>
     </row>
     <row r="448">
       <c r="A448" s="3" t="inlineStr">
         <is>
-          <t>Xalq banki</t>
+          <t>Ziraat Bank O'zbekiston</t>
         </is>
       </c>
       <c r="B448" s="3" t="inlineStr">
@@ -28100,27 +28084,31 @@
       </c>
       <c r="C448" s="3" t="inlineStr">
         <is>
-          <t>Iste'mol</t>
+          <t>Mikroqarz</t>
         </is>
       </c>
       <c r="D448" s="3" t="inlineStr">
         <is>
-          <t>Ish haqi loyihasi ishtirokchilari uchun</t>
+          <t>Mikroqarz</t>
         </is>
       </c>
       <c r="E448" s="3" t="n">
         <v>25</v>
       </c>
       <c r="F448" s="3" t="n">
-        <v>30</v>
+        <v>26.5</v>
       </c>
       <c r="G448" s="3" t="inlineStr"/>
       <c r="H448" s="3" t="inlineStr">
         <is>
-          <t>1–4 yil</t>
-        </is>
-      </c>
-      <c r="I448" s="3" t="inlineStr"/>
+          <t>1–36 oy</t>
+        </is>
+      </c>
+      <c r="I448" s="3" t="inlineStr">
+        <is>
+          <t>20 mln dan</t>
+        </is>
+      </c>
       <c r="J448" s="3" t="inlineStr">
         <is>
           <t>UZS</t>
@@ -28131,26 +28119,22 @@
           <t>Qo'lda tekshirilgan</t>
         </is>
       </c>
-      <c r="L448" s="3" t="inlineStr">
-        <is>
-          <t>2024-03</t>
-        </is>
-      </c>
+      <c r="L448" s="3" t="inlineStr"/>
       <c r="M448" s="3" t="inlineStr">
         <is>
-          <t>1 yil 25%, 2 yil 26%, 3 yil 28%, 4 yil 30%; 2024 yilgi hujjat</t>
+          <t>1–12 oy 25%, 13–24 oy 26%, 25–36 oy 26.5% (rasmiy daromadli)</t>
         </is>
       </c>
       <c r="N448" s="6" t="inlineStr">
         <is>
-          <t>https://xb.uz/cdn/2/uploads/2024/03/13/10/37/xFOk3qk78QLp4M9iml5Dtfxdpf4RAJg9WlWzWtIymDeLH1KET7RIL94TKXcXfUC7.pdf</t>
+          <t>https://ziraatbank.uz/uz/mikroqarz</t>
         </is>
       </c>
     </row>
     <row r="449">
       <c r="A449" s="3" t="inlineStr">
         <is>
-          <t>Xalq banki</t>
+          <t>Ziraat Bank O'zbekiston</t>
         </is>
       </c>
       <c r="B449" s="3" t="inlineStr">
@@ -28160,31 +28144,27 @@
       </c>
       <c r="C449" s="3" t="inlineStr">
         <is>
-          <t>Iste'mol</t>
+          <t>Mikroqarz</t>
         </is>
       </c>
       <c r="D449" s="3" t="inlineStr">
         <is>
-          <t>“MAHALLA LOYIHASI” KREDITI</t>
+          <t>Mikroqarz</t>
         </is>
       </c>
       <c r="E449" s="3" t="n">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="F449" s="3" t="n">
-        <v>27</v>
+        <v>26.5</v>
       </c>
       <c r="G449" s="3" t="inlineStr"/>
       <c r="H449" s="3" t="inlineStr">
         <is>
-          <t>6 oy – 5 yil</t>
-        </is>
-      </c>
-      <c r="I449" s="3" t="inlineStr">
-        <is>
-          <t>50 mln – 10 mlrd</t>
-        </is>
-      </c>
+          <t>1 oy – 3 yil</t>
+        </is>
+      </c>
+      <c r="I449" s="3" t="inlineStr"/>
       <c r="J449" s="3" t="inlineStr">
         <is>
           <t>UZS</t>
@@ -28197,718 +28177,18 @@
       </c>
       <c r="L449" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="M449" s="3" t="inlineStr"/>
       <c r="N449" s="6" t="inlineStr">
         <is>
-          <t>https://xb.uz/page/aylanma-mablaglarni-toldirish-kredit-liniyalari</t>
-        </is>
-      </c>
-    </row>
-    <row r="450">
-      <c r="A450" s="3" t="inlineStr">
-        <is>
-          <t>Xalq banki</t>
-        </is>
-      </c>
-      <c r="B450" s="3" t="inlineStr">
-        <is>
-          <t>Jismoniy</t>
-        </is>
-      </c>
-      <c r="C450" s="3" t="inlineStr">
-        <is>
-          <t>Iste'mol</t>
-        </is>
-      </c>
-      <c r="D450" s="3" t="inlineStr">
-        <is>
-          <t>"Moliyaviy ommabop" krediti</t>
-        </is>
-      </c>
-      <c r="E450" s="3" t="n">
-        <v>23</v>
-      </c>
-      <c r="F450" s="3" t="n">
-        <v>24</v>
-      </c>
-      <c r="G450" s="3" t="inlineStr"/>
-      <c r="H450" s="3" t="inlineStr">
-        <is>
-          <t>3 yilgacha</t>
-        </is>
-      </c>
-      <c r="I450" s="3" t="inlineStr"/>
-      <c r="J450" s="3" t="inlineStr">
-        <is>
-          <t>UZS</t>
-        </is>
-      </c>
-      <c r="K450" s="3" t="inlineStr">
-        <is>
-          <t>Saytdan avtomatik</t>
-        </is>
-      </c>
-      <c r="L450" s="3" t="inlineStr">
-        <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="M450" s="3" t="inlineStr"/>
-      <c r="N450" s="6" t="inlineStr">
-        <is>
-          <t>https://xb.uz/page/moliyaviy-ommabop-krediti</t>
-        </is>
-      </c>
-    </row>
-    <row r="451">
-      <c r="A451" s="3" t="inlineStr">
-        <is>
-          <t>Xalq banki</t>
-        </is>
-      </c>
-      <c r="B451" s="3" t="inlineStr">
-        <is>
-          <t>Jismoniy</t>
-        </is>
-      </c>
-      <c r="C451" s="3" t="inlineStr">
-        <is>
-          <t>Iste'mol</t>
-        </is>
-      </c>
-      <c r="D451" s="3" t="inlineStr">
-        <is>
-          <t>Talaba ta’lim krediti</t>
-        </is>
-      </c>
-      <c r="E451" s="3" t="n">
-        <v>24</v>
-      </c>
-      <c r="F451" s="3" t="n">
-        <v>24</v>
-      </c>
-      <c r="G451" s="3" t="inlineStr"/>
-      <c r="H451" s="3" t="inlineStr">
-        <is>
-          <t>1 yil – 7 yil</t>
-        </is>
-      </c>
-      <c r="I451" s="3" t="inlineStr">
-        <is>
-          <t>30 mln – 100 mln</t>
-        </is>
-      </c>
-      <c r="J451" s="3" t="inlineStr">
-        <is>
-          <t>UZS</t>
-        </is>
-      </c>
-      <c r="K451" s="3" t="inlineStr">
-        <is>
-          <t>Saytdan avtomatik</t>
-        </is>
-      </c>
-      <c r="L451" s="3" t="inlineStr">
-        <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="M451" s="3" t="inlineStr"/>
-      <c r="N451" s="6" t="inlineStr">
-        <is>
-          <t>https://xb.uz/page/istemol-kreditlari</t>
-        </is>
-      </c>
-    </row>
-    <row r="452">
-      <c r="A452" s="3" t="inlineStr">
-        <is>
-          <t>Xalq banki</t>
-        </is>
-      </c>
-      <c r="B452" s="3" t="inlineStr">
-        <is>
-          <t>Jismoniy</t>
-        </is>
-      </c>
-      <c r="C452" s="3" t="inlineStr">
-        <is>
-          <t>Iste'mol</t>
-        </is>
-      </c>
-      <c r="D452" s="3" t="inlineStr">
-        <is>
-          <t>“Hamroh” krediti (xotin-qizlar uchun)</t>
-        </is>
-      </c>
-      <c r="E452" s="3" t="n">
-        <v>17.5</v>
-      </c>
-      <c r="F452" s="3" t="n">
-        <v>21</v>
-      </c>
-      <c r="G452" s="3" t="inlineStr"/>
-      <c r="H452" s="3" t="inlineStr">
-        <is>
-          <t>1 yil – 7 yil</t>
-        </is>
-      </c>
-      <c r="I452" s="3" t="inlineStr">
-        <is>
-          <t>300 mln gacha</t>
-        </is>
-      </c>
-      <c r="J452" s="3" t="inlineStr">
-        <is>
-          <t>UZS</t>
-        </is>
-      </c>
-      <c r="K452" s="3" t="inlineStr">
-        <is>
-          <t>Saytdan avtomatik</t>
-        </is>
-      </c>
-      <c r="L452" s="3" t="inlineStr">
-        <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="M452" s="3" t="inlineStr"/>
-      <c r="N452" s="6" t="inlineStr">
-        <is>
-          <t>https://xb.uz/page/ijtimoiy-kreditlar</t>
-        </is>
-      </c>
-    </row>
-    <row r="453">
-      <c r="A453" s="3" t="inlineStr">
-        <is>
-          <t>Xalq banki</t>
-        </is>
-      </c>
-      <c r="B453" s="3" t="inlineStr">
-        <is>
-          <t>Jismoniy</t>
-        </is>
-      </c>
-      <c r="C453" s="3" t="inlineStr">
-        <is>
-          <t>Iste'mol</t>
-        </is>
-      </c>
-      <c r="D453" s="3" t="inlineStr">
-        <is>
-          <t>"Green" iste'mol krediti</t>
-        </is>
-      </c>
-      <c r="E453" s="3" t="n">
-        <v>20</v>
-      </c>
-      <c r="F453" s="3" t="n">
-        <v>20</v>
-      </c>
-      <c r="G453" s="3" t="inlineStr"/>
-      <c r="H453" s="3" t="inlineStr">
-        <is>
-          <t>1 oy – 5 yil</t>
-        </is>
-      </c>
-      <c r="I453" s="3" t="inlineStr">
-        <is>
-          <t>264.939 ming – 100 mln</t>
-        </is>
-      </c>
-      <c r="J453" s="3" t="inlineStr">
-        <is>
-          <t>UZS</t>
-        </is>
-      </c>
-      <c r="K453" s="3" t="inlineStr">
-        <is>
-          <t>Saytdan avtomatik</t>
-        </is>
-      </c>
-      <c r="L453" s="3" t="inlineStr">
-        <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="M453" s="3" t="inlineStr"/>
-      <c r="N453" s="6" t="inlineStr">
-        <is>
-          <t>https://xb.uz/page/yashil-makon-istemol-krediti</t>
-        </is>
-      </c>
-    </row>
-    <row r="454">
-      <c r="A454" s="3" t="inlineStr">
-        <is>
-          <t>Xalq banki</t>
-        </is>
-      </c>
-      <c r="B454" s="3" t="inlineStr">
-        <is>
-          <t>Jismoniy</t>
-        </is>
-      </c>
-      <c r="C454" s="3" t="inlineStr">
-        <is>
-          <t>Mikroqarz</t>
-        </is>
-      </c>
-      <c r="D454" s="3" t="inlineStr">
-        <is>
-          <t>Onlayn mikroqarz</t>
-        </is>
-      </c>
-      <c r="E454" s="3" t="n">
-        <v>24</v>
-      </c>
-      <c r="F454" s="3" t="n">
-        <v>29</v>
-      </c>
-      <c r="G454" s="3" t="inlineStr"/>
-      <c r="H454" s="3" t="inlineStr">
-        <is>
-          <t>1 oy – 4 yil</t>
-        </is>
-      </c>
-      <c r="I454" s="3" t="inlineStr">
-        <is>
-          <t>111.327 ming – 100 mln</t>
-        </is>
-      </c>
-      <c r="J454" s="3" t="inlineStr">
-        <is>
-          <t>UZS</t>
-        </is>
-      </c>
-      <c r="K454" s="3" t="inlineStr">
-        <is>
-          <t>Saytdan avtomatik</t>
-        </is>
-      </c>
-      <c r="L454" s="3" t="inlineStr">
-        <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="M454" s="3" t="inlineStr"/>
-      <c r="N454" s="6" t="inlineStr">
-        <is>
-          <t>https://xb.uz/page/onlayn-mikroqarz</t>
-        </is>
-      </c>
-    </row>
-    <row r="455">
-      <c r="A455" s="3" t="inlineStr">
-        <is>
-          <t>Xalq banki</t>
-        </is>
-      </c>
-      <c r="B455" s="3" t="inlineStr">
-        <is>
-          <t>Jismoniy</t>
-        </is>
-      </c>
-      <c r="C455" s="3" t="inlineStr">
-        <is>
-          <t>Mikroqarz</t>
-        </is>
-      </c>
-      <c r="D455" s="3" t="inlineStr">
-        <is>
-          <t>Onlayn mikroqarz</t>
-        </is>
-      </c>
-      <c r="E455" s="3" t="n">
-        <v>21</v>
-      </c>
-      <c r="F455" s="3" t="n">
-        <v>25</v>
-      </c>
-      <c r="G455" s="3" t="inlineStr"/>
-      <c r="H455" s="3" t="inlineStr">
-        <is>
-          <t>2 yil – 4 yil</t>
-        </is>
-      </c>
-      <c r="I455" s="3" t="inlineStr">
-        <is>
-          <t>30 mln – 100 mln</t>
-        </is>
-      </c>
-      <c r="J455" s="3" t="inlineStr">
-        <is>
-          <t>UZS</t>
-        </is>
-      </c>
-      <c r="K455" s="3" t="inlineStr">
-        <is>
-          <t>Saytdan avtomatik</t>
-        </is>
-      </c>
-      <c r="L455" s="3" t="inlineStr">
-        <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="M455" s="3" t="inlineStr"/>
-      <c r="N455" s="6" t="inlineStr">
-        <is>
-          <t>https://xb.uz/page/mikrokreditlar</t>
-        </is>
-      </c>
-    </row>
-    <row r="456">
-      <c r="A456" s="3" t="inlineStr">
-        <is>
-          <t>Xalq banki</t>
-        </is>
-      </c>
-      <c r="B456" s="3" t="inlineStr">
-        <is>
-          <t>Jismoniy</t>
-        </is>
-      </c>
-      <c r="C456" s="3" t="inlineStr">
-        <is>
-          <t>Mikroqarz</t>
-        </is>
-      </c>
-      <c r="D456" s="3" t="inlineStr">
-        <is>
-          <t>Pensiya mikroqarzi</t>
-        </is>
-      </c>
-      <c r="E456" s="3" t="n">
-        <v>21</v>
-      </c>
-      <c r="F456" s="3" t="n">
-        <v>21</v>
-      </c>
-      <c r="G456" s="3" t="inlineStr"/>
-      <c r="H456" s="3" t="inlineStr">
-        <is>
-          <t>1 oy – 2 yil</t>
-        </is>
-      </c>
-      <c r="I456" s="3" t="inlineStr">
-        <is>
-          <t>1.54157 mln – 30 mln</t>
-        </is>
-      </c>
-      <c r="J456" s="3" t="inlineStr">
-        <is>
-          <t>UZS</t>
-        </is>
-      </c>
-      <c r="K456" s="3" t="inlineStr">
-        <is>
-          <t>Saytdan avtomatik</t>
-        </is>
-      </c>
-      <c r="L456" s="3" t="inlineStr">
-        <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="M456" s="3" t="inlineStr"/>
-      <c r="N456" s="6" t="inlineStr">
-        <is>
-          <t>https://xb.uz/page/pensiya-mikroqarzi</t>
-        </is>
-      </c>
-    </row>
-    <row r="457">
-      <c r="A457" s="3" t="inlineStr">
-        <is>
-          <t>Ziraat Bank O'zbekiston</t>
-        </is>
-      </c>
-      <c r="B457" s="3" t="inlineStr">
-        <is>
-          <t>Jismoniy</t>
-        </is>
-      </c>
-      <c r="C457" s="3" t="inlineStr">
-        <is>
-          <t>Iste'mol</t>
-        </is>
-      </c>
-      <c r="D457" s="3" t="inlineStr">
-        <is>
-          <t>Iste`mol kredit "Shinam uy"</t>
-        </is>
-      </c>
-      <c r="E457" s="3" t="n">
-        <v>25</v>
-      </c>
-      <c r="F457" s="3" t="n">
-        <v>28</v>
-      </c>
-      <c r="G457" s="3" t="inlineStr"/>
-      <c r="H457" s="3" t="inlineStr">
-        <is>
-          <t>1 oy – 3 yil</t>
-        </is>
-      </c>
-      <c r="I457" s="3" t="inlineStr"/>
-      <c r="J457" s="3" t="inlineStr">
-        <is>
-          <t>UZS</t>
-        </is>
-      </c>
-      <c r="K457" s="3" t="inlineStr">
-        <is>
-          <t>Saytdan avtomatik</t>
-        </is>
-      </c>
-      <c r="L457" s="3" t="inlineStr">
-        <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="M457" s="3" t="inlineStr"/>
-      <c r="N457" s="6" t="inlineStr">
-        <is>
-          <t>https://ziraatbank.uz/uz/%D1%88%D0%B8%D0%BD%D0%B0%D0%BC-%D1%83%D0%B9</t>
-        </is>
-      </c>
-    </row>
-    <row r="458">
-      <c r="A458" s="3" t="inlineStr">
-        <is>
-          <t>Ziraat Bank O'zbekiston</t>
-        </is>
-      </c>
-      <c r="B458" s="3" t="inlineStr">
-        <is>
-          <t>Jismoniy</t>
-        </is>
-      </c>
-      <c r="C458" s="3" t="inlineStr">
-        <is>
-          <t>Iste'mol</t>
-        </is>
-      </c>
-      <c r="D458" s="3" t="inlineStr">
-        <is>
-          <t>Iste'mol kredit "Yashil Komfort"</t>
-        </is>
-      </c>
-      <c r="E458" s="3" t="n">
-        <v>24</v>
-      </c>
-      <c r="F458" s="3" t="n">
-        <v>25</v>
-      </c>
-      <c r="G458" s="3" t="inlineStr"/>
-      <c r="H458" s="3" t="inlineStr">
-        <is>
-          <t>6 oy – 5 yil</t>
-        </is>
-      </c>
-      <c r="I458" s="3" t="inlineStr"/>
-      <c r="J458" s="3" t="inlineStr">
-        <is>
-          <t>UZS</t>
-        </is>
-      </c>
-      <c r="K458" s="3" t="inlineStr">
-        <is>
-          <t>Saytdan avtomatik</t>
-        </is>
-      </c>
-      <c r="L458" s="3" t="inlineStr">
-        <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="M458" s="3" t="inlineStr"/>
-      <c r="N458" s="6" t="inlineStr">
-        <is>
-          <t>https://ziraatbank.uz/uz/iste-mol-kredit----yashil-komfort---</t>
-        </is>
-      </c>
-    </row>
-    <row r="459">
-      <c r="A459" s="3" t="inlineStr">
-        <is>
-          <t>Ziraat Bank O'zbekiston</t>
-        </is>
-      </c>
-      <c r="B459" s="3" t="inlineStr">
-        <is>
-          <t>Jismoniy</t>
-        </is>
-      </c>
-      <c r="C459" s="3" t="inlineStr">
-        <is>
-          <t>Iste'mol</t>
-        </is>
-      </c>
-      <c r="D459" s="3" t="inlineStr">
-        <is>
-          <t>ECO SARMOYA</t>
-        </is>
-      </c>
-      <c r="E459" s="3" t="n">
-        <v>23.5</v>
-      </c>
-      <c r="F459" s="3" t="n">
-        <v>25</v>
-      </c>
-      <c r="G459" s="3" t="inlineStr"/>
-      <c r="H459" s="3" t="inlineStr">
-        <is>
-          <t>6 oy – 5 yil</t>
-        </is>
-      </c>
-      <c r="I459" s="3" t="inlineStr"/>
-      <c r="J459" s="3" t="inlineStr">
-        <is>
-          <t>UZS</t>
-        </is>
-      </c>
-      <c r="K459" s="3" t="inlineStr">
-        <is>
-          <t>Saytdan avtomatik</t>
-        </is>
-      </c>
-      <c r="L459" s="3" t="inlineStr">
-        <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="M459" s="3" t="inlineStr"/>
-      <c r="N459" s="6" t="inlineStr">
-        <is>
-          <t>https://ziraatbank.uz/uz/eco-sarmoya</t>
-        </is>
-      </c>
-    </row>
-    <row r="460">
-      <c r="A460" s="3" t="inlineStr">
-        <is>
-          <t>Ziraat Bank O'zbekiston</t>
-        </is>
-      </c>
-      <c r="B460" s="3" t="inlineStr">
-        <is>
-          <t>Jismoniy</t>
-        </is>
-      </c>
-      <c r="C460" s="3" t="inlineStr">
-        <is>
-          <t>Mikroqarz</t>
-        </is>
-      </c>
-      <c r="D460" s="3" t="inlineStr">
-        <is>
-          <t>Mikroqarz</t>
-        </is>
-      </c>
-      <c r="E460" s="3" t="n">
-        <v>25</v>
-      </c>
-      <c r="F460" s="3" t="n">
-        <v>26.5</v>
-      </c>
-      <c r="G460" s="3" t="inlineStr"/>
-      <c r="H460" s="3" t="inlineStr">
-        <is>
-          <t>1–36 oy</t>
-        </is>
-      </c>
-      <c r="I460" s="3" t="inlineStr">
-        <is>
-          <t>20 mln dan</t>
-        </is>
-      </c>
-      <c r="J460" s="3" t="inlineStr">
-        <is>
-          <t>UZS</t>
-        </is>
-      </c>
-      <c r="K460" s="3" t="inlineStr">
-        <is>
-          <t>Qo'lda tekshirilgan</t>
-        </is>
-      </c>
-      <c r="L460" s="3" t="inlineStr"/>
-      <c r="M460" s="3" t="inlineStr">
-        <is>
-          <t>1–12 oy 25%, 13–24 oy 26%, 25–36 oy 26.5% (rasmiy daromadli)</t>
-        </is>
-      </c>
-      <c r="N460" s="6" t="inlineStr">
-        <is>
           <t>https://ziraatbank.uz/uz/mikroqarz</t>
         </is>
       </c>
     </row>
-    <row r="461">
-      <c r="A461" s="3" t="inlineStr">
-        <is>
-          <t>Ziraat Bank O'zbekiston</t>
-        </is>
-      </c>
-      <c r="B461" s="3" t="inlineStr">
-        <is>
-          <t>Jismoniy</t>
-        </is>
-      </c>
-      <c r="C461" s="3" t="inlineStr">
-        <is>
-          <t>Mikroqarz</t>
-        </is>
-      </c>
-      <c r="D461" s="3" t="inlineStr">
-        <is>
-          <t>Mikroqarz</t>
-        </is>
-      </c>
-      <c r="E461" s="3" t="n">
-        <v>25</v>
-      </c>
-      <c r="F461" s="3" t="n">
-        <v>26.5</v>
-      </c>
-      <c r="G461" s="3" t="inlineStr"/>
-      <c r="H461" s="3" t="inlineStr">
-        <is>
-          <t>1 oy – 3 yil</t>
-        </is>
-      </c>
-      <c r="I461" s="3" t="inlineStr"/>
-      <c r="J461" s="3" t="inlineStr">
-        <is>
-          <t>UZS</t>
-        </is>
-      </c>
-      <c r="K461" s="3" t="inlineStr">
-        <is>
-          <t>Saytdan avtomatik</t>
-        </is>
-      </c>
-      <c r="L461" s="3" t="inlineStr">
-        <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="M461" s="3" t="inlineStr"/>
-      <c r="N461" s="6" t="inlineStr">
-        <is>
-          <t>https://ziraatbank.uz/uz/mikroqarz</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:N461"/>
+  <autoFilter ref="A1:N449"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N3" r:id="rId2"/>
@@ -29358,18 +28638,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N447" r:id="rId446"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N448" r:id="rId447"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N449" r:id="rId448"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N450" r:id="rId449"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N451" r:id="rId450"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N452" r:id="rId451"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N453" r:id="rId452"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N454" r:id="rId453"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N455" r:id="rId454"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N456" r:id="rId455"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N457" r:id="rId456"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N458" r:id="rId457"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N459" r:id="rId458"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N460" r:id="rId459"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N461" r:id="rId460"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -30209,18 +29477,18 @@
         </is>
       </c>
       <c r="B30" s="3" t="n">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="C30" s="3" t="n">
         <v>0</v>
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>15 – 32</t>
+          <t>23 – 32</t>
         </is>
       </c>
       <c r="E30" s="3" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="F30" s="3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Ma'lumot avtomatik yangilandi (2026-10-19)
</commit_message>
<xml_diff>
--- a/docs/banklar_kreditlar.xlsx
+++ b/docs/banklar_kreditlar.xlsx
@@ -2223,7 +2223,7 @@
       </c>
       <c r="L3" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M3" s="3" t="inlineStr"/>
@@ -2283,7 +2283,7 @@
       </c>
       <c r="L4" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M4" s="3" t="inlineStr"/>
@@ -2343,7 +2343,7 @@
       </c>
       <c r="L5" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M5" s="3" t="inlineStr"/>
@@ -2403,7 +2403,7 @@
       </c>
       <c r="L6" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M6" s="3" t="inlineStr"/>
@@ -2463,7 +2463,7 @@
       </c>
       <c r="L7" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M7" s="3" t="inlineStr"/>
@@ -2523,7 +2523,7 @@
       </c>
       <c r="L8" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M8" s="3" t="inlineStr"/>
@@ -2639,7 +2639,7 @@
       </c>
       <c r="L10" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M10" s="3" t="inlineStr"/>
@@ -2699,7 +2699,7 @@
       </c>
       <c r="L11" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M11" s="3" t="inlineStr"/>
@@ -2815,7 +2815,7 @@
       </c>
       <c r="L13" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M13" s="3" t="inlineStr"/>
@@ -2875,7 +2875,7 @@
       </c>
       <c r="L14" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M14" s="3" t="inlineStr"/>
@@ -2935,7 +2935,7 @@
       </c>
       <c r="L15" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M15" s="3" t="inlineStr"/>
@@ -3047,7 +3047,7 @@
       </c>
       <c r="L17" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M17" s="3" t="inlineStr"/>
@@ -3107,7 +3107,7 @@
       </c>
       <c r="L18" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M18" s="3" t="inlineStr"/>
@@ -3223,7 +3223,7 @@
       </c>
       <c r="L20" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M20" s="3" t="inlineStr"/>
@@ -3283,7 +3283,7 @@
       </c>
       <c r="L21" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M21" s="3" t="inlineStr"/>
@@ -3343,7 +3343,7 @@
       </c>
       <c r="L22" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M22" s="3" t="inlineStr"/>
@@ -3403,7 +3403,7 @@
       </c>
       <c r="L23" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M23" s="3" t="inlineStr"/>
@@ -3463,7 +3463,7 @@
       </c>
       <c r="L24" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M24" s="3" t="inlineStr"/>
@@ -3631,7 +3631,7 @@
       </c>
       <c r="L27" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M27" s="3" t="inlineStr"/>
@@ -3691,7 +3691,7 @@
       </c>
       <c r="L28" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M28" s="3" t="inlineStr"/>
@@ -3751,7 +3751,7 @@
       </c>
       <c r="L29" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M29" s="3" t="inlineStr"/>
@@ -3811,7 +3811,7 @@
       </c>
       <c r="L30" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M30" s="3" t="inlineStr"/>
@@ -3871,7 +3871,7 @@
       </c>
       <c r="L31" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M31" s="3" t="inlineStr"/>
@@ -3931,7 +3931,7 @@
       </c>
       <c r="L32" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M32" s="3" t="inlineStr"/>
@@ -3991,7 +3991,7 @@
       </c>
       <c r="L33" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M33" s="3" t="inlineStr"/>
@@ -4051,7 +4051,7 @@
       </c>
       <c r="L34" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M34" s="3" t="inlineStr"/>
@@ -4111,7 +4111,7 @@
       </c>
       <c r="L35" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M35" s="3" t="inlineStr"/>
@@ -4171,7 +4171,7 @@
       </c>
       <c r="L36" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M36" s="3" t="inlineStr"/>
@@ -4227,7 +4227,7 @@
       </c>
       <c r="L37" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M37" s="3" t="inlineStr"/>
@@ -4339,7 +4339,7 @@
       </c>
       <c r="L39" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M39" s="3" t="inlineStr"/>
@@ -4395,7 +4395,7 @@
       </c>
       <c r="L40" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M40" s="3" t="inlineStr"/>
@@ -4451,7 +4451,7 @@
       </c>
       <c r="L41" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M41" s="3" t="inlineStr"/>
@@ -4507,7 +4507,7 @@
       </c>
       <c r="L42" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M42" s="3" t="inlineStr"/>
@@ -4567,7 +4567,7 @@
       </c>
       <c r="L43" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M43" s="3" t="inlineStr"/>
@@ -4627,7 +4627,7 @@
       </c>
       <c r="L44" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M44" s="3" t="inlineStr"/>
@@ -4687,7 +4687,7 @@
       </c>
       <c r="L45" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M45" s="3" t="inlineStr"/>
@@ -4743,7 +4743,7 @@
       </c>
       <c r="L46" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M46" s="3" t="inlineStr"/>
@@ -4799,7 +4799,7 @@
       </c>
       <c r="L47" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M47" s="3" t="inlineStr"/>
@@ -4859,7 +4859,7 @@
       </c>
       <c r="L48" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M48" s="3" t="inlineStr"/>
@@ -4919,7 +4919,7 @@
       </c>
       <c r="L49" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M49" s="3" t="inlineStr"/>
@@ -4979,7 +4979,7 @@
       </c>
       <c r="L50" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M50" s="3" t="inlineStr"/>
@@ -5093,7 +5093,7 @@
       </c>
       <c r="L52" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M52" s="3" t="inlineStr"/>
@@ -5153,7 +5153,7 @@
       </c>
       <c r="L53" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M53" s="3" t="inlineStr"/>
@@ -5213,7 +5213,7 @@
       </c>
       <c r="L54" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M54" s="3" t="inlineStr"/>
@@ -5273,7 +5273,7 @@
       </c>
       <c r="L55" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M55" s="3" t="inlineStr"/>
@@ -5333,7 +5333,7 @@
       </c>
       <c r="L56" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M56" s="3" t="inlineStr"/>
@@ -5445,7 +5445,7 @@
       </c>
       <c r="L58" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M58" s="3" t="inlineStr"/>
@@ -5501,7 +5501,7 @@
       </c>
       <c r="L59" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M59" s="3" t="inlineStr"/>
@@ -6257,7 +6257,7 @@
       </c>
       <c r="L72" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M72" s="3" t="inlineStr"/>
@@ -6369,7 +6369,7 @@
       </c>
       <c r="L74" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M74" s="3" t="inlineStr"/>
@@ -6481,7 +6481,7 @@
       </c>
       <c r="L76" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M76" s="3" t="inlineStr"/>
@@ -6537,7 +6537,7 @@
       </c>
       <c r="L77" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M77" s="3" t="inlineStr"/>
@@ -6593,7 +6593,7 @@
       </c>
       <c r="L78" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M78" s="3" t="inlineStr"/>
@@ -6649,7 +6649,7 @@
       </c>
       <c r="L79" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M79" s="3" t="inlineStr"/>
@@ -6705,7 +6705,7 @@
       </c>
       <c r="L80" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M80" s="3" t="inlineStr"/>
@@ -6761,7 +6761,7 @@
       </c>
       <c r="L81" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M81" s="3" t="inlineStr"/>
@@ -6817,7 +6817,7 @@
       </c>
       <c r="L82" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M82" s="3" t="inlineStr"/>
@@ -6869,7 +6869,7 @@
       </c>
       <c r="L83" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M83" s="3" t="inlineStr"/>
@@ -6929,7 +6929,7 @@
       </c>
       <c r="L84" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M84" s="3" t="inlineStr"/>
@@ -6989,7 +6989,7 @@
       </c>
       <c r="L85" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M85" s="3" t="inlineStr"/>
@@ -7049,7 +7049,7 @@
       </c>
       <c r="L86" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M86" s="3" t="inlineStr"/>
@@ -7109,7 +7109,7 @@
       </c>
       <c r="L87" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M87" s="3" t="inlineStr"/>
@@ -7169,7 +7169,7 @@
       </c>
       <c r="L88" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M88" s="3" t="inlineStr"/>
@@ -7225,7 +7225,7 @@
       </c>
       <c r="L89" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M89" s="3" t="inlineStr"/>
@@ -7277,7 +7277,7 @@
       </c>
       <c r="L90" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M90" s="3" t="inlineStr"/>
@@ -7389,7 +7389,7 @@
       </c>
       <c r="L92" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M92" s="3" t="inlineStr"/>
@@ -7445,7 +7445,7 @@
       </c>
       <c r="L93" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M93" s="3" t="inlineStr"/>
@@ -7505,7 +7505,7 @@
       </c>
       <c r="L94" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M94" s="3" t="inlineStr"/>
@@ -7565,7 +7565,7 @@
       </c>
       <c r="L95" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M95" s="3" t="inlineStr"/>
@@ -7625,7 +7625,7 @@
       </c>
       <c r="L96" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M96" s="3" t="inlineStr"/>
@@ -7685,7 +7685,7 @@
       </c>
       <c r="L97" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M97" s="3" t="inlineStr"/>
@@ -7745,7 +7745,7 @@
       </c>
       <c r="L98" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M98" s="3" t="inlineStr"/>
@@ -7805,7 +7805,7 @@
       </c>
       <c r="L99" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M99" s="3" t="inlineStr"/>
@@ -7865,7 +7865,7 @@
       </c>
       <c r="L100" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M100" s="3" t="inlineStr"/>
@@ -7985,7 +7985,7 @@
       </c>
       <c r="L102" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M102" s="3" t="inlineStr"/>
@@ -8045,7 +8045,7 @@
       </c>
       <c r="L103" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M103" s="3" t="inlineStr"/>
@@ -8105,7 +8105,7 @@
       </c>
       <c r="L104" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M104" s="3" t="inlineStr"/>
@@ -8165,7 +8165,7 @@
       </c>
       <c r="L105" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M105" s="3" t="inlineStr"/>
@@ -8281,7 +8281,7 @@
       </c>
       <c r="L107" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M107" s="3" t="inlineStr"/>
@@ -8341,7 +8341,7 @@
       </c>
       <c r="L108" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M108" s="3" t="inlineStr"/>
@@ -8401,7 +8401,7 @@
       </c>
       <c r="L109" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M109" s="3" t="inlineStr"/>
@@ -8461,7 +8461,7 @@
       </c>
       <c r="L110" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M110" s="3" t="inlineStr"/>
@@ -8521,7 +8521,7 @@
       </c>
       <c r="L111" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M111" s="3" t="inlineStr"/>
@@ -8581,7 +8581,7 @@
       </c>
       <c r="L112" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M112" s="3" t="inlineStr"/>
@@ -8637,7 +8637,7 @@
       </c>
       <c r="L113" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M113" s="3" t="inlineStr"/>
@@ -8693,7 +8693,7 @@
       </c>
       <c r="L114" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M114" s="3" t="inlineStr"/>
@@ -8749,7 +8749,7 @@
       </c>
       <c r="L115" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M115" s="3" t="inlineStr"/>
@@ -8809,7 +8809,7 @@
       </c>
       <c r="L116" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M116" s="3" t="inlineStr"/>
@@ -8869,7 +8869,7 @@
       </c>
       <c r="L117" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M117" s="3" t="inlineStr"/>
@@ -8929,7 +8929,7 @@
       </c>
       <c r="L118" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M118" s="3" t="inlineStr"/>
@@ -8989,7 +8989,7 @@
       </c>
       <c r="L119" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M119" s="3" t="inlineStr"/>
@@ -9049,7 +9049,7 @@
       </c>
       <c r="L120" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M120" s="3" t="inlineStr"/>
@@ -9109,7 +9109,7 @@
       </c>
       <c r="L121" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M121" s="3" t="inlineStr"/>
@@ -9169,7 +9169,7 @@
       </c>
       <c r="L122" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M122" s="3" t="inlineStr"/>
@@ -9229,7 +9229,7 @@
       </c>
       <c r="L123" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M123" s="3" t="inlineStr"/>
@@ -9289,7 +9289,7 @@
       </c>
       <c r="L124" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M124" s="3" t="inlineStr"/>
@@ -9349,7 +9349,7 @@
       </c>
       <c r="L125" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M125" s="3" t="inlineStr"/>
@@ -9409,7 +9409,7 @@
       </c>
       <c r="L126" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M126" s="3" t="inlineStr"/>
@@ -9469,7 +9469,7 @@
       </c>
       <c r="L127" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M127" s="3" t="inlineStr"/>
@@ -9529,7 +9529,7 @@
       </c>
       <c r="L128" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M128" s="3" t="inlineStr"/>
@@ -9589,7 +9589,7 @@
       </c>
       <c r="L129" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M129" s="3" t="inlineStr"/>
@@ -9821,7 +9821,7 @@
       </c>
       <c r="L133" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M133" s="3" t="inlineStr"/>
@@ -9881,7 +9881,7 @@
       </c>
       <c r="L134" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M134" s="3" t="inlineStr"/>
@@ -9941,7 +9941,7 @@
       </c>
       <c r="L135" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M135" s="3" t="inlineStr"/>
@@ -10001,7 +10001,7 @@
       </c>
       <c r="L136" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M136" s="3" t="inlineStr"/>
@@ -10169,7 +10169,7 @@
       </c>
       <c r="L139" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M139" s="3" t="inlineStr"/>
@@ -10457,7 +10457,7 @@
       </c>
       <c r="L144" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M144" s="3" t="inlineStr"/>
@@ -10577,7 +10577,7 @@
       </c>
       <c r="L146" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M146" s="3" t="inlineStr"/>
@@ -10841,7 +10841,7 @@
       </c>
       <c r="L151" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M151" s="3" t="inlineStr"/>
@@ -10957,7 +10957,7 @@
       </c>
       <c r="L153" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M153" s="3" t="inlineStr"/>
@@ -11017,7 +11017,7 @@
       </c>
       <c r="L154" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M154" s="3" t="inlineStr"/>
@@ -11077,7 +11077,7 @@
       </c>
       <c r="L155" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M155" s="3" t="inlineStr"/>
@@ -11247,7 +11247,7 @@
       </c>
       <c r="L158" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M158" s="3" t="inlineStr"/>
@@ -11303,7 +11303,7 @@
       </c>
       <c r="L159" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M159" s="3" t="inlineStr"/>
@@ -11363,7 +11363,7 @@
       </c>
       <c r="L160" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M160" s="3" t="inlineStr"/>
@@ -11423,7 +11423,7 @@
       </c>
       <c r="L161" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M161" s="3" t="inlineStr"/>
@@ -11533,7 +11533,7 @@
       </c>
       <c r="L163" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M163" s="3" t="inlineStr"/>
@@ -11593,7 +11593,7 @@
       </c>
       <c r="L164" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M164" s="3" t="inlineStr"/>
@@ -11649,7 +11649,7 @@
       </c>
       <c r="L165" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M165" s="3" t="inlineStr"/>
@@ -11709,7 +11709,7 @@
       </c>
       <c r="L166" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M166" s="3" t="inlineStr"/>
@@ -11889,7 +11889,7 @@
       </c>
       <c r="L169" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M169" s="3" t="inlineStr"/>
@@ -11949,7 +11949,7 @@
       </c>
       <c r="L170" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M170" s="3" t="inlineStr"/>
@@ -12065,7 +12065,7 @@
       </c>
       <c r="L172" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M172" s="3" t="inlineStr"/>
@@ -12125,7 +12125,7 @@
       </c>
       <c r="L173" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M173" s="3" t="inlineStr"/>
@@ -12181,7 +12181,7 @@
       </c>
       <c r="L174" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M174" s="3" t="inlineStr"/>
@@ -12241,7 +12241,7 @@
       </c>
       <c r="L175" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M175" s="3" t="inlineStr"/>
@@ -12301,7 +12301,7 @@
       </c>
       <c r="L176" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M176" s="3" t="inlineStr"/>
@@ -12357,7 +12357,7 @@
       </c>
       <c r="L177" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M177" s="3" t="inlineStr"/>
@@ -12413,7 +12413,7 @@
       </c>
       <c r="L178" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M178" s="3" t="inlineStr"/>
@@ -12465,7 +12465,7 @@
       </c>
       <c r="L179" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M179" s="3" t="inlineStr"/>
@@ -12637,7 +12637,7 @@
       </c>
       <c r="L182" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M182" s="3" t="inlineStr"/>
@@ -12693,7 +12693,7 @@
       </c>
       <c r="L183" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M183" s="3" t="inlineStr"/>
@@ -12749,7 +12749,7 @@
       </c>
       <c r="L184" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M184" s="3" t="inlineStr"/>
@@ -12805,7 +12805,7 @@
       </c>
       <c r="L185" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M185" s="3" t="inlineStr"/>
@@ -12865,7 +12865,7 @@
       </c>
       <c r="L186" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M186" s="3" t="inlineStr"/>
@@ -12985,7 +12985,7 @@
       </c>
       <c r="L188" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M188" s="3" t="inlineStr"/>
@@ -13045,7 +13045,7 @@
       </c>
       <c r="L189" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M189" s="3" t="inlineStr"/>
@@ -13161,7 +13161,7 @@
       </c>
       <c r="L191" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M191" s="3" t="inlineStr"/>
@@ -13221,7 +13221,7 @@
       </c>
       <c r="L192" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M192" s="3" t="inlineStr"/>
@@ -13281,7 +13281,7 @@
       </c>
       <c r="L193" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M193" s="3" t="inlineStr"/>
@@ -13341,7 +13341,7 @@
       </c>
       <c r="L194" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M194" s="3" t="inlineStr"/>
@@ -13401,7 +13401,7 @@
       </c>
       <c r="L195" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M195" s="3" t="inlineStr"/>
@@ -13461,7 +13461,7 @@
       </c>
       <c r="L196" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M196" s="3" t="inlineStr"/>
@@ -13581,7 +13581,7 @@
       </c>
       <c r="L198" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M198" s="3" t="inlineStr"/>
@@ -13641,7 +13641,7 @@
       </c>
       <c r="L199" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M199" s="3" t="inlineStr"/>
@@ -13701,7 +13701,7 @@
       </c>
       <c r="L200" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M200" s="3" t="inlineStr"/>
@@ -13761,7 +13761,7 @@
       </c>
       <c r="L201" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M201" s="3" t="inlineStr"/>
@@ -13821,7 +13821,7 @@
       </c>
       <c r="L202" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M202" s="3" t="inlineStr"/>
@@ -13881,7 +13881,7 @@
       </c>
       <c r="L203" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M203" s="3" t="inlineStr"/>
@@ -13941,7 +13941,7 @@
       </c>
       <c r="L204" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M204" s="3" t="inlineStr"/>
@@ -14065,7 +14065,7 @@
       </c>
       <c r="L206" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M206" s="3" t="inlineStr"/>
@@ -14183,7 +14183,7 @@
       </c>
       <c r="L208" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M208" s="3" t="inlineStr"/>
@@ -14243,7 +14243,7 @@
       </c>
       <c r="L209" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M209" s="3" t="inlineStr"/>
@@ -14357,7 +14357,7 @@
       </c>
       <c r="L211" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M211" s="3" t="inlineStr"/>
@@ -14473,7 +14473,7 @@
       </c>
       <c r="L213" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M213" s="3" t="inlineStr"/>
@@ -14525,7 +14525,7 @@
       </c>
       <c r="L214" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M214" s="3" t="inlineStr"/>
@@ -14577,7 +14577,7 @@
       </c>
       <c r="L215" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M215" s="3" t="inlineStr"/>
@@ -14687,7 +14687,7 @@
       </c>
       <c r="L217" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M217" s="3" t="inlineStr"/>
@@ -14747,7 +14747,7 @@
       </c>
       <c r="L218" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M218" s="3" t="inlineStr"/>
@@ -14915,7 +14915,7 @@
       </c>
       <c r="L221" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M221" s="3" t="inlineStr"/>
@@ -15023,7 +15023,7 @@
       </c>
       <c r="L223" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M223" s="3" t="inlineStr"/>
@@ -15083,7 +15083,7 @@
       </c>
       <c r="L224" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M224" s="3" t="inlineStr"/>
@@ -15143,7 +15143,7 @@
       </c>
       <c r="L225" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M225" s="3" t="inlineStr"/>
@@ -15203,7 +15203,7 @@
       </c>
       <c r="L226" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M226" s="3" t="inlineStr"/>
@@ -15259,7 +15259,7 @@
       </c>
       <c r="L227" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M227" s="3" t="inlineStr"/>
@@ -15319,7 +15319,7 @@
       </c>
       <c r="L228" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M228" s="3" t="inlineStr"/>
@@ -15379,7 +15379,7 @@
       </c>
       <c r="L229" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M229" s="3" t="inlineStr"/>
@@ -15439,7 +15439,7 @@
       </c>
       <c r="L230" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M230" s="3" t="inlineStr"/>
@@ -15559,7 +15559,7 @@
       </c>
       <c r="L232" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M232" s="3" t="inlineStr"/>
@@ -15619,7 +15619,7 @@
       </c>
       <c r="L233" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M233" s="3" t="inlineStr"/>
@@ -15679,7 +15679,7 @@
       </c>
       <c r="L234" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M234" s="3" t="inlineStr"/>
@@ -15735,7 +15735,7 @@
       </c>
       <c r="L235" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M235" s="3" t="inlineStr"/>
@@ -15959,7 +15959,7 @@
       </c>
       <c r="L239" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M239" s="3" t="inlineStr"/>
@@ -16071,7 +16071,7 @@
       </c>
       <c r="L241" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M241" s="3" t="inlineStr"/>
@@ -16127,7 +16127,7 @@
       </c>
       <c r="L242" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M242" s="3" t="inlineStr"/>
@@ -16187,7 +16187,7 @@
       </c>
       <c r="L243" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M243" s="3" t="inlineStr"/>
@@ -16301,7 +16301,7 @@
       </c>
       <c r="L245" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M245" s="3" t="inlineStr"/>
@@ -16357,7 +16357,7 @@
       </c>
       <c r="L246" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M246" s="3" t="inlineStr"/>
@@ -16417,7 +16417,7 @@
       </c>
       <c r="L247" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M247" s="3" t="inlineStr"/>
@@ -16477,7 +16477,7 @@
       </c>
       <c r="L248" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M248" s="3" t="inlineStr"/>
@@ -16537,7 +16537,7 @@
       </c>
       <c r="L249" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M249" s="3" t="inlineStr"/>
@@ -16597,7 +16597,7 @@
       </c>
       <c r="L250" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M250" s="3" t="inlineStr"/>
@@ -16657,7 +16657,7 @@
       </c>
       <c r="L251" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M251" s="3" t="inlineStr"/>
@@ -16717,7 +16717,7 @@
       </c>
       <c r="L252" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M252" s="3" t="inlineStr"/>
@@ -16777,7 +16777,7 @@
       </c>
       <c r="L253" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M253" s="3" t="inlineStr"/>
@@ -16837,7 +16837,7 @@
       </c>
       <c r="L254" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M254" s="3" t="inlineStr"/>
@@ -16897,7 +16897,7 @@
       </c>
       <c r="L255" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M255" s="3" t="inlineStr"/>
@@ -16957,7 +16957,7 @@
       </c>
       <c r="L256" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M256" s="3" t="inlineStr"/>
@@ -17017,7 +17017,7 @@
       </c>
       <c r="L257" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M257" s="3" t="inlineStr"/>
@@ -17073,7 +17073,7 @@
       </c>
       <c r="L258" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M258" s="3" t="inlineStr"/>
@@ -17133,7 +17133,7 @@
       </c>
       <c r="L259" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M259" s="3" t="inlineStr"/>
@@ -17257,7 +17257,7 @@
       </c>
       <c r="L261" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M261" s="3" t="inlineStr"/>
@@ -17377,7 +17377,7 @@
       </c>
       <c r="L263" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M263" s="3" t="inlineStr"/>
@@ -17437,7 +17437,7 @@
       </c>
       <c r="L264" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M264" s="3" t="inlineStr"/>
@@ -17557,7 +17557,7 @@
       </c>
       <c r="L266" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M266" s="3" t="inlineStr"/>
@@ -17617,7 +17617,7 @@
       </c>
       <c r="L267" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M267" s="3" t="inlineStr"/>
@@ -17677,7 +17677,7 @@
       </c>
       <c r="L268" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M268" s="3" t="inlineStr"/>
@@ -17733,7 +17733,7 @@
       </c>
       <c r="L269" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M269" s="3" t="inlineStr"/>
@@ -17793,7 +17793,7 @@
       </c>
       <c r="L270" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M270" s="3" t="inlineStr"/>
@@ -17973,7 +17973,7 @@
       </c>
       <c r="L273" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M273" s="3" t="inlineStr"/>
@@ -18033,7 +18033,7 @@
       </c>
       <c r="L274" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M274" s="3" t="inlineStr"/>
@@ -18093,7 +18093,7 @@
       </c>
       <c r="L275" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M275" s="3" t="inlineStr"/>
@@ -18153,7 +18153,7 @@
       </c>
       <c r="L276" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M276" s="3" t="inlineStr"/>
@@ -18213,7 +18213,7 @@
       </c>
       <c r="L277" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M277" s="3" t="inlineStr"/>
@@ -18273,7 +18273,7 @@
       </c>
       <c r="L278" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M278" s="3" t="inlineStr"/>
@@ -18333,7 +18333,7 @@
       </c>
       <c r="L279" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M279" s="3" t="inlineStr"/>
@@ -18393,7 +18393,7 @@
       </c>
       <c r="L280" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M280" s="3" t="inlineStr"/>
@@ -18453,7 +18453,7 @@
       </c>
       <c r="L281" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M281" s="3" t="inlineStr"/>
@@ -18513,7 +18513,7 @@
       </c>
       <c r="L282" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M282" s="3" t="inlineStr"/>
@@ -18573,7 +18573,7 @@
       </c>
       <c r="L283" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M283" s="3" t="inlineStr"/>
@@ -18625,7 +18625,7 @@
       </c>
       <c r="L284" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M284" s="3" t="inlineStr"/>
@@ -18685,7 +18685,7 @@
       </c>
       <c r="L285" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M285" s="3" t="inlineStr"/>
@@ -18745,7 +18745,7 @@
       </c>
       <c r="L286" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M286" s="3" t="inlineStr"/>
@@ -18805,7 +18805,7 @@
       </c>
       <c r="L287" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M287" s="3" t="inlineStr"/>
@@ -18917,7 +18917,7 @@
       </c>
       <c r="L289" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M289" s="3" t="inlineStr"/>
@@ -18977,7 +18977,7 @@
       </c>
       <c r="L290" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M290" s="3" t="inlineStr"/>
@@ -19037,7 +19037,7 @@
       </c>
       <c r="L291" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M291" s="3" t="inlineStr"/>
@@ -19097,7 +19097,7 @@
       </c>
       <c r="L292" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M292" s="3" t="inlineStr"/>
@@ -19269,7 +19269,7 @@
       </c>
       <c r="L295" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M295" s="3" t="inlineStr"/>
@@ -19329,7 +19329,7 @@
       </c>
       <c r="L296" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M296" s="3" t="inlineStr"/>
@@ -19389,7 +19389,7 @@
       </c>
       <c r="L297" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M297" s="3" t="inlineStr"/>
@@ -19507,7 +19507,7 @@
       </c>
       <c r="L299" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M299" s="3" t="inlineStr"/>
@@ -19567,7 +19567,7 @@
       </c>
       <c r="L300" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M300" s="3" t="inlineStr"/>
@@ -19627,7 +19627,7 @@
       </c>
       <c r="L301" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M301" s="3" t="inlineStr"/>
@@ -19687,7 +19687,7 @@
       </c>
       <c r="L302" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M302" s="3" t="inlineStr"/>
@@ -19747,7 +19747,7 @@
       </c>
       <c r="L303" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M303" s="3" t="inlineStr"/>
@@ -19807,7 +19807,7 @@
       </c>
       <c r="L304" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M304" s="3" t="inlineStr"/>
@@ -19867,7 +19867,7 @@
       </c>
       <c r="L305" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M305" s="3" t="inlineStr"/>
@@ -19927,7 +19927,7 @@
       </c>
       <c r="L306" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M306" s="3" t="inlineStr"/>
@@ -19983,7 +19983,7 @@
       </c>
       <c r="L307" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M307" s="3" t="inlineStr"/>
@@ -20195,7 +20195,7 @@
       <c r="G311" s="3" t="inlineStr"/>
       <c r="H311" s="3" t="inlineStr">
         <is>
-          <t>2.43 oygacha</t>
+          <t>2.4 oygacha</t>
         </is>
       </c>
       <c r="I311" s="3" t="inlineStr"/>
@@ -20211,7 +20211,7 @@
       </c>
       <c r="L311" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M311" s="3" t="inlineStr"/>
@@ -20607,7 +20607,7 @@
       </c>
       <c r="L318" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M318" s="3" t="inlineStr"/>
@@ -20667,7 +20667,7 @@
       </c>
       <c r="L319" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M319" s="3" t="inlineStr"/>
@@ -20727,7 +20727,7 @@
       </c>
       <c r="L320" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M320" s="3" t="inlineStr"/>
@@ -20787,7 +20787,7 @@
       </c>
       <c r="L321" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M321" s="3" t="inlineStr"/>
@@ -20967,7 +20967,7 @@
       </c>
       <c r="L324" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M324" s="3" t="inlineStr"/>
@@ -21027,7 +21027,7 @@
       </c>
       <c r="L325" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M325" s="3" t="inlineStr"/>
@@ -21087,7 +21087,7 @@
       </c>
       <c r="L326" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M326" s="3" t="inlineStr"/>
@@ -21147,7 +21147,7 @@
       </c>
       <c r="L327" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M327" s="3" t="inlineStr"/>
@@ -21207,7 +21207,7 @@
       </c>
       <c r="L328" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M328" s="3" t="inlineStr"/>
@@ -21267,7 +21267,7 @@
       </c>
       <c r="L329" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M329" s="3" t="inlineStr"/>
@@ -21327,7 +21327,7 @@
       </c>
       <c r="L330" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M330" s="3" t="inlineStr"/>
@@ -21443,7 +21443,7 @@
       </c>
       <c r="L332" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M332" s="3" t="inlineStr"/>
@@ -21503,7 +21503,7 @@
       </c>
       <c r="L333" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M333" s="3" t="inlineStr"/>
@@ -21563,7 +21563,7 @@
       </c>
       <c r="L334" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M334" s="3" t="inlineStr"/>
@@ -21623,7 +21623,7 @@
       </c>
       <c r="L335" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M335" s="3" t="inlineStr"/>
@@ -21683,7 +21683,7 @@
       </c>
       <c r="L336" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M336" s="3" t="inlineStr"/>
@@ -21743,7 +21743,7 @@
       </c>
       <c r="L337" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M337" s="3" t="inlineStr"/>
@@ -21803,7 +21803,7 @@
       </c>
       <c r="L338" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M338" s="3" t="inlineStr"/>
@@ -21863,7 +21863,7 @@
       </c>
       <c r="L339" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M339" s="3" t="inlineStr"/>
@@ -21919,7 +21919,7 @@
       </c>
       <c r="L340" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M340" s="3" t="inlineStr"/>
@@ -21979,7 +21979,7 @@
       </c>
       <c r="L341" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M341" s="3" t="inlineStr"/>
@@ -22039,7 +22039,7 @@
       </c>
       <c r="L342" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M342" s="3" t="inlineStr"/>
@@ -22099,7 +22099,7 @@
       </c>
       <c r="L343" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M343" s="3" t="inlineStr"/>
@@ -22211,7 +22211,7 @@
       </c>
       <c r="L345" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M345" s="3" t="inlineStr"/>
@@ -22271,7 +22271,7 @@
       </c>
       <c r="L346" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M346" s="3" t="inlineStr"/>
@@ -22331,7 +22331,7 @@
       </c>
       <c r="L347" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M347" s="3" t="inlineStr"/>
@@ -22391,7 +22391,7 @@
       </c>
       <c r="L348" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M348" s="3" t="inlineStr"/>
@@ -22511,7 +22511,7 @@
       </c>
       <c r="L350" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M350" s="3" t="inlineStr"/>
@@ -22571,7 +22571,7 @@
       </c>
       <c r="L351" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M351" s="3" t="inlineStr"/>
@@ -22631,7 +22631,7 @@
       </c>
       <c r="L352" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M352" s="3" t="inlineStr"/>
@@ -22747,7 +22747,7 @@
       </c>
       <c r="L354" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M354" s="3" t="inlineStr"/>
@@ -22861,7 +22861,7 @@
       </c>
       <c r="L356" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M356" s="3" t="inlineStr"/>
@@ -22917,7 +22917,7 @@
       </c>
       <c r="L357" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M357" s="3" t="inlineStr"/>
@@ -23029,7 +23029,7 @@
       </c>
       <c r="L359" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M359" s="3" t="inlineStr"/>
@@ -23085,7 +23085,7 @@
       </c>
       <c r="L360" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M360" s="3" t="inlineStr"/>
@@ -23141,7 +23141,7 @@
       </c>
       <c r="L361" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M361" s="3" t="inlineStr"/>
@@ -23253,7 +23253,7 @@
       </c>
       <c r="L363" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M363" s="3" t="inlineStr"/>
@@ -23365,7 +23365,7 @@
       </c>
       <c r="L365" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M365" s="3" t="inlineStr"/>
@@ -23481,7 +23481,7 @@
       </c>
       <c r="L367" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M367" s="3" t="inlineStr"/>
@@ -23537,7 +23537,7 @@
       </c>
       <c r="L368" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M368" s="3" t="inlineStr"/>
@@ -23593,7 +23593,7 @@
       </c>
       <c r="L369" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M369" s="3" t="inlineStr"/>
@@ -23649,7 +23649,7 @@
       </c>
       <c r="L370" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M370" s="3" t="inlineStr"/>
@@ -23705,7 +23705,7 @@
       </c>
       <c r="L371" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M371" s="3" t="inlineStr"/>
@@ -23761,7 +23761,7 @@
       </c>
       <c r="L372" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M372" s="3" t="inlineStr"/>
@@ -23817,7 +23817,7 @@
       </c>
       <c r="L373" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M373" s="3" t="inlineStr"/>
@@ -23873,7 +23873,7 @@
       </c>
       <c r="L374" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M374" s="3" t="inlineStr"/>
@@ -23929,7 +23929,7 @@
       </c>
       <c r="L375" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M375" s="3" t="inlineStr"/>
@@ -23985,7 +23985,7 @@
       </c>
       <c r="L376" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M376" s="3" t="inlineStr"/>
@@ -24041,7 +24041,7 @@
       </c>
       <c r="L377" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M377" s="3" t="inlineStr"/>
@@ -24097,7 +24097,7 @@
       </c>
       <c r="L378" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M378" s="3" t="inlineStr"/>
@@ -24153,7 +24153,7 @@
       </c>
       <c r="L379" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M379" s="3" t="inlineStr"/>
@@ -24213,7 +24213,7 @@
       </c>
       <c r="L380" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M380" s="3" t="inlineStr"/>
@@ -24273,7 +24273,7 @@
       </c>
       <c r="L381" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M381" s="3" t="inlineStr"/>
@@ -24333,7 +24333,7 @@
       </c>
       <c r="L382" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M382" s="3" t="inlineStr"/>
@@ -24553,7 +24553,7 @@
       </c>
       <c r="L386" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M386" s="3" t="inlineStr"/>
@@ -24609,7 +24609,7 @@
       </c>
       <c r="L387" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M387" s="3" t="inlineStr"/>
@@ -24665,7 +24665,7 @@
       </c>
       <c r="L388" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M388" s="3" t="inlineStr"/>
@@ -24785,7 +24785,7 @@
       </c>
       <c r="L390" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M390" s="3" t="inlineStr"/>
@@ -24841,7 +24841,7 @@
       </c>
       <c r="L391" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M391" s="3" t="inlineStr"/>
@@ -25073,7 +25073,7 @@
       </c>
       <c r="L395" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M395" s="3" t="inlineStr"/>
@@ -25129,7 +25129,7 @@
       </c>
       <c r="L396" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M396" s="3" t="inlineStr"/>
@@ -25189,7 +25189,7 @@
       </c>
       <c r="L397" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M397" s="3" t="inlineStr"/>
@@ -25301,7 +25301,7 @@
       </c>
       <c r="L399" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M399" s="3" t="inlineStr"/>
@@ -25357,7 +25357,7 @@
       </c>
       <c r="L400" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M400" s="3" t="inlineStr"/>
@@ -25413,7 +25413,7 @@
       </c>
       <c r="L401" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M401" s="3" t="inlineStr"/>
@@ -25469,7 +25469,7 @@
       </c>
       <c r="L402" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M402" s="3" t="inlineStr"/>
@@ -25525,7 +25525,7 @@
       </c>
       <c r="L403" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M403" s="3" t="inlineStr"/>
@@ -25581,7 +25581,7 @@
       </c>
       <c r="L404" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M404" s="3" t="inlineStr"/>
@@ -25637,7 +25637,7 @@
       </c>
       <c r="L405" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M405" s="3" t="inlineStr"/>
@@ -25745,7 +25745,7 @@
       </c>
       <c r="L407" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M407" s="3" t="inlineStr"/>
@@ -25805,7 +25805,7 @@
       </c>
       <c r="L408" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M408" s="3" t="inlineStr"/>
@@ -25865,7 +25865,7 @@
       </c>
       <c r="L409" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M409" s="3" t="inlineStr"/>
@@ -25981,7 +25981,7 @@
       </c>
       <c r="L411" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M411" s="3" t="inlineStr"/>
@@ -26149,7 +26149,7 @@
       </c>
       <c r="L414" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M414" s="3" t="inlineStr"/>
@@ -26209,7 +26209,7 @@
       </c>
       <c r="L415" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M415" s="3" t="inlineStr"/>
@@ -26269,7 +26269,7 @@
       </c>
       <c r="L416" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M416" s="3" t="inlineStr"/>
@@ -26329,7 +26329,7 @@
       </c>
       <c r="L417" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M417" s="3" t="inlineStr"/>
@@ -26665,7 +26665,7 @@
       </c>
       <c r="L423" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M423" s="3" t="inlineStr"/>
@@ -26725,7 +26725,7 @@
       </c>
       <c r="L424" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M424" s="3" t="inlineStr"/>
@@ -26785,7 +26785,7 @@
       </c>
       <c r="L425" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M425" s="3" t="inlineStr"/>
@@ -26845,7 +26845,7 @@
       </c>
       <c r="L426" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M426" s="3" t="inlineStr"/>
@@ -26901,7 +26901,7 @@
       </c>
       <c r="L427" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M427" s="3" t="inlineStr"/>
@@ -27141,7 +27141,7 @@
       </c>
       <c r="L431" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M431" s="3" t="inlineStr"/>
@@ -27201,7 +27201,7 @@
       </c>
       <c r="L432" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M432" s="3" t="inlineStr"/>
@@ -27313,7 +27313,7 @@
       </c>
       <c r="L434" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M434" s="3" t="inlineStr"/>
@@ -27369,7 +27369,7 @@
       </c>
       <c r="L435" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M435" s="3" t="inlineStr"/>
@@ -27425,7 +27425,7 @@
       </c>
       <c r="L436" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M436" s="3" t="inlineStr"/>
@@ -27481,7 +27481,7 @@
       </c>
       <c r="L437" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M437" s="3" t="inlineStr"/>
@@ -27537,7 +27537,7 @@
       </c>
       <c r="L438" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M438" s="3" t="inlineStr"/>
@@ -27597,7 +27597,7 @@
       </c>
       <c r="L439" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M439" s="3" t="inlineStr"/>
@@ -27657,7 +27657,7 @@
       </c>
       <c r="L440" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M440" s="3" t="inlineStr"/>
@@ -27893,7 +27893,7 @@
       </c>
       <c r="L444" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M444" s="3" t="inlineStr"/>
@@ -27949,7 +27949,7 @@
       </c>
       <c r="L445" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M445" s="3" t="inlineStr"/>
@@ -28005,7 +28005,7 @@
       </c>
       <c r="L446" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M446" s="3" t="inlineStr"/>
@@ -28061,7 +28061,7 @@
       </c>
       <c r="L447" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M447" s="3" t="inlineStr"/>
@@ -28177,7 +28177,7 @@
       </c>
       <c r="L449" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M449" s="3" t="inlineStr"/>

</xml_diff>

<commit_message>
Ma'lumot avtomatik yangilandi (2026-10-22)
</commit_message>
<xml_diff>
--- a/docs/banklar_kreditlar.xlsx
+++ b/docs/banklar_kreditlar.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Izoh" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Kreditlar'!$A$1:$N$439</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Kreditlar'!$A$1:$N$441</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Banklar xulosasi'!$A$1:$G$31</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Izoh'!$A$1:$A$9</definedName>
   </definedNames>
@@ -2028,7 +2028,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N439"/>
+  <dimension ref="A1:N441"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -2223,7 +2223,7 @@
       </c>
       <c r="L3" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M3" s="3" t="inlineStr"/>
@@ -2283,7 +2283,7 @@
       </c>
       <c r="L4" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M4" s="3" t="inlineStr"/>
@@ -2343,7 +2343,7 @@
       </c>
       <c r="L5" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M5" s="3" t="inlineStr"/>
@@ -2403,7 +2403,7 @@
       </c>
       <c r="L6" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M6" s="3" t="inlineStr"/>
@@ -2463,7 +2463,7 @@
       </c>
       <c r="L7" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M7" s="3" t="inlineStr"/>
@@ -2523,7 +2523,7 @@
       </c>
       <c r="L8" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M8" s="3" t="inlineStr"/>
@@ -2639,7 +2639,7 @@
       </c>
       <c r="L10" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M10" s="3" t="inlineStr"/>
@@ -2699,7 +2699,7 @@
       </c>
       <c r="L11" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M11" s="3" t="inlineStr"/>
@@ -2815,7 +2815,7 @@
       </c>
       <c r="L13" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M13" s="3" t="inlineStr"/>
@@ -2875,7 +2875,7 @@
       </c>
       <c r="L14" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M14" s="3" t="inlineStr"/>
@@ -2935,7 +2935,7 @@
       </c>
       <c r="L15" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M15" s="3" t="inlineStr"/>
@@ -3047,7 +3047,7 @@
       </c>
       <c r="L17" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M17" s="3" t="inlineStr"/>
@@ -3107,7 +3107,7 @@
       </c>
       <c r="L18" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M18" s="3" t="inlineStr"/>
@@ -3223,7 +3223,7 @@
       </c>
       <c r="L20" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M20" s="3" t="inlineStr"/>
@@ -3283,7 +3283,7 @@
       </c>
       <c r="L21" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M21" s="3" t="inlineStr"/>
@@ -3343,7 +3343,7 @@
       </c>
       <c r="L22" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M22" s="3" t="inlineStr"/>
@@ -3403,7 +3403,7 @@
       </c>
       <c r="L23" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M23" s="3" t="inlineStr"/>
@@ -3463,7 +3463,7 @@
       </c>
       <c r="L24" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M24" s="3" t="inlineStr"/>
@@ -3631,7 +3631,7 @@
       </c>
       <c r="L27" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M27" s="3" t="inlineStr"/>
@@ -3691,7 +3691,7 @@
       </c>
       <c r="L28" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M28" s="3" t="inlineStr"/>
@@ -3751,7 +3751,7 @@
       </c>
       <c r="L29" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M29" s="3" t="inlineStr"/>
@@ -3811,7 +3811,7 @@
       </c>
       <c r="L30" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M30" s="3" t="inlineStr"/>
@@ -3871,7 +3871,7 @@
       </c>
       <c r="L31" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M31" s="3" t="inlineStr"/>
@@ -3931,7 +3931,7 @@
       </c>
       <c r="L32" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M32" s="3" t="inlineStr"/>
@@ -3991,7 +3991,7 @@
       </c>
       <c r="L33" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M33" s="3" t="inlineStr"/>
@@ -4051,7 +4051,7 @@
       </c>
       <c r="L34" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M34" s="3" t="inlineStr"/>
@@ -4111,7 +4111,7 @@
       </c>
       <c r="L35" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M35" s="3" t="inlineStr"/>
@@ -4171,7 +4171,7 @@
       </c>
       <c r="L36" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M36" s="3" t="inlineStr"/>
@@ -4227,7 +4227,7 @@
       </c>
       <c r="L37" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M37" s="3" t="inlineStr"/>
@@ -4339,7 +4339,7 @@
       </c>
       <c r="L39" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M39" s="3" t="inlineStr"/>
@@ -4395,7 +4395,7 @@
       </c>
       <c r="L40" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M40" s="3" t="inlineStr"/>
@@ -4451,7 +4451,7 @@
       </c>
       <c r="L41" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M41" s="3" t="inlineStr"/>
@@ -4507,7 +4507,7 @@
       </c>
       <c r="L42" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M42" s="3" t="inlineStr"/>
@@ -4567,7 +4567,7 @@
       </c>
       <c r="L43" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M43" s="3" t="inlineStr"/>
@@ -4627,7 +4627,7 @@
       </c>
       <c r="L44" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M44" s="3" t="inlineStr"/>
@@ -4687,7 +4687,7 @@
       </c>
       <c r="L45" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M45" s="3" t="inlineStr"/>
@@ -4743,7 +4743,7 @@
       </c>
       <c r="L46" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M46" s="3" t="inlineStr"/>
@@ -4799,7 +4799,7 @@
       </c>
       <c r="L47" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M47" s="3" t="inlineStr"/>
@@ -4859,7 +4859,7 @@
       </c>
       <c r="L48" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M48" s="3" t="inlineStr"/>
@@ -4919,7 +4919,7 @@
       </c>
       <c r="L49" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M49" s="3" t="inlineStr"/>
@@ -4979,7 +4979,7 @@
       </c>
       <c r="L50" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M50" s="3" t="inlineStr"/>
@@ -5093,7 +5093,7 @@
       </c>
       <c r="L52" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M52" s="3" t="inlineStr"/>
@@ -5153,7 +5153,7 @@
       </c>
       <c r="L53" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M53" s="3" t="inlineStr"/>
@@ -5213,7 +5213,7 @@
       </c>
       <c r="L54" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M54" s="3" t="inlineStr"/>
@@ -5273,7 +5273,7 @@
       </c>
       <c r="L55" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M55" s="3" t="inlineStr"/>
@@ -5333,7 +5333,7 @@
       </c>
       <c r="L56" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M56" s="3" t="inlineStr"/>
@@ -5445,7 +5445,7 @@
       </c>
       <c r="L58" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M58" s="3" t="inlineStr"/>
@@ -5501,7 +5501,7 @@
       </c>
       <c r="L59" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M59" s="3" t="inlineStr"/>
@@ -7389,7 +7389,7 @@
       </c>
       <c r="L92" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M92" s="3" t="inlineStr"/>
@@ -7445,7 +7445,7 @@
       </c>
       <c r="L93" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M93" s="3" t="inlineStr"/>
@@ -7505,7 +7505,7 @@
       </c>
       <c r="L94" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M94" s="3" t="inlineStr"/>
@@ -7565,7 +7565,7 @@
       </c>
       <c r="L95" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M95" s="3" t="inlineStr"/>
@@ -7625,7 +7625,7 @@
       </c>
       <c r="L96" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M96" s="3" t="inlineStr"/>
@@ -7685,7 +7685,7 @@
       </c>
       <c r="L97" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M97" s="3" t="inlineStr"/>
@@ -7745,7 +7745,7 @@
       </c>
       <c r="L98" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M98" s="3" t="inlineStr"/>
@@ -7805,7 +7805,7 @@
       </c>
       <c r="L99" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M99" s="3" t="inlineStr"/>
@@ -7865,7 +7865,7 @@
       </c>
       <c r="L100" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M100" s="3" t="inlineStr"/>
@@ -7925,7 +7925,7 @@
       </c>
       <c r="L101" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M101" s="3" t="inlineStr"/>
@@ -7985,7 +7985,7 @@
       </c>
       <c r="L102" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M102" s="3" t="inlineStr"/>
@@ -8105,7 +8105,7 @@
       </c>
       <c r="L104" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M104" s="3" t="inlineStr"/>
@@ -8165,7 +8165,7 @@
       </c>
       <c r="L105" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M105" s="3" t="inlineStr"/>
@@ -8225,7 +8225,7 @@
       </c>
       <c r="L106" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M106" s="3" t="inlineStr"/>
@@ -8285,7 +8285,7 @@
       </c>
       <c r="L107" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M107" s="3" t="inlineStr"/>
@@ -8345,7 +8345,7 @@
       </c>
       <c r="L108" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M108" s="3" t="inlineStr"/>
@@ -8461,7 +8461,7 @@
       </c>
       <c r="L110" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M110" s="3" t="inlineStr"/>
@@ -8521,7 +8521,7 @@
       </c>
       <c r="L111" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M111" s="3" t="inlineStr"/>
@@ -8581,7 +8581,7 @@
       </c>
       <c r="L112" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M112" s="3" t="inlineStr"/>
@@ -8641,7 +8641,7 @@
       </c>
       <c r="L113" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M113" s="3" t="inlineStr"/>
@@ -8701,7 +8701,7 @@
       </c>
       <c r="L114" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M114" s="3" t="inlineStr"/>
@@ -8757,7 +8757,7 @@
       </c>
       <c r="L115" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M115" s="3" t="inlineStr"/>
@@ -8817,7 +8817,7 @@
       </c>
       <c r="L116" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M116" s="3" t="inlineStr"/>
@@ -8877,7 +8877,7 @@
       </c>
       <c r="L117" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M117" s="3" t="inlineStr"/>
@@ -8933,7 +8933,7 @@
       </c>
       <c r="L118" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M118" s="3" t="inlineStr"/>
@@ -8993,7 +8993,7 @@
       </c>
       <c r="L119" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M119" s="3" t="inlineStr"/>
@@ -9049,7 +9049,7 @@
       </c>
       <c r="L120" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M120" s="3" t="inlineStr"/>
@@ -9105,7 +9105,7 @@
       </c>
       <c r="L121" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M121" s="3" t="inlineStr"/>
@@ -9165,7 +9165,7 @@
       </c>
       <c r="L122" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M122" s="3" t="inlineStr"/>
@@ -9225,7 +9225,7 @@
       </c>
       <c r="L123" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M123" s="3" t="inlineStr"/>
@@ -9285,7 +9285,7 @@
       </c>
       <c r="L124" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M124" s="3" t="inlineStr"/>
@@ -9313,7 +9313,7 @@
       </c>
       <c r="D125" s="3" t="inlineStr">
         <is>
-          <t>BRB mikroqarzi bilan tezkor yechimlar</t>
+          <t>Mikroqarz</t>
         </is>
       </c>
       <c r="E125" s="3" t="n">
@@ -9325,12 +9325,12 @@
       <c r="G125" s="3" t="inlineStr"/>
       <c r="H125" s="3" t="inlineStr">
         <is>
-          <t>6 oy – 4 yil</t>
+          <t>4 yilgacha</t>
         </is>
       </c>
       <c r="I125" s="3" t="inlineStr">
         <is>
-          <t>34.104 – 100 mln</t>
+          <t>100 mln gacha</t>
         </is>
       </c>
       <c r="J125" s="3" t="inlineStr">
@@ -9345,7 +9345,7 @@
       </c>
       <c r="L125" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M125" s="3" t="inlineStr"/>
@@ -9405,7 +9405,7 @@
       </c>
       <c r="L126" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M126" s="3" t="inlineStr"/>
@@ -9465,7 +9465,7 @@
       </c>
       <c r="L127" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M127" s="3" t="inlineStr"/>
@@ -9525,7 +9525,7 @@
       </c>
       <c r="L128" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M128" s="3" t="inlineStr"/>
@@ -9585,7 +9585,7 @@
       </c>
       <c r="L129" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M129" s="3" t="inlineStr"/>
@@ -9645,7 +9645,7 @@
       </c>
       <c r="L130" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M130" s="3" t="inlineStr"/>
@@ -9705,7 +9705,7 @@
       </c>
       <c r="L131" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M131" s="3" t="inlineStr"/>
@@ -9765,7 +9765,7 @@
       </c>
       <c r="L132" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M132" s="3" t="inlineStr"/>
@@ -9825,7 +9825,7 @@
       </c>
       <c r="L133" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M133" s="3" t="inlineStr"/>
@@ -9885,7 +9885,7 @@
       </c>
       <c r="L134" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M134" s="3" t="inlineStr"/>
@@ -9945,7 +9945,7 @@
       </c>
       <c r="L135" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M135" s="3" t="inlineStr"/>
@@ -10005,7 +10005,7 @@
       </c>
       <c r="L136" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M136" s="3" t="inlineStr"/>
@@ -10237,7 +10237,7 @@
       </c>
       <c r="L140" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M140" s="3" t="inlineStr"/>
@@ -10297,7 +10297,7 @@
       </c>
       <c r="L141" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M141" s="3" t="inlineStr"/>
@@ -10357,7 +10357,7 @@
       </c>
       <c r="L142" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M142" s="3" t="inlineStr"/>
@@ -10417,7 +10417,7 @@
       </c>
       <c r="L143" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M143" s="3" t="inlineStr"/>
@@ -10585,7 +10585,7 @@
       </c>
       <c r="L146" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M146" s="3" t="inlineStr"/>
@@ -10873,7 +10873,7 @@
       </c>
       <c r="L151" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M151" s="3" t="inlineStr"/>
@@ -10993,7 +10993,7 @@
       </c>
       <c r="L153" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M153" s="3" t="inlineStr"/>
@@ -11257,7 +11257,7 @@
       </c>
       <c r="L158" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M158" s="3" t="inlineStr"/>
@@ -11373,7 +11373,7 @@
       </c>
       <c r="L160" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M160" s="3" t="inlineStr"/>
@@ -11433,7 +11433,7 @@
       </c>
       <c r="L161" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M161" s="3" t="inlineStr"/>
@@ -11493,7 +11493,7 @@
       </c>
       <c r="L162" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M162" s="3" t="inlineStr"/>
@@ -11663,7 +11663,7 @@
       </c>
       <c r="L165" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M165" s="3" t="inlineStr"/>
@@ -11719,7 +11719,7 @@
       </c>
       <c r="L166" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M166" s="3" t="inlineStr"/>
@@ -11779,7 +11779,7 @@
       </c>
       <c r="L167" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M167" s="3" t="inlineStr"/>
@@ -11839,7 +11839,7 @@
       </c>
       <c r="L168" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M168" s="3" t="inlineStr"/>
@@ -11949,7 +11949,7 @@
       </c>
       <c r="L170" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M170" s="3" t="inlineStr"/>
@@ -12009,7 +12009,7 @@
       </c>
       <c r="L171" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M171" s="3" t="inlineStr"/>
@@ -12065,7 +12065,7 @@
       </c>
       <c r="L172" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M172" s="3" t="inlineStr"/>
@@ -12125,7 +12125,7 @@
       </c>
       <c r="L173" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M173" s="3" t="inlineStr"/>
@@ -12305,7 +12305,7 @@
       </c>
       <c r="L176" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M176" s="3" t="inlineStr"/>
@@ -12365,7 +12365,7 @@
       </c>
       <c r="L177" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M177" s="3" t="inlineStr"/>
@@ -12481,7 +12481,7 @@
       </c>
       <c r="L179" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M179" s="3" t="inlineStr"/>
@@ -12541,7 +12541,7 @@
       </c>
       <c r="L180" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M180" s="3" t="inlineStr"/>
@@ -12597,7 +12597,7 @@
       </c>
       <c r="L181" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M181" s="3" t="inlineStr"/>
@@ -12657,7 +12657,7 @@
       </c>
       <c r="L182" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M182" s="3" t="inlineStr"/>
@@ -12717,7 +12717,7 @@
       </c>
       <c r="L183" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M183" s="3" t="inlineStr"/>
@@ -12773,7 +12773,7 @@
       </c>
       <c r="L184" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M184" s="3" t="inlineStr"/>
@@ -12829,7 +12829,7 @@
       </c>
       <c r="L185" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M185" s="3" t="inlineStr"/>
@@ -12881,7 +12881,7 @@
       </c>
       <c r="L186" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M186" s="3" t="inlineStr"/>
@@ -13053,7 +13053,7 @@
       </c>
       <c r="L189" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M189" s="3" t="inlineStr"/>
@@ -13109,7 +13109,7 @@
       </c>
       <c r="L190" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M190" s="3" t="inlineStr"/>
@@ -13165,7 +13165,7 @@
       </c>
       <c r="L191" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M191" s="3" t="inlineStr"/>
@@ -13221,7 +13221,7 @@
       </c>
       <c r="L192" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M192" s="3" t="inlineStr"/>
@@ -13281,7 +13281,7 @@
       </c>
       <c r="L193" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M193" s="3" t="inlineStr"/>
@@ -13401,7 +13401,7 @@
       </c>
       <c r="L195" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M195" s="3" t="inlineStr"/>
@@ -13517,7 +13517,7 @@
       </c>
       <c r="L197" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M197" s="3" t="inlineStr"/>
@@ -13577,7 +13577,7 @@
       </c>
       <c r="L198" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M198" s="3" t="inlineStr"/>
@@ -13637,7 +13637,7 @@
       </c>
       <c r="L199" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M199" s="3" t="inlineStr"/>
@@ -13757,7 +13757,7 @@
       </c>
       <c r="L201" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M201" s="3" t="inlineStr"/>
@@ -13817,7 +13817,7 @@
       </c>
       <c r="L202" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M202" s="3" t="inlineStr"/>
@@ -13877,7 +13877,7 @@
       </c>
       <c r="L203" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M203" s="3" t="inlineStr"/>
@@ -13937,7 +13937,7 @@
       </c>
       <c r="L204" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M204" s="3" t="inlineStr"/>
@@ -13997,7 +13997,7 @@
       </c>
       <c r="L205" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M205" s="3" t="inlineStr"/>
@@ -14057,7 +14057,7 @@
       </c>
       <c r="L206" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M206" s="3" t="inlineStr"/>
@@ -14117,7 +14117,7 @@
       </c>
       <c r="L207" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M207" s="3" t="inlineStr"/>
@@ -14241,7 +14241,7 @@
       </c>
       <c r="L209" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M209" s="3" t="inlineStr"/>
@@ -14359,7 +14359,7 @@
       </c>
       <c r="L211" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M211" s="3" t="inlineStr"/>
@@ -14533,7 +14533,7 @@
       </c>
       <c r="L214" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M214" s="3" t="inlineStr"/>
@@ -14585,7 +14585,7 @@
       </c>
       <c r="L215" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M215" s="3" t="inlineStr"/>
@@ -14637,7 +14637,7 @@
       </c>
       <c r="L216" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M216" s="3" t="inlineStr"/>
@@ -14747,7 +14747,7 @@
       </c>
       <c r="L218" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M218" s="3" t="inlineStr"/>
@@ -14807,7 +14807,7 @@
       </c>
       <c r="L219" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M219" s="3" t="inlineStr"/>
@@ -14975,7 +14975,7 @@
       </c>
       <c r="L222" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M222" s="3" t="inlineStr"/>
@@ -15379,7 +15379,7 @@
       </c>
       <c r="L229" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M229" s="3" t="inlineStr"/>
@@ -15439,7 +15439,7 @@
       </c>
       <c r="L230" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M230" s="3" t="inlineStr"/>
@@ -15499,7 +15499,7 @@
       </c>
       <c r="L231" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M231" s="3" t="inlineStr"/>
@@ -15619,7 +15619,7 @@
       </c>
       <c r="L233" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M233" s="3" t="inlineStr"/>
@@ -15679,7 +15679,7 @@
       </c>
       <c r="L234" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M234" s="3" t="inlineStr"/>
@@ -15739,7 +15739,7 @@
       </c>
       <c r="L235" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M235" s="3" t="inlineStr"/>
@@ -15795,7 +15795,7 @@
       </c>
       <c r="L236" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M236" s="3" t="inlineStr"/>
@@ -16019,7 +16019,7 @@
       </c>
       <c r="L240" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M240" s="3" t="inlineStr"/>
@@ -16131,7 +16131,7 @@
       </c>
       <c r="L242" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M242" s="3" t="inlineStr"/>
@@ -16187,7 +16187,7 @@
       </c>
       <c r="L243" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M243" s="3" t="inlineStr"/>
@@ -16247,7 +16247,7 @@
       </c>
       <c r="L244" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M244" s="3" t="inlineStr"/>
@@ -16361,7 +16361,7 @@
       </c>
       <c r="L246" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M246" s="3" t="inlineStr"/>
@@ -16417,7 +16417,7 @@
       </c>
       <c r="L247" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M247" s="3" t="inlineStr"/>
@@ -16477,7 +16477,7 @@
       </c>
       <c r="L248" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M248" s="3" t="inlineStr"/>
@@ -16537,7 +16537,7 @@
       </c>
       <c r="L249" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M249" s="3" t="inlineStr"/>
@@ -16597,7 +16597,7 @@
       </c>
       <c r="L250" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M250" s="3" t="inlineStr"/>
@@ -16657,7 +16657,7 @@
       </c>
       <c r="L251" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M251" s="3" t="inlineStr"/>
@@ -16717,7 +16717,7 @@
       </c>
       <c r="L252" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M252" s="3" t="inlineStr"/>
@@ -16777,7 +16777,7 @@
       </c>
       <c r="L253" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M253" s="3" t="inlineStr"/>
@@ -16837,7 +16837,7 @@
       </c>
       <c r="L254" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M254" s="3" t="inlineStr"/>
@@ -16897,7 +16897,7 @@
       </c>
       <c r="L255" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M255" s="3" t="inlineStr"/>
@@ -16957,7 +16957,7 @@
       </c>
       <c r="L256" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M256" s="3" t="inlineStr"/>
@@ -17017,7 +17017,7 @@
       </c>
       <c r="L257" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M257" s="3" t="inlineStr"/>
@@ -17077,7 +17077,7 @@
       </c>
       <c r="L258" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M258" s="3" t="inlineStr"/>
@@ -17133,7 +17133,7 @@
       </c>
       <c r="L259" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M259" s="3" t="inlineStr"/>
@@ -17193,7 +17193,7 @@
       </c>
       <c r="L260" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M260" s="3" t="inlineStr"/>
@@ -17317,7 +17317,7 @@
       </c>
       <c r="L262" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M262" s="3" t="inlineStr"/>
@@ -17437,7 +17437,7 @@
       </c>
       <c r="L264" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M264" s="3" t="inlineStr"/>
@@ -17497,7 +17497,7 @@
       </c>
       <c r="L265" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M265" s="3" t="inlineStr"/>
@@ -17617,7 +17617,7 @@
       </c>
       <c r="L267" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M267" s="3" t="inlineStr"/>
@@ -17677,7 +17677,7 @@
       </c>
       <c r="L268" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M268" s="3" t="inlineStr"/>
@@ -17737,7 +17737,7 @@
       </c>
       <c r="L269" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M269" s="3" t="inlineStr"/>
@@ -17793,7 +17793,7 @@
       </c>
       <c r="L270" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M270" s="3" t="inlineStr"/>
@@ -17853,7 +17853,7 @@
       </c>
       <c r="L271" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M271" s="3" t="inlineStr"/>
@@ -18033,7 +18033,7 @@
       </c>
       <c r="L274" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M274" s="3" t="inlineStr"/>
@@ -18093,7 +18093,7 @@
       </c>
       <c r="L275" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M275" s="3" t="inlineStr"/>
@@ -18153,7 +18153,7 @@
       </c>
       <c r="L276" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M276" s="3" t="inlineStr"/>
@@ -18213,7 +18213,7 @@
       </c>
       <c r="L277" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M277" s="3" t="inlineStr"/>
@@ -18273,7 +18273,7 @@
       </c>
       <c r="L278" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M278" s="3" t="inlineStr"/>
@@ -18333,7 +18333,7 @@
       </c>
       <c r="L279" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M279" s="3" t="inlineStr"/>
@@ -18393,7 +18393,7 @@
       </c>
       <c r="L280" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M280" s="3" t="inlineStr"/>
@@ -18453,7 +18453,7 @@
       </c>
       <c r="L281" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M281" s="3" t="inlineStr"/>
@@ -18513,7 +18513,7 @@
       </c>
       <c r="L282" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M282" s="3" t="inlineStr"/>
@@ -18573,7 +18573,7 @@
       </c>
       <c r="L283" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M283" s="3" t="inlineStr"/>
@@ -18633,7 +18633,7 @@
       </c>
       <c r="L284" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M284" s="3" t="inlineStr"/>
@@ -18685,13 +18685,13 @@
       </c>
       <c r="L285" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M285" s="3" t="inlineStr"/>
       <c r="N285" s="6" t="inlineStr">
         <is>
-          <t>https://sqb.uz/uz/individuals/ipoteka/ipoteka-na-pervichnoe-zhile-uz/</t>
+          <t>https://sqb.uz/uz/individuals/ipoteka/new-house-ipoteka-2-uz/</t>
         </is>
       </c>
     </row>
@@ -18745,7 +18745,7 @@
       </c>
       <c r="L286" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M286" s="3" t="inlineStr"/>
@@ -18805,7 +18805,7 @@
       </c>
       <c r="L287" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M287" s="3" t="inlineStr"/>
@@ -18865,7 +18865,7 @@
       </c>
       <c r="L288" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M288" s="3" t="inlineStr"/>
@@ -18977,7 +18977,7 @@
       </c>
       <c r="L290" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M290" s="3" t="inlineStr"/>
@@ -19037,7 +19037,7 @@
       </c>
       <c r="L291" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M291" s="3" t="inlineStr"/>
@@ -19097,7 +19097,7 @@
       </c>
       <c r="L292" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M292" s="3" t="inlineStr"/>
@@ -19157,7 +19157,7 @@
       </c>
       <c r="L293" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M293" s="3" t="inlineStr"/>
@@ -19329,7 +19329,7 @@
       </c>
       <c r="L296" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M296" s="3" t="inlineStr"/>
@@ -19389,7 +19389,7 @@
       </c>
       <c r="L297" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M297" s="3" t="inlineStr"/>
@@ -19449,7 +19449,7 @@
       </c>
       <c r="L298" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M298" s="3" t="inlineStr"/>
@@ -19563,7 +19563,7 @@
       </c>
       <c r="L300" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M300" s="3" t="inlineStr"/>
@@ -19623,7 +19623,7 @@
       </c>
       <c r="L301" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M301" s="3" t="inlineStr"/>
@@ -19683,7 +19683,7 @@
       </c>
       <c r="L302" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M302" s="3" t="inlineStr"/>
@@ -19743,7 +19743,7 @@
       </c>
       <c r="L303" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M303" s="3" t="inlineStr"/>
@@ -19803,7 +19803,7 @@
       </c>
       <c r="L304" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M304" s="3" t="inlineStr"/>
@@ -19863,7 +19863,7 @@
       </c>
       <c r="L305" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M305" s="3" t="inlineStr"/>
@@ -19923,7 +19923,7 @@
       </c>
       <c r="L306" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M306" s="3" t="inlineStr"/>
@@ -19983,7 +19983,7 @@
       </c>
       <c r="L307" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M307" s="3" t="inlineStr"/>
@@ -20039,7 +20039,7 @@
       </c>
       <c r="L308" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M308" s="3" t="inlineStr"/>
@@ -20251,7 +20251,7 @@
       <c r="G312" s="3" t="inlineStr"/>
       <c r="H312" s="3" t="inlineStr">
         <is>
-          <t>2.33 oygacha</t>
+          <t>2.3 oygacha</t>
         </is>
       </c>
       <c r="I312" s="3" t="inlineStr"/>
@@ -20267,7 +20267,7 @@
       </c>
       <c r="L312" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M312" s="3" t="inlineStr"/>
@@ -20663,7 +20663,7 @@
       </c>
       <c r="L319" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M319" s="3" t="inlineStr"/>
@@ -20723,7 +20723,7 @@
       </c>
       <c r="L320" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M320" s="3" t="inlineStr"/>
@@ -20899,7 +20899,7 @@
       </c>
       <c r="L323" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M323" s="3" t="inlineStr"/>
@@ -21015,7 +21015,7 @@
       </c>
       <c r="L325" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M325" s="3" t="inlineStr"/>
@@ -21075,7 +21075,7 @@
       </c>
       <c r="L326" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M326" s="3" t="inlineStr"/>
@@ -21135,7 +21135,7 @@
       </c>
       <c r="L327" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M327" s="3" t="inlineStr"/>
@@ -21195,7 +21195,7 @@
       </c>
       <c r="L328" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M328" s="3" t="inlineStr"/>
@@ -21255,7 +21255,7 @@
       </c>
       <c r="L329" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M329" s="3" t="inlineStr"/>
@@ -21315,7 +21315,7 @@
       </c>
       <c r="L330" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M330" s="3" t="inlineStr"/>
@@ -21375,7 +21375,7 @@
       </c>
       <c r="L331" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M331" s="3" t="inlineStr"/>
@@ -21435,7 +21435,7 @@
       </c>
       <c r="L332" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M332" s="3" t="inlineStr"/>
@@ -21491,7 +21491,7 @@
       </c>
       <c r="L333" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M333" s="3" t="inlineStr"/>
@@ -21551,7 +21551,7 @@
       </c>
       <c r="L334" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M334" s="3" t="inlineStr"/>
@@ -21663,7 +21663,7 @@
       </c>
       <c r="L336" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M336" s="3" t="inlineStr"/>
@@ -21723,7 +21723,7 @@
       </c>
       <c r="L337" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M337" s="3" t="inlineStr"/>
@@ -21783,7 +21783,7 @@
       </c>
       <c r="L338" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M338" s="3" t="inlineStr"/>
@@ -21843,7 +21843,7 @@
       </c>
       <c r="L339" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M339" s="3" t="inlineStr"/>
@@ -21963,7 +21963,7 @@
       </c>
       <c r="L341" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M341" s="3" t="inlineStr"/>
@@ -22023,7 +22023,7 @@
       </c>
       <c r="L342" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M342" s="3" t="inlineStr"/>
@@ -22083,7 +22083,7 @@
       </c>
       <c r="L343" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M343" s="3" t="inlineStr"/>
@@ -22199,7 +22199,7 @@
       </c>
       <c r="L345" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M345" s="3" t="inlineStr"/>
@@ -22313,7 +22313,7 @@
       </c>
       <c r="L347" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M347" s="3" t="inlineStr"/>
@@ -22369,7 +22369,7 @@
       </c>
       <c r="L348" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M348" s="3" t="inlineStr"/>
@@ -22481,7 +22481,7 @@
       </c>
       <c r="L350" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M350" s="3" t="inlineStr"/>
@@ -22537,7 +22537,7 @@
       </c>
       <c r="L351" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M351" s="3" t="inlineStr"/>
@@ -22593,7 +22593,7 @@
       </c>
       <c r="L352" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M352" s="3" t="inlineStr"/>
@@ -22705,7 +22705,7 @@
       </c>
       <c r="L354" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M354" s="3" t="inlineStr"/>
@@ -22817,7 +22817,7 @@
       </c>
       <c r="L356" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M356" s="3" t="inlineStr"/>
@@ -22933,7 +22933,7 @@
       </c>
       <c r="L358" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M358" s="3" t="inlineStr"/>
@@ -22989,7 +22989,7 @@
       </c>
       <c r="L359" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M359" s="3" t="inlineStr"/>
@@ -23045,7 +23045,7 @@
       </c>
       <c r="L360" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M360" s="3" t="inlineStr"/>
@@ -23101,7 +23101,7 @@
       </c>
       <c r="L361" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M361" s="3" t="inlineStr"/>
@@ -23157,7 +23157,7 @@
       </c>
       <c r="L362" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M362" s="3" t="inlineStr"/>
@@ -23213,7 +23213,7 @@
       </c>
       <c r="L363" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M363" s="3" t="inlineStr"/>
@@ -23269,7 +23269,7 @@
       </c>
       <c r="L364" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M364" s="3" t="inlineStr"/>
@@ -23325,7 +23325,7 @@
       </c>
       <c r="L365" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M365" s="3" t="inlineStr"/>
@@ -23381,7 +23381,7 @@
       </c>
       <c r="L366" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M366" s="3" t="inlineStr"/>
@@ -23437,7 +23437,7 @@
       </c>
       <c r="L367" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M367" s="3" t="inlineStr"/>
@@ -23493,7 +23493,7 @@
       </c>
       <c r="L368" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M368" s="3" t="inlineStr"/>
@@ -23549,7 +23549,7 @@
       </c>
       <c r="L369" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M369" s="3" t="inlineStr"/>
@@ -23605,7 +23605,7 @@
       </c>
       <c r="L370" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M370" s="3" t="inlineStr"/>
@@ -23665,7 +23665,7 @@
       </c>
       <c r="L371" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M371" s="3" t="inlineStr"/>
@@ -23725,7 +23725,7 @@
       </c>
       <c r="L372" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M372" s="3" t="inlineStr"/>
@@ -23785,7 +23785,7 @@
       </c>
       <c r="L373" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M373" s="3" t="inlineStr"/>
@@ -23837,7 +23837,7 @@
       </c>
       <c r="L374" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M374" s="3" t="inlineStr"/>
@@ -24057,7 +24057,7 @@
       </c>
       <c r="L378" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M378" s="3" t="inlineStr"/>
@@ -24113,7 +24113,7 @@
       </c>
       <c r="L379" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M379" s="3" t="inlineStr"/>
@@ -24169,7 +24169,7 @@
       </c>
       <c r="L380" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M380" s="3" t="inlineStr"/>
@@ -24289,7 +24289,7 @@
       </c>
       <c r="L382" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M382" s="3" t="inlineStr"/>
@@ -24345,7 +24345,7 @@
       </c>
       <c r="L383" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M383" s="3" t="inlineStr"/>
@@ -24577,7 +24577,7 @@
       </c>
       <c r="L387" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M387" s="3" t="inlineStr"/>
@@ -24633,7 +24633,7 @@
       </c>
       <c r="L388" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M388" s="3" t="inlineStr"/>
@@ -24693,7 +24693,7 @@
       </c>
       <c r="L389" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M389" s="3" t="inlineStr"/>
@@ -24805,7 +24805,7 @@
       </c>
       <c r="L391" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M391" s="3" t="inlineStr"/>
@@ -24861,7 +24861,7 @@
       </c>
       <c r="L392" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M392" s="3" t="inlineStr"/>
@@ -24917,7 +24917,7 @@
       </c>
       <c r="L393" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M393" s="3" t="inlineStr"/>
@@ -24973,7 +24973,7 @@
       </c>
       <c r="L394" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M394" s="3" t="inlineStr"/>
@@ -25029,7 +25029,7 @@
       </c>
       <c r="L395" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M395" s="3" t="inlineStr"/>
@@ -25085,7 +25085,7 @@
       </c>
       <c r="L396" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M396" s="3" t="inlineStr"/>
@@ -25141,7 +25141,7 @@
       </c>
       <c r="L397" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M397" s="3" t="inlineStr"/>
@@ -25249,7 +25249,7 @@
       </c>
       <c r="L399" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M399" s="3" t="inlineStr"/>
@@ -25309,7 +25309,7 @@
       </c>
       <c r="L400" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M400" s="3" t="inlineStr"/>
@@ -25369,7 +25369,7 @@
       </c>
       <c r="L401" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M401" s="3" t="inlineStr"/>
@@ -25485,7 +25485,7 @@
       </c>
       <c r="L403" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M403" s="3" t="inlineStr"/>
@@ -25653,7 +25653,7 @@
       </c>
       <c r="L406" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M406" s="3" t="inlineStr"/>
@@ -25713,7 +25713,7 @@
       </c>
       <c r="L407" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M407" s="3" t="inlineStr"/>
@@ -25773,7 +25773,7 @@
       </c>
       <c r="L408" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M408" s="3" t="inlineStr"/>
@@ -25833,7 +25833,7 @@
       </c>
       <c r="L409" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M409" s="3" t="inlineStr"/>
@@ -26086,7 +26086,11 @@
       <c r="F414" s="3" t="n">
         <v>27</v>
       </c>
-      <c r="G414" s="3" t="inlineStr"/>
+      <c r="G414" s="3" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
       <c r="H414" s="3" t="inlineStr">
         <is>
           <t>36 oy</t>
@@ -26128,27 +26132,31 @@
       </c>
       <c r="C415" s="3" t="inlineStr">
         <is>
-          <t>Avtokredit</t>
+          <t>Biznes</t>
         </is>
       </c>
       <c r="D415" s="3" t="inlineStr">
         <is>
-          <t>Avtokredit</t>
+          <t>Biznesga birinchi qadam – “Lux”</t>
         </is>
       </c>
       <c r="E415" s="3" t="n">
-        <v>27</v>
+        <v>36</v>
       </c>
       <c r="F415" s="3" t="n">
-        <v>27</v>
+        <v>36</v>
       </c>
       <c r="G415" s="3" t="inlineStr"/>
       <c r="H415" s="3" t="inlineStr">
         <is>
-          <t>3 yil – 5 yil</t>
-        </is>
-      </c>
-      <c r="I415" s="3" t="inlineStr"/>
+          <t>1 oy – 3 yil</t>
+        </is>
+      </c>
+      <c r="I415" s="3" t="inlineStr">
+        <is>
+          <t>1 mln – 100 mln</t>
+        </is>
+      </c>
       <c r="J415" s="3" t="inlineStr">
         <is>
           <t>UZS</t>
@@ -26161,13 +26169,13 @@
       </c>
       <c r="L415" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M415" s="3" t="inlineStr"/>
       <c r="N415" s="6" t="inlineStr">
         <is>
-          <t>https://universalbank.uz/credit/avtokredit-ikkilamchi-bozor-uc</t>
+          <t>https://universalbank.uz/credit/biznesga-birinchi-qadam-lux</t>
         </is>
       </c>
     </row>
@@ -26189,7 +26197,7 @@
       </c>
       <c r="D416" s="3" t="inlineStr">
         <is>
-          <t>Biznesga birinchi qadam</t>
+          <t>Biznesga birinchi qadam – “Premium”</t>
         </is>
       </c>
       <c r="E416" s="3" t="n">
@@ -26204,7 +26212,11 @@
           <t>1 oy – 3 yil</t>
         </is>
       </c>
-      <c r="I416" s="3" t="inlineStr"/>
+      <c r="I416" s="3" t="inlineStr">
+        <is>
+          <t>45.804 – 30 mln</t>
+        </is>
+      </c>
       <c r="J416" s="3" t="inlineStr">
         <is>
           <t>UZS</t>
@@ -26217,13 +26229,13 @@
       </c>
       <c r="L416" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M416" s="3" t="inlineStr"/>
       <c r="N416" s="6" t="inlineStr">
         <is>
-          <t>https://universalbank.uz/credit/biznesga-birinchi-qadam-lux</t>
+          <t>https://universalbank.uz/credit/biznesga-birinchi-qadam-premiu</t>
         </is>
       </c>
     </row>
@@ -26245,7 +26257,7 @@
       </c>
       <c r="D417" s="3" t="inlineStr">
         <is>
-          <t>Biznesga birinchi qadam</t>
+          <t>Biznesga birinchi qadam – “Standart”</t>
         </is>
       </c>
       <c r="E417" s="3" t="n">
@@ -26257,10 +26269,14 @@
       <c r="G417" s="3" t="inlineStr"/>
       <c r="H417" s="3" t="inlineStr">
         <is>
-          <t>2 oy – 2 yil</t>
-        </is>
-      </c>
-      <c r="I417" s="3" t="inlineStr"/>
+          <t>1 oy – 2 yil</t>
+        </is>
+      </c>
+      <c r="I417" s="3" t="inlineStr">
+        <is>
+          <t>57.992 – 20 mln</t>
+        </is>
+      </c>
       <c r="J417" s="3" t="inlineStr">
         <is>
           <t>UZS</t>
@@ -26273,7 +26289,7 @@
       </c>
       <c r="L417" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M417" s="3" t="inlineStr"/>
@@ -26301,7 +26317,7 @@
       </c>
       <c r="D418" s="3" t="inlineStr">
         <is>
-          <t>Biznesga birinchi qadam</t>
+          <t>Biznesga birinchi qadam – “Econom”</t>
         </is>
       </c>
       <c r="E418" s="3" t="n">
@@ -26316,7 +26332,11 @@
           <t>1 oy – 1 yil</t>
         </is>
       </c>
-      <c r="I418" s="3" t="inlineStr"/>
+      <c r="I418" s="3" t="inlineStr">
+        <is>
+          <t>98.474 – 10 mln</t>
+        </is>
+      </c>
       <c r="J418" s="3" t="inlineStr">
         <is>
           <t>UZS</t>
@@ -26329,7 +26349,7 @@
       </c>
       <c r="L418" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M418" s="3" t="inlineStr"/>
@@ -26357,7 +26377,7 @@
       </c>
       <c r="D419" s="3" t="inlineStr">
         <is>
-          <t>Ipoteka</t>
+          <t>Ipotekani qayta moliyalashtirish</t>
         </is>
       </c>
       <c r="E419" s="3" t="n">
@@ -26369,7 +26389,7 @@
       <c r="G419" s="3" t="inlineStr"/>
       <c r="H419" s="3" t="inlineStr">
         <is>
-          <t>10 yilgacha</t>
+          <t>3 oy – 10 yil</t>
         </is>
       </c>
       <c r="I419" s="3" t="inlineStr"/>
@@ -26385,13 +26405,13 @@
       </c>
       <c r="L419" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M419" s="3" t="inlineStr"/>
       <c r="N419" s="6" t="inlineStr">
         <is>
-          <t>https://universalbank.uz/credit/ipoteka-ikkilamchi-bozor-uchun</t>
+          <t>https://universalbank.uz/credit/ipotekani-qayta-moliyalashtiri</t>
         </is>
       </c>
     </row>
@@ -26408,27 +26428,35 @@
       </c>
       <c r="C420" s="3" t="inlineStr">
         <is>
-          <t>Ipoteka</t>
+          <t>Iste'mol</t>
         </is>
       </c>
       <c r="D420" s="3" t="inlineStr">
         <is>
-          <t>Ipotekani qayta moliyalashtirish</t>
+          <t>Iste'mol krediti</t>
         </is>
       </c>
       <c r="E420" s="3" t="n">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="F420" s="3" t="n">
-        <v>24</v>
-      </c>
-      <c r="G420" s="3" t="inlineStr"/>
+        <v>32</v>
+      </c>
+      <c r="G420" s="3" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
       <c r="H420" s="3" t="inlineStr">
         <is>
-          <t>3 oy – 10 yil</t>
-        </is>
-      </c>
-      <c r="I420" s="3" t="inlineStr"/>
+          <t>36 oygacha</t>
+        </is>
+      </c>
+      <c r="I420" s="3" t="inlineStr">
+        <is>
+          <t>200 BHM gacha</t>
+        </is>
+      </c>
       <c r="J420" s="3" t="inlineStr">
         <is>
           <t>UZS</t>
@@ -26436,18 +26464,18 @@
       </c>
       <c r="K420" s="3" t="inlineStr">
         <is>
-          <t>Saytdan avtomatik</t>
-        </is>
-      </c>
-      <c r="L420" s="3" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="M420" s="3" t="inlineStr"/>
+          <t>Qo'lda tekshirilgan</t>
+        </is>
+      </c>
+      <c r="L420" s="3" t="inlineStr"/>
+      <c r="M420" s="3" t="inlineStr">
+        <is>
+          <t>Byudjet xodimlari uchun 30%</t>
+        </is>
+      </c>
       <c r="N420" s="6" t="inlineStr">
         <is>
-          <t>https://universalbank.uz/credit/ipotekani-qayta-moliyalashtiri</t>
+          <t>https://universalbank.uz/credit/iste'mol-krediti</t>
         </is>
       </c>
     </row>
@@ -26464,24 +26492,24 @@
       </c>
       <c r="C421" s="3" t="inlineStr">
         <is>
-          <t>Ipoteka</t>
+          <t>Mikroqarz</t>
         </is>
       </c>
       <c r="D421" s="3" t="inlineStr">
         <is>
-          <t>Yashil ta’mir</t>
+          <t>ISHONCH</t>
         </is>
       </c>
       <c r="E421" s="3" t="n">
-        <v>24</v>
+        <v>31</v>
       </c>
       <c r="F421" s="3" t="n">
-        <v>24</v>
+        <v>31</v>
       </c>
       <c r="G421" s="3" t="inlineStr"/>
       <c r="H421" s="3" t="inlineStr">
         <is>
-          <t>5 yilgacha</t>
+          <t>36 oygacha</t>
         </is>
       </c>
       <c r="I421" s="3" t="inlineStr"/>
@@ -26492,18 +26520,18 @@
       </c>
       <c r="K421" s="3" t="inlineStr">
         <is>
-          <t>Saytdan avtomatik</t>
-        </is>
-      </c>
-      <c r="L421" s="3" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="M421" s="3" t="inlineStr"/>
+          <t>Qo'lda tekshirilgan</t>
+        </is>
+      </c>
+      <c r="L421" s="3" t="inlineStr"/>
+      <c r="M421" s="3" t="inlineStr">
+        <is>
+          <t>1 oygacha imtiyoz</t>
+        </is>
+      </c>
       <c r="N421" s="6" t="inlineStr">
         <is>
-          <t>https://universalbank.uz/credit/yashil-tamir-ipoteka-krediti</t>
+          <t>https://universalbank.uz/credit/mikroqarz-ishonch</t>
         </is>
       </c>
     </row>
@@ -26520,33 +26548,29 @@
       </c>
       <c r="C422" s="3" t="inlineStr">
         <is>
-          <t>Iste'mol</t>
+          <t>Mikroqarz</t>
         </is>
       </c>
       <c r="D422" s="3" t="inlineStr">
         <is>
-          <t>Iste'mol krediti</t>
+          <t>Mikroqarz (byudjet)</t>
         </is>
       </c>
       <c r="E422" s="3" t="n">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="F422" s="3" t="n">
-        <v>32</v>
-      </c>
-      <c r="G422" s="3" t="inlineStr">
-        <is>
-          <t>26</t>
-        </is>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="G422" s="3" t="inlineStr"/>
       <c r="H422" s="3" t="inlineStr">
         <is>
-          <t>36 oygacha</t>
+          <t>12 oygacha</t>
         </is>
       </c>
       <c r="I422" s="3" t="inlineStr">
         <is>
-          <t>200 BHM gacha</t>
+          <t>50 mln gacha</t>
         </is>
       </c>
       <c r="J422" s="3" t="inlineStr">
@@ -26562,12 +26586,12 @@
       <c r="L422" s="3" t="inlineStr"/>
       <c r="M422" s="3" t="inlineStr">
         <is>
-          <t>Byudjet xodimlari uchun 30%</t>
+          <t>6 oygacha 24%, 6–12 oy 26%</t>
         </is>
       </c>
       <c r="N422" s="6" t="inlineStr">
         <is>
-          <t>https://universalbank.uz/credit/iste'mol-krediti</t>
+          <t>https://universalbank.uz/credit/mikroqarz-byudjet</t>
         </is>
       </c>
     </row>
@@ -26584,27 +26608,31 @@
       </c>
       <c r="C423" s="3" t="inlineStr">
         <is>
-          <t>Iste'mol</t>
+          <t>Mikroqarz</t>
         </is>
       </c>
       <c r="D423" s="3" t="inlineStr">
         <is>
-          <t>Comfort house</t>
+          <t>Mikrokredit - 300</t>
         </is>
       </c>
       <c r="E423" s="3" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="F423" s="3" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="G423" s="3" t="inlineStr"/>
       <c r="H423" s="3" t="inlineStr">
         <is>
-          <t>10 yilgacha</t>
-        </is>
-      </c>
-      <c r="I423" s="3" t="inlineStr"/>
+          <t>1 oy – 5 yil</t>
+        </is>
+      </c>
+      <c r="I423" s="3" t="inlineStr">
+        <is>
+          <t>300 mln gacha</t>
+        </is>
+      </c>
       <c r="J423" s="3" t="inlineStr">
         <is>
           <t>UZS</t>
@@ -26617,13 +26645,13 @@
       </c>
       <c r="L423" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M423" s="3" t="inlineStr"/>
       <c r="N423" s="6" t="inlineStr">
         <is>
-          <t>https://universalbank.uz/credit/comfort-house-iste'mol-krediti</t>
+          <t>https://universalbank.uz/credit/mikrokredit-300</t>
         </is>
       </c>
     </row>
@@ -26645,22 +26673,26 @@
       </c>
       <c r="D424" s="3" t="inlineStr">
         <is>
-          <t>ISHONCH</t>
+          <t>Mikroqarz</t>
         </is>
       </c>
       <c r="E424" s="3" t="n">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="F424" s="3" t="n">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="G424" s="3" t="inlineStr"/>
       <c r="H424" s="3" t="inlineStr">
         <is>
-          <t>36 oygacha</t>
-        </is>
-      </c>
-      <c r="I424" s="3" t="inlineStr"/>
+          <t>3 yil – 5 yil</t>
+        </is>
+      </c>
+      <c r="I424" s="3" t="inlineStr">
+        <is>
+          <t>100 mln gacha</t>
+        </is>
+      </c>
       <c r="J424" s="3" t="inlineStr">
         <is>
           <t>UZS</t>
@@ -26668,18 +26700,18 @@
       </c>
       <c r="K424" s="3" t="inlineStr">
         <is>
-          <t>Qo'lda tekshirilgan</t>
-        </is>
-      </c>
-      <c r="L424" s="3" t="inlineStr"/>
-      <c r="M424" s="3" t="inlineStr">
-        <is>
-          <t>1 oygacha imtiyoz</t>
-        </is>
-      </c>
+          <t>Saytdan avtomatik</t>
+        </is>
+      </c>
+      <c r="L424" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="M424" s="3" t="inlineStr"/>
       <c r="N424" s="6" t="inlineStr">
         <is>
-          <t>https://universalbank.uz/credit/mikroqarz-ishonch</t>
+          <t>https://universalbank.uz/credit/mikroqarz</t>
         </is>
       </c>
     </row>
@@ -26691,36 +26723,32 @@
       </c>
       <c r="B425" s="3" t="inlineStr">
         <is>
-          <t>Jismoniy</t>
+          <t>Yuridik</t>
         </is>
       </c>
       <c r="C425" s="3" t="inlineStr">
         <is>
-          <t>Mikroqarz</t>
+          <t>Biznes</t>
         </is>
       </c>
       <c r="D425" s="3" t="inlineStr">
         <is>
-          <t>Mikroqarz</t>
+          <t>Biznes kreditlari</t>
         </is>
       </c>
       <c r="E425" s="3" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F425" s="3" t="n">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="G425" s="3" t="inlineStr"/>
       <c r="H425" s="3" t="inlineStr">
         <is>
-          <t>3 yilgacha</t>
-        </is>
-      </c>
-      <c r="I425" s="3" t="inlineStr">
-        <is>
-          <t>50 mln gacha</t>
-        </is>
-      </c>
+          <t>36–120 oy</t>
+        </is>
+      </c>
+      <c r="I425" s="3" t="inlineStr"/>
       <c r="J425" s="3" t="inlineStr">
         <is>
           <t>UZS</t>
@@ -26728,18 +26756,18 @@
       </c>
       <c r="K425" s="3" t="inlineStr">
         <is>
-          <t>Saytdan avtomatik</t>
-        </is>
-      </c>
-      <c r="L425" s="3" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="M425" s="3" t="inlineStr"/>
+          <t>Qo'lda tekshirilgan</t>
+        </is>
+      </c>
+      <c r="L425" s="3" t="inlineStr"/>
+      <c r="M425" s="3" t="inlineStr">
+        <is>
+          <t>USD da 12–14%</t>
+        </is>
+      </c>
       <c r="N425" s="6" t="inlineStr">
         <is>
-          <t>https://universalbank.uz/credit/mikroqarz-ishonch</t>
+          <t>https://universalbank.uz/juristic/kreditlar</t>
         </is>
       </c>
     </row>
@@ -26751,36 +26779,32 @@
       </c>
       <c r="B426" s="3" t="inlineStr">
         <is>
-          <t>Jismoniy</t>
+          <t>Yuridik</t>
         </is>
       </c>
       <c r="C426" s="3" t="inlineStr">
         <is>
-          <t>Mikroqarz</t>
+          <t>Biznes</t>
         </is>
       </c>
       <c r="D426" s="3" t="inlineStr">
         <is>
-          <t>Mikroqarz (byudjet)</t>
+          <t>Good customer 100</t>
         </is>
       </c>
       <c r="E426" s="3" t="n">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="F426" s="3" t="n">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="G426" s="3" t="inlineStr"/>
       <c r="H426" s="3" t="inlineStr">
         <is>
-          <t>12 oygacha</t>
-        </is>
-      </c>
-      <c r="I426" s="3" t="inlineStr">
-        <is>
-          <t>50 mln gacha</t>
-        </is>
-      </c>
+          <t>3 oy – 3 yil</t>
+        </is>
+      </c>
+      <c r="I426" s="3" t="inlineStr"/>
       <c r="J426" s="3" t="inlineStr">
         <is>
           <t>UZS</t>
@@ -26788,18 +26812,18 @@
       </c>
       <c r="K426" s="3" t="inlineStr">
         <is>
-          <t>Qo'lda tekshirilgan</t>
-        </is>
-      </c>
-      <c r="L426" s="3" t="inlineStr"/>
-      <c r="M426" s="3" t="inlineStr">
-        <is>
-          <t>6 oygacha 24%, 6–12 oy 26%</t>
-        </is>
-      </c>
+          <t>Saytdan avtomatik</t>
+        </is>
+      </c>
+      <c r="L426" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="M426" s="3" t="inlineStr"/>
       <c r="N426" s="6" t="inlineStr">
         <is>
-          <t>https://universalbank.uz/credit/mikroqarz-byudjet</t>
+          <t>https://universalbank.uz/juristic/credit/good-customer-100</t>
         </is>
       </c>
     </row>
@@ -26811,36 +26835,32 @@
       </c>
       <c r="B427" s="3" t="inlineStr">
         <is>
-          <t>Jismoniy</t>
+          <t>Yuridik</t>
         </is>
       </c>
       <c r="C427" s="3" t="inlineStr">
         <is>
-          <t>Mikroqarz</t>
+          <t>Biznes</t>
         </is>
       </c>
       <c r="D427" s="3" t="inlineStr">
         <is>
-          <t>Mikrokredit - 300</t>
+          <t>Good customer 300</t>
         </is>
       </c>
       <c r="E427" s="3" t="n">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="F427" s="3" t="n">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="G427" s="3" t="inlineStr"/>
       <c r="H427" s="3" t="inlineStr">
         <is>
-          <t>5 yilgacha</t>
-        </is>
-      </c>
-      <c r="I427" s="3" t="inlineStr">
-        <is>
-          <t>300 mln gacha</t>
-        </is>
-      </c>
+          <t>3 oy – 3 yil</t>
+        </is>
+      </c>
+      <c r="I427" s="3" t="inlineStr"/>
       <c r="J427" s="3" t="inlineStr">
         <is>
           <t>UZS</t>
@@ -26853,13 +26873,13 @@
       </c>
       <c r="L427" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M427" s="3" t="inlineStr"/>
       <c r="N427" s="6" t="inlineStr">
         <is>
-          <t>https://universalbank.uz/credit/mikrokredit-300</t>
+          <t>https://universalbank.uz/juristic/credit/good-customer-300</t>
         </is>
       </c>
     </row>
@@ -26871,29 +26891,29 @@
       </c>
       <c r="B428" s="3" t="inlineStr">
         <is>
-          <t>Jismoniy</t>
+          <t>Yuridik</t>
         </is>
       </c>
       <c r="C428" s="3" t="inlineStr">
         <is>
-          <t>Mikroqarz</t>
+          <t>Biznes</t>
         </is>
       </c>
       <c r="D428" s="3" t="inlineStr">
         <is>
-          <t>Mikroqarz</t>
+          <t>Good customer 500</t>
         </is>
       </c>
       <c r="E428" s="3" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="F428" s="3" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="G428" s="3" t="inlineStr"/>
       <c r="H428" s="3" t="inlineStr">
         <is>
-          <t>3 yil – 5 yil</t>
+          <t>3 oy – 3 yil</t>
         </is>
       </c>
       <c r="I428" s="3" t="inlineStr"/>
@@ -26909,13 +26929,13 @@
       </c>
       <c r="L428" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M428" s="3" t="inlineStr"/>
       <c r="N428" s="6" t="inlineStr">
         <is>
-          <t>https://universalbank.uz/credit/mikroqarz</t>
+          <t>https://universalbank.uz/juristic/credit/good-customer-500</t>
         </is>
       </c>
     </row>
@@ -26927,36 +26947,32 @@
       </c>
       <c r="B429" s="3" t="inlineStr">
         <is>
-          <t>Jismoniy</t>
+          <t>Yuridik</t>
         </is>
       </c>
       <c r="C429" s="3" t="inlineStr">
         <is>
-          <t>Mikroqarz</t>
+          <t>Biznes</t>
         </is>
       </c>
       <c r="D429" s="3" t="inlineStr">
         <is>
-          <t>Mikroqarz</t>
+          <t>BlueOrchard</t>
         </is>
       </c>
       <c r="E429" s="3" t="n">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="F429" s="3" t="n">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="G429" s="3" t="inlineStr"/>
       <c r="H429" s="3" t="inlineStr">
         <is>
-          <t>1 yilgacha</t>
-        </is>
-      </c>
-      <c r="I429" s="3" t="inlineStr">
-        <is>
-          <t>50 mln gacha</t>
-        </is>
-      </c>
+          <t>6 oy – 5 yil</t>
+        </is>
+      </c>
+      <c r="I429" s="3" t="inlineStr"/>
       <c r="J429" s="3" t="inlineStr">
         <is>
           <t>UZS</t>
@@ -26969,13 +26985,13 @@
       </c>
       <c r="L429" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M429" s="3" t="inlineStr"/>
       <c r="N429" s="6" t="inlineStr">
         <is>
-          <t>https://universalbank.uz/credit/mikroqarz-byudjet</t>
+          <t>https://universalbank.uz/juristic/credit/blueorchard</t>
         </is>
       </c>
     </row>
@@ -26997,11 +27013,11 @@
       </c>
       <c r="D430" s="3" t="inlineStr">
         <is>
-          <t>Biznes kreditlari</t>
+          <t>Simbiotics</t>
         </is>
       </c>
       <c r="E430" s="3" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="F430" s="3" t="n">
         <v>30</v>
@@ -27009,7 +27025,7 @@
       <c r="G430" s="3" t="inlineStr"/>
       <c r="H430" s="3" t="inlineStr">
         <is>
-          <t>36–120 oy</t>
+          <t>6 oy – 5 yil</t>
         </is>
       </c>
       <c r="I430" s="3" t="inlineStr"/>
@@ -27020,57 +27036,57 @@
       </c>
       <c r="K430" s="3" t="inlineStr">
         <is>
-          <t>Qo'lda tekshirilgan</t>
-        </is>
-      </c>
-      <c r="L430" s="3" t="inlineStr"/>
-      <c r="M430" s="3" t="inlineStr">
-        <is>
-          <t>USD da 12–14%</t>
-        </is>
-      </c>
+          <t>Saytdan avtomatik</t>
+        </is>
+      </c>
+      <c r="L430" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="M430" s="3" t="inlineStr"/>
       <c r="N430" s="6" t="inlineStr">
         <is>
-          <t>https://universalbank.uz/juristic/kreditlar</t>
+          <t>https://universalbank.uz/juristic/credit/simbiotics</t>
         </is>
       </c>
     </row>
     <row r="431">
       <c r="A431" s="3" t="inlineStr">
         <is>
-          <t>Uzum Bank</t>
+          <t>Universal bank</t>
         </is>
       </c>
       <c r="B431" s="3" t="inlineStr">
         <is>
-          <t>Jismoniy</t>
+          <t>Yuridik</t>
         </is>
       </c>
       <c r="C431" s="3" t="inlineStr">
         <is>
-          <t>Mikroqarz</t>
+          <t>Biznes</t>
         </is>
       </c>
       <c r="D431" s="3" t="inlineStr">
         <is>
-          <t>Mikroqarz (Uzum Nasiya orqali)</t>
+          <t>Qulay</t>
         </is>
       </c>
       <c r="E431" s="3" t="n">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="F431" s="3" t="n">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="G431" s="3" t="inlineStr"/>
       <c r="H431" s="3" t="inlineStr">
         <is>
-          <t>30 kun</t>
+          <t>3 oy – 3 yil</t>
         </is>
       </c>
       <c r="I431" s="3" t="inlineStr">
         <is>
-          <t>25 mln gacha</t>
+          <t>3 mlrd gacha</t>
         </is>
       </c>
       <c r="J431" s="3" t="inlineStr">
@@ -27080,55 +27096,59 @@
       </c>
       <c r="K431" s="3" t="inlineStr">
         <is>
-          <t>Qo'lda tekshirilgan</t>
-        </is>
-      </c>
-      <c r="L431" s="3" t="inlineStr"/>
-      <c r="M431" s="3" t="inlineStr">
-        <is>
-          <t>30 kundan keyin qarz 12 ta to'lovga bo'linadi (Uzum Nasiya komissiyasi bilan); kartaga o'tkazish 5%</t>
-        </is>
-      </c>
+          <t>Saytdan avtomatik</t>
+        </is>
+      </c>
+      <c r="L431" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="M431" s="3" t="inlineStr"/>
       <c r="N431" s="6" t="inlineStr">
         <is>
-          <t>https://uzumbank.uz/en/card/</t>
+          <t>https://universalbank.uz/juristic/credit/qulay</t>
         </is>
       </c>
     </row>
     <row r="432">
       <c r="A432" s="3" t="inlineStr">
         <is>
-          <t>Xalq banki</t>
+          <t>Universal bank</t>
         </is>
       </c>
       <c r="B432" s="3" t="inlineStr">
         <is>
-          <t>Jismoniy</t>
+          <t>Yuridik</t>
         </is>
       </c>
       <c r="C432" s="3" t="inlineStr">
         <is>
-          <t>Iste'mol</t>
+          <t>Biznes</t>
         </is>
       </c>
       <c r="D432" s="3" t="inlineStr">
         <is>
-          <t>Byudjet tashkiloti xodimlari uchun</t>
+          <t>ESG Finance</t>
         </is>
       </c>
       <c r="E432" s="3" t="n">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="F432" s="3" t="n">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="G432" s="3" t="inlineStr"/>
       <c r="H432" s="3" t="inlineStr">
         <is>
-          <t>4 yilgacha</t>
-        </is>
-      </c>
-      <c r="I432" s="3" t="inlineStr"/>
+          <t>6 oy – 5 yil</t>
+        </is>
+      </c>
+      <c r="I432" s="3" t="inlineStr">
+        <is>
+          <t>3 mlrd gacha</t>
+        </is>
+      </c>
       <c r="J432" s="3" t="inlineStr">
         <is>
           <t>UZS</t>
@@ -27136,29 +27156,25 @@
       </c>
       <c r="K432" s="3" t="inlineStr">
         <is>
-          <t>Qo'lda tekshirilgan</t>
+          <t>Saytdan avtomatik</t>
         </is>
       </c>
       <c r="L432" s="3" t="inlineStr">
         <is>
-          <t>2024-03</t>
-        </is>
-      </c>
-      <c r="M432" s="3" t="inlineStr">
-        <is>
-          <t>2024 yilgi hujjat</t>
-        </is>
-      </c>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="M432" s="3" t="inlineStr"/>
       <c r="N432" s="6" t="inlineStr">
         <is>
-          <t>https://xb.uz/cdn/2/uploads/2024/03/13/10/37/xFOk3qk78QLp4M9iml5Dtfxdpf4RAJg9WlWzWtIymDeLH1KET7RIL94TKXcXfUC7.pdf</t>
+          <t>https://universalbank.uz/juristic/credit/esg-finance</t>
         </is>
       </c>
     </row>
     <row r="433">
       <c r="A433" s="3" t="inlineStr">
         <is>
-          <t>Xalq banki</t>
+          <t>Uzum Bank</t>
         </is>
       </c>
       <c r="B433" s="3" t="inlineStr">
@@ -27168,27 +27184,31 @@
       </c>
       <c r="C433" s="3" t="inlineStr">
         <is>
-          <t>Iste'mol</t>
+          <t>Mikroqarz</t>
         </is>
       </c>
       <c r="D433" s="3" t="inlineStr">
         <is>
-          <t>Ish haqi loyihasi ishtirokchilari uchun</t>
+          <t>Mikroqarz (Uzum Nasiya orqali)</t>
         </is>
       </c>
       <c r="E433" s="3" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="F433" s="3" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="G433" s="3" t="inlineStr"/>
       <c r="H433" s="3" t="inlineStr">
         <is>
-          <t>1–4 yil</t>
-        </is>
-      </c>
-      <c r="I433" s="3" t="inlineStr"/>
+          <t>30 kun</t>
+        </is>
+      </c>
+      <c r="I433" s="3" t="inlineStr">
+        <is>
+          <t>25 mln gacha</t>
+        </is>
+      </c>
       <c r="J433" s="3" t="inlineStr">
         <is>
           <t>UZS</t>
@@ -27199,19 +27219,15 @@
           <t>Qo'lda tekshirilgan</t>
         </is>
       </c>
-      <c r="L433" s="3" t="inlineStr">
-        <is>
-          <t>2024-03</t>
-        </is>
-      </c>
+      <c r="L433" s="3" t="inlineStr"/>
       <c r="M433" s="3" t="inlineStr">
         <is>
-          <t>1 yil 25%, 2 yil 26%, 3 yil 28%, 4 yil 30%; 2024 yilgi hujjat</t>
+          <t>30 kundan keyin qarz 12 ta to'lovga bo'linadi (Uzum Nasiya komissiyasi bilan); kartaga o'tkazish 5%</t>
         </is>
       </c>
       <c r="N433" s="6" t="inlineStr">
         <is>
-          <t>https://xb.uz/cdn/2/uploads/2024/03/13/10/37/xFOk3qk78QLp4M9iml5Dtfxdpf4RAJg9WlWzWtIymDeLH1KET7RIL94TKXcXfUC7.pdf</t>
+          <t>https://uzumbank.uz/en/card/</t>
         </is>
       </c>
     </row>
@@ -27233,19 +27249,19 @@
       </c>
       <c r="D434" s="3" t="inlineStr">
         <is>
-          <t>"Moliyaviy ommabop" krediti</t>
+          <t>Byudjet tashkiloti xodimlari uchun</t>
         </is>
       </c>
       <c r="E434" s="3" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="F434" s="3" t="n">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="G434" s="3" t="inlineStr"/>
       <c r="H434" s="3" t="inlineStr">
         <is>
-          <t>3 yilgacha</t>
+          <t>4 yilgacha</t>
         </is>
       </c>
       <c r="I434" s="3" t="inlineStr"/>
@@ -27256,25 +27272,29 @@
       </c>
       <c r="K434" s="3" t="inlineStr">
         <is>
-          <t>Saytdan avtomatik</t>
+          <t>Qo'lda tekshirilgan</t>
         </is>
       </c>
       <c r="L434" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="M434" s="3" t="inlineStr"/>
+          <t>2024-03</t>
+        </is>
+      </c>
+      <c r="M434" s="3" t="inlineStr">
+        <is>
+          <t>2024 yilgi hujjat</t>
+        </is>
+      </c>
       <c r="N434" s="6" t="inlineStr">
         <is>
-          <t>https://xb.uz/page/moliyaviy-ommabop-krediti</t>
+          <t>https://xb.uz/cdn/2/uploads/2024/03/13/10/37/xFOk3qk78QLp4M9iml5Dtfxdpf4RAJg9WlWzWtIymDeLH1KET7RIL94TKXcXfUC7.pdf</t>
         </is>
       </c>
     </row>
     <row r="435">
       <c r="A435" s="3" t="inlineStr">
         <is>
-          <t>Ziraat Bank O'zbekiston</t>
+          <t>Xalq banki</t>
         </is>
       </c>
       <c r="B435" s="3" t="inlineStr">
@@ -27289,19 +27309,19 @@
       </c>
       <c r="D435" s="3" t="inlineStr">
         <is>
-          <t>Iste`mol kredit "Shinam uy"</t>
+          <t>Ish haqi loyihasi ishtirokchilari uchun</t>
         </is>
       </c>
       <c r="E435" s="3" t="n">
         <v>25</v>
       </c>
       <c r="F435" s="3" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="G435" s="3" t="inlineStr"/>
       <c r="H435" s="3" t="inlineStr">
         <is>
-          <t>1 oy – 3 yil</t>
+          <t>1–4 yil</t>
         </is>
       </c>
       <c r="I435" s="3" t="inlineStr"/>
@@ -27312,25 +27332,29 @@
       </c>
       <c r="K435" s="3" t="inlineStr">
         <is>
-          <t>Saytdan avtomatik</t>
+          <t>Qo'lda tekshirilgan</t>
         </is>
       </c>
       <c r="L435" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="M435" s="3" t="inlineStr"/>
+          <t>2024-03</t>
+        </is>
+      </c>
+      <c r="M435" s="3" t="inlineStr">
+        <is>
+          <t>1 yil 25%, 2 yil 26%, 3 yil 28%, 4 yil 30%; 2024 yilgi hujjat</t>
+        </is>
+      </c>
       <c r="N435" s="6" t="inlineStr">
         <is>
-          <t>https://ziraatbank.uz/uz/%D1%88%D0%B8%D0%BD%D0%B0%D0%BC-%D1%83%D0%B9</t>
+          <t>https://xb.uz/cdn/2/uploads/2024/03/13/10/37/xFOk3qk78QLp4M9iml5Dtfxdpf4RAJg9WlWzWtIymDeLH1KET7RIL94TKXcXfUC7.pdf</t>
         </is>
       </c>
     </row>
     <row r="436">
       <c r="A436" s="3" t="inlineStr">
         <is>
-          <t>Ziraat Bank O'zbekiston</t>
+          <t>Xalq banki</t>
         </is>
       </c>
       <c r="B436" s="3" t="inlineStr">
@@ -27345,19 +27369,19 @@
       </c>
       <c r="D436" s="3" t="inlineStr">
         <is>
-          <t>Iste'mol kredit "Yashil Komfort"</t>
+          <t>"Moliyaviy ommabop" krediti</t>
         </is>
       </c>
       <c r="E436" s="3" t="n">
+        <v>23</v>
+      </c>
+      <c r="F436" s="3" t="n">
         <v>24</v>
-      </c>
-      <c r="F436" s="3" t="n">
-        <v>25</v>
       </c>
       <c r="G436" s="3" t="inlineStr"/>
       <c r="H436" s="3" t="inlineStr">
         <is>
-          <t>6 oy – 5 yil</t>
+          <t>3 yilgacha</t>
         </is>
       </c>
       <c r="I436" s="3" t="inlineStr"/>
@@ -27373,13 +27397,13 @@
       </c>
       <c r="L436" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M436" s="3" t="inlineStr"/>
       <c r="N436" s="6" t="inlineStr">
         <is>
-          <t>https://ziraatbank.uz/uz/iste-mol-kredit----yashil-komfort---</t>
+          <t>https://xb.uz/page/moliyaviy-ommabop-krediti</t>
         </is>
       </c>
     </row>
@@ -27401,19 +27425,19 @@
       </c>
       <c r="D437" s="3" t="inlineStr">
         <is>
-          <t>ECO SARMOYA</t>
+          <t>Iste`mol kredit "Shinam uy"</t>
         </is>
       </c>
       <c r="E437" s="3" t="n">
-        <v>23.5</v>
+        <v>25</v>
       </c>
       <c r="F437" s="3" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="G437" s="3" t="inlineStr"/>
       <c r="H437" s="3" t="inlineStr">
         <is>
-          <t>6 oy – 5 yil</t>
+          <t>1 oy – 3 yil</t>
         </is>
       </c>
       <c r="I437" s="3" t="inlineStr"/>
@@ -27429,13 +27453,13 @@
       </c>
       <c r="L437" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M437" s="3" t="inlineStr"/>
       <c r="N437" s="6" t="inlineStr">
         <is>
-          <t>https://ziraatbank.uz/uz/eco-sarmoya</t>
+          <t>https://ziraatbank.uz/uz/%D1%88%D0%B8%D0%BD%D0%B0%D0%BC-%D1%83%D0%B9</t>
         </is>
       </c>
     </row>
@@ -27452,31 +27476,27 @@
       </c>
       <c r="C438" s="3" t="inlineStr">
         <is>
-          <t>Mikroqarz</t>
+          <t>Iste'mol</t>
         </is>
       </c>
       <c r="D438" s="3" t="inlineStr">
         <is>
-          <t>Mikroqarz</t>
+          <t>Iste'mol kredit "Yashil Komfort"</t>
         </is>
       </c>
       <c r="E438" s="3" t="n">
+        <v>24</v>
+      </c>
+      <c r="F438" s="3" t="n">
         <v>25</v>
-      </c>
-      <c r="F438" s="3" t="n">
-        <v>26.5</v>
       </c>
       <c r="G438" s="3" t="inlineStr"/>
       <c r="H438" s="3" t="inlineStr">
         <is>
-          <t>1–36 oy</t>
-        </is>
-      </c>
-      <c r="I438" s="3" t="inlineStr">
-        <is>
-          <t>20 mln dan</t>
-        </is>
-      </c>
+          <t>6 oy – 5 yil</t>
+        </is>
+      </c>
+      <c r="I438" s="3" t="inlineStr"/>
       <c r="J438" s="3" t="inlineStr">
         <is>
           <t>UZS</t>
@@ -27484,18 +27504,18 @@
       </c>
       <c r="K438" s="3" t="inlineStr">
         <is>
-          <t>Qo'lda tekshirilgan</t>
-        </is>
-      </c>
-      <c r="L438" s="3" t="inlineStr"/>
-      <c r="M438" s="3" t="inlineStr">
-        <is>
-          <t>1–12 oy 25%, 13–24 oy 26%, 25–36 oy 26.5% (rasmiy daromadli)</t>
-        </is>
-      </c>
+          <t>Saytdan avtomatik</t>
+        </is>
+      </c>
+      <c r="L438" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="M438" s="3" t="inlineStr"/>
       <c r="N438" s="6" t="inlineStr">
         <is>
-          <t>https://ziraatbank.uz/uz/mikroqarz</t>
+          <t>https://ziraatbank.uz/uz/iste-mol-kredit----yashil-komfort---</t>
         </is>
       </c>
     </row>
@@ -27512,24 +27532,24 @@
       </c>
       <c r="C439" s="3" t="inlineStr">
         <is>
-          <t>Mikroqarz</t>
+          <t>Iste'mol</t>
         </is>
       </c>
       <c r="D439" s="3" t="inlineStr">
         <is>
-          <t>Mikroqarz</t>
+          <t>ECO SARMOYA</t>
         </is>
       </c>
       <c r="E439" s="3" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="F439" s="3" t="n">
         <v>25</v>
-      </c>
-      <c r="F439" s="3" t="n">
-        <v>26.5</v>
       </c>
       <c r="G439" s="3" t="inlineStr"/>
       <c r="H439" s="3" t="inlineStr">
         <is>
-          <t>1 oy – 3 yil</t>
+          <t>6 oy – 5 yil</t>
         </is>
       </c>
       <c r="I439" s="3" t="inlineStr"/>
@@ -27545,18 +27565,134 @@
       </c>
       <c r="L439" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M439" s="3" t="inlineStr"/>
       <c r="N439" s="6" t="inlineStr">
         <is>
+          <t>https://ziraatbank.uz/uz/eco-sarmoya</t>
+        </is>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" s="3" t="inlineStr">
+        <is>
+          <t>Ziraat Bank O'zbekiston</t>
+        </is>
+      </c>
+      <c r="B440" s="3" t="inlineStr">
+        <is>
+          <t>Jismoniy</t>
+        </is>
+      </c>
+      <c r="C440" s="3" t="inlineStr">
+        <is>
+          <t>Mikroqarz</t>
+        </is>
+      </c>
+      <c r="D440" s="3" t="inlineStr">
+        <is>
+          <t>Mikroqarz</t>
+        </is>
+      </c>
+      <c r="E440" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="F440" s="3" t="n">
+        <v>26.5</v>
+      </c>
+      <c r="G440" s="3" t="inlineStr"/>
+      <c r="H440" s="3" t="inlineStr">
+        <is>
+          <t>1–36 oy</t>
+        </is>
+      </c>
+      <c r="I440" s="3" t="inlineStr">
+        <is>
+          <t>20 mln dan</t>
+        </is>
+      </c>
+      <c r="J440" s="3" t="inlineStr">
+        <is>
+          <t>UZS</t>
+        </is>
+      </c>
+      <c r="K440" s="3" t="inlineStr">
+        <is>
+          <t>Qo'lda tekshirilgan</t>
+        </is>
+      </c>
+      <c r="L440" s="3" t="inlineStr"/>
+      <c r="M440" s="3" t="inlineStr">
+        <is>
+          <t>1–12 oy 25%, 13–24 oy 26%, 25–36 oy 26.5% (rasmiy daromadli)</t>
+        </is>
+      </c>
+      <c r="N440" s="6" t="inlineStr">
+        <is>
           <t>https://ziraatbank.uz/uz/mikroqarz</t>
         </is>
       </c>
     </row>
+    <row r="441">
+      <c r="A441" s="3" t="inlineStr">
+        <is>
+          <t>Ziraat Bank O'zbekiston</t>
+        </is>
+      </c>
+      <c r="B441" s="3" t="inlineStr">
+        <is>
+          <t>Jismoniy</t>
+        </is>
+      </c>
+      <c r="C441" s="3" t="inlineStr">
+        <is>
+          <t>Mikroqarz</t>
+        </is>
+      </c>
+      <c r="D441" s="3" t="inlineStr">
+        <is>
+          <t>Mikroqarz</t>
+        </is>
+      </c>
+      <c r="E441" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="F441" s="3" t="n">
+        <v>26.5</v>
+      </c>
+      <c r="G441" s="3" t="inlineStr"/>
+      <c r="H441" s="3" t="inlineStr">
+        <is>
+          <t>1 oy – 3 yil</t>
+        </is>
+      </c>
+      <c r="I441" s="3" t="inlineStr"/>
+      <c r="J441" s="3" t="inlineStr">
+        <is>
+          <t>UZS</t>
+        </is>
+      </c>
+      <c r="K441" s="3" t="inlineStr">
+        <is>
+          <t>Saytdan avtomatik</t>
+        </is>
+      </c>
+      <c r="L441" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="M441" s="3" t="inlineStr"/>
+      <c r="N441" s="6" t="inlineStr">
+        <is>
+          <t>https://ziraatbank.uz/uz/mikroqarz</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N439"/>
+  <autoFilter ref="A1:N441"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N3" r:id="rId2"/>
@@ -27996,6 +28132,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N437" r:id="rId436"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N438" r:id="rId437"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N439" r:id="rId438"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N440" r:id="rId439"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N441" r:id="rId440"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -28781,10 +28919,10 @@
         </is>
       </c>
       <c r="B28" s="3" t="n">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="C28" s="3" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
@@ -28792,7 +28930,7 @@
         </is>
       </c>
       <c r="E28" s="3" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F28" s="3" t="inlineStr"/>
       <c r="G28" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Ma'lumot avtomatik yangilandi (2026-10-23)
</commit_message>
<xml_diff>
--- a/docs/banklar_kreditlar.xlsx
+++ b/docs/banklar_kreditlar.xlsx
@@ -2223,7 +2223,7 @@
       </c>
       <c r="L3" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M3" s="3" t="inlineStr"/>
@@ -2283,7 +2283,7 @@
       </c>
       <c r="L4" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M4" s="3" t="inlineStr"/>
@@ -2343,7 +2343,7 @@
       </c>
       <c r="L5" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M5" s="3" t="inlineStr"/>
@@ -2403,7 +2403,7 @@
       </c>
       <c r="L6" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M6" s="3" t="inlineStr"/>
@@ -2463,7 +2463,7 @@
       </c>
       <c r="L7" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M7" s="3" t="inlineStr"/>
@@ -2523,7 +2523,7 @@
       </c>
       <c r="L8" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M8" s="3" t="inlineStr"/>
@@ -2639,7 +2639,7 @@
       </c>
       <c r="L10" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M10" s="3" t="inlineStr"/>
@@ -2699,7 +2699,7 @@
       </c>
       <c r="L11" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M11" s="3" t="inlineStr"/>
@@ -2815,7 +2815,7 @@
       </c>
       <c r="L13" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M13" s="3" t="inlineStr"/>
@@ -2875,7 +2875,7 @@
       </c>
       <c r="L14" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M14" s="3" t="inlineStr"/>
@@ -2935,7 +2935,7 @@
       </c>
       <c r="L15" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M15" s="3" t="inlineStr"/>
@@ -3047,7 +3047,7 @@
       </c>
       <c r="L17" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M17" s="3" t="inlineStr"/>
@@ -3107,7 +3107,7 @@
       </c>
       <c r="L18" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M18" s="3" t="inlineStr"/>
@@ -3223,7 +3223,7 @@
       </c>
       <c r="L20" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M20" s="3" t="inlineStr"/>
@@ -3283,7 +3283,7 @@
       </c>
       <c r="L21" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M21" s="3" t="inlineStr"/>
@@ -3343,7 +3343,7 @@
       </c>
       <c r="L22" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M22" s="3" t="inlineStr"/>
@@ -3403,7 +3403,7 @@
       </c>
       <c r="L23" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M23" s="3" t="inlineStr"/>
@@ -3463,7 +3463,7 @@
       </c>
       <c r="L24" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M24" s="3" t="inlineStr"/>
@@ -3631,7 +3631,7 @@
       </c>
       <c r="L27" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M27" s="3" t="inlineStr"/>
@@ -3691,7 +3691,7 @@
       </c>
       <c r="L28" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M28" s="3" t="inlineStr"/>
@@ -3751,7 +3751,7 @@
       </c>
       <c r="L29" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M29" s="3" t="inlineStr"/>
@@ -3811,7 +3811,7 @@
       </c>
       <c r="L30" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M30" s="3" t="inlineStr"/>
@@ -3871,7 +3871,7 @@
       </c>
       <c r="L31" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M31" s="3" t="inlineStr"/>
@@ -3931,7 +3931,7 @@
       </c>
       <c r="L32" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M32" s="3" t="inlineStr"/>
@@ -3991,7 +3991,7 @@
       </c>
       <c r="L33" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M33" s="3" t="inlineStr"/>
@@ -4051,7 +4051,7 @@
       </c>
       <c r="L34" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M34" s="3" t="inlineStr"/>
@@ -4111,7 +4111,7 @@
       </c>
       <c r="L35" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M35" s="3" t="inlineStr"/>
@@ -4171,7 +4171,7 @@
       </c>
       <c r="L36" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M36" s="3" t="inlineStr"/>
@@ -4227,7 +4227,7 @@
       </c>
       <c r="L37" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M37" s="3" t="inlineStr"/>
@@ -4339,7 +4339,7 @@
       </c>
       <c r="L39" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M39" s="3" t="inlineStr"/>
@@ -4395,7 +4395,7 @@
       </c>
       <c r="L40" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M40" s="3" t="inlineStr"/>
@@ -4451,7 +4451,7 @@
       </c>
       <c r="L41" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M41" s="3" t="inlineStr"/>
@@ -4507,7 +4507,7 @@
       </c>
       <c r="L42" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M42" s="3" t="inlineStr"/>
@@ -4567,7 +4567,7 @@
       </c>
       <c r="L43" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M43" s="3" t="inlineStr"/>
@@ -4627,7 +4627,7 @@
       </c>
       <c r="L44" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M44" s="3" t="inlineStr"/>
@@ -4687,7 +4687,7 @@
       </c>
       <c r="L45" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M45" s="3" t="inlineStr"/>
@@ -4743,7 +4743,7 @@
       </c>
       <c r="L46" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M46" s="3" t="inlineStr"/>
@@ -4799,7 +4799,7 @@
       </c>
       <c r="L47" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M47" s="3" t="inlineStr"/>
@@ -4859,7 +4859,7 @@
       </c>
       <c r="L48" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M48" s="3" t="inlineStr"/>
@@ -4919,7 +4919,7 @@
       </c>
       <c r="L49" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M49" s="3" t="inlineStr"/>
@@ -4979,7 +4979,7 @@
       </c>
       <c r="L50" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M50" s="3" t="inlineStr"/>
@@ -5093,7 +5093,7 @@
       </c>
       <c r="L52" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M52" s="3" t="inlineStr"/>
@@ -5153,7 +5153,7 @@
       </c>
       <c r="L53" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M53" s="3" t="inlineStr"/>
@@ -5213,7 +5213,7 @@
       </c>
       <c r="L54" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M54" s="3" t="inlineStr"/>
@@ -5273,7 +5273,7 @@
       </c>
       <c r="L55" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M55" s="3" t="inlineStr"/>
@@ -5333,7 +5333,7 @@
       </c>
       <c r="L56" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M56" s="3" t="inlineStr"/>
@@ -5445,7 +5445,7 @@
       </c>
       <c r="L58" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M58" s="3" t="inlineStr"/>
@@ -5501,7 +5501,7 @@
       </c>
       <c r="L59" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M59" s="3" t="inlineStr"/>
@@ -6257,7 +6257,7 @@
       </c>
       <c r="L72" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M72" s="3" t="inlineStr"/>
@@ -6369,7 +6369,7 @@
       </c>
       <c r="L74" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M74" s="3" t="inlineStr"/>
@@ -6481,7 +6481,7 @@
       </c>
       <c r="L76" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M76" s="3" t="inlineStr"/>
@@ -6537,7 +6537,7 @@
       </c>
       <c r="L77" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M77" s="3" t="inlineStr"/>
@@ -6593,7 +6593,7 @@
       </c>
       <c r="L78" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M78" s="3" t="inlineStr"/>
@@ -6649,7 +6649,7 @@
       </c>
       <c r="L79" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M79" s="3" t="inlineStr"/>
@@ -6705,7 +6705,7 @@
       </c>
       <c r="L80" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M80" s="3" t="inlineStr"/>
@@ -6761,7 +6761,7 @@
       </c>
       <c r="L81" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M81" s="3" t="inlineStr"/>
@@ -6817,7 +6817,7 @@
       </c>
       <c r="L82" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M82" s="3" t="inlineStr"/>
@@ -6869,7 +6869,7 @@
       </c>
       <c r="L83" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M83" s="3" t="inlineStr"/>
@@ -6929,7 +6929,7 @@
       </c>
       <c r="L84" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M84" s="3" t="inlineStr"/>
@@ -6989,7 +6989,7 @@
       </c>
       <c r="L85" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M85" s="3" t="inlineStr"/>
@@ -7049,7 +7049,7 @@
       </c>
       <c r="L86" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M86" s="3" t="inlineStr"/>
@@ -7109,7 +7109,7 @@
       </c>
       <c r="L87" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M87" s="3" t="inlineStr"/>
@@ -7169,7 +7169,7 @@
       </c>
       <c r="L88" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M88" s="3" t="inlineStr"/>
@@ -7225,7 +7225,7 @@
       </c>
       <c r="L89" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M89" s="3" t="inlineStr"/>
@@ -7277,7 +7277,7 @@
       </c>
       <c r="L90" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M90" s="3" t="inlineStr"/>
@@ -7389,7 +7389,7 @@
       </c>
       <c r="L92" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M92" s="3" t="inlineStr"/>
@@ -7445,7 +7445,7 @@
       </c>
       <c r="L93" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M93" s="3" t="inlineStr"/>
@@ -7505,7 +7505,7 @@
       </c>
       <c r="L94" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M94" s="3" t="inlineStr"/>
@@ -7565,7 +7565,7 @@
       </c>
       <c r="L95" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M95" s="3" t="inlineStr"/>
@@ -7625,7 +7625,7 @@
       </c>
       <c r="L96" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M96" s="3" t="inlineStr"/>
@@ -7685,7 +7685,7 @@
       </c>
       <c r="L97" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M97" s="3" t="inlineStr"/>
@@ -7745,7 +7745,7 @@
       </c>
       <c r="L98" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M98" s="3" t="inlineStr"/>
@@ -7805,7 +7805,7 @@
       </c>
       <c r="L99" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M99" s="3" t="inlineStr"/>
@@ -7865,7 +7865,7 @@
       </c>
       <c r="L100" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M100" s="3" t="inlineStr"/>
@@ -7925,7 +7925,7 @@
       </c>
       <c r="L101" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M101" s="3" t="inlineStr"/>
@@ -7985,7 +7985,7 @@
       </c>
       <c r="L102" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M102" s="3" t="inlineStr"/>
@@ -8105,7 +8105,7 @@
       </c>
       <c r="L104" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M104" s="3" t="inlineStr"/>
@@ -8165,7 +8165,7 @@
       </c>
       <c r="L105" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M105" s="3" t="inlineStr"/>
@@ -8225,7 +8225,7 @@
       </c>
       <c r="L106" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M106" s="3" t="inlineStr"/>
@@ -8285,7 +8285,7 @@
       </c>
       <c r="L107" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M107" s="3" t="inlineStr"/>
@@ -8345,7 +8345,7 @@
       </c>
       <c r="L108" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M108" s="3" t="inlineStr"/>
@@ -8461,7 +8461,7 @@
       </c>
       <c r="L110" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M110" s="3" t="inlineStr"/>
@@ -8521,7 +8521,7 @@
       </c>
       <c r="L111" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M111" s="3" t="inlineStr"/>
@@ -8581,7 +8581,7 @@
       </c>
       <c r="L112" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M112" s="3" t="inlineStr"/>
@@ -8641,7 +8641,7 @@
       </c>
       <c r="L113" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M113" s="3" t="inlineStr"/>
@@ -8701,7 +8701,7 @@
       </c>
       <c r="L114" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M114" s="3" t="inlineStr"/>
@@ -8757,7 +8757,7 @@
       </c>
       <c r="L115" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M115" s="3" t="inlineStr"/>
@@ -8817,7 +8817,7 @@
       </c>
       <c r="L116" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M116" s="3" t="inlineStr"/>
@@ -8877,7 +8877,7 @@
       </c>
       <c r="L117" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M117" s="3" t="inlineStr"/>
@@ -8933,7 +8933,7 @@
       </c>
       <c r="L118" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M118" s="3" t="inlineStr"/>
@@ -8993,7 +8993,7 @@
       </c>
       <c r="L119" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M119" s="3" t="inlineStr"/>
@@ -9049,7 +9049,7 @@
       </c>
       <c r="L120" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M120" s="3" t="inlineStr"/>
@@ -9105,7 +9105,7 @@
       </c>
       <c r="L121" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M121" s="3" t="inlineStr"/>
@@ -9165,7 +9165,7 @@
       </c>
       <c r="L122" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M122" s="3" t="inlineStr"/>
@@ -9225,7 +9225,7 @@
       </c>
       <c r="L123" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M123" s="3" t="inlineStr"/>
@@ -9285,7 +9285,7 @@
       </c>
       <c r="L124" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M124" s="3" t="inlineStr"/>
@@ -9345,7 +9345,7 @@
       </c>
       <c r="L125" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M125" s="3" t="inlineStr"/>
@@ -9405,7 +9405,7 @@
       </c>
       <c r="L126" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M126" s="3" t="inlineStr"/>
@@ -9465,7 +9465,7 @@
       </c>
       <c r="L127" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M127" s="3" t="inlineStr"/>
@@ -9525,7 +9525,7 @@
       </c>
       <c r="L128" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M128" s="3" t="inlineStr"/>
@@ -9585,7 +9585,7 @@
       </c>
       <c r="L129" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M129" s="3" t="inlineStr"/>
@@ -9645,7 +9645,7 @@
       </c>
       <c r="L130" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M130" s="3" t="inlineStr"/>
@@ -9705,7 +9705,7 @@
       </c>
       <c r="L131" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M131" s="3" t="inlineStr"/>
@@ -9765,7 +9765,7 @@
       </c>
       <c r="L132" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M132" s="3" t="inlineStr"/>
@@ -9825,7 +9825,7 @@
       </c>
       <c r="L133" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M133" s="3" t="inlineStr"/>
@@ -9885,7 +9885,7 @@
       </c>
       <c r="L134" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M134" s="3" t="inlineStr"/>
@@ -9945,7 +9945,7 @@
       </c>
       <c r="L135" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M135" s="3" t="inlineStr"/>
@@ -10005,7 +10005,7 @@
       </c>
       <c r="L136" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M136" s="3" t="inlineStr"/>
@@ -10237,7 +10237,7 @@
       </c>
       <c r="L140" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M140" s="3" t="inlineStr"/>
@@ -10297,7 +10297,7 @@
       </c>
       <c r="L141" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M141" s="3" t="inlineStr"/>
@@ -10357,7 +10357,7 @@
       </c>
       <c r="L142" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M142" s="3" t="inlineStr"/>
@@ -10417,7 +10417,7 @@
       </c>
       <c r="L143" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M143" s="3" t="inlineStr"/>
@@ -10585,7 +10585,7 @@
       </c>
       <c r="L146" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M146" s="3" t="inlineStr"/>
@@ -10873,7 +10873,7 @@
       </c>
       <c r="L151" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M151" s="3" t="inlineStr"/>
@@ -10993,7 +10993,7 @@
       </c>
       <c r="L153" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M153" s="3" t="inlineStr"/>
@@ -11257,7 +11257,7 @@
       </c>
       <c r="L158" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M158" s="3" t="inlineStr"/>
@@ -11373,7 +11373,7 @@
       </c>
       <c r="L160" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M160" s="3" t="inlineStr"/>
@@ -11433,7 +11433,7 @@
       </c>
       <c r="L161" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M161" s="3" t="inlineStr"/>
@@ -11493,7 +11493,7 @@
       </c>
       <c r="L162" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M162" s="3" t="inlineStr"/>
@@ -11663,7 +11663,7 @@
       </c>
       <c r="L165" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M165" s="3" t="inlineStr"/>
@@ -11719,7 +11719,7 @@
       </c>
       <c r="L166" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M166" s="3" t="inlineStr"/>
@@ -11779,7 +11779,7 @@
       </c>
       <c r="L167" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M167" s="3" t="inlineStr"/>
@@ -11839,7 +11839,7 @@
       </c>
       <c r="L168" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M168" s="3" t="inlineStr"/>
@@ -11949,7 +11949,7 @@
       </c>
       <c r="L170" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M170" s="3" t="inlineStr"/>
@@ -12009,7 +12009,7 @@
       </c>
       <c r="L171" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M171" s="3" t="inlineStr"/>
@@ -12065,7 +12065,7 @@
       </c>
       <c r="L172" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M172" s="3" t="inlineStr"/>
@@ -12125,7 +12125,7 @@
       </c>
       <c r="L173" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M173" s="3" t="inlineStr"/>
@@ -12305,7 +12305,7 @@
       </c>
       <c r="L176" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M176" s="3" t="inlineStr"/>
@@ -12365,7 +12365,7 @@
       </c>
       <c r="L177" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M177" s="3" t="inlineStr"/>
@@ -12481,7 +12481,7 @@
       </c>
       <c r="L179" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M179" s="3" t="inlineStr"/>
@@ -12541,7 +12541,7 @@
       </c>
       <c r="L180" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M180" s="3" t="inlineStr"/>
@@ -12597,7 +12597,7 @@
       </c>
       <c r="L181" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M181" s="3" t="inlineStr"/>
@@ -12657,7 +12657,7 @@
       </c>
       <c r="L182" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M182" s="3" t="inlineStr"/>
@@ -12717,7 +12717,7 @@
       </c>
       <c r="L183" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M183" s="3" t="inlineStr"/>
@@ -12773,7 +12773,7 @@
       </c>
       <c r="L184" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M184" s="3" t="inlineStr"/>
@@ -12829,7 +12829,7 @@
       </c>
       <c r="L185" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M185" s="3" t="inlineStr"/>
@@ -12881,7 +12881,7 @@
       </c>
       <c r="L186" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M186" s="3" t="inlineStr"/>
@@ -13053,7 +13053,7 @@
       </c>
       <c r="L189" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M189" s="3" t="inlineStr"/>
@@ -13109,7 +13109,7 @@
       </c>
       <c r="L190" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M190" s="3" t="inlineStr"/>
@@ -13165,7 +13165,7 @@
       </c>
       <c r="L191" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M191" s="3" t="inlineStr"/>
@@ -13221,7 +13221,7 @@
       </c>
       <c r="L192" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M192" s="3" t="inlineStr"/>
@@ -13281,7 +13281,7 @@
       </c>
       <c r="L193" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M193" s="3" t="inlineStr"/>
@@ -13401,7 +13401,7 @@
       </c>
       <c r="L195" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M195" s="3" t="inlineStr"/>
@@ -13517,7 +13517,7 @@
       </c>
       <c r="L197" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M197" s="3" t="inlineStr"/>
@@ -13577,7 +13577,7 @@
       </c>
       <c r="L198" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M198" s="3" t="inlineStr"/>
@@ -13637,7 +13637,7 @@
       </c>
       <c r="L199" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M199" s="3" t="inlineStr"/>
@@ -13757,7 +13757,7 @@
       </c>
       <c r="L201" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M201" s="3" t="inlineStr"/>
@@ -13817,7 +13817,7 @@
       </c>
       <c r="L202" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M202" s="3" t="inlineStr"/>
@@ -13877,7 +13877,7 @@
       </c>
       <c r="L203" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M203" s="3" t="inlineStr"/>
@@ -13937,7 +13937,7 @@
       </c>
       <c r="L204" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M204" s="3" t="inlineStr"/>
@@ -13997,7 +13997,7 @@
       </c>
       <c r="L205" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M205" s="3" t="inlineStr"/>
@@ -14057,7 +14057,7 @@
       </c>
       <c r="L206" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M206" s="3" t="inlineStr"/>
@@ -14117,7 +14117,7 @@
       </c>
       <c r="L207" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M207" s="3" t="inlineStr"/>
@@ -14241,7 +14241,7 @@
       </c>
       <c r="L209" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M209" s="3" t="inlineStr"/>
@@ -14359,7 +14359,7 @@
       </c>
       <c r="L211" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M211" s="3" t="inlineStr"/>
@@ -14533,7 +14533,7 @@
       </c>
       <c r="L214" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M214" s="3" t="inlineStr"/>
@@ -14585,7 +14585,7 @@
       </c>
       <c r="L215" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M215" s="3" t="inlineStr"/>
@@ -14637,7 +14637,7 @@
       </c>
       <c r="L216" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M216" s="3" t="inlineStr"/>
@@ -14747,7 +14747,7 @@
       </c>
       <c r="L218" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M218" s="3" t="inlineStr"/>
@@ -14807,7 +14807,7 @@
       </c>
       <c r="L219" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M219" s="3" t="inlineStr"/>
@@ -14975,7 +14975,7 @@
       </c>
       <c r="L222" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M222" s="3" t="inlineStr"/>
@@ -15379,7 +15379,7 @@
       </c>
       <c r="L229" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M229" s="3" t="inlineStr"/>
@@ -15439,7 +15439,7 @@
       </c>
       <c r="L230" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M230" s="3" t="inlineStr"/>
@@ -15499,7 +15499,7 @@
       </c>
       <c r="L231" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M231" s="3" t="inlineStr"/>
@@ -15619,7 +15619,7 @@
       </c>
       <c r="L233" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M233" s="3" t="inlineStr"/>
@@ -15679,7 +15679,7 @@
       </c>
       <c r="L234" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M234" s="3" t="inlineStr"/>
@@ -15739,7 +15739,7 @@
       </c>
       <c r="L235" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M235" s="3" t="inlineStr"/>
@@ -15795,7 +15795,7 @@
       </c>
       <c r="L236" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M236" s="3" t="inlineStr"/>
@@ -16019,7 +16019,7 @@
       </c>
       <c r="L240" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M240" s="3" t="inlineStr"/>
@@ -16131,7 +16131,7 @@
       </c>
       <c r="L242" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M242" s="3" t="inlineStr"/>
@@ -16187,7 +16187,7 @@
       </c>
       <c r="L243" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M243" s="3" t="inlineStr"/>
@@ -16247,7 +16247,7 @@
       </c>
       <c r="L244" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M244" s="3" t="inlineStr"/>
@@ -16361,7 +16361,7 @@
       </c>
       <c r="L246" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M246" s="3" t="inlineStr"/>
@@ -16417,7 +16417,7 @@
       </c>
       <c r="L247" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M247" s="3" t="inlineStr"/>
@@ -16477,7 +16477,7 @@
       </c>
       <c r="L248" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M248" s="3" t="inlineStr"/>
@@ -16537,7 +16537,7 @@
       </c>
       <c r="L249" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M249" s="3" t="inlineStr"/>
@@ -16597,7 +16597,7 @@
       </c>
       <c r="L250" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M250" s="3" t="inlineStr"/>
@@ -16625,7 +16625,7 @@
       </c>
       <c r="D251" s="3" t="inlineStr">
         <is>
-          <t>NBU’dan UzAuto Motors avtomobillari uchun avtokredit</t>
+          <t>Alyans Auto'dan avtokredit</t>
         </is>
       </c>
       <c r="E251" s="3" t="n">
@@ -16637,12 +16637,12 @@
       <c r="G251" s="3" t="inlineStr"/>
       <c r="H251" s="3" t="inlineStr">
         <is>
-          <t>10 oy – 5 yil</t>
+          <t>2 oy – 5 yil</t>
         </is>
       </c>
       <c r="I251" s="3" t="inlineStr">
         <is>
-          <t>50 mln – 300 mln</t>
+          <t>50 mln – 1 mlrd</t>
         </is>
       </c>
       <c r="J251" s="3" t="inlineStr">
@@ -16657,13 +16657,13 @@
       </c>
       <c r="L251" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M251" s="3" t="inlineStr"/>
       <c r="N251" s="6" t="inlineStr">
         <is>
-          <t>https://nbu.uz/jismoniy-shaxslarga-kreditlar/uzauto-motorsdan-avtokredit</t>
+          <t>https://nbu.uz/jismoniy-shaxslarga-kreditlar/alyans-autodan-avtokredit</t>
         </is>
       </c>
     </row>
@@ -16685,7 +16685,7 @@
       </c>
       <c r="D252" s="3" t="inlineStr">
         <is>
-          <t>Avtokredit KIA</t>
+          <t>NBU’dan UzAuto Motors avtomobillari uchun avtokredit</t>
         </is>
       </c>
       <c r="E252" s="3" t="n">
@@ -16697,12 +16697,12 @@
       <c r="G252" s="3" t="inlineStr"/>
       <c r="H252" s="3" t="inlineStr">
         <is>
-          <t>1 yil – 5 yil</t>
+          <t>10 oy – 5 yil</t>
         </is>
       </c>
       <c r="I252" s="3" t="inlineStr">
         <is>
-          <t>50 mln – 1 mlrd</t>
+          <t>50 mln – 300 mln</t>
         </is>
       </c>
       <c r="J252" s="3" t="inlineStr">
@@ -16717,13 +16717,13 @@
       </c>
       <c r="L252" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M252" s="3" t="inlineStr"/>
       <c r="N252" s="6" t="inlineStr">
         <is>
-          <t>https://nbu.uz/jismoniy-shaxslarga-kreditlar/avtokredit-kia-haval</t>
+          <t>https://nbu.uz/jismoniy-shaxslarga-kreditlar/uzauto-motorsdan-avtokredit</t>
         </is>
       </c>
     </row>
@@ -16745,7 +16745,7 @@
       </c>
       <c r="D253" s="3" t="inlineStr">
         <is>
-          <t>Avtokredit Changan</t>
+          <t>Avtokredit KIA</t>
         </is>
       </c>
       <c r="E253" s="3" t="n">
@@ -16762,7 +16762,7 @@
       </c>
       <c r="I253" s="3" t="inlineStr">
         <is>
-          <t>20 mln – 500 mln</t>
+          <t>50 mln – 1 mlrd</t>
         </is>
       </c>
       <c r="J253" s="3" t="inlineStr">
@@ -16777,13 +16777,13 @@
       </c>
       <c r="L253" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M253" s="3" t="inlineStr"/>
       <c r="N253" s="6" t="inlineStr">
         <is>
-          <t>https://nbu.uz/jismoniy-shaxslarga-kreditlar/changan-avtokrediti</t>
+          <t>https://nbu.uz/jismoniy-shaxslarga-kreditlar/avtokredit-kia-haval</t>
         </is>
       </c>
     </row>
@@ -16805,7 +16805,7 @@
       </c>
       <c r="D254" s="3" t="inlineStr">
         <is>
-          <t>Avtokredit Haval</t>
+          <t>Avtokredit Changan</t>
         </is>
       </c>
       <c r="E254" s="3" t="n">
@@ -16822,7 +16822,7 @@
       </c>
       <c r="I254" s="3" t="inlineStr">
         <is>
-          <t>50 mln – 500 mln</t>
+          <t>20 mln – 500 mln</t>
         </is>
       </c>
       <c r="J254" s="3" t="inlineStr">
@@ -16837,13 +16837,13 @@
       </c>
       <c r="L254" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M254" s="3" t="inlineStr"/>
       <c r="N254" s="6" t="inlineStr">
         <is>
-          <t>https://nbu.uz/jismoniy-shaxslarga-kreditlar/avtokredit-haval</t>
+          <t>https://nbu.uz/jismoniy-shaxslarga-kreditlar/changan-avtokrediti</t>
         </is>
       </c>
     </row>
@@ -16865,24 +16865,24 @@
       </c>
       <c r="D255" s="3" t="inlineStr">
         <is>
-          <t>Elektromobil va gibrid avtomobillar uchun avtokredit</t>
+          <t>Avtokredit Haval</t>
         </is>
       </c>
       <c r="E255" s="3" t="n">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="F255" s="3" t="n">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="G255" s="3" t="inlineStr"/>
       <c r="H255" s="3" t="inlineStr">
         <is>
-          <t>6 oy – 4 yil</t>
+          <t>1 yil – 5 yil</t>
         </is>
       </c>
       <c r="I255" s="3" t="inlineStr">
         <is>
-          <t>100 mln – 500 mln</t>
+          <t>50 mln – 500 mln</t>
         </is>
       </c>
       <c r="J255" s="3" t="inlineStr">
@@ -16897,13 +16897,13 @@
       </c>
       <c r="L255" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M255" s="3" t="inlineStr"/>
       <c r="N255" s="6" t="inlineStr">
         <is>
-          <t>https://nbu.uz/jismoniy-shaxslarga-kreditlar/elektromobillar-va-gibridlar-uchun-avtokredit</t>
+          <t>https://nbu.uz/jismoniy-shaxslarga-kreditlar/avtokredit-haval</t>
         </is>
       </c>
     </row>
@@ -16925,24 +16925,24 @@
       </c>
       <c r="D256" s="3" t="inlineStr">
         <is>
-          <t>Yangi avtomobillar uchun avtokredit</t>
+          <t>Elektromobil va gibrid avtomobillar uchun avtokredit</t>
         </is>
       </c>
       <c r="E256" s="3" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F256" s="3" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G256" s="3" t="inlineStr"/>
       <c r="H256" s="3" t="inlineStr">
         <is>
-          <t>6 oy – 5 yil</t>
+          <t>6 oy – 4 yil</t>
         </is>
       </c>
       <c r="I256" s="3" t="inlineStr">
         <is>
-          <t>50 mln – 1 mlrd</t>
+          <t>100 mln – 500 mln</t>
         </is>
       </c>
       <c r="J256" s="3" t="inlineStr">
@@ -16957,13 +16957,13 @@
       </c>
       <c r="L256" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M256" s="3" t="inlineStr"/>
       <c r="N256" s="6" t="inlineStr">
         <is>
-          <t>https://nbu.uz/jismoniy-shaxslarga-kreditlar/yangi-avtomobillar-uchun-avtokredit</t>
+          <t>https://nbu.uz/jismoniy-shaxslarga-kreditlar/elektromobillar-va-gibridlar-uchun-avtokredit</t>
         </is>
       </c>
     </row>
@@ -16980,29 +16980,29 @@
       </c>
       <c r="C257" s="3" t="inlineStr">
         <is>
-          <t>Biznes</t>
+          <t>Avtokredit</t>
         </is>
       </c>
       <c r="D257" s="3" t="inlineStr">
         <is>
-          <t>"Tezkor" krediti</t>
+          <t>Yangi avtomobillar uchun avtokredit</t>
         </is>
       </c>
       <c r="E257" s="3" t="n">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="F257" s="3" t="n">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="G257" s="3" t="inlineStr"/>
       <c r="H257" s="3" t="inlineStr">
         <is>
-          <t>3 oy – 18 oy</t>
+          <t>6 oy – 5 yil</t>
         </is>
       </c>
       <c r="I257" s="3" t="inlineStr">
         <is>
-          <t>100 mln – 1.5 mlrd</t>
+          <t>50 mln – 1 mlrd</t>
         </is>
       </c>
       <c r="J257" s="3" t="inlineStr">
@@ -17017,13 +17017,13 @@
       </c>
       <c r="L257" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M257" s="3" t="inlineStr"/>
       <c r="N257" s="6" t="inlineStr">
         <is>
-          <t>https://nbu.uz/kichik-biznes/kreditlar/tezkor</t>
+          <t>https://nbu.uz/jismoniy-shaxslarga-kreditlar/yangi-avtomobillar-uchun-avtokredit</t>
         </is>
       </c>
     </row>
@@ -17045,24 +17045,24 @@
       </c>
       <c r="D258" s="3" t="inlineStr">
         <is>
-          <t>"Yengil start" krediti</t>
+          <t>"Tezkor" krediti</t>
         </is>
       </c>
       <c r="E258" s="3" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="F258" s="3" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="G258" s="3" t="inlineStr"/>
       <c r="H258" s="3" t="inlineStr">
         <is>
-          <t>6 oy – 3 yil</t>
+          <t>3 oy – 18 oy</t>
         </is>
       </c>
       <c r="I258" s="3" t="inlineStr">
         <is>
-          <t>100 mln gacha</t>
+          <t>100 mln – 1.5 mlrd</t>
         </is>
       </c>
       <c r="J258" s="3" t="inlineStr">
@@ -17077,13 +17077,13 @@
       </c>
       <c r="L258" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M258" s="3" t="inlineStr"/>
       <c r="N258" s="6" t="inlineStr">
         <is>
-          <t>https://nbu.uz/kichik-biznes/kreditlar/kredit-engil-start</t>
+          <t>https://nbu.uz/kichik-biznes/kreditlar/tezkor</t>
         </is>
       </c>
     </row>
@@ -17133,7 +17133,7 @@
       </c>
       <c r="L259" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M259" s="3" t="inlineStr"/>
@@ -17193,7 +17193,7 @@
       </c>
       <c r="L260" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M260" s="3" t="inlineStr"/>
@@ -17317,7 +17317,7 @@
       </c>
       <c r="L262" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M262" s="3" t="inlineStr"/>
@@ -17437,7 +17437,7 @@
       </c>
       <c r="L264" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M264" s="3" t="inlineStr"/>
@@ -17497,7 +17497,7 @@
       </c>
       <c r="L265" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M265" s="3" t="inlineStr"/>
@@ -17617,7 +17617,7 @@
       </c>
       <c r="L267" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M267" s="3" t="inlineStr"/>
@@ -17677,7 +17677,7 @@
       </c>
       <c r="L268" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M268" s="3" t="inlineStr"/>
@@ -17737,7 +17737,7 @@
       </c>
       <c r="L269" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M269" s="3" t="inlineStr"/>
@@ -17793,7 +17793,7 @@
       </c>
       <c r="L270" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M270" s="3" t="inlineStr"/>
@@ -17853,7 +17853,7 @@
       </c>
       <c r="L271" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M271" s="3" t="inlineStr"/>
@@ -18033,7 +18033,7 @@
       </c>
       <c r="L274" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M274" s="3" t="inlineStr"/>
@@ -18093,7 +18093,7 @@
       </c>
       <c r="L275" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M275" s="3" t="inlineStr"/>
@@ -18153,7 +18153,7 @@
       </c>
       <c r="L276" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M276" s="3" t="inlineStr"/>
@@ -18213,7 +18213,7 @@
       </c>
       <c r="L277" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M277" s="3" t="inlineStr"/>
@@ -18273,7 +18273,7 @@
       </c>
       <c r="L278" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M278" s="3" t="inlineStr"/>
@@ -18333,7 +18333,7 @@
       </c>
       <c r="L279" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M279" s="3" t="inlineStr"/>
@@ -18393,7 +18393,7 @@
       </c>
       <c r="L280" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M280" s="3" t="inlineStr"/>
@@ -18453,7 +18453,7 @@
       </c>
       <c r="L281" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M281" s="3" t="inlineStr"/>
@@ -18513,7 +18513,7 @@
       </c>
       <c r="L282" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M282" s="3" t="inlineStr"/>
@@ -18573,7 +18573,7 @@
       </c>
       <c r="L283" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M283" s="3" t="inlineStr"/>
@@ -18633,7 +18633,7 @@
       </c>
       <c r="L284" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M284" s="3" t="inlineStr"/>
@@ -18685,7 +18685,7 @@
       </c>
       <c r="L285" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M285" s="3" t="inlineStr"/>
@@ -18745,7 +18745,7 @@
       </c>
       <c r="L286" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M286" s="3" t="inlineStr"/>
@@ -18805,7 +18805,7 @@
       </c>
       <c r="L287" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M287" s="3" t="inlineStr"/>
@@ -18865,7 +18865,7 @@
       </c>
       <c r="L288" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M288" s="3" t="inlineStr"/>
@@ -18977,7 +18977,7 @@
       </c>
       <c r="L290" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M290" s="3" t="inlineStr"/>
@@ -19037,7 +19037,7 @@
       </c>
       <c r="L291" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M291" s="3" t="inlineStr"/>
@@ -19097,7 +19097,7 @@
       </c>
       <c r="L292" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M292" s="3" t="inlineStr"/>
@@ -19157,7 +19157,7 @@
       </c>
       <c r="L293" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M293" s="3" t="inlineStr"/>
@@ -19329,7 +19329,7 @@
       </c>
       <c r="L296" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M296" s="3" t="inlineStr"/>
@@ -19389,7 +19389,7 @@
       </c>
       <c r="L297" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M297" s="3" t="inlineStr"/>
@@ -19417,24 +19417,22 @@
       </c>
       <c r="D298" s="3" t="inlineStr">
         <is>
-          <t>«Mahalla tadbirkori» mikroqarzi</t>
+          <t>SQB Mobile onlayn mikroqarz</t>
         </is>
       </c>
       <c r="E298" s="3" t="n">
-        <v>25</v>
-      </c>
-      <c r="F298" s="3" t="n">
-        <v>25</v>
-      </c>
+        <v>24</v>
+      </c>
+      <c r="F298" s="3" t="n"/>
       <c r="G298" s="3" t="inlineStr"/>
       <c r="H298" s="3" t="inlineStr">
         <is>
-          <t>5 yilgacha</t>
+          <t>12–48 oy</t>
         </is>
       </c>
       <c r="I298" s="3" t="inlineStr">
         <is>
-          <t>300 mln gacha</t>
+          <t>2–100 mln</t>
         </is>
       </c>
       <c r="J298" s="3" t="inlineStr">
@@ -19444,18 +19442,14 @@
       </c>
       <c r="K298" s="3" t="inlineStr">
         <is>
-          <t>Saytdan avtomatik</t>
-        </is>
-      </c>
-      <c r="L298" s="3" t="inlineStr">
-        <is>
-          <t>2026-10-22</t>
-        </is>
-      </c>
+          <t>Qo'lda tekshirilgan</t>
+        </is>
+      </c>
+      <c r="L298" s="3" t="inlineStr"/>
       <c r="M298" s="3" t="inlineStr"/>
       <c r="N298" s="6" t="inlineStr">
         <is>
-          <t>https://sqb.uz/uz/individuals/credits/mikrokredit-mahalla-tadbirkori-uz/</t>
+          <t>https://sqb.uz/en/individuals/credits/sqb-mobile-ilovasida-mikroqarz-uz/</t>
         </is>
       </c>
     </row>
@@ -19477,22 +19471,24 @@
       </c>
       <c r="D299" s="3" t="inlineStr">
         <is>
-          <t>SQB Mobile onlayn mikroqarz</t>
+          <t>«Mahalla» mikroqarzi</t>
         </is>
       </c>
       <c r="E299" s="3" t="n">
         <v>24</v>
       </c>
-      <c r="F299" s="3" t="n"/>
+      <c r="F299" s="3" t="n">
+        <v>24</v>
+      </c>
       <c r="G299" s="3" t="inlineStr"/>
       <c r="H299" s="3" t="inlineStr">
         <is>
-          <t>12–48 oy</t>
+          <t>5 yilgacha</t>
         </is>
       </c>
       <c r="I299" s="3" t="inlineStr">
         <is>
-          <t>2–100 mln</t>
+          <t>15 mln gacha</t>
         </is>
       </c>
       <c r="J299" s="3" t="inlineStr">
@@ -19502,14 +19498,18 @@
       </c>
       <c r="K299" s="3" t="inlineStr">
         <is>
-          <t>Qo'lda tekshirilgan</t>
-        </is>
-      </c>
-      <c r="L299" s="3" t="inlineStr"/>
+          <t>Saytdan avtomatik</t>
+        </is>
+      </c>
+      <c r="L299" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
       <c r="M299" s="3" t="inlineStr"/>
       <c r="N299" s="6" t="inlineStr">
         <is>
-          <t>https://sqb.uz/en/individuals/credits/sqb-mobile-ilovasida-mikroqarz-uz/</t>
+          <t>https://sqb.uz/uz/individuals/credits/mahalla-mikroqarz-uz/</t>
         </is>
       </c>
     </row>
@@ -19531,24 +19531,24 @@
       </c>
       <c r="D300" s="3" t="inlineStr">
         <is>
-          <t>«Mahalla» mikroqarzi</t>
+          <t>«MikroMadad» mikroqarzi</t>
         </is>
       </c>
       <c r="E300" s="3" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F300" s="3" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="G300" s="3" t="inlineStr"/>
       <c r="H300" s="3" t="inlineStr">
         <is>
-          <t>5 yilgacha</t>
+          <t>4 yilgacha</t>
         </is>
       </c>
       <c r="I300" s="3" t="inlineStr">
         <is>
-          <t>15 mln gacha</t>
+          <t>100 mln gacha</t>
         </is>
       </c>
       <c r="J300" s="3" t="inlineStr">
@@ -19563,13 +19563,13 @@
       </c>
       <c r="L300" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M300" s="3" t="inlineStr"/>
       <c r="N300" s="6" t="inlineStr">
         <is>
-          <t>https://sqb.uz/uz/individuals/credits/mahalla-mikroqarz-uz/</t>
+          <t>https://sqb.uz/uz/individuals/credits/mikromadad-mikroqarz-uz/</t>
         </is>
       </c>
     </row>
@@ -19591,24 +19591,24 @@
       </c>
       <c r="D301" s="3" t="inlineStr">
         <is>
-          <t>«MikroMadad» mikroqarzi</t>
+          <t>«Bir kontur — bir mahsulot» mikroqarzi</t>
         </is>
       </c>
       <c r="E301" s="3" t="n">
-        <v>23</v>
+        <v>22.9</v>
       </c>
       <c r="F301" s="3" t="n">
-        <v>23</v>
+        <v>22.9</v>
       </c>
       <c r="G301" s="3" t="inlineStr"/>
       <c r="H301" s="3" t="inlineStr">
         <is>
-          <t>4 yilgacha</t>
+          <t>18 oygacha</t>
         </is>
       </c>
       <c r="I301" s="3" t="inlineStr">
         <is>
-          <t>100 mln gacha</t>
+          <t>20 mln gacha</t>
         </is>
       </c>
       <c r="J301" s="3" t="inlineStr">
@@ -19623,13 +19623,13 @@
       </c>
       <c r="L301" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M301" s="3" t="inlineStr"/>
       <c r="N301" s="6" t="inlineStr">
         <is>
-          <t>https://sqb.uz/uz/individuals/credits/mikromadad-mikroqarz-uz/</t>
+          <t>https://sqb.uz/uz/individuals/credits/mikrozaym-bir-kontur-bir-mahsulot-uz/</t>
         </is>
       </c>
     </row>
@@ -19651,24 +19651,24 @@
       </c>
       <c r="D302" s="3" t="inlineStr">
         <is>
-          <t>«Bir kontur — bir mahsulot» mikroqarzi</t>
+          <t>«Istiqlol online» mikroqarz</t>
         </is>
       </c>
       <c r="E302" s="3" t="n">
-        <v>22.9</v>
+        <v>21</v>
       </c>
       <c r="F302" s="3" t="n">
-        <v>22.9</v>
+        <v>21</v>
       </c>
       <c r="G302" s="3" t="inlineStr"/>
       <c r="H302" s="3" t="inlineStr">
         <is>
-          <t>18 oygacha</t>
+          <t>3 yilgacha</t>
         </is>
       </c>
       <c r="I302" s="3" t="inlineStr">
         <is>
-          <t>20 mln gacha</t>
+          <t>100 mln gacha</t>
         </is>
       </c>
       <c r="J302" s="3" t="inlineStr">
@@ -19683,13 +19683,13 @@
       </c>
       <c r="L302" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M302" s="3" t="inlineStr"/>
       <c r="N302" s="6" t="inlineStr">
         <is>
-          <t>https://sqb.uz/uz/individuals/credits/mikrozaym-bir-kontur-bir-mahsulot-uz/</t>
+          <t>https://sqb.uz/uz/individuals/credits/mikrozaym-istiqlol-online-uz/</t>
         </is>
       </c>
     </row>
@@ -19743,7 +19743,7 @@
       </c>
       <c r="L303" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M303" s="3" t="inlineStr"/>
@@ -19771,14 +19771,14 @@
       </c>
       <c r="D304" s="3" t="inlineStr">
         <is>
-          <t>«Istiqlol online» mikroqarz</t>
+          <t>«Istiqlol» mikroqarzi</t>
         </is>
       </c>
       <c r="E304" s="3" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F304" s="3" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G304" s="3" t="inlineStr"/>
       <c r="H304" s="3" t="inlineStr">
@@ -19803,13 +19803,13 @@
       </c>
       <c r="L304" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M304" s="3" t="inlineStr"/>
       <c r="N304" s="6" t="inlineStr">
         <is>
-          <t>https://sqb.uz/uz/individuals/credits/mikrozaym-istiqlol-online-uz/</t>
+          <t>https://sqb.uz/uz/individuals/credits/istiqlol-mikroqarz-uz/</t>
         </is>
       </c>
     </row>
@@ -19831,24 +19831,24 @@
       </c>
       <c r="D305" s="3" t="inlineStr">
         <is>
-          <t>«Istiqlol» mikroqarzi</t>
+          <t>«Mahalla tadbirkori» mikroqarzi</t>
         </is>
       </c>
       <c r="E305" s="3" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="F305" s="3" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="G305" s="3" t="inlineStr"/>
       <c r="H305" s="3" t="inlineStr">
         <is>
-          <t>3 yilgacha</t>
+          <t>5 yilgacha</t>
         </is>
       </c>
       <c r="I305" s="3" t="inlineStr">
         <is>
-          <t>100 mln gacha</t>
+          <t>150 mln gacha</t>
         </is>
       </c>
       <c r="J305" s="3" t="inlineStr">
@@ -19863,13 +19863,13 @@
       </c>
       <c r="L305" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M305" s="3" t="inlineStr"/>
       <c r="N305" s="6" t="inlineStr">
         <is>
-          <t>https://sqb.uz/uz/individuals/credits/istiqlol-mikroqarz-uz/</t>
+          <t>https://sqb.uz/uz/individuals/credits/mikrokredit-mahalla-tadbirkori-uz/</t>
         </is>
       </c>
     </row>
@@ -19923,7 +19923,7 @@
       </c>
       <c r="L306" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M306" s="3" t="inlineStr"/>
@@ -19983,7 +19983,7 @@
       </c>
       <c r="L307" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M307" s="3" t="inlineStr"/>
@@ -20039,7 +20039,7 @@
       </c>
       <c r="L308" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M308" s="3" t="inlineStr"/>
@@ -20663,7 +20663,7 @@
       </c>
       <c r="L319" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M319" s="3" t="inlineStr"/>
@@ -20723,7 +20723,7 @@
       </c>
       <c r="L320" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M320" s="3" t="inlineStr"/>
@@ -20899,7 +20899,7 @@
       </c>
       <c r="L323" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M323" s="3" t="inlineStr"/>
@@ -21015,7 +21015,7 @@
       </c>
       <c r="L325" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M325" s="3" t="inlineStr"/>
@@ -21075,7 +21075,7 @@
       </c>
       <c r="L326" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M326" s="3" t="inlineStr"/>
@@ -21135,7 +21135,7 @@
       </c>
       <c r="L327" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M327" s="3" t="inlineStr"/>
@@ -21195,7 +21195,7 @@
       </c>
       <c r="L328" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M328" s="3" t="inlineStr"/>
@@ -21255,7 +21255,7 @@
       </c>
       <c r="L329" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M329" s="3" t="inlineStr"/>
@@ -21315,7 +21315,7 @@
       </c>
       <c r="L330" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M330" s="3" t="inlineStr"/>
@@ -21375,7 +21375,7 @@
       </c>
       <c r="L331" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M331" s="3" t="inlineStr"/>
@@ -21435,7 +21435,7 @@
       </c>
       <c r="L332" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M332" s="3" t="inlineStr"/>
@@ -21491,7 +21491,7 @@
       </c>
       <c r="L333" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M333" s="3" t="inlineStr"/>
@@ -21551,7 +21551,7 @@
       </c>
       <c r="L334" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M334" s="3" t="inlineStr"/>
@@ -21663,7 +21663,7 @@
       </c>
       <c r="L336" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M336" s="3" t="inlineStr"/>
@@ -21723,7 +21723,7 @@
       </c>
       <c r="L337" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M337" s="3" t="inlineStr"/>
@@ -21783,7 +21783,7 @@
       </c>
       <c r="L338" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M338" s="3" t="inlineStr"/>
@@ -21843,7 +21843,7 @@
       </c>
       <c r="L339" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M339" s="3" t="inlineStr"/>
@@ -21963,7 +21963,7 @@
       </c>
       <c r="L341" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M341" s="3" t="inlineStr"/>
@@ -22023,7 +22023,7 @@
       </c>
       <c r="L342" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M342" s="3" t="inlineStr"/>
@@ -22083,7 +22083,7 @@
       </c>
       <c r="L343" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M343" s="3" t="inlineStr"/>
@@ -22199,7 +22199,7 @@
       </c>
       <c r="L345" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M345" s="3" t="inlineStr"/>
@@ -22313,7 +22313,7 @@
       </c>
       <c r="L347" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M347" s="3" t="inlineStr"/>
@@ -22369,7 +22369,7 @@
       </c>
       <c r="L348" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M348" s="3" t="inlineStr"/>
@@ -22481,7 +22481,7 @@
       </c>
       <c r="L350" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M350" s="3" t="inlineStr"/>
@@ -22537,7 +22537,7 @@
       </c>
       <c r="L351" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M351" s="3" t="inlineStr"/>
@@ -22593,7 +22593,7 @@
       </c>
       <c r="L352" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M352" s="3" t="inlineStr"/>
@@ -22705,7 +22705,7 @@
       </c>
       <c r="L354" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M354" s="3" t="inlineStr"/>
@@ -22817,7 +22817,7 @@
       </c>
       <c r="L356" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M356" s="3" t="inlineStr"/>
@@ -22933,7 +22933,7 @@
       </c>
       <c r="L358" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M358" s="3" t="inlineStr"/>
@@ -22989,7 +22989,7 @@
       </c>
       <c r="L359" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M359" s="3" t="inlineStr"/>
@@ -23045,7 +23045,7 @@
       </c>
       <c r="L360" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M360" s="3" t="inlineStr"/>
@@ -23101,7 +23101,7 @@
       </c>
       <c r="L361" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M361" s="3" t="inlineStr"/>
@@ -23157,7 +23157,7 @@
       </c>
       <c r="L362" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M362" s="3" t="inlineStr"/>
@@ -23213,7 +23213,7 @@
       </c>
       <c r="L363" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M363" s="3" t="inlineStr"/>
@@ -23269,7 +23269,7 @@
       </c>
       <c r="L364" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M364" s="3" t="inlineStr"/>
@@ -23325,7 +23325,7 @@
       </c>
       <c r="L365" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M365" s="3" t="inlineStr"/>
@@ -23381,7 +23381,7 @@
       </c>
       <c r="L366" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M366" s="3" t="inlineStr"/>
@@ -23437,7 +23437,7 @@
       </c>
       <c r="L367" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M367" s="3" t="inlineStr"/>
@@ -23493,7 +23493,7 @@
       </c>
       <c r="L368" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M368" s="3" t="inlineStr"/>
@@ -23549,7 +23549,7 @@
       </c>
       <c r="L369" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M369" s="3" t="inlineStr"/>
@@ -23605,7 +23605,7 @@
       </c>
       <c r="L370" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M370" s="3" t="inlineStr"/>
@@ -23665,7 +23665,7 @@
       </c>
       <c r="L371" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M371" s="3" t="inlineStr"/>
@@ -23725,7 +23725,7 @@
       </c>
       <c r="L372" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M372" s="3" t="inlineStr"/>
@@ -23785,7 +23785,7 @@
       </c>
       <c r="L373" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M373" s="3" t="inlineStr"/>
@@ -23837,7 +23837,7 @@
       </c>
       <c r="L374" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M374" s="3" t="inlineStr"/>
@@ -24057,7 +24057,7 @@
       </c>
       <c r="L378" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M378" s="3" t="inlineStr"/>
@@ -24113,7 +24113,7 @@
       </c>
       <c r="L379" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M379" s="3" t="inlineStr"/>
@@ -24169,7 +24169,7 @@
       </c>
       <c r="L380" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M380" s="3" t="inlineStr"/>
@@ -24289,7 +24289,7 @@
       </c>
       <c r="L382" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M382" s="3" t="inlineStr"/>
@@ -24345,7 +24345,7 @@
       </c>
       <c r="L383" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M383" s="3" t="inlineStr"/>
@@ -24577,7 +24577,7 @@
       </c>
       <c r="L387" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M387" s="3" t="inlineStr"/>
@@ -24633,7 +24633,7 @@
       </c>
       <c r="L388" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M388" s="3" t="inlineStr"/>
@@ -24693,7 +24693,7 @@
       </c>
       <c r="L389" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M389" s="3" t="inlineStr"/>
@@ -24805,7 +24805,7 @@
       </c>
       <c r="L391" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M391" s="3" t="inlineStr"/>
@@ -24861,7 +24861,7 @@
       </c>
       <c r="L392" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M392" s="3" t="inlineStr"/>
@@ -24917,7 +24917,7 @@
       </c>
       <c r="L393" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M393" s="3" t="inlineStr"/>
@@ -24973,7 +24973,7 @@
       </c>
       <c r="L394" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M394" s="3" t="inlineStr"/>
@@ -25029,7 +25029,7 @@
       </c>
       <c r="L395" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M395" s="3" t="inlineStr"/>
@@ -25085,7 +25085,7 @@
       </c>
       <c r="L396" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M396" s="3" t="inlineStr"/>
@@ -25141,7 +25141,7 @@
       </c>
       <c r="L397" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M397" s="3" t="inlineStr"/>
@@ -25249,7 +25249,7 @@
       </c>
       <c r="L399" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M399" s="3" t="inlineStr"/>
@@ -25309,7 +25309,7 @@
       </c>
       <c r="L400" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M400" s="3" t="inlineStr"/>
@@ -25369,7 +25369,7 @@
       </c>
       <c r="L401" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M401" s="3" t="inlineStr"/>
@@ -25485,7 +25485,7 @@
       </c>
       <c r="L403" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M403" s="3" t="inlineStr"/>
@@ -25653,7 +25653,7 @@
       </c>
       <c r="L406" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M406" s="3" t="inlineStr"/>
@@ -25713,7 +25713,7 @@
       </c>
       <c r="L407" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M407" s="3" t="inlineStr"/>
@@ -25773,7 +25773,7 @@
       </c>
       <c r="L408" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M408" s="3" t="inlineStr"/>
@@ -25833,7 +25833,7 @@
       </c>
       <c r="L409" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M409" s="3" t="inlineStr"/>
@@ -26154,7 +26154,7 @@
       </c>
       <c r="I415" s="3" t="inlineStr">
         <is>
-          <t>1 mln – 100 mln</t>
+          <t>45.804 – 100 mln</t>
         </is>
       </c>
       <c r="J415" s="3" t="inlineStr">
@@ -26169,7 +26169,7 @@
       </c>
       <c r="L415" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M415" s="3" t="inlineStr"/>
@@ -26229,7 +26229,7 @@
       </c>
       <c r="L416" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M416" s="3" t="inlineStr"/>
@@ -26289,7 +26289,7 @@
       </c>
       <c r="L417" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M417" s="3" t="inlineStr"/>
@@ -26349,7 +26349,7 @@
       </c>
       <c r="L418" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M418" s="3" t="inlineStr"/>
@@ -26405,7 +26405,7 @@
       </c>
       <c r="L419" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M419" s="3" t="inlineStr"/>
@@ -26645,7 +26645,7 @@
       </c>
       <c r="L423" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M423" s="3" t="inlineStr"/>
@@ -26705,7 +26705,7 @@
       </c>
       <c r="L424" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M424" s="3" t="inlineStr"/>
@@ -26817,7 +26817,7 @@
       </c>
       <c r="L426" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M426" s="3" t="inlineStr"/>
@@ -26873,7 +26873,7 @@
       </c>
       <c r="L427" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M427" s="3" t="inlineStr"/>
@@ -26929,7 +26929,7 @@
       </c>
       <c r="L428" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M428" s="3" t="inlineStr"/>
@@ -26985,7 +26985,7 @@
       </c>
       <c r="L429" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M429" s="3" t="inlineStr"/>
@@ -27041,7 +27041,7 @@
       </c>
       <c r="L430" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M430" s="3" t="inlineStr"/>
@@ -27101,7 +27101,7 @@
       </c>
       <c r="L431" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M431" s="3" t="inlineStr"/>
@@ -27161,7 +27161,7 @@
       </c>
       <c r="L432" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M432" s="3" t="inlineStr"/>
@@ -27397,7 +27397,7 @@
       </c>
       <c r="L436" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M436" s="3" t="inlineStr"/>
@@ -27453,7 +27453,7 @@
       </c>
       <c r="L437" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M437" s="3" t="inlineStr"/>
@@ -27509,7 +27509,7 @@
       </c>
       <c r="L438" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M438" s="3" t="inlineStr"/>
@@ -27565,7 +27565,7 @@
       </c>
       <c r="L439" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M439" s="3" t="inlineStr"/>
@@ -27681,7 +27681,7 @@
       </c>
       <c r="L441" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M441" s="3" t="inlineStr"/>

</xml_diff>

<commit_message>
Ma'lumot avtomatik yangilandi (2026-10-26)
</commit_message>
<xml_diff>
--- a/docs/banklar_kreditlar.xlsx
+++ b/docs/banklar_kreditlar.xlsx
@@ -2223,7 +2223,7 @@
       </c>
       <c r="L3" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M3" s="3" t="inlineStr"/>
@@ -2283,7 +2283,7 @@
       </c>
       <c r="L4" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M4" s="3" t="inlineStr"/>
@@ -2343,7 +2343,7 @@
       </c>
       <c r="L5" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M5" s="3" t="inlineStr"/>
@@ -2403,7 +2403,7 @@
       </c>
       <c r="L6" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M6" s="3" t="inlineStr"/>
@@ -2463,7 +2463,7 @@
       </c>
       <c r="L7" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M7" s="3" t="inlineStr"/>
@@ -2523,7 +2523,7 @@
       </c>
       <c r="L8" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M8" s="3" t="inlineStr"/>
@@ -2639,7 +2639,7 @@
       </c>
       <c r="L10" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M10" s="3" t="inlineStr"/>
@@ -2699,7 +2699,7 @@
       </c>
       <c r="L11" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M11" s="3" t="inlineStr"/>
@@ -2815,7 +2815,7 @@
       </c>
       <c r="L13" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M13" s="3" t="inlineStr"/>
@@ -2875,7 +2875,7 @@
       </c>
       <c r="L14" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M14" s="3" t="inlineStr"/>
@@ -2935,7 +2935,7 @@
       </c>
       <c r="L15" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M15" s="3" t="inlineStr"/>
@@ -3047,7 +3047,7 @@
       </c>
       <c r="L17" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M17" s="3" t="inlineStr"/>
@@ -3107,7 +3107,7 @@
       </c>
       <c r="L18" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M18" s="3" t="inlineStr"/>
@@ -3223,7 +3223,7 @@
       </c>
       <c r="L20" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M20" s="3" t="inlineStr"/>
@@ -3283,7 +3283,7 @@
       </c>
       <c r="L21" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M21" s="3" t="inlineStr"/>
@@ -3343,7 +3343,7 @@
       </c>
       <c r="L22" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M22" s="3" t="inlineStr"/>
@@ -3403,7 +3403,7 @@
       </c>
       <c r="L23" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M23" s="3" t="inlineStr"/>
@@ -3463,7 +3463,7 @@
       </c>
       <c r="L24" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M24" s="3" t="inlineStr"/>
@@ -3631,7 +3631,7 @@
       </c>
       <c r="L27" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M27" s="3" t="inlineStr"/>
@@ -3691,7 +3691,7 @@
       </c>
       <c r="L28" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M28" s="3" t="inlineStr"/>
@@ -3751,7 +3751,7 @@
       </c>
       <c r="L29" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M29" s="3" t="inlineStr"/>
@@ -3811,7 +3811,7 @@
       </c>
       <c r="L30" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M30" s="3" t="inlineStr"/>
@@ -3871,7 +3871,7 @@
       </c>
       <c r="L31" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M31" s="3" t="inlineStr"/>
@@ -3931,7 +3931,7 @@
       </c>
       <c r="L32" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M32" s="3" t="inlineStr"/>
@@ -3991,7 +3991,7 @@
       </c>
       <c r="L33" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M33" s="3" t="inlineStr"/>
@@ -4051,7 +4051,7 @@
       </c>
       <c r="L34" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M34" s="3" t="inlineStr"/>
@@ -4111,7 +4111,7 @@
       </c>
       <c r="L35" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M35" s="3" t="inlineStr"/>
@@ -4171,7 +4171,7 @@
       </c>
       <c r="L36" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M36" s="3" t="inlineStr"/>
@@ -4227,7 +4227,7 @@
       </c>
       <c r="L37" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M37" s="3" t="inlineStr"/>
@@ -4339,7 +4339,7 @@
       </c>
       <c r="L39" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M39" s="3" t="inlineStr"/>
@@ -4395,7 +4395,7 @@
       </c>
       <c r="L40" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M40" s="3" t="inlineStr"/>
@@ -4451,7 +4451,7 @@
       </c>
       <c r="L41" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M41" s="3" t="inlineStr"/>
@@ -4507,7 +4507,7 @@
       </c>
       <c r="L42" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M42" s="3" t="inlineStr"/>
@@ -4567,7 +4567,7 @@
       </c>
       <c r="L43" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M43" s="3" t="inlineStr"/>
@@ -4627,7 +4627,7 @@
       </c>
       <c r="L44" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M44" s="3" t="inlineStr"/>
@@ -4687,7 +4687,7 @@
       </c>
       <c r="L45" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M45" s="3" t="inlineStr"/>
@@ -4743,7 +4743,7 @@
       </c>
       <c r="L46" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M46" s="3" t="inlineStr"/>
@@ -4799,7 +4799,7 @@
       </c>
       <c r="L47" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M47" s="3" t="inlineStr"/>
@@ -4859,7 +4859,7 @@
       </c>
       <c r="L48" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M48" s="3" t="inlineStr"/>
@@ -4919,7 +4919,7 @@
       </c>
       <c r="L49" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M49" s="3" t="inlineStr"/>
@@ -4979,7 +4979,7 @@
       </c>
       <c r="L50" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M50" s="3" t="inlineStr"/>
@@ -5093,7 +5093,7 @@
       </c>
       <c r="L52" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M52" s="3" t="inlineStr"/>
@@ -5153,7 +5153,7 @@
       </c>
       <c r="L53" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M53" s="3" t="inlineStr"/>
@@ -5213,7 +5213,7 @@
       </c>
       <c r="L54" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M54" s="3" t="inlineStr"/>
@@ -5273,7 +5273,7 @@
       </c>
       <c r="L55" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M55" s="3" t="inlineStr"/>
@@ -5333,7 +5333,7 @@
       </c>
       <c r="L56" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M56" s="3" t="inlineStr"/>
@@ -5445,7 +5445,7 @@
       </c>
       <c r="L58" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M58" s="3" t="inlineStr"/>
@@ -5501,7 +5501,7 @@
       </c>
       <c r="L59" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M59" s="3" t="inlineStr"/>
@@ -6257,7 +6257,7 @@
       </c>
       <c r="L72" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M72" s="3" t="inlineStr"/>
@@ -6369,7 +6369,7 @@
       </c>
       <c r="L74" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M74" s="3" t="inlineStr"/>
@@ -6481,7 +6481,7 @@
       </c>
       <c r="L76" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M76" s="3" t="inlineStr"/>
@@ -6537,7 +6537,7 @@
       </c>
       <c r="L77" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M77" s="3" t="inlineStr"/>
@@ -6593,7 +6593,7 @@
       </c>
       <c r="L78" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M78" s="3" t="inlineStr"/>
@@ -6649,7 +6649,7 @@
       </c>
       <c r="L79" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M79" s="3" t="inlineStr"/>
@@ -6705,7 +6705,7 @@
       </c>
       <c r="L80" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M80" s="3" t="inlineStr"/>
@@ -6761,7 +6761,7 @@
       </c>
       <c r="L81" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M81" s="3" t="inlineStr"/>
@@ -6817,7 +6817,7 @@
       </c>
       <c r="L82" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M82" s="3" t="inlineStr"/>
@@ -6869,7 +6869,7 @@
       </c>
       <c r="L83" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M83" s="3" t="inlineStr"/>
@@ -6929,7 +6929,7 @@
       </c>
       <c r="L84" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M84" s="3" t="inlineStr"/>
@@ -6989,7 +6989,7 @@
       </c>
       <c r="L85" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M85" s="3" t="inlineStr"/>
@@ -7049,7 +7049,7 @@
       </c>
       <c r="L86" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M86" s="3" t="inlineStr"/>
@@ -7109,7 +7109,7 @@
       </c>
       <c r="L87" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M87" s="3" t="inlineStr"/>
@@ -7169,7 +7169,7 @@
       </c>
       <c r="L88" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M88" s="3" t="inlineStr"/>
@@ -7225,7 +7225,7 @@
       </c>
       <c r="L89" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M89" s="3" t="inlineStr"/>
@@ -7277,7 +7277,7 @@
       </c>
       <c r="L90" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M90" s="3" t="inlineStr"/>
@@ -7389,7 +7389,7 @@
       </c>
       <c r="L92" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M92" s="3" t="inlineStr"/>
@@ -7445,7 +7445,7 @@
       </c>
       <c r="L93" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M93" s="3" t="inlineStr"/>
@@ -7505,7 +7505,7 @@
       </c>
       <c r="L94" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M94" s="3" t="inlineStr"/>
@@ -7565,7 +7565,7 @@
       </c>
       <c r="L95" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M95" s="3" t="inlineStr"/>
@@ -7625,7 +7625,7 @@
       </c>
       <c r="L96" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M96" s="3" t="inlineStr"/>
@@ -7685,7 +7685,7 @@
       </c>
       <c r="L97" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M97" s="3" t="inlineStr"/>
@@ -7745,7 +7745,7 @@
       </c>
       <c r="L98" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M98" s="3" t="inlineStr"/>
@@ -7805,7 +7805,7 @@
       </c>
       <c r="L99" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M99" s="3" t="inlineStr"/>
@@ -7865,7 +7865,7 @@
       </c>
       <c r="L100" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M100" s="3" t="inlineStr"/>
@@ -7925,7 +7925,7 @@
       </c>
       <c r="L101" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M101" s="3" t="inlineStr"/>
@@ -7985,7 +7985,7 @@
       </c>
       <c r="L102" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M102" s="3" t="inlineStr"/>
@@ -8105,7 +8105,7 @@
       </c>
       <c r="L104" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M104" s="3" t="inlineStr"/>
@@ -8165,7 +8165,7 @@
       </c>
       <c r="L105" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M105" s="3" t="inlineStr"/>
@@ -8225,7 +8225,7 @@
       </c>
       <c r="L106" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M106" s="3" t="inlineStr"/>
@@ -8285,7 +8285,7 @@
       </c>
       <c r="L107" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M107" s="3" t="inlineStr"/>
@@ -8345,7 +8345,7 @@
       </c>
       <c r="L108" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M108" s="3" t="inlineStr"/>
@@ -8461,7 +8461,7 @@
       </c>
       <c r="L110" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M110" s="3" t="inlineStr"/>
@@ -8521,7 +8521,7 @@
       </c>
       <c r="L111" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M111" s="3" t="inlineStr"/>
@@ -8581,7 +8581,7 @@
       </c>
       <c r="L112" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M112" s="3" t="inlineStr"/>
@@ -8641,7 +8641,7 @@
       </c>
       <c r="L113" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M113" s="3" t="inlineStr"/>
@@ -8701,7 +8701,7 @@
       </c>
       <c r="L114" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M114" s="3" t="inlineStr"/>
@@ -8757,7 +8757,7 @@
       </c>
       <c r="L115" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M115" s="3" t="inlineStr"/>
@@ -8817,7 +8817,7 @@
       </c>
       <c r="L116" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M116" s="3" t="inlineStr"/>
@@ -8877,7 +8877,7 @@
       </c>
       <c r="L117" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M117" s="3" t="inlineStr"/>
@@ -8933,7 +8933,7 @@
       </c>
       <c r="L118" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M118" s="3" t="inlineStr"/>
@@ -8993,7 +8993,7 @@
       </c>
       <c r="L119" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M119" s="3" t="inlineStr"/>
@@ -9049,7 +9049,7 @@
       </c>
       <c r="L120" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M120" s="3" t="inlineStr"/>
@@ -9105,7 +9105,7 @@
       </c>
       <c r="L121" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M121" s="3" t="inlineStr"/>
@@ -9165,7 +9165,7 @@
       </c>
       <c r="L122" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M122" s="3" t="inlineStr"/>
@@ -9225,7 +9225,7 @@
       </c>
       <c r="L123" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M123" s="3" t="inlineStr"/>
@@ -9285,7 +9285,7 @@
       </c>
       <c r="L124" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M124" s="3" t="inlineStr"/>
@@ -9345,7 +9345,7 @@
       </c>
       <c r="L125" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M125" s="3" t="inlineStr"/>
@@ -9405,7 +9405,7 @@
       </c>
       <c r="L126" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M126" s="3" t="inlineStr"/>
@@ -9465,7 +9465,7 @@
       </c>
       <c r="L127" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M127" s="3" t="inlineStr"/>
@@ -9525,7 +9525,7 @@
       </c>
       <c r="L128" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M128" s="3" t="inlineStr"/>
@@ -9585,7 +9585,7 @@
       </c>
       <c r="L129" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M129" s="3" t="inlineStr"/>
@@ -9645,7 +9645,7 @@
       </c>
       <c r="L130" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M130" s="3" t="inlineStr"/>
@@ -9705,7 +9705,7 @@
       </c>
       <c r="L131" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M131" s="3" t="inlineStr"/>
@@ -9765,7 +9765,7 @@
       </c>
       <c r="L132" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M132" s="3" t="inlineStr"/>
@@ -9825,7 +9825,7 @@
       </c>
       <c r="L133" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M133" s="3" t="inlineStr"/>
@@ -9885,7 +9885,7 @@
       </c>
       <c r="L134" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M134" s="3" t="inlineStr"/>
@@ -9945,7 +9945,7 @@
       </c>
       <c r="L135" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M135" s="3" t="inlineStr"/>
@@ -10005,7 +10005,7 @@
       </c>
       <c r="L136" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M136" s="3" t="inlineStr"/>
@@ -10237,7 +10237,7 @@
       </c>
       <c r="L140" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M140" s="3" t="inlineStr"/>
@@ -10297,7 +10297,7 @@
       </c>
       <c r="L141" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M141" s="3" t="inlineStr"/>
@@ -10357,7 +10357,7 @@
       </c>
       <c r="L142" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M142" s="3" t="inlineStr"/>
@@ -10417,7 +10417,7 @@
       </c>
       <c r="L143" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M143" s="3" t="inlineStr"/>
@@ -10585,7 +10585,7 @@
       </c>
       <c r="L146" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M146" s="3" t="inlineStr"/>
@@ -10873,7 +10873,7 @@
       </c>
       <c r="L151" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M151" s="3" t="inlineStr"/>
@@ -10993,7 +10993,7 @@
       </c>
       <c r="L153" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M153" s="3" t="inlineStr"/>
@@ -11257,7 +11257,7 @@
       </c>
       <c r="L158" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M158" s="3" t="inlineStr"/>
@@ -11373,7 +11373,7 @@
       </c>
       <c r="L160" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M160" s="3" t="inlineStr"/>
@@ -11433,7 +11433,7 @@
       </c>
       <c r="L161" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M161" s="3" t="inlineStr"/>
@@ -11493,7 +11493,7 @@
       </c>
       <c r="L162" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M162" s="3" t="inlineStr"/>
@@ -11663,7 +11663,7 @@
       </c>
       <c r="L165" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M165" s="3" t="inlineStr"/>
@@ -11719,7 +11719,7 @@
       </c>
       <c r="L166" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M166" s="3" t="inlineStr"/>
@@ -11779,7 +11779,7 @@
       </c>
       <c r="L167" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M167" s="3" t="inlineStr"/>
@@ -11839,7 +11839,7 @@
       </c>
       <c r="L168" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M168" s="3" t="inlineStr"/>
@@ -11949,7 +11949,7 @@
       </c>
       <c r="L170" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M170" s="3" t="inlineStr"/>
@@ -12009,7 +12009,7 @@
       </c>
       <c r="L171" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M171" s="3" t="inlineStr"/>
@@ -12065,7 +12065,7 @@
       </c>
       <c r="L172" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M172" s="3" t="inlineStr"/>
@@ -12125,7 +12125,7 @@
       </c>
       <c r="L173" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M173" s="3" t="inlineStr"/>
@@ -12305,7 +12305,7 @@
       </c>
       <c r="L176" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M176" s="3" t="inlineStr"/>
@@ -12365,7 +12365,7 @@
       </c>
       <c r="L177" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M177" s="3" t="inlineStr"/>
@@ -12481,7 +12481,7 @@
       </c>
       <c r="L179" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M179" s="3" t="inlineStr"/>
@@ -12541,7 +12541,7 @@
       </c>
       <c r="L180" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M180" s="3" t="inlineStr"/>
@@ -12597,7 +12597,7 @@
       </c>
       <c r="L181" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M181" s="3" t="inlineStr"/>
@@ -12657,7 +12657,7 @@
       </c>
       <c r="L182" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M182" s="3" t="inlineStr"/>
@@ -12717,7 +12717,7 @@
       </c>
       <c r="L183" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M183" s="3" t="inlineStr"/>
@@ -12773,7 +12773,7 @@
       </c>
       <c r="L184" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M184" s="3" t="inlineStr"/>
@@ -12829,7 +12829,7 @@
       </c>
       <c r="L185" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M185" s="3" t="inlineStr"/>
@@ -12881,7 +12881,7 @@
       </c>
       <c r="L186" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M186" s="3" t="inlineStr"/>
@@ -13053,7 +13053,7 @@
       </c>
       <c r="L189" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M189" s="3" t="inlineStr"/>
@@ -13109,7 +13109,7 @@
       </c>
       <c r="L190" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M190" s="3" t="inlineStr"/>
@@ -13165,7 +13165,7 @@
       </c>
       <c r="L191" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M191" s="3" t="inlineStr"/>
@@ -13221,7 +13221,7 @@
       </c>
       <c r="L192" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M192" s="3" t="inlineStr"/>
@@ -13281,7 +13281,7 @@
       </c>
       <c r="L193" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M193" s="3" t="inlineStr"/>
@@ -13401,7 +13401,7 @@
       </c>
       <c r="L195" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M195" s="3" t="inlineStr"/>
@@ -13517,7 +13517,7 @@
       </c>
       <c r="L197" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M197" s="3" t="inlineStr"/>
@@ -13577,7 +13577,7 @@
       </c>
       <c r="L198" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M198" s="3" t="inlineStr"/>
@@ -13637,7 +13637,7 @@
       </c>
       <c r="L199" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M199" s="3" t="inlineStr"/>
@@ -13757,7 +13757,7 @@
       </c>
       <c r="L201" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M201" s="3" t="inlineStr"/>
@@ -13817,7 +13817,7 @@
       </c>
       <c r="L202" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M202" s="3" t="inlineStr"/>
@@ -13877,7 +13877,7 @@
       </c>
       <c r="L203" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M203" s="3" t="inlineStr"/>
@@ -13937,7 +13937,7 @@
       </c>
       <c r="L204" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M204" s="3" t="inlineStr"/>
@@ -13997,7 +13997,7 @@
       </c>
       <c r="L205" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M205" s="3" t="inlineStr"/>
@@ -14057,7 +14057,7 @@
       </c>
       <c r="L206" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M206" s="3" t="inlineStr"/>
@@ -14117,7 +14117,7 @@
       </c>
       <c r="L207" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M207" s="3" t="inlineStr"/>
@@ -14241,7 +14241,7 @@
       </c>
       <c r="L209" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M209" s="3" t="inlineStr"/>
@@ -14359,7 +14359,7 @@
       </c>
       <c r="L211" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M211" s="3" t="inlineStr"/>
@@ -14533,7 +14533,7 @@
       </c>
       <c r="L214" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M214" s="3" t="inlineStr"/>
@@ -14585,7 +14585,7 @@
       </c>
       <c r="L215" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M215" s="3" t="inlineStr"/>
@@ -14637,7 +14637,7 @@
       </c>
       <c r="L216" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M216" s="3" t="inlineStr"/>
@@ -14747,7 +14747,7 @@
       </c>
       <c r="L218" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M218" s="3" t="inlineStr"/>
@@ -14807,7 +14807,7 @@
       </c>
       <c r="L219" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M219" s="3" t="inlineStr"/>
@@ -14975,7 +14975,7 @@
       </c>
       <c r="L222" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M222" s="3" t="inlineStr"/>
@@ -15379,7 +15379,7 @@
       </c>
       <c r="L229" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M229" s="3" t="inlineStr"/>
@@ -15439,7 +15439,7 @@
       </c>
       <c r="L230" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M230" s="3" t="inlineStr"/>
@@ -15499,7 +15499,7 @@
       </c>
       <c r="L231" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M231" s="3" t="inlineStr"/>
@@ -15619,7 +15619,7 @@
       </c>
       <c r="L233" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M233" s="3" t="inlineStr"/>
@@ -15679,7 +15679,7 @@
       </c>
       <c r="L234" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M234" s="3" t="inlineStr"/>
@@ -15739,7 +15739,7 @@
       </c>
       <c r="L235" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M235" s="3" t="inlineStr"/>
@@ -15795,7 +15795,7 @@
       </c>
       <c r="L236" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M236" s="3" t="inlineStr"/>
@@ -16019,7 +16019,7 @@
       </c>
       <c r="L240" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M240" s="3" t="inlineStr"/>
@@ -16131,7 +16131,7 @@
       </c>
       <c r="L242" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M242" s="3" t="inlineStr"/>
@@ -16187,7 +16187,7 @@
       </c>
       <c r="L243" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M243" s="3" t="inlineStr"/>
@@ -16247,7 +16247,7 @@
       </c>
       <c r="L244" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M244" s="3" t="inlineStr"/>
@@ -16361,7 +16361,7 @@
       </c>
       <c r="L246" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M246" s="3" t="inlineStr"/>
@@ -16417,7 +16417,7 @@
       </c>
       <c r="L247" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M247" s="3" t="inlineStr"/>
@@ -16477,7 +16477,7 @@
       </c>
       <c r="L248" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M248" s="3" t="inlineStr"/>
@@ -16537,7 +16537,7 @@
       </c>
       <c r="L249" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M249" s="3" t="inlineStr"/>
@@ -16597,7 +16597,7 @@
       </c>
       <c r="L250" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M250" s="3" t="inlineStr"/>
@@ -16657,7 +16657,7 @@
       </c>
       <c r="L251" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M251" s="3" t="inlineStr"/>
@@ -16717,7 +16717,7 @@
       </c>
       <c r="L252" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M252" s="3" t="inlineStr"/>
@@ -16777,7 +16777,7 @@
       </c>
       <c r="L253" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M253" s="3" t="inlineStr"/>
@@ -16837,7 +16837,7 @@
       </c>
       <c r="L254" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M254" s="3" t="inlineStr"/>
@@ -16897,7 +16897,7 @@
       </c>
       <c r="L255" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M255" s="3" t="inlineStr"/>
@@ -16957,7 +16957,7 @@
       </c>
       <c r="L256" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M256" s="3" t="inlineStr"/>
@@ -17017,7 +17017,7 @@
       </c>
       <c r="L257" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M257" s="3" t="inlineStr"/>
@@ -17077,7 +17077,7 @@
       </c>
       <c r="L258" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M258" s="3" t="inlineStr"/>
@@ -17133,7 +17133,7 @@
       </c>
       <c r="L259" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M259" s="3" t="inlineStr"/>
@@ -17193,7 +17193,7 @@
       </c>
       <c r="L260" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M260" s="3" t="inlineStr"/>
@@ -17317,7 +17317,7 @@
       </c>
       <c r="L262" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M262" s="3" t="inlineStr"/>
@@ -17437,7 +17437,7 @@
       </c>
       <c r="L264" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M264" s="3" t="inlineStr"/>
@@ -17497,7 +17497,7 @@
       </c>
       <c r="L265" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M265" s="3" t="inlineStr"/>
@@ -17617,7 +17617,7 @@
       </c>
       <c r="L267" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M267" s="3" t="inlineStr"/>
@@ -17677,7 +17677,7 @@
       </c>
       <c r="L268" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M268" s="3" t="inlineStr"/>
@@ -17737,7 +17737,7 @@
       </c>
       <c r="L269" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M269" s="3" t="inlineStr"/>
@@ -17793,7 +17793,7 @@
       </c>
       <c r="L270" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M270" s="3" t="inlineStr"/>
@@ -17853,7 +17853,7 @@
       </c>
       <c r="L271" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M271" s="3" t="inlineStr"/>
@@ -18033,7 +18033,7 @@
       </c>
       <c r="L274" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M274" s="3" t="inlineStr"/>
@@ -18093,7 +18093,7 @@
       </c>
       <c r="L275" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M275" s="3" t="inlineStr"/>
@@ -18153,7 +18153,7 @@
       </c>
       <c r="L276" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M276" s="3" t="inlineStr"/>
@@ -18213,7 +18213,7 @@
       </c>
       <c r="L277" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M277" s="3" t="inlineStr"/>
@@ -18273,7 +18273,7 @@
       </c>
       <c r="L278" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M278" s="3" t="inlineStr"/>
@@ -18333,7 +18333,7 @@
       </c>
       <c r="L279" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M279" s="3" t="inlineStr"/>
@@ -18393,7 +18393,7 @@
       </c>
       <c r="L280" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M280" s="3" t="inlineStr"/>
@@ -18453,7 +18453,7 @@
       </c>
       <c r="L281" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M281" s="3" t="inlineStr"/>
@@ -18513,7 +18513,7 @@
       </c>
       <c r="L282" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M282" s="3" t="inlineStr"/>
@@ -18573,7 +18573,7 @@
       </c>
       <c r="L283" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M283" s="3" t="inlineStr"/>
@@ -18633,7 +18633,7 @@
       </c>
       <c r="L284" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M284" s="3" t="inlineStr"/>
@@ -18685,7 +18685,7 @@
       </c>
       <c r="L285" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M285" s="3" t="inlineStr"/>
@@ -18745,7 +18745,7 @@
       </c>
       <c r="L286" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M286" s="3" t="inlineStr"/>
@@ -18805,7 +18805,7 @@
       </c>
       <c r="L287" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M287" s="3" t="inlineStr"/>
@@ -18865,7 +18865,7 @@
       </c>
       <c r="L288" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M288" s="3" t="inlineStr"/>
@@ -18977,7 +18977,7 @@
       </c>
       <c r="L290" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M290" s="3" t="inlineStr"/>
@@ -19037,7 +19037,7 @@
       </c>
       <c r="L291" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M291" s="3" t="inlineStr"/>
@@ -19097,7 +19097,7 @@
       </c>
       <c r="L292" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M292" s="3" t="inlineStr"/>
@@ -19157,7 +19157,7 @@
       </c>
       <c r="L293" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M293" s="3" t="inlineStr"/>
@@ -19329,7 +19329,7 @@
       </c>
       <c r="L296" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M296" s="3" t="inlineStr"/>
@@ -19389,7 +19389,7 @@
       </c>
       <c r="L297" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M297" s="3" t="inlineStr"/>
@@ -19503,7 +19503,7 @@
       </c>
       <c r="L299" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M299" s="3" t="inlineStr"/>
@@ -19563,7 +19563,7 @@
       </c>
       <c r="L300" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M300" s="3" t="inlineStr"/>
@@ -19623,7 +19623,7 @@
       </c>
       <c r="L301" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M301" s="3" t="inlineStr"/>
@@ -19683,7 +19683,7 @@
       </c>
       <c r="L302" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M302" s="3" t="inlineStr"/>
@@ -19743,7 +19743,7 @@
       </c>
       <c r="L303" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M303" s="3" t="inlineStr"/>
@@ -19803,7 +19803,7 @@
       </c>
       <c r="L304" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M304" s="3" t="inlineStr"/>
@@ -19863,7 +19863,7 @@
       </c>
       <c r="L305" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M305" s="3" t="inlineStr"/>
@@ -19923,7 +19923,7 @@
       </c>
       <c r="L306" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M306" s="3" t="inlineStr"/>
@@ -19983,7 +19983,7 @@
       </c>
       <c r="L307" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M307" s="3" t="inlineStr"/>
@@ -20039,7 +20039,7 @@
       </c>
       <c r="L308" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M308" s="3" t="inlineStr"/>
@@ -20163,7 +20163,7 @@
       </c>
       <c r="L310" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M310" s="3" t="inlineStr"/>
@@ -20279,7 +20279,7 @@
       </c>
       <c r="L312" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M312" s="3" t="inlineStr"/>
@@ -20335,7 +20335,7 @@
       </c>
       <c r="L313" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M313" s="3" t="inlineStr"/>
@@ -20447,7 +20447,7 @@
       </c>
       <c r="L315" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M315" s="3" t="inlineStr"/>
@@ -20487,7 +20487,7 @@
       <c r="G316" s="3" t="inlineStr"/>
       <c r="H316" s="3" t="inlineStr">
         <is>
-          <t>2.2 oygacha</t>
+          <t>2.17 oygacha</t>
         </is>
       </c>
       <c r="I316" s="3" t="inlineStr"/>
@@ -20503,7 +20503,7 @@
       </c>
       <c r="L316" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M316" s="3" t="inlineStr"/>
@@ -20899,7 +20899,7 @@
       </c>
       <c r="L323" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M323" s="3" t="inlineStr"/>
@@ -20959,7 +20959,7 @@
       </c>
       <c r="L324" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M324" s="3" t="inlineStr"/>
@@ -21135,7 +21135,7 @@
       </c>
       <c r="L327" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M327" s="3" t="inlineStr"/>
@@ -21251,7 +21251,7 @@
       </c>
       <c r="L329" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M329" s="3" t="inlineStr"/>
@@ -21311,7 +21311,7 @@
       </c>
       <c r="L330" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M330" s="3" t="inlineStr"/>
@@ -21371,7 +21371,7 @@
       </c>
       <c r="L331" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M331" s="3" t="inlineStr"/>
@@ -21431,7 +21431,7 @@
       </c>
       <c r="L332" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M332" s="3" t="inlineStr"/>
@@ -21491,7 +21491,7 @@
       </c>
       <c r="L333" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M333" s="3" t="inlineStr"/>
@@ -21551,7 +21551,7 @@
       </c>
       <c r="L334" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M334" s="3" t="inlineStr"/>
@@ -21611,7 +21611,7 @@
       </c>
       <c r="L335" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M335" s="3" t="inlineStr"/>
@@ -21671,7 +21671,7 @@
       </c>
       <c r="L336" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M336" s="3" t="inlineStr"/>
@@ -21727,7 +21727,7 @@
       </c>
       <c r="L337" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M337" s="3" t="inlineStr"/>
@@ -21787,7 +21787,7 @@
       </c>
       <c r="L338" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M338" s="3" t="inlineStr"/>
@@ -21899,7 +21899,7 @@
       </c>
       <c r="L340" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M340" s="3" t="inlineStr"/>
@@ -21959,7 +21959,7 @@
       </c>
       <c r="L341" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M341" s="3" t="inlineStr"/>
@@ -22019,7 +22019,7 @@
       </c>
       <c r="L342" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M342" s="3" t="inlineStr"/>
@@ -22079,7 +22079,7 @@
       </c>
       <c r="L343" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M343" s="3" t="inlineStr"/>
@@ -22199,7 +22199,7 @@
       </c>
       <c r="L345" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M345" s="3" t="inlineStr"/>
@@ -22259,7 +22259,7 @@
       </c>
       <c r="L346" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M346" s="3" t="inlineStr"/>
@@ -22319,7 +22319,7 @@
       </c>
       <c r="L347" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M347" s="3" t="inlineStr"/>
@@ -22435,7 +22435,7 @@
       </c>
       <c r="L349" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M349" s="3" t="inlineStr"/>
@@ -22549,7 +22549,7 @@
       </c>
       <c r="L351" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M351" s="3" t="inlineStr"/>
@@ -22605,7 +22605,7 @@
       </c>
       <c r="L352" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M352" s="3" t="inlineStr"/>
@@ -22717,7 +22717,7 @@
       </c>
       <c r="L354" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M354" s="3" t="inlineStr"/>
@@ -22773,7 +22773,7 @@
       </c>
       <c r="L355" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M355" s="3" t="inlineStr"/>
@@ -22829,7 +22829,7 @@
       </c>
       <c r="L356" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M356" s="3" t="inlineStr"/>
@@ -22941,7 +22941,7 @@
       </c>
       <c r="L358" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M358" s="3" t="inlineStr"/>
@@ -23053,7 +23053,7 @@
       </c>
       <c r="L360" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M360" s="3" t="inlineStr"/>
@@ -23169,7 +23169,7 @@
       </c>
       <c r="L362" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M362" s="3" t="inlineStr"/>
@@ -23225,7 +23225,7 @@
       </c>
       <c r="L363" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M363" s="3" t="inlineStr"/>
@@ -23281,7 +23281,7 @@
       </c>
       <c r="L364" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M364" s="3" t="inlineStr"/>
@@ -23337,7 +23337,7 @@
       </c>
       <c r="L365" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M365" s="3" t="inlineStr"/>
@@ -23393,7 +23393,7 @@
       </c>
       <c r="L366" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M366" s="3" t="inlineStr"/>
@@ -23449,7 +23449,7 @@
       </c>
       <c r="L367" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M367" s="3" t="inlineStr"/>
@@ -23505,7 +23505,7 @@
       </c>
       <c r="L368" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M368" s="3" t="inlineStr"/>
@@ -23561,7 +23561,7 @@
       </c>
       <c r="L369" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M369" s="3" t="inlineStr"/>
@@ -23617,7 +23617,7 @@
       </c>
       <c r="L370" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M370" s="3" t="inlineStr"/>
@@ -23673,7 +23673,7 @@
       </c>
       <c r="L371" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M371" s="3" t="inlineStr"/>
@@ -23729,7 +23729,7 @@
       </c>
       <c r="L372" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M372" s="3" t="inlineStr"/>
@@ -23785,7 +23785,7 @@
       </c>
       <c r="L373" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M373" s="3" t="inlineStr"/>
@@ -23841,7 +23841,7 @@
       </c>
       <c r="L374" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M374" s="3" t="inlineStr"/>
@@ -23901,7 +23901,7 @@
       </c>
       <c r="L375" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M375" s="3" t="inlineStr"/>
@@ -23961,7 +23961,7 @@
       </c>
       <c r="L376" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M376" s="3" t="inlineStr"/>
@@ -24021,7 +24021,7 @@
       </c>
       <c r="L377" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M377" s="3" t="inlineStr"/>
@@ -24073,7 +24073,7 @@
       </c>
       <c r="L378" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M378" s="3" t="inlineStr"/>
@@ -24293,7 +24293,7 @@
       </c>
       <c r="L382" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M382" s="3" t="inlineStr"/>
@@ -24349,7 +24349,7 @@
       </c>
       <c r="L383" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M383" s="3" t="inlineStr"/>
@@ -24405,7 +24405,7 @@
       </c>
       <c r="L384" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M384" s="3" t="inlineStr"/>
@@ -24525,7 +24525,7 @@
       </c>
       <c r="L386" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M386" s="3" t="inlineStr"/>
@@ -24581,7 +24581,7 @@
       </c>
       <c r="L387" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M387" s="3" t="inlineStr"/>
@@ -24813,7 +24813,7 @@
       </c>
       <c r="L391" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M391" s="3" t="inlineStr"/>
@@ -24869,7 +24869,7 @@
       </c>
       <c r="L392" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M392" s="3" t="inlineStr"/>
@@ -24929,7 +24929,7 @@
       </c>
       <c r="L393" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M393" s="3" t="inlineStr"/>
@@ -25041,7 +25041,7 @@
       </c>
       <c r="L395" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M395" s="3" t="inlineStr"/>
@@ -25097,7 +25097,7 @@
       </c>
       <c r="L396" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M396" s="3" t="inlineStr"/>
@@ -25153,7 +25153,7 @@
       </c>
       <c r="L397" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M397" s="3" t="inlineStr"/>
@@ -25209,7 +25209,7 @@
       </c>
       <c r="L398" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M398" s="3" t="inlineStr"/>
@@ -25265,7 +25265,7 @@
       </c>
       <c r="L399" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M399" s="3" t="inlineStr"/>
@@ -25321,7 +25321,7 @@
       </c>
       <c r="L400" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M400" s="3" t="inlineStr"/>
@@ -25377,7 +25377,7 @@
       </c>
       <c r="L401" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M401" s="3" t="inlineStr"/>
@@ -25485,7 +25485,7 @@
       </c>
       <c r="L403" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M403" s="3" t="inlineStr"/>
@@ -25545,7 +25545,7 @@
       </c>
       <c r="L404" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M404" s="3" t="inlineStr"/>
@@ -25605,7 +25605,7 @@
       </c>
       <c r="L405" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M405" s="3" t="inlineStr"/>
@@ -25721,7 +25721,7 @@
       </c>
       <c r="L407" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M407" s="3" t="inlineStr"/>
@@ -25889,7 +25889,7 @@
       </c>
       <c r="L410" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M410" s="3" t="inlineStr"/>
@@ -25949,7 +25949,7 @@
       </c>
       <c r="L411" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M411" s="3" t="inlineStr"/>
@@ -26009,7 +26009,7 @@
       </c>
       <c r="L412" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M412" s="3" t="inlineStr"/>
@@ -26069,7 +26069,7 @@
       </c>
       <c r="L413" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M413" s="3" t="inlineStr"/>
@@ -26405,7 +26405,7 @@
       </c>
       <c r="L419" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M419" s="3" t="inlineStr"/>
@@ -26465,7 +26465,7 @@
       </c>
       <c r="L420" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M420" s="3" t="inlineStr"/>
@@ -26525,7 +26525,7 @@
       </c>
       <c r="L421" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M421" s="3" t="inlineStr"/>
@@ -26585,7 +26585,7 @@
       </c>
       <c r="L422" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M422" s="3" t="inlineStr"/>
@@ -26641,7 +26641,7 @@
       </c>
       <c r="L423" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M423" s="3" t="inlineStr"/>
@@ -26881,7 +26881,7 @@
       </c>
       <c r="L427" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M427" s="3" t="inlineStr"/>
@@ -26941,7 +26941,7 @@
       </c>
       <c r="L428" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M428" s="3" t="inlineStr"/>
@@ -27053,7 +27053,7 @@
       </c>
       <c r="L430" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M430" s="3" t="inlineStr"/>
@@ -27109,7 +27109,7 @@
       </c>
       <c r="L431" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M431" s="3" t="inlineStr"/>
@@ -27165,7 +27165,7 @@
       </c>
       <c r="L432" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M432" s="3" t="inlineStr"/>
@@ -27221,7 +27221,7 @@
       </c>
       <c r="L433" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M433" s="3" t="inlineStr"/>
@@ -27277,7 +27277,7 @@
       </c>
       <c r="L434" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M434" s="3" t="inlineStr"/>
@@ -27337,7 +27337,7 @@
       </c>
       <c r="L435" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M435" s="3" t="inlineStr"/>
@@ -27397,7 +27397,7 @@
       </c>
       <c r="L436" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M436" s="3" t="inlineStr"/>
@@ -27633,7 +27633,7 @@
       </c>
       <c r="L440" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M440" s="3" t="inlineStr"/>
@@ -27689,7 +27689,7 @@
       </c>
       <c r="L441" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M441" s="3" t="inlineStr"/>
@@ -27745,7 +27745,7 @@
       </c>
       <c r="L442" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M442" s="3" t="inlineStr"/>
@@ -27801,7 +27801,7 @@
       </c>
       <c r="L443" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M443" s="3" t="inlineStr"/>
@@ -27917,7 +27917,7 @@
       </c>
       <c r="L445" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M445" s="3" t="inlineStr"/>

</xml_diff>